<commit_message>
Pooja and main door to the east side; kitchen entered from the north
- Master back to 9'-6" x 14'; Bedroom 2 15 x 14'-6"; sitting area
  24 x 7'-6" (takes the old pooja bay); dining 11 ft wide, now holding
  the plot centre.
- Pooja (4 x 4 ft, opens west) on the living's east wall, just south of
  the main door, which moves to the north end of the east face.
  Verandah steps, pillars, swing and seat realigned to the door.
- Corner below the pooja joins the kitchen as a fridge corner; kitchen
  entry is now a 3 ft sliding door from the living on the north; the
  dining-side door is closed and the south counter runs full length.
- TV taken off the plan; its wall is logged as an open issue.
- Room label offsets for crowded rooms.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Schedules/KH-P1_Schedules_RevB.xlsx
+++ b/03_Schedules/KH-P1_Schedules_RevB.xlsx
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E8" s="4" t="n">
         <v>24</v>
@@ -919,7 +919,7 @@
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>23.4</v>
+        <v>21.4</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>22.4</v>
@@ -943,7 +943,7 @@
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>27.8</v>
+        <v>25.8</v>
       </c>
       <c r="E10" s="4" t="n">
         <v>20.3</v>
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>28.1</v>
+        <v>26.1</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>24</v>
@@ -995,7 +995,7 @@
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>24.2</v>
@@ -1023,7 +1023,7 @@
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>25.3</v>
+        <v>23.3</v>
       </c>
       <c r="E13" s="4" t="n">
         <v>20.6</v>
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="D26" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E26" s="4" t="n">
         <v>26.6</v>
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="D31" s="4" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>26</v>
@@ -2549,7 +2549,7 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Fridge at the kitchen's west end, by the wet-area door, well away from the hob.</t>
+          <t>Fridge in its own corner below the pooja, beside the north entry and well away from the hob; nothing blocks the counter.</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -2572,7 +2572,7 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>The kitchen door faces the dining directly: a 3 ft sliding glass door, open when serving, closed when frying.</t>
+          <t>The kitchen is entered from the living on the north through a 3 ft sliding glass door, open when serving, closed when frying; the fridge corner sits beside it.</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -2710,7 +2710,7 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Here the pooja opens west onto the basin nook and hall, so the family sits facing east; idols are on its east wall. It shares a wall with the open wet area (not a toilet): that wall carries no pipes, and the pooja floor is 3 in higher.</t>
+          <t>Here the pooja sits on the living's east wall, just south of the main door (no toilet on any side). It opens west into the living, idols on its east wall, so the family faces east; the floor is 3 in higher.</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -4158,7 +4158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4201,17 +4201,17 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Land</t>
+          <t>Layout</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Agricultural land: confirm conversion to non-agricultural use with the gram panchayat / collector (AP repealed the NALA Act in 2025; new process to be confirmed)</t>
+          <t>TV wall to be decided: the main door now takes the north end of the east wall, so the TV (50-55 in, with data and 2 sockets) needs a new wall</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Owner / surveyor</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
@@ -4231,12 +4231,12 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Building permission route (panchayat vs DTCP / APCRDA via APDPMS) and setbacks under AP Building Rules 2017</t>
+          <t>Agricultural land: confirm conversion to non-agricultural use with the gram panchayat / collector (AP repealed the NALA Act in 2025; new process to be confirmed)</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Owner / surveyor</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
@@ -4256,7 +4256,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Plot 27 ft x 70 ft: north wall is 2 ft from the plot line and eaves overhang the owned north strip; septic and soak pit sit in the strip</t>
+          <t>Building permission route (panchayat vs DTCP / APCRDA via APDPMS) and setbacks under AP Building Rules 2017</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -4276,17 +4276,17 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Soil</t>
+          <t>Land</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Soil test (bore holes to 3 m min): black cotton soil is common in Guntur. Foundation type (isolated footings below active zone, under-reamed piles, or soil replacement) depends on it</t>
+          <t>Plot 27 ft x 75 ft (length to confirm by survey): north wall is 2 ft from the plot line and eaves overhang the owned north strip; septic and soak pit sit in the strip</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Structural engineer</t>
+          <t>Architect</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -4301,12 +4301,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>Soil</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>RCC frame with AAC infill: columns, plinth beam, lintel band, ring beam; steel truss with cyclone tie-downs</t>
+          <t>Soil test (bore holes to 3 m min): black cotton soil is common in Guntur. Foundation type (isolated footings below active zone, under-reamed piles, or soil replacement) depends on it</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -4326,17 +4326,17 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Structure</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Wet area is open to the walkway: lockable steel/WPC kitchen-to-wet-area door, compound wall and gate at the back; optional MS grille shutter across the wet area opening</t>
+          <t>RCC frame with AAC infill: columns, plinth beam, lintel band, ring beam; steel truss with cyclone tie-downs</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Owner / architect</t>
+          <t>Structural engineer</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -4351,17 +4351,17 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Services</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Groundwater: test TDS, hardness, fluoride. Plan RO for drinking and a softener for bathrooms if hardness is high</t>
+          <t>Wet area is open to the walkway: lockable steel/WPC kitchen-to-wet-area door, compound wall and gate at the back; optional MS grille shutter across the wet area opening</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Plumber / owner</t>
+          <t>Owner / architect</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -4381,12 +4381,12 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Septic and soak pit sizes; keep soak pits and gardens 6 ft+ from foundations in expansive soil</t>
+          <t>Groundwater: test TDS, hardness, fluoride. Plan RO for drinking and a softener for bathrooms if hardness is high</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Plumber / owner</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -4406,12 +4406,12 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Electrical load (with ACs), service connection size, earthing, inverter / solar PV</t>
+          <t>Septic and soak pit sizes; keep soak pits and gardens 6 ft+ from foundations in expansive soil</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Electrical engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -4426,22 +4426,22 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Services</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Phase 2 on the north strip will block north light and sits on the septic: plan the split now</t>
+          <t>Electrical load (with ACs), service connection size, earthing, inverter / solar PV</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Electrical engineer</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Deferred by owner</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -4451,22 +4451,22 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Vastu</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Bed head east (master), NW ensuite, Bedroom 2's attached bath north-west of centre on the outer wall (no common toilet), central dining, pooja south of centre opening west (devotees face east), beside the open wet area with a dry shared wall, DB in SE-ish living wall</t>
+          <t>Phase 2 on the north strip will block north light and sits on the septic: plan the split now</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Vastu consultant</t>
+          <t>Architect</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>To confirm</t>
+          <t>Deferred by owner</t>
         </is>
       </c>
     </row>
@@ -4476,22 +4476,22 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Climate</t>
+          <t>Vastu</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Roof heat: insulation, ventilated attic, ventilator lantern louvres and shutters; ODU positions on shaded walls</t>
+          <t>Bed head east (master), NW ensuite, Bedroom 2's attached bath north-west of centre on the outer wall (no common toilet), dining at the plot centre, pooja on the living's east wall just south of the main door, opening west (devotees face east), DB on the living's south wall</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Vastu consultant</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -4501,20 +4501,45 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>Climate</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Roof heat: insulation, ventilated attic, ventilator lantern louvres and shutters; ODU positions on shaded walls</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
           <t>Levels</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Survey road and field levels; plinth at 2 ft above finished ground (raise if site floods)</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Surveyor / architect</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -4531,7 +4556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4676,7 +4701,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master suite takes 2 ft (master bedroom 11'-6" x 14', master bay 9 x 8 ft) and Bedroom 2 takes 3 ft (15 x 16 ft); the sitting area in front of them grows to 18 ft. Everything east of Bedroom 2 moves 5 ft east; the plot centre now falls inside Bedroom 2, near its east wall, with the dining and ventilator about 5 ft east of it (Vastu to confirm).</t>
+          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
         </is>
       </c>
     </row>
@@ -4686,7 +4711,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
+          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
         </is>
       </c>
     </row>
@@ -4696,7 +4721,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
+          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
         </is>
       </c>
     </row>
@@ -4706,7 +4731,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
+          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
         </is>
       </c>
     </row>
@@ -4716,7 +4741,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
+          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
         </is>
       </c>
     </row>
@@ -4726,7 +4751,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
+          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
         </is>
       </c>
     </row>
@@ -4736,7 +4761,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
+          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
         </is>
       </c>
     </row>
@@ -4746,7 +4771,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
+          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
         </is>
       </c>
     </row>
@@ -4756,7 +4781,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
+          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
         </is>
       </c>
     </row>
@@ -4766,7 +4791,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
+          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4801,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
+          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
         </is>
       </c>
     </row>
@@ -4786,7 +4811,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
+          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
         </is>
       </c>
     </row>
@@ -4796,7 +4821,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
+          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
         </is>
       </c>
     </row>
@@ -4806,7 +4831,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
+          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
         </is>
       </c>
     </row>
@@ -4816,7 +4841,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
         </is>
       </c>
     </row>
@@ -4826,7 +4851,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
         </is>
       </c>
     </row>
@@ -4835,6 +4860,36 @@
         <v>29</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>Roof: Mangalore clay tiles on steel truss over insulated cement-fibre deck; all edge tiles mechanically fixed.</t>
         </is>
@@ -4851,7 +4906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5005,7 +5060,7 @@
         </is>
       </c>
       <c r="D3" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E3" s="4" t="n">
         <v>8</v>
@@ -5019,7 +5074,7 @@
         <v/>
       </c>
       <c r="H3" s="5" t="n">
-        <v>8.789999999999999</v>
+        <v>6.79</v>
       </c>
       <c r="I3" s="5" t="n">
         <v>7.62</v>
@@ -5165,7 +5220,7 @@
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>11.5</v>
+        <v>9.5</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>14</v>
@@ -5179,7 +5234,7 @@
         <v/>
       </c>
       <c r="H6" s="5" t="n">
-        <v>11.08</v>
+        <v>9.08</v>
       </c>
       <c r="I6" s="5" t="n">
         <v>13.62</v>
@@ -5272,7 +5327,7 @@
         <v>15</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>16</v>
+        <v>14.5</v>
       </c>
       <c r="F8" s="5">
         <f>D8*E8</f>
@@ -5286,7 +5341,7 @@
         <v>14.58</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>15.41</v>
+        <v>13.91</v>
       </c>
       <c r="J8" s="5">
         <f>H8*I8</f>
@@ -5325,7 +5380,7 @@
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>8</v>
@@ -5339,7 +5394,7 @@
         <v/>
       </c>
       <c r="H9" s="5" t="n">
-        <v>8.789999999999999</v>
+        <v>10.79</v>
       </c>
       <c r="I9" s="5" t="n">
         <v>8</v>
@@ -5381,7 +5436,7 @@
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E10" s="4" t="n">
         <v>6</v>
@@ -5395,7 +5450,7 @@
         <v/>
       </c>
       <c r="H10" s="5" t="n">
-        <v>8.789999999999999</v>
+        <v>10.79</v>
       </c>
       <c r="I10" s="5" t="n">
         <v>5.62</v>
@@ -5419,21 +5474,21 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>R11</t>
+          <t>R13</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Pooja</t>
+          <t>Wet area (open to the walkway)</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>6</v>
@@ -5447,10 +5502,10 @@
         <v/>
       </c>
       <c r="H11" s="5" t="n">
-        <v>3.58</v>
+        <v>5.58</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>5.42</v>
+        <v>5.71</v>
       </c>
       <c r="J11" s="5">
         <f>H11*I11</f>
@@ -5458,37 +5513,41 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>+2'-3"</t>
+          <t>+1'-9"</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Flat 9'-6"</t>
-        </is>
-      </c>
-      <c r="M11" s="4" t="inlineStr"/>
+          <t>Sloped (open truss)</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>Semi-open, jali on south wall</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>R13</t>
+          <t>R14</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Wet area (open to the walkway)</t>
+          <t>Sitting and serving area (open)</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="F12" s="5">
         <f>D12*E12</f>
@@ -5499,10 +5558,10 @@
         <v/>
       </c>
       <c r="H12" s="5" t="n">
-        <v>5.58</v>
+        <v>23.58</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>5.71</v>
+        <v>6.92</v>
       </c>
       <c r="J12" s="5">
         <f>H12*I12</f>
@@ -5510,41 +5569,37 @@
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>+1'-9"</t>
+          <t>+2'-0"</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>Sloped (open truss)</t>
-        </is>
-      </c>
-      <c r="M12" s="4" t="inlineStr">
-        <is>
-          <t>Semi-open, jali on south wall</t>
-        </is>
-      </c>
+          <t>Flat 9'-6"</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>R14</t>
+          <t>R15</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area (open)</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F13" s="5">
         <f>D13*E13</f>
@@ -5555,10 +5610,10 @@
         <v/>
       </c>
       <c r="H13" s="5" t="n">
-        <v>17.58</v>
+        <v>13.41</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>5.42</v>
+        <v>9.25</v>
       </c>
       <c r="J13" s="5">
         <f>H13*I13</f>
@@ -5579,24 +5634,24 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>R15</t>
+          <t>R16</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="D14" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F14" s="5">
         <f>D14*E14</f>
@@ -5607,10 +5662,10 @@
         <v/>
       </c>
       <c r="H14" s="5" t="n">
-        <v>13.41</v>
+        <v>11.62</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>9.25</v>
+        <v>11.25</v>
       </c>
       <c r="J14" s="5">
         <f>H14*I14</f>
@@ -5623,7 +5678,7 @@
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>Flat 9'-6"</t>
+          <t>Sloped (follows roof)</t>
         </is>
       </c>
       <c r="M14" s="4" t="inlineStr"/>
@@ -5631,24 +5686,24 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>R16</t>
+          <t>R11</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
+          <t>Pooja</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
           <t>Living</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Living</t>
-        </is>
-      </c>
       <c r="D15" s="4" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F15" s="5">
         <f>D15*E15</f>
@@ -5659,10 +5714,10 @@
         <v/>
       </c>
       <c r="H15" s="5" t="n">
-        <v>11.62</v>
+        <v>3.42</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>11.25</v>
+        <v>3.58</v>
       </c>
       <c r="J15" s="5">
         <f>H15*I15</f>
@@ -5670,12 +5725,12 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>+2'-0"</t>
+          <t>+2'-3"</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>Sloped (follows roof)</t>
+          <t>Flat 9'-6"</t>
         </is>
       </c>
       <c r="M15" s="4" t="inlineStr"/>
@@ -5683,24 +5738,24 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>R17</t>
+          <t>R20</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Poomukham (verandah)</t>
+          <t>Fridge corner</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Entry</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="D16" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>12</v>
+        <v>3.5</v>
       </c>
       <c r="F16" s="5">
         <f>D16*E16</f>
@@ -5711,10 +5766,10 @@
         <v/>
       </c>
       <c r="H16" s="5" t="n">
-        <v>5.62</v>
+        <v>3.42</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>11.62</v>
+        <v>3.29</v>
       </c>
       <c r="J16" s="5">
         <f>H16*I16</f>
@@ -5722,47 +5777,99 @@
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
+          <t>+2'-0"</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Flat 9'-6"</t>
+        </is>
+      </c>
+      <c r="M16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>R17</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Poomukham (verandah)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Entry</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="F17" s="5">
+        <f>D17*E17</f>
+        <v/>
+      </c>
+      <c r="G17" s="5">
+        <f>F17*0.092903</f>
+        <v/>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>5.62</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>11.62</v>
+      </c>
+      <c r="J17" s="5">
+        <f>H17*I17</f>
+        <v/>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
           <t>+1'-6"</t>
         </is>
       </c>
-      <c r="L16" s="4" t="inlineStr">
+      <c r="L17" s="4" t="inlineStr">
         <is>
           <t>Sloped (exposed rafters)</t>
         </is>
       </c>
-      <c r="M16" s="4" t="inlineStr">
+      <c r="M17" s="4" t="inlineStr">
         <is>
           <t>Open verandah</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr"/>
-      <c r="B17" s="6" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr"/>
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr"/>
-      <c r="D17" s="6" t="inlineStr"/>
-      <c r="E17" s="6" t="inlineStr"/>
-      <c r="F17" s="7">
-        <f>SUM(F2:F16)</f>
+      <c r="C18" s="6" t="inlineStr"/>
+      <c r="D18" s="6" t="inlineStr"/>
+      <c r="E18" s="6" t="inlineStr"/>
+      <c r="F18" s="7">
+        <f>SUM(F2:F17)</f>
         <v/>
       </c>
-      <c r="G17" s="7">
-        <f>SUM(G2:G16)</f>
+      <c r="G18" s="7">
+        <f>SUM(G2:G17)</f>
         <v/>
       </c>
-      <c r="H17" s="7" t="inlineStr"/>
-      <c r="I17" s="7" t="inlineStr"/>
-      <c r="J17" s="7">
-        <f>SUM(J2:J16)</f>
+      <c r="H18" s="7" t="inlineStr"/>
+      <c r="I18" s="7" t="inlineStr"/>
+      <c r="J18" s="7">
+        <f>SUM(J2:J17)</f>
         <v/>
       </c>
-      <c r="K17" s="6" t="inlineStr"/>
-      <c r="L17" s="6" t="inlineStr"/>
-      <c r="M17" s="6" t="inlineStr">
+      <c r="K18" s="6" t="inlineStr"/>
+      <c r="L18" s="6" t="inlineStr"/>
+      <c r="M18" s="6" t="inlineStr">
         <is>
           <t>Built footprint 60' x 22' = 1,320 sq ft</t>
         </is>
@@ -6040,7 +6147,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Carved teak, double leaf (opens west; family sits facing east)</t>
+          <t>Carved teak, double leaf (opens west into the living; family faces east)</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -6094,7 +6201,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Kitchen entry from dining</t>
+          <t>Kitchen entry from the living (north)</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
@@ -6232,12 +6339,12 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>W02</t>
+          <t>W03</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Master bay</t>
+          <t>Sitting and serving area</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -6246,7 +6353,7 @@
         </is>
       </c>
       <c r="D3" s="9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E3" s="9" t="n">
         <v>3</v>
@@ -6260,7 +6367,7 @@
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Teak casement, glazed (south light, deep sunshade)</t>
+          <t>Timber jali + glazed shutters</t>
         </is>
       </c>
       <c r="I3" s="8" t="inlineStr"/>
@@ -6268,12 +6375,12 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>W03</t>
+          <t>W04</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area</t>
+          <t>Basin and crockery nook</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -6282,10 +6389,10 @@
         </is>
       </c>
       <c r="D4" s="9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="F4" s="9" t="n">
         <v>7</v>
@@ -6296,7 +6403,7 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Timber jali + glazed shutters</t>
+          <t>Timber jali + glazed shutters (over the serving counter)</t>
         </is>
       </c>
       <c r="I4" s="8" t="inlineStr"/>
@@ -6304,24 +6411,24 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>W04</t>
+          <t>W17</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Basin and crockery nook</t>
+          <t>Pooja</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>East (to verandah)</t>
         </is>
       </c>
       <c r="D5" s="9" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>3.5</v>
+        <v>5.5</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>7</v>
@@ -6332,7 +6439,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Timber jali + glazed shutters (over the serving counter)</t>
+          <t>High vent to the poomukham, jali + mesh (lamp smoke out)</t>
         </is>
       </c>
       <c r="I5" s="8" t="inlineStr"/>
@@ -6340,12 +6447,12 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>W17</t>
+          <t>W19</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Pooja</t>
+          <t>Sitting and serving area</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -6354,10 +6461,10 @@
         </is>
       </c>
       <c r="D6" s="9" t="n">
-        <v>2</v>
+        <v>2.8</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>5.5</v>
+        <v>3.5</v>
       </c>
       <c r="F6" s="9" t="n">
         <v>7</v>
@@ -6368,7 +6475,7 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>High vent, jali + mesh (lamp smoke out)</t>
+          <t>Timber jali + glazed shutters</t>
         </is>
       </c>
       <c r="I6" s="8" t="inlineStr"/>
@@ -6834,7 +6941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -7055,7 +7162,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Built-in wardrobe 6 ft, south wall, sliding doors, lofts above</t>
+          <t>Built-in wardrobe 6'-5", south wall, sliding doors, lofts above</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -7064,7 +7171,7 @@
         </is>
       </c>
       <c r="E5" s="4" t="n">
-        <v>6</v>
+        <v>6.4</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>2</v>
@@ -7915,7 +8022,7 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Washing machine bay 2' x 2' (covered back corner, 2 in clear of the pooja wall)</t>
+          <t>Washing machine bay 2' x 2' (covered back corner, 2 in clear of the west wall)</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -8044,7 +8151,7 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Counter-top wash basin at the west end of the serving counter, away from the pooja</t>
+          <t>Counter-top wash basin at the west end of the serving counter</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -8139,7 +8246,7 @@
         </is>
       </c>
       <c r="E30" s="4" t="n">
-        <v>10.7</v>
+        <v>13.2</v>
       </c>
       <c r="F30" s="4" t="n">
         <v>2</v>
@@ -8216,7 +8323,7 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Refrigerator space (west end, away from the hob)</t>
+          <t>Refrigerator space (in the corner below the pooja, door facing south)</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -8225,10 +8332,10 @@
         </is>
       </c>
       <c r="E32" s="4" t="n">
-        <v>2.3</v>
+        <v>2.5</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="G32" s="4" t="n">
         <v>1</v>
@@ -8249,7 +8356,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>F37</t>
+          <t>F38</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -8259,26 +8366,26 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>TV unit + 50-55 in TV (east wall, north of the door)</t>
+          <t>Three-seat sofa 6'6" facing the TV</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Appliance / joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
-        <v>1.2</v>
+        <v>2.7</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>4.5</v>
+        <v>6.3</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Teak; north window to the side, no glare</t>
+          <t>Teak frame, cotton cushions</t>
         </is>
       </c>
       <c r="I33" s="10" t="n"/>
@@ -8292,7 +8399,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>F38</t>
+          <t>F39</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -8302,7 +8409,7 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Three-seat sofa 6'6" facing the TV</t>
+          <t>Coffee table 3'6" x 2'</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -8311,17 +8418,17 @@
         </is>
       </c>
       <c r="E34" s="4" t="n">
-        <v>2.7</v>
+        <v>2</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>6.3</v>
+        <v>3.3</v>
       </c>
       <c r="G34" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>Teak frame, cotton cushions</t>
+          <t>Teak</t>
         </is>
       </c>
       <c r="I34" s="10" t="n"/>
@@ -8335,7 +8442,7 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>F39</t>
+          <t>F40</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -8345,7 +8452,7 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Coffee table 3'6" x 2'</t>
+          <t>Armchair by the north window</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -8357,14 +8464,14 @@
         <v>2</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>3.3</v>
+        <v>1.6</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>Teak</t>
+          <t>Cane / teak</t>
         </is>
       </c>
       <c r="I35" s="10" t="n"/>
@@ -8378,17 +8485,17 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>F40</t>
+          <t>F41</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Poomukham (verandah)</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Armchair by the north window</t>
+          <t>Oonjal (swing) 3'6"</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -8397,17 +8504,17 @@
         </is>
       </c>
       <c r="E36" s="4" t="n">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="G36" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>Cane / teak</t>
+          <t>Teak, chains to beam</t>
         </is>
       </c>
       <c r="I36" s="10" t="n"/>
@@ -8421,7 +8528,7 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>F41</t>
+          <t>F42</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -8431,26 +8538,26 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Oonjal (swing) 3'6"</t>
+          <t>Arugu seat (built-in, south end)</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E37" s="4" t="n">
-        <v>3.5</v>
+        <v>1.2</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>1.5</v>
+        <v>2.4</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>Teak, chains to beam</t>
+          <t>Laterite base, teak top</t>
         </is>
       </c>
       <c r="I37" s="10" t="n"/>
@@ -8462,71 +8569,28 @@
       <c r="L37" s="8" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>F42</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>Poomukham (verandah)</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>Arugu seats (built-in)</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>Built-in joinery</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="F38" s="4" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="G38" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H38" s="4" t="inlineStr">
-        <is>
-          <t>Laterite base, teak top</t>
-        </is>
-      </c>
-      <c r="I38" s="10" t="n"/>
-      <c r="J38" s="11">
-        <f>G38*I38</f>
+      <c r="A38" s="6" t="inlineStr"/>
+      <c r="B38" s="6" t="inlineStr"/>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr"/>
+      <c r="E38" s="6" t="inlineStr"/>
+      <c r="F38" s="6" t="inlineStr"/>
+      <c r="G38" s="6">
+        <f>SUM(G2:G37)</f>
         <v/>
       </c>
-      <c r="K38" s="8" t="inlineStr"/>
-      <c r="L38" s="8" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="6" t="inlineStr"/>
-      <c r="B39" s="6" t="inlineStr"/>
-      <c r="C39" s="6" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="D39" s="6" t="inlineStr"/>
-      <c r="E39" s="6" t="inlineStr"/>
-      <c r="F39" s="6" t="inlineStr"/>
-      <c r="G39" s="6">
-        <f>SUM(G2:G38)</f>
+      <c r="H38" s="6" t="inlineStr"/>
+      <c r="I38" s="12" t="inlineStr"/>
+      <c r="J38" s="12">
+        <f>SUM(J2:J37)</f>
         <v/>
       </c>
-      <c r="H39" s="6" t="inlineStr"/>
-      <c r="I39" s="12" t="inlineStr"/>
-      <c r="J39" s="12">
-        <f>SUM(J2:J38)</f>
-        <v/>
-      </c>
-      <c r="K39" s="6" t="inlineStr"/>
-      <c r="L39" s="6" t="inlineStr"/>
+      <c r="K38" s="6" t="inlineStr"/>
+      <c r="L38" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8662,7 +8726,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Idol on west wall facing east; lamp niche with heat-proof back</t>
+          <t>Idols on the east wall facing west (family faces east); lamp niche with heat-proof back</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr"/>
@@ -9633,7 +9697,7 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>21.83</v>
+        <v>20.74</v>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
@@ -9693,7 +9757,7 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>6.28</v>
+        <v>6.8</v>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
@@ -9753,7 +9817,7 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>265</v>
+        <v>269.9</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
@@ -9783,7 +9847,7 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>140.3</v>
+        <v>134.8</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
@@ -9813,7 +9877,7 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>50.5</v>
+        <v>44.5</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
@@ -9873,7 +9937,7 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>32.1</v>
+        <v>41</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
@@ -9899,11 +9963,11 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Marble / teak (pooja)</t>
+          <t>Rough Cuddapah / Kota, falls</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1.8</v>
+        <v>3</v>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
@@ -9929,11 +9993,11 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Rough Cuddapah / Kota, falls</t>
+          <t>Anti-skid matt vitrified</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>3</v>
+        <v>12.6</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
@@ -9959,11 +10023,11 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Anti-skid matt vitrified</t>
+          <t>Marble / teak (pooja)</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>11.5</v>
+        <v>1.1</v>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
@@ -10023,7 +10087,7 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>112.7</v>
+        <v>114.7</v>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
@@ -10443,7 +10507,7 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>23.7</v>
+        <v>24</v>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
@@ -10485,7 +10549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G105"/>
+  <dimension ref="A1:G107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -10837,7 +10901,7 @@
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>18.5</v>
+        <v>17.5</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>7.5</v>
@@ -10866,7 +10930,7 @@
         </is>
       </c>
       <c r="E12" s="4" t="n">
-        <v>17</v>
+        <v>14.5</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>8.6</v>
@@ -10895,7 +10959,7 @@
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>22.6</v>
+        <v>20.6</v>
       </c>
       <c r="F13" s="4" t="n">
         <v>8.6</v>
@@ -11180,7 +11244,7 @@
         </is>
       </c>
       <c r="E22" s="4" t="n">
-        <v>17.25</v>
+        <v>16.25</v>
       </c>
       <c r="F22" s="4" t="n">
         <v>18</v>
@@ -11209,7 +11273,7 @@
         </is>
       </c>
       <c r="E23" s="4" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F23" s="4" t="n">
         <v>23.5</v>
@@ -11296,7 +11360,7 @@
         </is>
       </c>
       <c r="E26" s="4" t="n">
-        <v>22.6</v>
+        <v>20.6</v>
       </c>
       <c r="F26" s="4" t="n">
         <v>9.4</v>
@@ -11329,7 +11393,7 @@
         </is>
       </c>
       <c r="E27" s="4" t="n">
-        <v>22.6</v>
+        <v>20.6</v>
       </c>
       <c r="F27" s="4" t="n">
         <v>21.6</v>
@@ -11362,7 +11426,7 @@
         </is>
       </c>
       <c r="E28" s="4" t="n">
-        <v>22.6</v>
+        <v>20.6</v>
       </c>
       <c r="F28" s="4" t="n">
         <v>15.4</v>
@@ -11395,7 +11459,7 @@
         </is>
       </c>
       <c r="E29" s="4" t="n">
-        <v>22.6</v>
+        <v>20.6</v>
       </c>
       <c r="F29" s="4" t="n">
         <v>22.2</v>
@@ -11461,7 +11525,7 @@
         </is>
       </c>
       <c r="E31" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F31" s="4" t="n">
         <v>25.6</v>
@@ -11527,10 +11591,10 @@
         </is>
       </c>
       <c r="E33" s="4" t="n">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>6</v>
+        <v>18.5</v>
       </c>
       <c r="G33" s="4" t="inlineStr"/>
     </row>
@@ -11556,10 +11620,10 @@
         </is>
       </c>
       <c r="E34" s="4" t="n">
-        <v>44.6</v>
+        <v>58.4</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>6</v>
+        <v>18.5</v>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
@@ -11589,10 +11653,10 @@
         </is>
       </c>
       <c r="E35" s="4" t="n">
-        <v>42</v>
+        <v>55.4</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>3.4</v>
+        <v>20.1</v>
       </c>
       <c r="G35" s="4" t="inlineStr"/>
     </row>
@@ -11614,18 +11678,18 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area (open)</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="E36" s="4" t="n">
-        <v>40.6</v>
+        <v>54.6</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>8.4</v>
+        <v>16.3</v>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>pooja switches outside, nook side</t>
+          <t>pooja switches outside, living side</t>
         </is>
       </c>
     </row>
@@ -11651,27 +11715,27 @@
         </is>
       </c>
       <c r="E37" s="4" t="n">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>6.5</v>
+        <v>6.75</v>
       </c>
       <c r="G37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>6 A socket at counter</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -11680,16 +11744,12 @@
         </is>
       </c>
       <c r="E38" s="4" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="G38" s="4" t="inlineStr">
-        <is>
-          <t>serving counter</t>
-        </is>
-      </c>
+        <v>6.5</v>
+      </c>
+      <c r="G38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -11713,7 +11773,7 @@
         </is>
       </c>
       <c r="E39" s="4" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F39" s="4" t="n">
         <v>3.4</v>
@@ -11727,46 +11787,50 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>6 A socket at counter</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Bath 2 (attached to Bedroom 2)</t>
+          <t>Sitting and serving area (open)</t>
         </is>
       </c>
       <c r="E40" s="4" t="n">
-        <v>25.5</v>
+        <v>38</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>21.5</v>
-      </c>
-      <c r="G40" s="4" t="inlineStr"/>
+        <v>3.4</v>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>serving counter</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>EF</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Exhaust fan</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>7'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -11775,31 +11839,27 @@
         </is>
       </c>
       <c r="E41" s="4" t="n">
-        <v>26.6</v>
+        <v>23.5</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>24.6</v>
-      </c>
-      <c r="G41" s="4" t="inlineStr">
-        <is>
-          <t>out through the north wall</t>
-        </is>
-      </c>
+        <v>21.5</v>
+      </c>
+      <c r="G41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>EF</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Geyser (16 A)</t>
+          <t>Exhaust fan</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>7'-0"</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -11808,31 +11868,31 @@
         </is>
       </c>
       <c r="E42" s="4" t="n">
-        <v>28.1</v>
+        <v>24.6</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>23</v>
+        <v>24.6</v>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>over shower</t>
+          <t>out through the north wall</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>G</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>6 A socket at counter</t>
+          <t>Geyser (16 A)</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -11841,64 +11901,64 @@
         </is>
       </c>
       <c r="E43" s="4" t="n">
-        <v>28.1</v>
+        <v>26.1</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>21.6</v>
+        <v>23</v>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>by basin</t>
+          <t>over shower</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>6 A socket at counter</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Bedroom 2</t>
+          <t>Bath 2 (attached to Bedroom 2)</t>
         </is>
       </c>
       <c r="E44" s="4" t="n">
-        <v>26.8</v>
+        <v>26.1</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>18.8</v>
+        <v>21.6</v>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>Bath 2 switches outside the bath door</t>
+          <t>by basin</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Ceiling fan point</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -11907,22 +11967,26 @@
         </is>
       </c>
       <c r="E45" s="4" t="n">
-        <v>30.5</v>
+        <v>24.8</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="G45" s="4" t="inlineStr"/>
+        <v>18.8</v>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>Bath 2 switches outside the bath door</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Ceiling fan point</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -11936,10 +12000,10 @@
         </is>
       </c>
       <c r="E46" s="4" t="n">
-        <v>30.5</v>
+        <v>28.5</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>12.5</v>
+        <v>17</v>
       </c>
       <c r="G46" s="4" t="inlineStr"/>
     </row>
@@ -11965,10 +12029,10 @@
         </is>
       </c>
       <c r="E47" s="4" t="n">
-        <v>25.5</v>
+        <v>28.5</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>15.5</v>
+        <v>13.5</v>
       </c>
       <c r="G47" s="4" t="inlineStr"/>
     </row>
@@ -11994,27 +12058,27 @@
         </is>
       </c>
       <c r="E48" s="4" t="n">
-        <v>33</v>
+        <v>23.5</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -12023,16 +12087,12 @@
         </is>
       </c>
       <c r="E49" s="4" t="n">
-        <v>26.9</v>
+        <v>31</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="G49" s="4" t="inlineStr">
-        <is>
-          <t>at door</t>
-        </is>
-      </c>
+        <v>20.5</v>
+      </c>
+      <c r="G49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -12056,31 +12116,31 @@
         </is>
       </c>
       <c r="E50" s="4" t="n">
-        <v>37.4</v>
+        <v>24.9</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>9.4</v>
+        <v>10.9</v>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>bedside, 2-way</t>
+          <t>at door</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -12089,14 +12149,14 @@
         </is>
       </c>
       <c r="E51" s="4" t="n">
-        <v>37.6</v>
+        <v>35.4</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>9.9</v>
+        <v>10.9</v>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>bedside</t>
+          <t>bedside, 2-way</t>
         </is>
       </c>
     </row>
@@ -12122,10 +12182,10 @@
         </is>
       </c>
       <c r="E52" s="4" t="n">
-        <v>31.2</v>
+        <v>35.6</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>9.4</v>
+        <v>11.4</v>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
@@ -12155,26 +12215,26 @@
         </is>
       </c>
       <c r="E53" s="4" t="n">
-        <v>28.9</v>
+        <v>29.2</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>20</v>
+        <v>10.9</v>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>work table</t>
+          <t>bedside</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Inverter (UPS) socket</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
@@ -12188,26 +12248,26 @@
         </is>
       </c>
       <c r="E54" s="4" t="n">
-        <v>28.9</v>
+        <v>26.9</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>20.8</v>
+        <v>20</v>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>work table, monitor</t>
+          <t>work table</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Data point (Cat6)</t>
+          <t>Inverter (UPS) socket</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -12221,26 +12281,26 @@
         </is>
       </c>
       <c r="E55" s="4" t="n">
-        <v>28.9</v>
+        <v>26.9</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>21.6</v>
+        <v>20.8</v>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>work table</t>
+          <t>work table, monitor</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Inverter (UPS) socket</t>
+          <t>Data point (Cat6)</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -12254,10 +12314,10 @@
         </is>
       </c>
       <c r="E56" s="4" t="n">
-        <v>28.9</v>
+        <v>26.9</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>22.4</v>
+        <v>21.6</v>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
@@ -12268,17 +12328,17 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
+          <t>Inverter (UPS) socket</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>7'-6"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -12287,126 +12347,130 @@
         </is>
       </c>
       <c r="E57" s="4" t="n">
-        <v>37.6</v>
+        <v>26.9</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>18.6</v>
+        <v>22.4</v>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>east wall, not at the work table</t>
+          <t>work table</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>7'-6"</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area (open)</t>
+          <t>Bedroom 2</t>
         </is>
       </c>
       <c r="E58" s="4" t="n">
-        <v>32.2</v>
+        <v>35.6</v>
       </c>
       <c r="F58" s="4" t="n">
-        <v>3.4</v>
+        <v>18.6</v>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>over basin</t>
+          <t>east wall, not at the work table</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>ODU</t>
+          <t>WL</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>AC outdoor unit bracket</t>
+          <t>Wall light / mirror light</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>7'-0" outside</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Bedroom 2</t>
+          <t>Sitting and serving area (open)</t>
         </is>
       </c>
       <c r="E59" s="4" t="n">
-        <v>33</v>
+        <v>32.2</v>
       </c>
       <c r="F59" s="4" t="n">
-        <v>25.6</v>
+        <v>3.4</v>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>north wall, shaded</t>
+          <t>over basin</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>ODU</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>AC outdoor unit bracket</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>7'-0" outside</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>Dining bay (north window)</t>
+          <t>Bedroom 2</t>
         </is>
       </c>
       <c r="E60" s="4" t="n">
-        <v>42.5</v>
+        <v>31</v>
       </c>
       <c r="F60" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="G60" s="4" t="inlineStr"/>
+        <v>25.6</v>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>north wall, shaded</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -12415,60 +12479,56 @@
         </is>
       </c>
       <c r="E61" s="4" t="n">
-        <v>46.6</v>
+        <v>42.5</v>
       </c>
       <c r="F61" s="4" t="n">
-        <v>24.6</v>
+        <v>22</v>
       </c>
       <c r="G61" s="4" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Dining bay (north window)</t>
         </is>
       </c>
       <c r="E62" s="4" t="n">
-        <v>42.5</v>
+        <v>46.6</v>
       </c>
       <c r="F62" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G62" s="4" t="inlineStr">
-        <is>
-          <t>pendant</t>
-        </is>
-      </c>
+        <v>24.6</v>
+      </c>
+      <c r="G62" s="4" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -12477,27 +12537,31 @@
         </is>
       </c>
       <c r="E63" s="4" t="n">
-        <v>38.4</v>
+        <v>42.5</v>
       </c>
       <c r="F63" s="4" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="G63" s="4" t="inlineStr"/>
+        <v>15</v>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>pendant</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>WL</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Wall light / mirror light</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -12506,27 +12570,27 @@
         </is>
       </c>
       <c r="E64" s="4" t="n">
-        <v>38.4</v>
+        <v>36.4</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>16.2</v>
+        <v>17.5</v>
       </c>
       <c r="G64" s="4" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -12535,56 +12599,56 @@
         </is>
       </c>
       <c r="E65" s="4" t="n">
-        <v>46.6</v>
+        <v>36.4</v>
       </c>
       <c r="F65" s="4" t="n">
-        <v>17.8</v>
+        <v>16.2</v>
       </c>
       <c r="G65" s="4" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area (open)</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E66" s="4" t="n">
-        <v>28.5</v>
+        <v>46.6</v>
       </c>
       <c r="F66" s="4" t="n">
-        <v>6</v>
+        <v>17.8</v>
       </c>
       <c r="G66" s="4" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -12593,27 +12657,27 @@
         </is>
       </c>
       <c r="E67" s="4" t="n">
-        <v>23.4</v>
+        <v>28.5</v>
       </c>
       <c r="F67" s="4" t="n">
-        <v>6</v>
+        <v>6.75</v>
       </c>
       <c r="G67" s="4" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>INV</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Inverter + battery</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>floor</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -12622,64 +12686,60 @@
         </is>
       </c>
       <c r="E68" s="4" t="n">
-        <v>24</v>
+        <v>21.4</v>
       </c>
       <c r="F68" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="G68" s="4" t="inlineStr">
-        <is>
-          <t>lithium inverter in a ventilated cabinet under the bench</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="G68" s="4" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>INV</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Inverter + battery</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>floor</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>Wet area (open to the walkway)</t>
+          <t>Sitting and serving area (open)</t>
         </is>
       </c>
       <c r="E69" s="4" t="n">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="F69" s="4" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>weatherproof</t>
+          <t>lithium inverter in a ventilated cabinet under the bench</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>16 A power socket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -12688,31 +12748,31 @@
         </is>
       </c>
       <c r="E70" s="4" t="n">
-        <v>46.4</v>
+        <v>48</v>
       </c>
       <c r="F70" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>5.5</v>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>washing machine</t>
+          <t>weatherproof</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>16 A power socket</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>varies</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -12721,60 +12781,64 @@
         </is>
       </c>
       <c r="E71" s="4" t="n">
-        <v>50.6</v>
+        <v>46.4</v>
       </c>
       <c r="F71" s="4" t="n">
-        <v>6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>utility, weatherproof</t>
+          <t>washing machine</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Wet area (open to the walkway)</t>
         </is>
       </c>
       <c r="E72" s="4" t="n">
-        <v>60</v>
+        <v>50.6</v>
       </c>
       <c r="F72" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="G72" s="4" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="G72" s="4" t="inlineStr">
+        <is>
+          <t>utility, weatherproof</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
@@ -12783,16 +12847,12 @@
         </is>
       </c>
       <c r="E73" s="4" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F73" s="4" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="G73" s="4" t="inlineStr">
-        <is>
-          <t>under-cabinet</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="G73" s="4" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
@@ -12816,10 +12876,10 @@
         </is>
       </c>
       <c r="E74" s="4" t="n">
-        <v>64.5</v>
+        <v>59</v>
       </c>
       <c r="F74" s="4" t="n">
-        <v>9</v>
+        <v>3.5</v>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
@@ -12830,17 +12890,17 @@
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>WL</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Kitchen chimney point (16 A)</t>
+          <t>Wall light / mirror light</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>7'-0"</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -12849,31 +12909,31 @@
         </is>
       </c>
       <c r="E75" s="4" t="n">
-        <v>64.59999999999999</v>
+        <v>64.5</v>
       </c>
       <c r="F75" s="4" t="n">
-        <v>8.75</v>
+        <v>9</v>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>duct out through east wall</t>
+          <t>under-cabinet</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>16 A power socket</t>
+          <t>Kitchen chimney point (16 A)</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>7'-0"</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -12882,82 +12942,78 @@
         </is>
       </c>
       <c r="E76" s="4" t="n">
-        <v>51.6</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="F76" s="4" t="n">
-        <v>4.4</v>
+        <v>8.75</v>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>refrigerator, behind the fridge</t>
+          <t>duct out through east wall</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>6 A socket at counter</t>
+          <t>16 A power socket</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>varies</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Fridge corner</t>
         </is>
       </c>
       <c r="E77" s="4" t="n">
-        <v>56</v>
+        <v>56.75</v>
       </c>
       <c r="F77" s="4" t="n">
-        <v>3.5</v>
+        <v>16.2</v>
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>microwave / OTG</t>
+          <t>refrigerator, behind the fridge</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>6 A socket at counter</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Fridge corner</t>
         </is>
       </c>
       <c r="E78" s="4" t="n">
-        <v>61.5</v>
+        <v>57</v>
       </c>
       <c r="F78" s="4" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="G78" s="4" t="inlineStr">
-        <is>
-          <t>mixer</t>
-        </is>
-      </c>
+        <v>14.75</v>
+      </c>
+      <c r="G78" s="4" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -12981,10 +13037,10 @@
         </is>
       </c>
       <c r="E79" s="4" t="n">
-        <v>64.59999999999999</v>
+        <v>52.5</v>
       </c>
       <c r="F79" s="4" t="n">
-        <v>6</v>
+        <v>3.5</v>
       </c>
       <c r="G79" s="4" t="inlineStr"/>
     </row>
@@ -13010,12 +13066,16 @@
         </is>
       </c>
       <c r="E80" s="4" t="n">
-        <v>64.59999999999999</v>
+        <v>56</v>
       </c>
       <c r="F80" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="G80" s="4" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>microwave / OTG</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -13039,31 +13099,31 @@
         </is>
       </c>
       <c r="E81" s="4" t="n">
-        <v>57.3</v>
+        <v>61.5</v>
       </c>
       <c r="F81" s="4" t="n">
         <v>3.5</v>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>RO purifier, by sink</t>
+          <t>mixer</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>6 A socket at counter</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -13072,122 +13132,122 @@
         </is>
       </c>
       <c r="E82" s="4" t="n">
-        <v>51.6</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="F82" s="4" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="G82" s="4" t="inlineStr">
-        <is>
-          <t>beside the sliding entry</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="G82" s="4" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Ceiling fan point</t>
+          <t>6 A socket at counter</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="E83" s="4" t="n">
-        <v>53</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="F83" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="G83" s="4" t="inlineStr">
-        <is>
-          <t>long downrod</t>
-        </is>
-      </c>
+        <v>11.5</v>
+      </c>
+      <c r="G83" s="4" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>6 A socket at counter</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="E84" s="4" t="n">
-        <v>50</v>
+        <v>57.3</v>
       </c>
       <c r="F84" s="4" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="G84" s="4" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>RO purifier, by sink</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="E85" s="4" t="n">
-        <v>56</v>
+        <v>51.4</v>
       </c>
       <c r="F85" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="G85" s="4" t="inlineStr"/>
+        <v>12.6</v>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>beside the sliding entry</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>Ceiling fan point</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -13196,27 +13256,31 @@
         </is>
       </c>
       <c r="E86" s="4" t="n">
-        <v>47.4</v>
+        <v>53</v>
       </c>
       <c r="F86" s="4" t="n">
-        <v>24.2</v>
-      </c>
-      <c r="G86" s="4" t="inlineStr"/>
+        <v>19</v>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>long downrod</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>TV</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>TV + data point</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -13225,31 +13289,27 @@
         </is>
       </c>
       <c r="E87" s="4" t="n">
-        <v>58.6</v>
+        <v>50</v>
       </c>
       <c r="F87" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="G87" s="4" t="inlineStr">
-        <is>
-          <t>TV + data + 2 sockets, east wall</t>
-        </is>
-      </c>
+        <v>22.5</v>
+      </c>
+      <c r="G87" s="4" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -13258,31 +13318,27 @@
         </is>
       </c>
       <c r="E88" s="4" t="n">
-        <v>47.4</v>
+        <v>53</v>
       </c>
       <c r="F88" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="G88" s="4" t="inlineStr">
-        <is>
-          <t>sofa</t>
-        </is>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="G88" s="4" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>WL</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Wall light / mirror light</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
@@ -13291,31 +13347,27 @@
         </is>
       </c>
       <c r="E89" s="4" t="n">
-        <v>50.6</v>
+        <v>47.4</v>
       </c>
       <c r="F89" s="4" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="G89" s="4" t="inlineStr">
-        <is>
-          <t>floor socket, sofa end</t>
-        </is>
-      </c>
+        <v>24.2</v>
+      </c>
+      <c r="G89" s="4" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>7'-6"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -13327,28 +13379,28 @@
         <v>47.4</v>
       </c>
       <c r="F90" s="4" t="n">
-        <v>21.5</v>
+        <v>18</v>
       </c>
       <c r="G90" s="4" t="inlineStr">
         <is>
-          <t>west wall</t>
+          <t>sofa</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>ODU</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>AC outdoor unit bracket</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>7'-0" outside</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -13357,31 +13409,31 @@
         </is>
       </c>
       <c r="E91" s="4" t="n">
-        <v>57.5</v>
+        <v>50.6</v>
       </c>
       <c r="F91" s="4" t="n">
-        <v>25.6</v>
+        <v>17.8</v>
       </c>
       <c r="G91" s="4" t="inlineStr">
         <is>
-          <t>north wall, shaded</t>
+          <t>floor socket, sofa end</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>7'-6"</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
@@ -13390,31 +13442,31 @@
         </is>
       </c>
       <c r="E92" s="4" t="n">
-        <v>58.6</v>
+        <v>47.4</v>
       </c>
       <c r="F92" s="4" t="n">
-        <v>18.6</v>
+        <v>21.5</v>
       </c>
       <c r="G92" s="4" t="inlineStr">
         <is>
-          <t>main switch at door</t>
+          <t>west wall</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>ODU</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>Distribution board</t>
+          <t>AC outdoor unit bracket</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>5'-0" to top</t>
+          <t>7'-0" outside</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
@@ -13423,31 +13475,31 @@
         </is>
       </c>
       <c r="E93" s="4" t="n">
-        <v>57.2</v>
+        <v>57.5</v>
       </c>
       <c r="F93" s="4" t="n">
-        <v>13.4</v>
+        <v>25.6</v>
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>SE of living, near entry</t>
+          <t>north wall, shaded</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>Inverter (UPS) socket</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
@@ -13456,89 +13508,97 @@
         </is>
       </c>
       <c r="E94" s="4" t="n">
-        <v>58.4</v>
+        <v>58.6</v>
       </c>
       <c r="F94" s="4" t="n">
-        <v>13.4</v>
+        <v>21</v>
       </c>
       <c r="G94" s="4" t="inlineStr">
         <is>
-          <t>router</t>
+          <t>main switch at door</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Distribution board</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>5'-0" to top</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>Poomukham (verandah)</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="E95" s="4" t="n">
-        <v>62</v>
+        <v>54.6</v>
       </c>
       <c r="F95" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="G95" s="4" t="inlineStr"/>
+        <v>14</v>
+      </c>
+      <c r="G95" s="4" t="inlineStr">
+        <is>
+          <t>living side of the fridge-corner wall, near entry</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Inverter (UPS) socket</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>Poomukham (verandah)</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="E96" s="4" t="n">
-        <v>62</v>
+        <v>54.6</v>
       </c>
       <c r="F96" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="G96" s="4" t="inlineStr"/>
+        <v>15.4</v>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>router</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>BELL</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>Bell push</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>4'-6"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
@@ -13547,27 +13607,27 @@
         </is>
       </c>
       <c r="E97" s="4" t="n">
-        <v>59.4</v>
+        <v>62</v>
       </c>
       <c r="F97" s="4" t="n">
-        <v>18.6</v>
+        <v>16</v>
       </c>
       <c r="G97" s="4" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>CAM</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>CCTV point</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>8'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
@@ -13576,31 +13636,27 @@
         </is>
       </c>
       <c r="E98" s="4" t="n">
-        <v>64.5</v>
+        <v>62</v>
       </c>
       <c r="F98" s="4" t="n">
-        <v>24.6</v>
-      </c>
-      <c r="G98" s="4" t="inlineStr">
-        <is>
-          <t>covers gate and door</t>
-        </is>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="G98" s="4" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>BELL</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Bell push</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>4'-6"</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
@@ -13612,28 +13668,24 @@
         <v>59.4</v>
       </c>
       <c r="F99" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="G99" s="4" t="inlineStr">
-        <is>
-          <t>outdoor, weatherproof</t>
-        </is>
-      </c>
+        <v>20.4</v>
+      </c>
+      <c r="G99" s="4" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>CAM</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>CCTV point</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>8'-0"</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
@@ -13642,93 +13694,93 @@
         </is>
       </c>
       <c r="E100" s="4" t="n">
-        <v>59.4</v>
+        <v>64.5</v>
       </c>
       <c r="F100" s="4" t="n">
-        <v>19.2</v>
-      </c>
-      <c r="G100" s="4" t="inlineStr"/>
+        <v>24.6</v>
+      </c>
+      <c r="G100" s="4" t="inlineStr">
+        <is>
+          <t>covers gate and door</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>MTR</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>Meter at gate</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>5'-0"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>Site</t>
+          <t>Poomukham (verandah)</t>
         </is>
       </c>
       <c r="E101" s="4" t="n">
-        <v>74.59999999999999</v>
+        <v>59.4</v>
       </c>
       <c r="F101" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G101" s="4" t="inlineStr">
         <is>
-          <t>meter in compound wall by gate</t>
+          <t>outdoor, weatherproof</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>GL</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Outdoor / gate light</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>7'-0"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>Site</t>
+          <t>Poomukham (verandah)</t>
         </is>
       </c>
       <c r="E102" s="4" t="n">
-        <v>74.59999999999999</v>
+        <v>59.4</v>
       </c>
       <c r="F102" s="4" t="n">
-        <v>14.5</v>
-      </c>
-      <c r="G102" s="4" t="inlineStr">
-        <is>
-          <t>gate light</t>
-        </is>
-      </c>
+        <v>20.9</v>
+      </c>
+      <c r="G102" s="4" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>EP</t>
+          <t>MTR</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>Earth pit</t>
+          <t>Meter at gate</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>ground</t>
+          <t>5'-0"</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
@@ -13737,31 +13789,31 @@
         </is>
       </c>
       <c r="E103" s="4" t="n">
-        <v>66.2</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="F103" s="4" t="n">
-        <v>1.5</v>
+        <v>23</v>
       </c>
       <c r="G103" s="4" t="inlineStr">
         <is>
-          <t>earth pit 1</t>
+          <t>meter in compound wall by gate</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>EP</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>Earth pit</t>
+          <t>Outdoor / gate light</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>ground</t>
+          <t>7'-0"</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
@@ -13770,45 +13822,111 @@
         </is>
       </c>
       <c r="E104" s="4" t="n">
-        <v>73.5</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="F104" s="4" t="n">
-        <v>1.5</v>
+        <v>14.5</v>
       </c>
       <c r="G104" s="4" t="inlineStr">
         <is>
-          <t>earth pit 2</t>
+          <t>gate light</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
+          <t>EP</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>Earth pit</t>
+        </is>
+      </c>
+      <c r="C105" s="4" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="E105" s="4" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="F105" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G105" s="4" t="inlineStr">
+        <is>
+          <t>earth pit 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="4" t="inlineStr">
+        <is>
+          <t>EP</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>Earth pit</t>
+        </is>
+      </c>
+      <c r="C106" s="4" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="E106" s="4" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="F106" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G106" s="4" t="inlineStr">
+        <is>
+          <t>earth pit 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
           <t>GL</t>
         </is>
       </c>
-      <c r="B105" s="4" t="inlineStr">
+      <c r="B107" s="4" t="inlineStr">
         <is>
           <t>Outdoor / gate light</t>
         </is>
       </c>
-      <c r="C105" s="4" t="inlineStr">
+      <c r="C107" s="4" t="inlineStr">
         <is>
           <t>7'-0"</t>
         </is>
       </c>
-      <c r="D105" s="4" t="inlineStr">
+      <c r="D107" s="4" t="inlineStr">
         <is>
           <t>Site</t>
         </is>
       </c>
-      <c r="E105" s="4" t="n">
+      <c r="E107" s="4" t="n">
         <v>2.5</v>
       </c>
-      <c r="F105" s="4" t="n">
+      <c r="F107" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="G105" s="4" t="inlineStr">
+      <c r="G107" s="4" t="inlineStr">
         <is>
           <t>rear garden</t>
         </is>

</xml_diff>

<commit_message>
Reviews 15-16: TV wall, master bed, Bedroom 2 layout, kitchen entry, septic
Bath 2 enlarged then re-planned 7' x 6' with its door on the east wall so
Bedroom 2's bed (head west) has 1'-6" both sides; Bedroom 2 corner notched
to widen the way into the sitting area; Bedroom 2 door at the east end.
TV moves to Bedroom 2's east wall facing the dining bay; master bed moves
south with a window seat by the north window. Kitchen entered by a hinged
west door off the dining alcove (north sliding door walled up, pantry on
the north wall); hob and chimney on solid wall. Septic moved 6 ft+ from the
house with a soak trench; ensuite door outward; common bath WC, door,
geyser and shower fixed; DB moved to the dining wall. Drawing code supports
doors hinged at either jamb.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Schedules/KH-P1_Schedules_RevB.xlsx
+++ b/03_Schedules/KH-P1_Schedules_RevB.xlsx
@@ -894,11 +894,11 @@
         <v>45.6</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>7.6</v>
+        <v>7.35</v>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>wall-hung on the wet wall</t>
+          <t>on the wet wall</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
         <v>45.6</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>7</v>
+        <v>6.5</v>
       </c>
       <c r="F9" s="4" t="inlineStr"/>
     </row>
@@ -971,12 +971,16 @@
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>40.4</v>
+        <v>39.8</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="F11" s="4" t="inlineStr"/>
+        <v>3.9</v>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>west wall, clear of the window</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1051,14 +1055,14 @@
         </is>
       </c>
       <c r="D14" s="4" t="n">
-        <v>22</v>
+        <v>22.5</v>
       </c>
       <c r="E14" s="4" t="n">
         <v>24</v>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>wall-hung on the north (outer) wall</t>
+          <t>on the north (outer) wall, 15 in clear each side</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1086,7 @@
         <v>21.4</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>22.4</v>
+        <v>23.4</v>
       </c>
       <c r="F15" s="4" t="inlineStr"/>
     </row>
@@ -1103,14 +1107,14 @@
         </is>
       </c>
       <c r="D16" s="4" t="n">
-        <v>25.8</v>
+        <v>24.25</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>20.3</v>
+        <v>19.4</v>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>on 7 in wet wall</t>
+          <t>on 7 in wet wall (south)</t>
         </is>
       </c>
     </row>
@@ -1131,12 +1135,16 @@
         </is>
       </c>
       <c r="D17" s="4" t="n">
-        <v>26.1</v>
+        <v>27.6</v>
       </c>
       <c r="E17" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="F17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>east wall</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1155,10 +1163,10 @@
         </is>
       </c>
       <c r="D18" s="4" t="n">
-        <v>25</v>
+        <v>26.4</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>24.2</v>
+        <v>24.3</v>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
@@ -1183,7 +1191,7 @@
         </is>
       </c>
       <c r="D19" s="4" t="n">
-        <v>23.3</v>
+        <v>25.5</v>
       </c>
       <c r="E19" s="4" t="n">
         <v>20.6</v>
@@ -1791,7 +1799,7 @@
         </is>
       </c>
       <c r="D41" s="4" t="n">
-        <v>22</v>
+        <v>22.5</v>
       </c>
       <c r="E41" s="4" t="n">
         <v>26.6</v>
@@ -1819,7 +1827,7 @@
         </is>
       </c>
       <c r="D42" s="4" t="n">
-        <v>25</v>
+        <v>26.4</v>
       </c>
       <c r="E42" s="4" t="n">
         <v>26</v>
@@ -2328,7 +2336,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Check door swings against the furniture; put the DB away from the door and the pooja (here in the alcove between the dining and the kitchen).</t>
+          <t>Check door swings against the furniture; put the DB away from the door and the pooja (here on the dining face of Bedroom 2's east wall).</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -2765,7 +2773,7 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Fridge on the kitchen's north wall behind the pooja, beside the north entry and well away from the hob; nothing blocks the counter.</t>
+          <t>Fridge on the kitchen's north wall behind the pooja, beside the tall pantry and well away from the hob; nothing blocks the counter.</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -2788,7 +2796,7 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>The kitchen is entered from the living on the north through a 3 ft sliding glass door, open when serving, closed when frying; a second sliding door on the west takes food straight to the dining.</t>
+          <t>The kitchen is entered through a 3 ft hinged door on its west side, straight off the dining alcove: one short trip for serving, and it closes off cooking smoke. The pooja front stays quiet.</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -4007,7 +4015,7 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>Keep soil and grey water separate: soil to the septic, grey to a soak pit, with inspection chambers at every bend.</t>
+          <t>Keep soil and grey water separate: soil to the septic, grey to a soak trench, with inspection chambers at every bend.</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
@@ -4422,7 +4430,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>TV wall to be decided: the 4 ft east wall between the pooja and the main door now holds the shoe cupboard; options are a wall-mounted TV above a low shoe cabinet there, or a TV on a jali partition between the living and the dining (50-55 in, with data and 2 sockets)</t>
+          <t>TV on Bedroom 2's east wall facing the dining bay: confirm screen size (55-65 in at about 9 ft) and a concealed HDMI/data conduit from the unit</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -4497,7 +4505,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Plot 27 ft x 75 ft (length to confirm by survey): north wall is 2 ft from the plot line and eaves overhang the owned north strip; septic and soak pit sit in the strip</t>
+          <t>Plot 27 ft x 75 ft (length to confirm by survey): north wall is 2 ft from the plot line and eaves overhang the owned north strip; septic and soak trench sit in the strip</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -4622,7 +4630,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Septic and soak pit sizes; keep soak pits and gardens 6 ft+ from foundations in expansive soil</t>
+          <t>Septic tank size and soak trench length (percolation test); keep soak trenches and gardens 6 ft+ from foundations in expansive soil</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -4697,7 +4705,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Bed head east (master), NW ensuite, Bedroom 2's attached bath in its north-west corner on the north wall (north-west of the plot centre), common bath south of the plot centre beside the wet area (outside the central zone), dining at the plot centre, pooja in the living's south-east corner back to back with the kitchen, opening west (devotees face east), shoe cupboard between the pooja and the main door (behind the pooja's solid north wall), DB in the alcove between the dining and the kitchen</t>
+          <t>Bed head east (master), NW ensuite, Bedroom 2's attached bath in its north-west corner on the north wall (north-west of the plot centre), common bath south of the plot centre beside the wet area (outside the central zone), dining at the plot centre, pooja in the living's south-east corner back to back with the kitchen, opening west (devotees face east), shoe cupboard between the pooja and the main door (behind the pooja's solid north wall), DB on the dining face of Bedroom 2's east wall</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -4772,7 +4780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4917,7 +4925,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner (5'-6" x 6') and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
+          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
         </is>
       </c>
     </row>
@@ -4927,7 +4935,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
+          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
         </is>
       </c>
     </row>
@@ -4937,7 +4945,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
+          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
         </is>
       </c>
     </row>
@@ -4947,7 +4955,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
+          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
         </is>
       </c>
     </row>
@@ -4957,7 +4965,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
+          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
         </is>
       </c>
     </row>
@@ -4967,7 +4975,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
+          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
         </is>
       </c>
     </row>
@@ -4977,7 +4985,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
+          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
         </is>
       </c>
     </row>
@@ -4987,7 +4995,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
+          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
         </is>
       </c>
     </row>
@@ -4997,7 +5005,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
+          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
         </is>
       </c>
     </row>
@@ -5007,7 +5015,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
+          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
         </is>
       </c>
     </row>
@@ -5017,7 +5025,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
+          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
         </is>
       </c>
     </row>
@@ -5027,7 +5035,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
+          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
         </is>
       </c>
     </row>
@@ -5037,7 +5045,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
+          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
         </is>
       </c>
     </row>
@@ -5047,7 +5055,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
+          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
         </is>
       </c>
     </row>
@@ -5057,7 +5065,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
+          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
         </is>
       </c>
     </row>
@@ -5067,7 +5075,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
+          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
         </is>
       </c>
     </row>
@@ -5077,7 +5085,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
+          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
         </is>
       </c>
     </row>
@@ -5087,7 +5095,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
+          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
         </is>
       </c>
     </row>
@@ -5097,7 +5105,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
+          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
         </is>
       </c>
     </row>
@@ -5107,7 +5115,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
+          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
         </is>
       </c>
     </row>
@@ -5117,7 +5125,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
         </is>
       </c>
     </row>
@@ -5127,7 +5135,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
         </is>
       </c>
     </row>
@@ -5136,6 +5144,26 @@
         <v>35</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>Roof: Mangalore clay tiles on steel truss over insulated cement-fibre deck; all edge tiles mechanically fixed.</t>
         </is>
@@ -5518,7 +5546,7 @@
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>5.5</v>
+        <v>7</v>
       </c>
       <c r="E7" s="4" t="n">
         <v>6</v>
@@ -5532,10 +5560,10 @@
         <v/>
       </c>
       <c r="H7" s="5" t="n">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>5.42</v>
+        <v>5.33</v>
       </c>
       <c r="J7" s="5">
         <f>H7*I7</f>
@@ -6133,7 +6161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6237,7 +6265,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Ensuite</t>
+          <t>Ensuite (opens outward)</t>
         </is>
       </c>
       <c r="C3" s="4" t="n">
@@ -6307,7 +6335,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Bedroom 2 (from the sitting area)</t>
+          <t>Bedroom 2 (from the sitting area, east end; open leaf screens the bed)</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
@@ -6342,7 +6370,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Common bath (from the sitting area, opens outward)</t>
+          <t>Common bath (from the sitting area, opens outward, hinged at the north jamb so the open leaf stays clear of the counter)</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
@@ -6358,7 +6386,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Flush, waterproof (WPC/FRP)</t>
+          <t>Flush, waterproof (WPC/FRP), door closer</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -6377,7 +6405,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Bath 2 (from Bedroom 2, opens outward)</t>
+          <t>Bath 2 (east wall, from Bedroom 2, opens outward)</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
@@ -6477,12 +6505,12 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D17</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Kitchen entry from the living (north)</t>
+          <t>Kitchen entry (west, from the dining alcove; hinged at the north jamb)</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
@@ -6493,12 +6521,12 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Sliding</t>
+          <t>Hinged, single</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Sliding glass, 3 ft (closes off cooking smoke)</t>
+          <t>Teak frame, glazed upper panel, 3 ft (closes off cooking smoke)</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -6508,41 +6536,6 @@
       </c>
       <c r="H10" s="8" t="inlineStr"/>
       <c r="I10" s="8" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>D17</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Kitchen to dining (serving door, west)</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Sliding</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>Sliding glass, 2'-9" (food goes straight to the dining)</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H11" s="8" t="inlineStr"/>
-      <c r="I11" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6885,7 +6878,7 @@
         </is>
       </c>
       <c r="D9" s="9" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E9" s="9" t="n">
         <v>3.5</v>
@@ -6899,7 +6892,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Timber jali + glazed shutters</t>
+          <t>Timber jali + glazed shutters (2 ft, north end; hob wall kept solid)</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr"/>
@@ -7029,7 +7022,7 @@
         </is>
       </c>
       <c r="D13" s="9" t="n">
-        <v>6</v>
+        <v>5.2</v>
       </c>
       <c r="E13" s="9" t="n">
         <v>3</v>
@@ -7043,7 +7036,7 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Teak casement, glazed (6 ft)</t>
+          <t>Teak casement, glazed (5'-2")</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr"/>
@@ -7097,7 +7090,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr"/>
       <c r="D15" s="9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>7.5</v>
@@ -7111,7 +7104,7 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>High jali vent to the sitting area, above the bed head (cross-ventilation with W12 and W03)</t>
+          <t>High jali vent to the sitting area (cross-ventilation with W12 and W03)</t>
         </is>
       </c>
       <c r="I15" s="8" t="inlineStr"/>
@@ -7289,7 +7282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -7823,7 +7816,7 @@
         <v>1</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="G12" s="4" t="n">
         <v>2</v>
@@ -7887,36 +7880,36 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>F16</t>
+          <t>F54</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Common bath</t>
+          <t>Master bedroom</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>WC (EWC)</t>
+          <t>Window seat / diwan 5' x 2' under the north window, drawers below</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Sanitary / plumbing</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E14" s="4" t="n">
-        <v>1.7</v>
+        <v>5</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="G14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Wall-hung on the wet wall shared with the wet area, concealed cistern</t>
+          <t>Teak, cotton cushion</t>
         </is>
       </c>
       <c r="I14" s="10" t="n"/>
@@ -7930,7 +7923,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>F17</t>
+          <t>F16</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -7940,7 +7933,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Wash basin</t>
+          <t>WC (EWC), 17 in clear to the north wall</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -7949,7 +7942,7 @@
         </is>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.7</v>
+        <v>1.7</v>
       </c>
       <c r="F15" s="4" t="n">
         <v>1.2</v>
@@ -7959,7 +7952,7 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Wall-hung</t>
+          <t>Wall-hung on the wet wall shared with the wet area, concealed cistern</t>
         </is>
       </c>
       <c r="I15" s="10" t="n"/>
@@ -7973,7 +7966,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>F18</t>
+          <t>F17</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -7983,7 +7976,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Shower glass partition (3 x 3 ft shower in the south-west corner)</t>
+          <t>Wash basin</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -7992,17 +7985,17 @@
         </is>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.15</v>
+        <v>0.7</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>2.6</v>
+        <v>1.2</v>
       </c>
       <c r="G16" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>8 mm toughened glass</t>
+          <t>Wall-hung</t>
         </is>
       </c>
       <c r="I16" s="10" t="n"/>
@@ -8016,17 +8009,17 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>F48</t>
+          <t>F18</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Bath 2</t>
+          <t>Common bath</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>WC (EWC)</t>
+          <t>Shower glass partition (3 x 3 ft shower in the south-west corner)</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -8035,17 +8028,17 @@
         </is>
       </c>
       <c r="E17" s="4" t="n">
-        <v>1.2</v>
+        <v>0.15</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>1.8</v>
+        <v>2.6</v>
       </c>
       <c r="G17" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Wall-hung on the north (outer) wall, concealed cistern</t>
+          <t>8 mm toughened glass</t>
         </is>
       </c>
       <c r="I17" s="10" t="n"/>
@@ -8059,7 +8052,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>F49</t>
+          <t>F48</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -8069,7 +8062,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Wash basin</t>
+          <t>WC (EWC), 15 in clear each side of its centre</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -8078,17 +8071,17 @@
         </is>
       </c>
       <c r="E18" s="4" t="n">
-        <v>0.7</v>
+        <v>1.2</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="G18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Wall-hung on the wet wall</t>
+          <t>Wall-hung on the north (outer) wall, concealed cistern</t>
         </is>
       </c>
       <c r="I18" s="10" t="n"/>
@@ -8102,7 +8095,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>F50</t>
+          <t>F49</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -8112,7 +8105,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Shower glass partition (shower in the north-east corner)</t>
+          <t>Wash basin (south wall)</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -8121,17 +8114,17 @@
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>0.15</v>
+        <v>1.5</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>2.4</v>
+        <v>0.7</v>
       </c>
       <c r="G19" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>8 mm toughened glass</t>
+          <t>Wall-hung on the wet wall</t>
         </is>
       </c>
       <c r="I19" s="10" t="n"/>
@@ -8145,17 +8138,17 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>F20</t>
+          <t>F50</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Bedroom 2</t>
+          <t>Bath 2</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Queen bed 5' x 6'6" + headboard, head to the south wall</t>
+          <t>Fixed glass splash panel at the south edge of the 3' x 2'-9" wet zone (north-east), beside the door</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -8164,17 +8157,17 @@
         </is>
       </c>
       <c r="E20" s="4" t="n">
-        <v>5</v>
+        <v>1.5</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>6.4</v>
+        <v>0.15</v>
       </c>
       <c r="G20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Teak</t>
+          <t>8 mm toughened glass</t>
         </is>
       </c>
       <c r="I20" s="10" t="n"/>
@@ -8188,7 +8181,7 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>F51</t>
+          <t>F20</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -8198,7 +8191,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Bedside table</t>
+          <t>Queen bed 5' x 6'6" + headboard, head to the west wall, between the bath and the sitting area (1'-6" each side)</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -8207,13 +8200,13 @@
         </is>
       </c>
       <c r="E21" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G21" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="F21" s="4" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="G21" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
@@ -8231,7 +8224,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>F22</t>
+          <t>F51</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -8241,7 +8234,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Work table 4' x 2' with monitor (against the bath wall)</t>
+          <t>Bedside table</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -8250,17 +8243,17 @@
         </is>
       </c>
       <c r="E22" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G22" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F22" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="G22" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Teak / ply, cable tray, monitor arm</t>
+          <t>Teak</t>
         </is>
       </c>
       <c r="I22" s="10" t="n"/>
@@ -8274,7 +8267,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>F23</t>
+          <t>F22</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -8284,7 +8277,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Built-in wardrobe 6' (east wall, toward the house centre)</t>
+          <t>Work table 4' x 2' with monitor (east wall, south of the wardrobe)</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -8293,17 +8286,17 @@
         </is>
       </c>
       <c r="E23" s="4" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G23" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate</t>
+          <t>Teak / ply, cable tray, monitor arm</t>
         </is>
       </c>
       <c r="I23" s="10" t="n"/>
@@ -8317,36 +8310,36 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>F24</t>
+          <t>F23</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Bedroom 2</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Dining table 5' x 3', 6-seat</t>
+          <t>Built-in wardrobe 6' (east wall, toward the house centre)</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E24" s="4" t="n">
-        <v>5</v>
+        <v>1.8</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G24" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Teak or rosewood</t>
+          <t>Ply + laminate</t>
         </is>
       </c>
       <c r="I24" s="10" t="n"/>
@@ -8360,7 +8353,7 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F24</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -8370,7 +8363,7 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Dining chair</t>
+          <t>Dining table 5' x 3', 6-seat</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -8379,17 +8372,17 @@
         </is>
       </c>
       <c r="E25" s="4" t="n">
-        <v>1.1</v>
+        <v>5</v>
       </c>
       <c r="F25" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G25" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G25" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Teak + cane</t>
+          <t>Teak or rosewood</t>
         </is>
       </c>
       <c r="I25" s="10" t="n"/>
@@ -8403,36 +8396,36 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>F26</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Pooja</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Pooja mandapam on the east wall (idols face west; family faces east)</t>
+          <t>Dining chair</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E26" s="4" t="n">
-        <v>0.6</v>
+        <v>1.1</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Carved teak</t>
+          <t>Teak + cane</t>
         </is>
       </c>
       <c r="I26" s="10" t="n"/>
@@ -8446,36 +8439,36 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>F28</t>
+          <t>F26</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area</t>
+          <t>Pooja</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Built-in bench with storage drawers below</t>
+          <t>Pooja mandapam on the east wall (idols face west; family faces east)</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E27" s="4" t="n">
-        <v>1.5</v>
+        <v>0.6</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="G27" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Teak top, ply drawers, on legs</t>
+          <t>Carved teak</t>
         </is>
       </c>
       <c r="I27" s="10" t="n"/>
@@ -8489,36 +8482,36 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>F29</t>
+          <t>F28</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Wet area</t>
+          <t>Sitting and serving area</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Utility sink counter (on the kitchen wall)</t>
+          <t>Built-in bench with storage drawers below</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Sanitary / plumbing</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E28" s="4" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="G28" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Kadappa / granite, SS sinks</t>
+          <t>Teak top, ply drawers, on legs</t>
         </is>
       </c>
       <c r="I28" s="10" t="n"/>
@@ -8532,7 +8525,7 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>F30</t>
+          <t>F29</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -8542,26 +8535,26 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Washing machine bay 2' x 2' (covered back corner, 2 in clear of the bath wall)</t>
+          <t>Utility sink counter (on the kitchen wall)</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Appliance / joinery</t>
+          <t>Sanitary / plumbing</t>
         </is>
       </c>
       <c r="E29" s="4" t="n">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>1.9</v>
+        <v>2.5</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>Splash-proof socket, floor drain</t>
+          <t>Kadappa / granite, SS sinks</t>
         </is>
       </c>
       <c r="I29" s="10" t="n"/>
@@ -8575,7 +8568,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>F31</t>
+          <t>F30</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -8585,26 +8578,26 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Fold-away clothesline in the south walkway</t>
+          <t>Washing machine bay 2' x 2' (covered back corner, 2 in clear of the bath wall)</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Appliance / joinery</t>
         </is>
       </c>
       <c r="E30" s="4" t="n">
-        <v>4</v>
+        <v>1.9</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="G30" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>SS wire, wall brackets</t>
+          <t>Splash-proof socket, floor drain</t>
         </is>
       </c>
       <c r="I30" s="10" t="n"/>
@@ -8618,7 +8611,7 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>F44</t>
+          <t>F31</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -8628,26 +8621,26 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Tall slim utility cupboard (brooms, mops, detergents)</t>
+          <t>Fold-away clothesline in the south walkway</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E31" s="4" t="n">
-        <v>1.2</v>
+        <v>4</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate on legs, louvred doors</t>
+          <t>SS wire, wall brackets</t>
         </is>
       </c>
       <c r="I31" s="10" t="n"/>
@@ -8661,36 +8654,36 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>F32</t>
+          <t>F44</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area</t>
+          <t>Wet area</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Counter-top wash basin at the west end of the serving counter</t>
+          <t>Tall slim utility cupboard (brooms, mops, detergents)</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Sanitary / plumbing</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E32" s="4" t="n">
-        <v>1.9</v>
+        <v>1.2</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="G32" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>Ceramic basin in granite top</t>
+          <t>Ply + laminate on legs, louvred doors</t>
         </is>
       </c>
       <c r="I32" s="10" t="n"/>
@@ -8704,7 +8697,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>F33</t>
+          <t>F32</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -8714,16 +8707,16 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Serving counter with crockery cabinets above, 6 ft</t>
+          <t>Counter-top wash basin at the west end of the serving counter</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Sanitary / plumbing</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
-        <v>6</v>
+        <v>1.9</v>
       </c>
       <c r="F33" s="4" t="n">
         <v>2</v>
@@ -8733,7 +8726,7 @@
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Granite top, teak + glass shutters</t>
+          <t>Ceramic basin in granite top</t>
         </is>
       </c>
       <c r="I33" s="10" t="n"/>
@@ -8747,17 +8740,17 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>F34</t>
+          <t>F33</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Sitting and serving area</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>L-counter, south run</t>
+          <t>Serving counter with crockery cabinets above, 6 ft</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -8766,7 +8759,7 @@
         </is>
       </c>
       <c r="E34" s="4" t="n">
-        <v>13.2</v>
+        <v>6</v>
       </c>
       <c r="F34" s="4" t="n">
         <v>2</v>
@@ -8776,7 +8769,7 @@
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>Granite top, ply carcass</t>
+          <t>Granite top, teak + glass shutters</t>
         </is>
       </c>
       <c r="I34" s="10" t="n"/>
@@ -8790,7 +8783,7 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F34</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -8800,7 +8793,7 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>L-counter, east run (hob)</t>
+          <t>L-counter, south run</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -8809,17 +8802,17 @@
         </is>
       </c>
       <c r="E35" s="4" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="F35" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="F35" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>Granite top, cook faces east</t>
+          <t>Granite top, ply carcass</t>
         </is>
       </c>
       <c r="I35" s="10" t="n"/>
@@ -8833,7 +8826,7 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>F36</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -8843,26 +8836,26 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Refrigerator space (kitchen north wall, behind the pooja, door facing south)</t>
+          <t>L-counter, east run (hob centred 7'-6" from the south wall face, on solid wall)</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Appliance / joinery</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E36" s="4" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>2.4</v>
+        <v>7</v>
       </c>
       <c r="G36" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>Double-door, 2'6" wide</t>
+          <t>Granite top, cook faces east</t>
         </is>
       </c>
       <c r="I36" s="10" t="n"/>
@@ -8876,36 +8869,36 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>F38</t>
+          <t>F36</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Three-seat sofa 6'6" facing the TV</t>
+          <t>Refrigerator space (kitchen north wall, behind the pooja, door facing south)</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Appliance / joinery</t>
         </is>
       </c>
       <c r="E37" s="4" t="n">
-        <v>2.7</v>
+        <v>2.5</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>6.3</v>
+        <v>2.4</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>Teak frame, cotton cushions</t>
+          <t>Double-door, 2'6" wide</t>
         </is>
       </c>
       <c r="I37" s="10" t="n"/>
@@ -8919,17 +8912,17 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>F39</t>
+          <t>F55</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Coffee table 3'6" x 2'</t>
+          <t>Tall pantry 4'-5" x 2' on the north wall (provisions, rice, vessels)</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -8938,17 +8931,17 @@
         </is>
       </c>
       <c r="E38" s="4" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F38" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="F38" s="4" t="n">
-        <v>3.3</v>
       </c>
       <c r="G38" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Teak</t>
+          <t>Ply + laminate, full height with loft</t>
         </is>
       </c>
       <c r="I38" s="10" t="n"/>
@@ -8962,17 +8955,17 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>F40</t>
+          <t>F38</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Dining bay</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Armchair by the north window</t>
+          <t>Three-seat sofa 6'6" facing west to the TV</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -8981,17 +8974,17 @@
         </is>
       </c>
       <c r="E39" s="4" t="n">
-        <v>2</v>
+        <v>2.7</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>1.6</v>
+        <v>5.9</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Cane / teak</t>
+          <t>Teak frame, cotton cushions</t>
         </is>
       </c>
       <c r="I39" s="10" t="n"/>
@@ -9005,36 +8998,36 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>F52</t>
+          <t>F39</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Dining bay</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Shoe cupboard 3'-3" beside the main door (closed shutters, louvred for air)</t>
+          <t>Coffee table 3'6" x 2'</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E40" s="4" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>3.2</v>
+        <v>3.5</v>
       </c>
       <c r="G40" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate, 14 in deep</t>
+          <t>Teak</t>
         </is>
       </c>
       <c r="I40" s="10" t="n"/>
@@ -9048,36 +9041,36 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>F41</t>
+          <t>F53</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Poomukham (verandah)</t>
+          <t>Dining bay</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Oonjal (swing) 3'6"</t>
+          <t>TV unit 4'-5" on Bedroom 2's east wall (55-65 in TV wall-mounted above)</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Appliance / joinery</t>
         </is>
       </c>
       <c r="E41" s="4" t="n">
-        <v>3.5</v>
+        <v>1.3</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>1.5</v>
+        <v>4.4</v>
       </c>
       <c r="G41" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>Teak, chains to beam</t>
+          <t>Teak, low, open shelves</t>
         </is>
       </c>
       <c r="I41" s="10" t="n"/>
@@ -9091,36 +9084,36 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>F42</t>
+          <t>F40</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Poomukham (verandah)</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Arugu seat (built-in, south end)</t>
+          <t>Armchair by the north window</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E42" s="4" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
       <c r="G42" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>Laterite base, teak top</t>
+          <t>Cane / teak</t>
         </is>
       </c>
       <c r="I42" s="10" t="n"/>
@@ -9132,28 +9125,157 @@
       <c r="L42" s="8" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="inlineStr"/>
-      <c r="B43" s="6" t="inlineStr"/>
-      <c r="C43" s="6" t="inlineStr">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>F52</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Living</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Shoe cupboard 3'-3" beside the main door (closed shutters, louvred for air)</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Built-in joinery</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>Ply + laminate, 14 in deep</t>
+        </is>
+      </c>
+      <c r="I43" s="10" t="n"/>
+      <c r="J43" s="11">
+        <f>G43*I43</f>
+        <v/>
+      </c>
+      <c r="K43" s="8" t="inlineStr"/>
+      <c r="L43" s="8" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>F41</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Poomukham (verandah)</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Oonjal (swing) 3'6"</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Loose furniture</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F44" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G44" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>Teak, chains to beam</t>
+        </is>
+      </c>
+      <c r="I44" s="10" t="n"/>
+      <c r="J44" s="11">
+        <f>G44*I44</f>
+        <v/>
+      </c>
+      <c r="K44" s="8" t="inlineStr"/>
+      <c r="L44" s="8" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>F42</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Poomukham (verandah)</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Arugu seat (built-in, south end)</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Built-in joinery</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F45" s="4" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>Laterite base, teak top</t>
+        </is>
+      </c>
+      <c r="I45" s="10" t="n"/>
+      <c r="J45" s="11">
+        <f>G45*I45</f>
+        <v/>
+      </c>
+      <c r="K45" s="8" t="inlineStr"/>
+      <c r="L45" s="8" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr"/>
+      <c r="B46" s="6" t="inlineStr"/>
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D43" s="6" t="inlineStr"/>
-      <c r="E43" s="6" t="inlineStr"/>
-      <c r="F43" s="6" t="inlineStr"/>
-      <c r="G43" s="6">
-        <f>SUM(G2:G42)</f>
+      <c r="D46" s="6" t="inlineStr"/>
+      <c r="E46" s="6" t="inlineStr"/>
+      <c r="F46" s="6" t="inlineStr"/>
+      <c r="G46" s="6">
+        <f>SUM(G2:G45)</f>
         <v/>
       </c>
-      <c r="H43" s="6" t="inlineStr"/>
-      <c r="I43" s="12" t="inlineStr"/>
-      <c r="J43" s="12">
-        <f>SUM(J2:J42)</f>
+      <c r="H46" s="6" t="inlineStr"/>
+      <c r="I46" s="12" t="inlineStr"/>
+      <c r="J46" s="12">
+        <f>SUM(J2:J45)</f>
         <v/>
       </c>
-      <c r="K43" s="6" t="inlineStr"/>
-      <c r="L43" s="6" t="inlineStr"/>
+      <c r="K46" s="6" t="inlineStr"/>
+      <c r="L46" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10260,7 +10382,7 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>21.64</v>
+        <v>22.35</v>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
@@ -10290,7 +10412,7 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>2.86</v>
+        <v>3.47</v>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
@@ -10320,7 +10442,7 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>6.3</v>
+        <v>6.02</v>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
@@ -10350,7 +10472,7 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>87.2</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
@@ -10380,7 +10502,7 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>272.7</v>
+        <v>278.7</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
@@ -10410,7 +10532,7 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>139.3</v>
+        <v>142.9</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
@@ -10470,7 +10592,7 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>9.6</v>
+        <v>10.3</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
@@ -10800,7 +10922,7 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>11.9</v>
+        <v>13.8</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
@@ -10830,7 +10952,7 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>7.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
@@ -11070,7 +11192,7 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
@@ -11130,7 +11252,7 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>24.2</v>
+        <v>22.5</v>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
@@ -11172,7 +11294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G110"/>
+  <dimension ref="A1:G113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -11867,12 +11989,16 @@
         </is>
       </c>
       <c r="E22" s="4" t="n">
-        <v>16.25</v>
+        <v>17.4</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="G22" s="4" t="inlineStr"/>
+        <v>14.7</v>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>over the bed</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -12019,7 +12145,7 @@
         <v>20.6</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>21.6</v>
+        <v>18</v>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
@@ -12052,7 +12178,7 @@
         <v>20.6</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>15.4</v>
+        <v>11.6</v>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
@@ -12085,7 +12211,7 @@
         <v>20.6</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>22.2</v>
+        <v>17.6</v>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
@@ -12118,11 +12244,11 @@
         <v>11.9</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>22.5</v>
+        <v>18</v>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>west wall, throws toward the bed foot, not the head</t>
+          <t>west wall, throws along the bed, not on the head</t>
         </is>
       </c>
     </row>
@@ -12181,10 +12307,10 @@
         </is>
       </c>
       <c r="E32" s="4" t="n">
-        <v>23.5</v>
+        <v>24.5</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>21.5</v>
+        <v>21.8</v>
       </c>
       <c r="G32" s="4" t="inlineStr"/>
     </row>
@@ -12210,7 +12336,7 @@
         </is>
       </c>
       <c r="E33" s="4" t="n">
-        <v>24.6</v>
+        <v>25.6</v>
       </c>
       <c r="F33" s="4" t="n">
         <v>24.6</v>
@@ -12243,14 +12369,14 @@
         </is>
       </c>
       <c r="E34" s="4" t="n">
-        <v>26.1</v>
+        <v>27.6</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>23</v>
+        <v>23.6</v>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>over shower</t>
+          <t>over shower, east wall</t>
         </is>
       </c>
     </row>
@@ -12276,10 +12402,10 @@
         </is>
       </c>
       <c r="E35" s="4" t="n">
-        <v>26.1</v>
+        <v>25.3</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>21.6</v>
+        <v>19.4</v>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
@@ -12309,10 +12435,10 @@
         </is>
       </c>
       <c r="E36" s="4" t="n">
-        <v>24.8</v>
+        <v>28.4</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>18.8</v>
+        <v>22.2</v>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
@@ -12656,14 +12782,14 @@
         </is>
       </c>
       <c r="E47" s="4" t="n">
-        <v>41.2</v>
+        <v>39.8</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>3.4</v>
+        <v>4.5</v>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>over shower</t>
+          <t>over shower, west wall (clear of the window)</t>
         </is>
       </c>
     </row>
@@ -12755,10 +12881,10 @@
         </is>
       </c>
       <c r="E50" s="4" t="n">
-        <v>31</v>
+        <v>29.5</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>17.5</v>
+        <v>15.5</v>
       </c>
       <c r="G50" s="4" t="inlineStr"/>
     </row>
@@ -12784,10 +12910,10 @@
         </is>
       </c>
       <c r="E51" s="4" t="n">
-        <v>31</v>
+        <v>21.4</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>10.9</v>
+        <v>14.7</v>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
@@ -12817,10 +12943,10 @@
         </is>
       </c>
       <c r="E52" s="4" t="n">
-        <v>23.5</v>
+        <v>31</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G52" s="4" t="inlineStr"/>
     </row>
@@ -12875,14 +13001,14 @@
         </is>
       </c>
       <c r="E54" s="4" t="n">
-        <v>24.9</v>
+        <v>31.2</v>
       </c>
       <c r="F54" s="4" t="n">
         <v>10.9</v>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>at door</t>
+          <t>at the door, 2-way</t>
         </is>
       </c>
     </row>
@@ -12908,10 +13034,10 @@
         </is>
       </c>
       <c r="E55" s="4" t="n">
-        <v>34.4</v>
+        <v>21.4</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>10.9</v>
+        <v>11.9</v>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
@@ -12941,10 +13067,10 @@
         </is>
       </c>
       <c r="E56" s="4" t="n">
-        <v>34</v>
+        <v>21.4</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>10.9</v>
+        <v>11.2</v>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
@@ -12974,31 +13100,31 @@
         </is>
       </c>
       <c r="E57" s="4" t="n">
-        <v>28</v>
+        <v>21.4</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>10.9</v>
+        <v>18</v>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>bedside</t>
+          <t>bedside, north</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -13007,26 +13133,26 @@
         </is>
       </c>
       <c r="E58" s="4" t="n">
-        <v>26.9</v>
+        <v>21.4</v>
       </c>
       <c r="F58" s="4" t="n">
-        <v>20</v>
+        <v>18.5</v>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>work table</t>
+          <t>bedside, north, 2-way</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Inverter (UPS) socket</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -13040,26 +13166,26 @@
         </is>
       </c>
       <c r="E59" s="4" t="n">
-        <v>26.9</v>
+        <v>35.6</v>
       </c>
       <c r="F59" s="4" t="n">
-        <v>20.8</v>
+        <v>15</v>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>work table, monitor</t>
+          <t>work table</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Data point (Cat6)</t>
+          <t>Inverter (UPS) socket</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -13073,26 +13199,26 @@
         </is>
       </c>
       <c r="E60" s="4" t="n">
-        <v>26.9</v>
+        <v>35.6</v>
       </c>
       <c r="F60" s="4" t="n">
-        <v>21.6</v>
+        <v>15.8</v>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>work table</t>
+          <t>work table, monitor</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Inverter (UPS) socket</t>
+          <t>Data point (Cat6)</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -13106,10 +13232,10 @@
         </is>
       </c>
       <c r="E61" s="4" t="n">
-        <v>26.9</v>
+        <v>35.6</v>
       </c>
       <c r="F61" s="4" t="n">
-        <v>22.4</v>
+        <v>16.6</v>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
@@ -13120,17 +13246,17 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
+          <t>Inverter (UPS) socket</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>7'-6"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -13142,123 +13268,127 @@
         <v>35.6</v>
       </c>
       <c r="F62" s="4" t="n">
-        <v>18.6</v>
+        <v>17.4</v>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>east wall, not at the work table</t>
+          <t>work table</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>7'-6"</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area (open)</t>
+          <t>Bedroom 2</t>
         </is>
       </c>
       <c r="E63" s="4" t="n">
-        <v>32.2</v>
+        <v>35.6</v>
       </c>
       <c r="F63" s="4" t="n">
-        <v>3.4</v>
+        <v>18.6</v>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>over basin</t>
+          <t>east wall, not at the work table</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>ODU</t>
+          <t>WL</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>AC outdoor unit bracket</t>
+          <t>Wall light / mirror light</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>7'-0" outside</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>Bedroom 2</t>
+          <t>Sitting and serving area (open)</t>
         </is>
       </c>
       <c r="E64" s="4" t="n">
-        <v>31</v>
+        <v>32.2</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>25.6</v>
+        <v>3.4</v>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>north wall, shaded</t>
+          <t>over basin</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>ODU</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>AC outdoor unit bracket</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>7'-0" outside</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Dining bay (north window)</t>
+          <t>Bedroom 2</t>
         </is>
       </c>
       <c r="E65" s="4" t="n">
-        <v>42.5</v>
+        <v>31</v>
       </c>
       <c r="F65" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="G65" s="4" t="inlineStr"/>
+        <v>25.6</v>
+      </c>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t>north wall, shaded</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -13267,22 +13397,22 @@
         </is>
       </c>
       <c r="E66" s="4" t="n">
-        <v>46.6</v>
+        <v>39.5</v>
       </c>
       <c r="F66" s="4" t="n">
-        <v>24.6</v>
+        <v>21.5</v>
       </c>
       <c r="G66" s="4" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Ceiling fan point</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -13292,295 +13422,303 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Dining bay (north window)</t>
         </is>
       </c>
       <c r="E67" s="4" t="n">
-        <v>42.5</v>
+        <v>43</v>
       </c>
       <c r="F67" s="4" t="n">
-        <v>15</v>
+        <v>21.5</v>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>pendant</t>
+          <t>long downrod, over the seating</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Dining bay (north window)</t>
         </is>
       </c>
       <c r="E68" s="4" t="n">
-        <v>36.4</v>
+        <v>46.6</v>
       </c>
       <c r="F68" s="4" t="n">
-        <v>17.5</v>
+        <v>24.6</v>
       </c>
       <c r="G68" s="4" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>TV</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>TV + data point</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Dining bay (north window)</t>
         </is>
       </c>
       <c r="E69" s="4" t="n">
         <v>36.4</v>
       </c>
       <c r="F69" s="4" t="n">
-        <v>16.2</v>
-      </c>
-      <c r="G69" s="4" t="inlineStr"/>
+        <v>22.4</v>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>TV wall: 2 sockets + data + HDMI conduit to the unit</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Dining bay (north window)</t>
         </is>
       </c>
       <c r="E70" s="4" t="n">
-        <v>46.6</v>
+        <v>36.4</v>
       </c>
       <c r="F70" s="4" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="G70" s="4" t="inlineStr"/>
+        <v>21</v>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t>TV unit</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>7'-6"</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area (open)</t>
+          <t>Dining bay (north window)</t>
         </is>
       </c>
       <c r="E71" s="4" t="n">
-        <v>28.5</v>
+        <v>36.4</v>
       </c>
       <c r="F71" s="4" t="n">
-        <v>6.75</v>
-      </c>
-      <c r="G71" s="4" t="inlineStr"/>
+        <v>20</v>
+      </c>
+      <c r="G71" s="4" t="inlineStr">
+        <is>
+          <t>above the TV unit, throws east over the seating</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>ODU</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>AC outdoor unit bracket</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>7'-0" outside</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area (open)</t>
+          <t>Dining bay (north window)</t>
         </is>
       </c>
       <c r="E72" s="4" t="n">
-        <v>21.4</v>
+        <v>38</v>
       </c>
       <c r="F72" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="G72" s="4" t="inlineStr"/>
+        <v>25.6</v>
+      </c>
+      <c r="G72" s="4" t="inlineStr">
+        <is>
+          <t>north wall, shaded</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>INV</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Inverter + battery</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>floor</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area (open)</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E73" s="4" t="n">
-        <v>22</v>
+        <v>42.5</v>
       </c>
       <c r="F73" s="4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>lithium inverter in a ventilated cabinet under the bench</t>
+          <t>pendant</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>WL</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Wall light / mirror light</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>Wet area (open to the walkway)</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E74" s="4" t="n">
-        <v>48</v>
+        <v>36.4</v>
       </c>
       <c r="F74" s="4" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="G74" s="4" t="inlineStr">
-        <is>
-          <t>weatherproof</t>
-        </is>
-      </c>
+        <v>17.5</v>
+      </c>
+      <c r="G74" s="4" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>16 A power socket</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>Wet area (open to the walkway)</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E75" s="4" t="n">
-        <v>46.5</v>
+        <v>36.4</v>
       </c>
       <c r="F75" s="4" t="n">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="G75" s="4" t="inlineStr">
-        <is>
-          <t>washing machine</t>
-        </is>
-      </c>
+        <v>16.2</v>
+      </c>
+      <c r="G75" s="4" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>Wet area (open to the walkway)</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E76" s="4" t="n">
-        <v>50.6</v>
+        <v>36.4</v>
       </c>
       <c r="F76" s="4" t="n">
-        <v>6</v>
+        <v>13.7</v>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>utility, weatherproof</t>
+          <t>dining and bay, at the passage</t>
         </is>
       </c>
     </row>
@@ -13602,113 +13740,109 @@
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Sitting and serving area (open)</t>
         </is>
       </c>
       <c r="E77" s="4" t="n">
-        <v>60</v>
+        <v>28.5</v>
       </c>
       <c r="F77" s="4" t="n">
-        <v>8</v>
+        <v>6.75</v>
       </c>
       <c r="G77" s="4" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Sitting and serving area (open)</t>
         </is>
       </c>
       <c r="E78" s="4" t="n">
-        <v>59</v>
+        <v>21.4</v>
       </c>
       <c r="F78" s="4" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="G78" s="4" t="inlineStr">
-        <is>
-          <t>under-cabinet</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="G78" s="4" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>INV</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>Inverter + battery</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>floor</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Sitting and serving area (open)</t>
         </is>
       </c>
       <c r="E79" s="4" t="n">
-        <v>64.5</v>
+        <v>22</v>
       </c>
       <c r="F79" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>under-cabinet</t>
+          <t>lithium inverter in a ventilated cabinet under the bench</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Kitchen chimney point (16 A)</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>7'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Wet area (open to the walkway)</t>
         </is>
       </c>
       <c r="E80" s="4" t="n">
-        <v>64.59999999999999</v>
+        <v>48</v>
       </c>
       <c r="F80" s="4" t="n">
-        <v>8.75</v>
+        <v>5.5</v>
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>duct out through east wall</t>
+          <t>weatherproof</t>
         </is>
       </c>
     </row>
@@ -13730,64 +13864,68 @@
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Wet area (open to the walkway)</t>
         </is>
       </c>
       <c r="E81" s="4" t="n">
-        <v>56.75</v>
+        <v>46.5</v>
       </c>
       <c r="F81" s="4" t="n">
-        <v>12.7</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>refrigerator, behind the fridge</t>
+          <t>washing machine</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>6 A socket at counter</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Wet area (open to the walkway)</t>
         </is>
       </c>
       <c r="E82" s="4" t="n">
-        <v>52.5</v>
+        <v>50.6</v>
       </c>
       <c r="F82" s="4" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="G82" s="4" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>utility, weatherproof</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>6 A socket at counter</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
@@ -13796,31 +13934,27 @@
         </is>
       </c>
       <c r="E83" s="4" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="F83" s="4" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="G83" s="4" t="inlineStr">
-        <is>
-          <t>microwave / OTG</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="G83" s="4" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>WL</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>6 A socket at counter</t>
+          <t>Wall light / mirror light</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -13829,31 +13963,31 @@
         </is>
       </c>
       <c r="E84" s="4" t="n">
-        <v>61.5</v>
+        <v>59</v>
       </c>
       <c r="F84" s="4" t="n">
         <v>3.5</v>
       </c>
       <c r="G84" s="4" t="inlineStr">
         <is>
-          <t>mixer</t>
+          <t>under-cabinet</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>WL</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>6 A socket at counter</t>
+          <t>Wall light / mirror light</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
@@ -13862,27 +13996,31 @@
         </is>
       </c>
       <c r="E85" s="4" t="n">
-        <v>64.59999999999999</v>
+        <v>64.5</v>
       </c>
       <c r="F85" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="G85" s="4" t="inlineStr"/>
+        <v>9.6</v>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>under-cabinet</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>6 A socket at counter</t>
+          <t>Kitchen chimney point (16 A)</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>7'-0"</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -13894,24 +14032,28 @@
         <v>64.59999999999999</v>
       </c>
       <c r="F86" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="G86" s="4" t="inlineStr"/>
+        <v>7.5</v>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>3 ft chimney on solid wall, duct out through the east wall</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>6 A socket at counter</t>
+          <t>16 A power socket</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>varies</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -13920,31 +14062,31 @@
         </is>
       </c>
       <c r="E87" s="4" t="n">
-        <v>57.3</v>
+        <v>56.75</v>
       </c>
       <c r="F87" s="4" t="n">
-        <v>3.5</v>
+        <v>12.7</v>
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>RO purifier, by sink</t>
+          <t>refrigerator, behind the fridge</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>6 A socket at counter</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -13953,217 +14095,217 @@
         </is>
       </c>
       <c r="E88" s="4" t="n">
-        <v>51.4</v>
+        <v>52.5</v>
       </c>
       <c r="F88" s="4" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="G88" s="4" t="inlineStr">
-        <is>
-          <t>beside the sliding entry</t>
-        </is>
-      </c>
+        <v>3.5</v>
+      </c>
+      <c r="G88" s="4" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>Ceiling fan point</t>
+          <t>6 A socket at counter</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="E89" s="4" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F89" s="4" t="n">
-        <v>19</v>
+        <v>3.5</v>
       </c>
       <c r="G89" s="4" t="inlineStr">
         <is>
-          <t>long downrod</t>
+          <t>microwave / OTG</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>6 A socket at counter</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="E90" s="4" t="n">
-        <v>50</v>
+        <v>61.5</v>
       </c>
       <c r="F90" s="4" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="G90" s="4" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="G90" s="4" t="inlineStr">
+        <is>
+          <t>mixer</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>6 A socket at counter</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="E91" s="4" t="n">
-        <v>53</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="F91" s="4" t="n">
-        <v>16</v>
+        <v>5.6</v>
       </c>
       <c r="G91" s="4" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>6 A socket at counter</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="E92" s="4" t="n">
-        <v>47.4</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="F92" s="4" t="n">
-        <v>24.2</v>
+        <v>9.6</v>
       </c>
       <c r="G92" s="4" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>6 A socket at counter</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="E93" s="4" t="n">
-        <v>47.4</v>
+        <v>57.3</v>
       </c>
       <c r="F93" s="4" t="n">
-        <v>18</v>
+        <v>3.5</v>
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>sofa</t>
+          <t>RO purifier, by sink</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="E94" s="4" t="n">
-        <v>50.6</v>
+        <v>51.4</v>
       </c>
       <c r="F94" s="4" t="n">
-        <v>17.8</v>
+        <v>9</v>
       </c>
       <c r="G94" s="4" t="inlineStr">
         <is>
-          <t>floor socket, sofa end</t>
+          <t>beside the entry, latch side</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
+          <t>Ceiling fan point</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>7'-6"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
@@ -14172,31 +14314,31 @@
         </is>
       </c>
       <c r="E95" s="4" t="n">
-        <v>47.4</v>
+        <v>53</v>
       </c>
       <c r="F95" s="4" t="n">
-        <v>21.5</v>
+        <v>19</v>
       </c>
       <c r="G95" s="4" t="inlineStr">
         <is>
-          <t>west wall</t>
+          <t>long downrod</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>ODU</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>AC outdoor unit bracket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>7'-0" outside</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
@@ -14205,31 +14347,27 @@
         </is>
       </c>
       <c r="E96" s="4" t="n">
-        <v>57.5</v>
+        <v>50</v>
       </c>
       <c r="F96" s="4" t="n">
-        <v>25.6</v>
-      </c>
-      <c r="G96" s="4" t="inlineStr">
-        <is>
-          <t>north wall, shaded</t>
-        </is>
-      </c>
+        <v>22.5</v>
+      </c>
+      <c r="G96" s="4" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
@@ -14238,59 +14376,55 @@
         </is>
       </c>
       <c r="E97" s="4" t="n">
-        <v>58.6</v>
+        <v>53</v>
       </c>
       <c r="F97" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="G97" s="4" t="inlineStr">
-        <is>
-          <t>main switch at door</t>
-        </is>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="G97" s="4" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Distribution board</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>5'-0" to top</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Dining bay (north window)</t>
         </is>
       </c>
       <c r="E98" s="4" t="n">
-        <v>48</v>
+        <v>46.2</v>
       </c>
       <c r="F98" s="4" t="n">
-        <v>9.4</v>
+        <v>18.4</v>
       </c>
       <c r="G98" s="4" t="inlineStr">
         <is>
-          <t>alcove between the dining and the kitchen, near the entry, off the pooja wall</t>
+          <t>floor socket, sofa end</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>Inverter (UPS) socket</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
@@ -14300,122 +14434,134 @@
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="E99" s="4" t="n">
-        <v>49.6</v>
+        <v>50.6</v>
       </c>
       <c r="F99" s="4" t="n">
-        <v>9.4</v>
+        <v>17.8</v>
       </c>
       <c r="G99" s="4" t="inlineStr">
         <is>
-          <t>router</t>
+          <t>floor socket, armchair</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>Poomukham (verandah)</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="E100" s="4" t="n">
-        <v>62</v>
+        <v>58.6</v>
       </c>
       <c r="F100" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="G100" s="4" t="inlineStr"/>
+        <v>21</v>
+      </c>
+      <c r="G100" s="4" t="inlineStr">
+        <is>
+          <t>main switch at door</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Distribution board</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>5'-0" to top</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>Poomukham (verandah)</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E101" s="4" t="n">
-        <v>62</v>
+        <v>36.4</v>
       </c>
       <c r="F101" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="G101" s="4" t="inlineStr"/>
+        <v>12.6</v>
+      </c>
+      <c r="G101" s="4" t="inlineStr">
+        <is>
+          <t>dining face of Bedroom 2's east wall, by the passage; dry wall away from the pooja and wet area</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>BELL</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Bell push</t>
+          <t>Inverter (UPS) socket</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>4'-6"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>Poomukham (verandah)</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E102" s="4" t="n">
-        <v>59.4</v>
+        <v>36.4</v>
       </c>
       <c r="F102" s="4" t="n">
-        <v>20.4</v>
-      </c>
-      <c r="G102" s="4" t="inlineStr"/>
+        <v>14.6</v>
+      </c>
+      <c r="G102" s="4" t="inlineStr">
+        <is>
+          <t>router (central)</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>CAM</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>CCTV point</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>8'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
@@ -14424,31 +14570,27 @@
         </is>
       </c>
       <c r="E103" s="4" t="n">
-        <v>64.5</v>
+        <v>62</v>
       </c>
       <c r="F103" s="4" t="n">
-        <v>24.6</v>
-      </c>
-      <c r="G103" s="4" t="inlineStr">
-        <is>
-          <t>covers gate and door</t>
-        </is>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="G103" s="4" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
@@ -14457,31 +14599,27 @@
         </is>
       </c>
       <c r="E104" s="4" t="n">
-        <v>59.4</v>
+        <v>62</v>
       </c>
       <c r="F104" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="G104" s="4" t="inlineStr">
-        <is>
-          <t>outdoor, weatherproof</t>
-        </is>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="G104" s="4" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>BELL</t>
         </is>
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>Bell push</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>4'-6"</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
@@ -14493,123 +14631,119 @@
         <v>59.4</v>
       </c>
       <c r="F105" s="4" t="n">
-        <v>20.9</v>
+        <v>20.4</v>
       </c>
       <c r="G105" s="4" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>MTR</t>
+          <t>CAM</t>
         </is>
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>Meter at gate</t>
+          <t>CCTV point</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>5'-0"</t>
+          <t>8'-0"</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>Site</t>
+          <t>Poomukham (verandah)</t>
         </is>
       </c>
       <c r="E106" s="4" t="n">
-        <v>74.59999999999999</v>
+        <v>64.5</v>
       </c>
       <c r="F106" s="4" t="n">
-        <v>23</v>
+        <v>24.6</v>
       </c>
       <c r="G106" s="4" t="inlineStr">
         <is>
-          <t>meter in compound wall by gate</t>
+          <t>covers gate and door</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>GL</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>Outdoor / gate light</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>7'-0"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>Site</t>
+          <t>Poomukham (verandah)</t>
         </is>
       </c>
       <c r="E107" s="4" t="n">
-        <v>74.59999999999999</v>
+        <v>59.4</v>
       </c>
       <c r="F107" s="4" t="n">
-        <v>14.5</v>
+        <v>24</v>
       </c>
       <c r="G107" s="4" t="inlineStr">
         <is>
-          <t>gate light</t>
+          <t>outdoor, weatherproof</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>EP</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>Earth pit</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>ground</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>Site</t>
+          <t>Poomukham (verandah)</t>
         </is>
       </c>
       <c r="E108" s="4" t="n">
-        <v>66.2</v>
+        <v>59.4</v>
       </c>
       <c r="F108" s="4" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G108" s="4" t="inlineStr">
-        <is>
-          <t>earth pit 1</t>
-        </is>
-      </c>
+        <v>20.9</v>
+      </c>
+      <c r="G108" s="4" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>EP</t>
+          <t>MTR</t>
         </is>
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>Earth pit</t>
+          <t>Meter at gate</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>ground</t>
+          <t>5'-0"</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
@@ -14618,14 +14752,14 @@
         </is>
       </c>
       <c r="E109" s="4" t="n">
-        <v>73.5</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="F109" s="4" t="n">
-        <v>1.5</v>
+        <v>23</v>
       </c>
       <c r="G109" s="4" t="inlineStr">
         <is>
-          <t>earth pit 2</t>
+          <t>meter in compound wall by gate</t>
         </is>
       </c>
     </row>
@@ -14651,12 +14785,111 @@
         </is>
       </c>
       <c r="E110" s="4" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="F110" s="4" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="G110" s="4" t="inlineStr">
+        <is>
+          <t>gate light</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t>EP</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
+        <is>
+          <t>Earth pit</t>
+        </is>
+      </c>
+      <c r="C111" s="4" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="E111" s="4" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="F111" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G111" s="4" t="inlineStr">
+        <is>
+          <t>earth pit 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="4" t="inlineStr">
+        <is>
+          <t>EP</t>
+        </is>
+      </c>
+      <c r="B112" s="4" t="inlineStr">
+        <is>
+          <t>Earth pit</t>
+        </is>
+      </c>
+      <c r="C112" s="4" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="E112" s="4" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="F112" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G112" s="4" t="inlineStr">
+        <is>
+          <t>earth pit 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="4" t="inlineStr">
+        <is>
+          <t>GL</t>
+        </is>
+      </c>
+      <c r="B113" s="4" t="inlineStr">
+        <is>
+          <t>Outdoor / gate light</t>
+        </is>
+      </c>
+      <c r="C113" s="4" t="inlineStr">
+        <is>
+          <t>7'-0"</t>
+        </is>
+      </c>
+      <c r="D113" s="4" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="E113" s="4" t="n">
         <v>2.5</v>
       </c>
-      <c r="F110" s="4" t="n">
+      <c r="F113" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="G110" s="4" t="inlineStr">
+      <c r="G113" s="4" t="inlineStr">
         <is>
           <t>rear garden</t>
         </is>

</xml_diff>

<commit_message>
House lengthened to 62 ft for Bedroom 2; sitting-area cupboard and hand-wash basin
Everything east of Bedroom 2's middle moves 2 ft east: Bedroom 2 is 17 ft
wide, the sitting area 20'-6", the front yard 8 ft (setback to confirm).
Sheet, DXF and 3D code with hand-placed positions updated for the new
length. Sitting area gets a tall storage cupboard; the hand-wash basin
moves to the east end of the serving counter, outside the common bath.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Schedules/KH-P1_Schedules_RevB.xlsx
+++ b/03_Schedules/KH-P1_Schedules_RevB.xlsx
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>45.6</v>
+        <v>47.6</v>
       </c>
       <c r="E8" s="4" t="n">
         <v>7.35</v>
@@ -919,7 +919,7 @@
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>45.6</v>
+        <v>47.6</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>6.5</v>
@@ -943,7 +943,7 @@
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>45.6</v>
+        <v>47.6</v>
       </c>
       <c r="E10" s="4" t="n">
         <v>4.8</v>
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>39.8</v>
+        <v>41.8</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>3.9</v>
@@ -999,7 +999,7 @@
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>41.2</v>
+        <v>43.2</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>3.6</v>
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>44.3</v>
+        <v>46.3</v>
       </c>
       <c r="E13" s="4" t="n">
         <v>6</v>
@@ -1219,7 +1219,7 @@
         </is>
       </c>
       <c r="D20" s="4" t="n">
-        <v>49.85</v>
+        <v>51.85</v>
       </c>
       <c r="E20" s="4" t="n">
         <v>4.6</v>
@@ -1247,7 +1247,7 @@
         </is>
       </c>
       <c r="D21" s="4" t="n">
-        <v>47.35</v>
+        <v>49.35</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>7.85</v>
@@ -1271,7 +1271,7 @@
         </is>
       </c>
       <c r="D22" s="4" t="n">
-        <v>47.8</v>
+        <v>49.8</v>
       </c>
       <c r="E22" s="4" t="n">
         <v>3.6</v>
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="D23" s="4" t="n">
-        <v>50.6</v>
+        <v>52.6</v>
       </c>
       <c r="E23" s="4" t="n">
         <v>3.4</v>
@@ -1327,14 +1327,14 @@
         </is>
       </c>
       <c r="D24" s="4" t="n">
-        <v>32.2</v>
+        <v>40.2</v>
       </c>
       <c r="E24" s="4" t="n">
         <v>4.3</v>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>counter basin, waste straight out to the south walkway</t>
+          <t>hand-wash basin outside the common bath, waste straight out to the south walkway</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="D25" s="4" t="n">
-        <v>58.5</v>
+        <v>60.5</v>
       </c>
       <c r="E25" s="4" t="n">
         <v>3.5</v>
@@ -1383,7 +1383,7 @@
         </is>
       </c>
       <c r="D26" s="4" t="n">
-        <v>57.3</v>
+        <v>59.3</v>
       </c>
       <c r="E26" s="4" t="n">
         <v>3.5</v>
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="D27" s="4" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E27" s="4" t="n">
         <v>12.5</v>
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="D28" s="4" t="n">
-        <v>67.59999999999999</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="E28" s="4" t="n">
         <v>13.6</v>
@@ -1491,7 +1491,7 @@
         </is>
       </c>
       <c r="D30" s="4" t="n">
-        <v>70.5</v>
+        <v>71.2</v>
       </c>
       <c r="E30" s="4" t="n">
         <v>22</v>
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="D32" s="4" t="n">
-        <v>44.8</v>
+        <v>46.8</v>
       </c>
       <c r="E32" s="4" t="n">
         <v>1.8</v>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="D35" s="4" t="n">
-        <v>58.5</v>
+        <v>60.5</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>1</v>
@@ -1659,7 +1659,7 @@
         </is>
       </c>
       <c r="D36" s="4" t="n">
-        <v>47.8</v>
+        <v>49.8</v>
       </c>
       <c r="E36" s="4" t="n">
         <v>1</v>
@@ -4382,7 +4382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4425,17 +4425,17 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Layout</t>
+          <t>Land</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>TV on Bedroom 2's east wall facing the dining bay: confirm screen size (55-65 in at about 9 ft) and a concealed HDMI/data conduit from the unit</t>
+          <t>Front yard is now 8 ft (house 62 ft long): confirm the front setback allowed for this plot and road width before finalising; fall back to a 60 ft house if 10 ft is required</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Architect</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
@@ -4450,17 +4450,17 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Land</t>
+          <t>Layout</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Agricultural land: confirm conversion to non-agricultural use with the gram panchayat / collector (AP repealed the NALA Act in 2025; new process to be confirmed)</t>
+          <t>TV on Bedroom 2's east wall facing the dining bay: confirm screen size (55-65 in at about 9 ft) and a concealed HDMI/data conduit from the unit</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Owner / surveyor</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
@@ -4480,12 +4480,12 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Building permission route (panchayat vs DTCP / APCRDA via APDPMS) and setbacks under AP Building Rules 2017</t>
+          <t>Agricultural land: confirm conversion to non-agricultural use with the gram panchayat / collector (AP repealed the NALA Act in 2025; new process to be confirmed)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Owner / surveyor</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
@@ -4505,7 +4505,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Plot 27 ft x 75 ft (length to confirm by survey): north wall is 2 ft from the plot line and eaves overhang the owned north strip; septic and soak trench sit in the strip</t>
+          <t>Building permission route (panchayat vs DTCP / APCRDA via APDPMS) and setbacks under AP Building Rules 2017</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -4525,17 +4525,17 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Soil</t>
+          <t>Land</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Soil test (bore holes to 3 m min): black cotton soil is common in Guntur. Foundation type (isolated footings below active zone, under-reamed piles, or soil replacement) depends on it</t>
+          <t>Plot 27 ft x 75 ft (length to confirm by survey): north wall is 2 ft from the plot line and eaves overhang the owned north strip; septic and soak trench sit in the strip</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Structural engineer</t>
+          <t>Architect</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
@@ -4550,12 +4550,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>Soil</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>RCC frame with AAC infill: columns, plinth beam, lintel band, ring beam; steel truss with cyclone tie-downs</t>
+          <t>Soil test (bore holes to 3 m min): black cotton soil is common in Guntur. Foundation type (isolated footings below active zone, under-reamed piles, or soil replacement) depends on it</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -4575,17 +4575,17 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Structure</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Wet area is open to the walkway: lockable steel/WPC kitchen-to-wet-area door, compound wall and gate at the back; optional MS grille shutter across the wet area opening</t>
+          <t>RCC frame with AAC infill: columns, plinth beam, lintel band, ring beam; steel truss with cyclone tie-downs</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Owner / architect</t>
+          <t>Structural engineer</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -4600,17 +4600,17 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Services</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Groundwater: test TDS, hardness, fluoride. Plan RO for drinking and a softener for bathrooms if hardness is high</t>
+          <t>Wet area is open to the walkway: lockable steel/WPC kitchen-to-wet-area door, compound wall and gate at the back; optional MS grille shutter across the wet area opening</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Plumber / owner</t>
+          <t>Owner / architect</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -4630,12 +4630,12 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Septic tank size and soak trench length (percolation test); keep soak trenches and gardens 6 ft+ from foundations in expansive soil</t>
+          <t>Groundwater: test TDS, hardness, fluoride. Plan RO for drinking and a softener for bathrooms if hardness is high</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Plumber / owner</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -4655,12 +4655,12 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Electrical load (with ACs), service connection size, earthing, inverter / solar PV</t>
+          <t>Septic tank size and soak trench length (percolation test); keep soak trenches and gardens 6 ft+ from foundations in expansive soil</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Electrical engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -4675,22 +4675,22 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Services</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Phase 2 on the north strip will block north light and sits on the septic: plan the split now</t>
+          <t>Electrical load (with ACs), service connection size, earthing, inverter / solar PV</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Electrical engineer</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Deferred by owner</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -4700,22 +4700,22 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Vastu</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Bed head east (master), NW ensuite, Bedroom 2's attached bath in its north-west corner on the north wall (north-west of the plot centre), common bath south of the plot centre beside the wet area (outside the central zone), dining at the plot centre, pooja in the living's south-east corner back to back with the kitchen, opening west (devotees face east), shoe cupboard between the pooja and the main door (behind the pooja's solid north wall), DB on the dining face of Bedroom 2's east wall</t>
+          <t>Phase 2 on the north strip will block north light and sits on the septic: plan the split now</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Vastu consultant</t>
+          <t>Architect</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>To confirm</t>
+          <t>Deferred by owner</t>
         </is>
       </c>
     </row>
@@ -4725,22 +4725,22 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Climate</t>
+          <t>Vastu</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Roof heat: insulation, ventilated attic, ventilator lantern louvres and shutters; ODU positions on shaded walls</t>
+          <t>Bed head east (master), NW ensuite, Bedroom 2's attached bath in its north-west corner on the north wall (north-west of the plot centre), common bath south of the plot centre beside the wet area (outside the central zone), dining at the plot centre, pooja in the living's south-east corner back to back with the kitchen, opening west (devotees face east), shoe cupboard between the pooja and the main door (behind the pooja's solid north wall), DB on the dining face of Bedroom 2's east wall</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Vastu consultant</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -4750,20 +4750,45 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
+          <t>Climate</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Roof heat: insulation, ventilated attic, ventilator lantern louvres and shutters; ODU positions on shaded walls</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
           <t>Levels</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Survey road and field levels; plinth at 2 ft above finished ground (raise if site floods)</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Surveyor / architect</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -4780,7 +4805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4815,7 +4840,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Plot 27 ft x 75 ft (5 ft longer than first assumed; confirm by survey), road on east; house 60 ft x 22 ft with the same 10 ft front yard and 5 ft rear garden; owner accepts local practice on side setbacks (to be checked).</t>
+          <t>Plot 27 ft x 75 ft (5 ft longer than first assumed; confirm by survey), road on east; house 62 ft x 22 ft (lengthened 2 ft for Bedroom 2) with an 8 ft front yard and 5 ft rear garden; owner accepts local practice on side setbacks (to be checked).</t>
         </is>
       </c>
     </row>
@@ -4925,7 +4950,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
+          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
         </is>
       </c>
     </row>
@@ -4935,7 +4960,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
+          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
         </is>
       </c>
     </row>
@@ -4945,7 +4970,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
+          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
         </is>
       </c>
     </row>
@@ -4955,7 +4980,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
+          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4990,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
+          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
         </is>
       </c>
     </row>
@@ -4975,7 +5000,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
+          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
         </is>
       </c>
     </row>
@@ -4985,7 +5010,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
+          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
         </is>
       </c>
     </row>
@@ -4995,7 +5020,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
+          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
         </is>
       </c>
     </row>
@@ -5005,7 +5030,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
+          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
         </is>
       </c>
     </row>
@@ -5015,7 +5040,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
+          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
         </is>
       </c>
     </row>
@@ -5025,7 +5050,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
+          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
         </is>
       </c>
     </row>
@@ -5035,7 +5060,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
+          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
         </is>
       </c>
     </row>
@@ -5045,7 +5070,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
+          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
         </is>
       </c>
     </row>
@@ -5055,7 +5080,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
+          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
         </is>
       </c>
     </row>
@@ -5065,7 +5090,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
+          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
         </is>
       </c>
     </row>
@@ -5075,7 +5100,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
+          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
         </is>
       </c>
     </row>
@@ -5085,7 +5110,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
+          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
         </is>
       </c>
     </row>
@@ -5095,7 +5120,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
+          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
         </is>
       </c>
     </row>
@@ -5105,7 +5130,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
+          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
         </is>
       </c>
     </row>
@@ -5115,7 +5140,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
+          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
         </is>
       </c>
     </row>
@@ -5125,7 +5150,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
+          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
         </is>
       </c>
     </row>
@@ -5135,7 +5160,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
+          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
         </is>
       </c>
     </row>
@@ -5145,7 +5170,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
         </is>
       </c>
     </row>
@@ -5155,7 +5180,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
         </is>
       </c>
     </row>
@@ -5164,6 +5189,26 @@
         <v>37</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>Roof: Mangalore clay tiles on steel truss over insulated cement-fibre deck; all edge tiles mechanically fixed.</t>
         </is>
@@ -5650,7 +5695,7 @@
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>14.5</v>
@@ -5664,7 +5709,7 @@
         <v/>
       </c>
       <c r="H9" s="5" t="n">
-        <v>14.58</v>
+        <v>16.58</v>
       </c>
       <c r="I9" s="5" t="n">
         <v>13.91</v>
@@ -5870,7 +5915,7 @@
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>18.5</v>
+        <v>20.5</v>
       </c>
       <c r="E13" s="4" t="n">
         <v>7.5</v>
@@ -5884,7 +5929,7 @@
         <v/>
       </c>
       <c r="H13" s="5" t="n">
-        <v>18.08</v>
+        <v>20.08</v>
       </c>
       <c r="I13" s="5" t="n">
         <v>6.92</v>
@@ -6145,7 +6190,7 @@
       <c r="L18" s="6" t="inlineStr"/>
       <c r="M18" s="6" t="inlineStr">
         <is>
-          <t>Built footprint 60' x 22' = 1,320 sq ft</t>
+          <t>Built footprint 62' x 22' = 1,364 sq ft</t>
         </is>
       </c>
     </row>
@@ -7022,7 +7067,7 @@
         </is>
       </c>
       <c r="D13" s="9" t="n">
-        <v>5.2</v>
+        <v>6</v>
       </c>
       <c r="E13" s="9" t="n">
         <v>3</v>
@@ -7036,7 +7081,7 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Teak casement, glazed (5'-2")</t>
+          <t>Teak casement, glazed (6 ft)</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr"/>
@@ -7282,7 +7327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8707,7 +8752,7 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Counter-top wash basin at the west end of the serving counter</t>
+          <t>Hand-wash basin at the east end of the serving counter, just outside the common bath (after meals); mirror on the side wall</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -8783,17 +8828,17 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>F34</t>
+          <t>F56</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Sitting and serving area</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>L-counter, south run</t>
+          <t>Tall storage cupboard 5' x 2' (bedding, suitcases, festival vessels), loft above</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -8802,7 +8847,7 @@
         </is>
       </c>
       <c r="E35" s="4" t="n">
-        <v>13.2</v>
+        <v>5</v>
       </c>
       <c r="F35" s="4" t="n">
         <v>2</v>
@@ -8812,7 +8857,7 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>Granite top, ply carcass</t>
+          <t>Ply + laminate, full height</t>
         </is>
       </c>
       <c r="I35" s="10" t="n"/>
@@ -8826,7 +8871,7 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F34</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -8836,7 +8881,7 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>L-counter, east run (hob centred 7'-6" from the south wall face, on solid wall)</t>
+          <t>L-counter, south run</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -8845,17 +8890,17 @@
         </is>
       </c>
       <c r="E36" s="4" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="F36" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="F36" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="G36" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>Granite top, cook faces east</t>
+          <t>Granite top, ply carcass</t>
         </is>
       </c>
       <c r="I36" s="10" t="n"/>
@@ -8869,7 +8914,7 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>F36</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -8879,26 +8924,26 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Refrigerator space (kitchen north wall, behind the pooja, door facing south)</t>
+          <t>L-counter, east run (hob centred 7'-6" from the south wall face, on solid wall)</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Appliance / joinery</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E37" s="4" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>2.4</v>
+        <v>7</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>Double-door, 2'6" wide</t>
+          <t>Granite top, cook faces east</t>
         </is>
       </c>
       <c r="I37" s="10" t="n"/>
@@ -8912,7 +8957,7 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>F55</t>
+          <t>F36</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -8922,26 +8967,26 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Tall pantry 4'-5" x 2' on the north wall (provisions, rice, vessels)</t>
+          <t>Refrigerator space (kitchen north wall, behind the pooja, door facing south)</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Appliance / joinery</t>
         </is>
       </c>
       <c r="E38" s="4" t="n">
-        <v>4.4</v>
+        <v>2.5</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="G38" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate, full height with loft</t>
+          <t>Double-door, 2'6" wide</t>
         </is>
       </c>
       <c r="I38" s="10" t="n"/>
@@ -8955,17 +9000,17 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>F38</t>
+          <t>F55</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Dining bay</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Three-seat sofa 6'6" facing west to the TV</t>
+          <t>Tall pantry 4'-5" x 2' on the north wall (provisions, rice, vessels)</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -8974,17 +9019,17 @@
         </is>
       </c>
       <c r="E39" s="4" t="n">
-        <v>2.7</v>
+        <v>4.4</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>5.9</v>
+        <v>2</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Teak frame, cotton cushions</t>
+          <t>Ply + laminate, full height with loft</t>
         </is>
       </c>
       <c r="I39" s="10" t="n"/>
@@ -8998,7 +9043,7 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>F39</t>
+          <t>F38</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -9008,7 +9053,7 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Coffee table 3'6" x 2'</t>
+          <t>Three-seat sofa 6'6" facing west to the TV</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -9017,17 +9062,17 @@
         </is>
       </c>
       <c r="E40" s="4" t="n">
-        <v>2</v>
+        <v>2.7</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>3.5</v>
+        <v>5.9</v>
       </c>
       <c r="G40" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>Teak</t>
+          <t>Teak frame, cotton cushions</t>
         </is>
       </c>
       <c r="I40" s="10" t="n"/>
@@ -9041,7 +9086,7 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>F53</t>
+          <t>F39</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
@@ -9051,26 +9096,26 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>TV unit 4'-5" on Bedroom 2's east wall (55-65 in TV wall-mounted above)</t>
+          <t>Coffee table 3'6" x 2'</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Appliance / joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E41" s="4" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>4.4</v>
+        <v>3.5</v>
       </c>
       <c r="G41" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>Teak, low, open shelves</t>
+          <t>Teak</t>
         </is>
       </c>
       <c r="I41" s="10" t="n"/>
@@ -9084,36 +9129,36 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>F40</t>
+          <t>F53</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Dining bay</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Armchair by the north window</t>
+          <t>TV unit 4'-5" on Bedroom 2's east wall (55-65 in TV wall-mounted above)</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Appliance / joinery</t>
         </is>
       </c>
       <c r="E42" s="4" t="n">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>1.6</v>
+        <v>4.4</v>
       </c>
       <c r="G42" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>Cane / teak</t>
+          <t>Teak, low, open shelves</t>
         </is>
       </c>
       <c r="I42" s="10" t="n"/>
@@ -9127,7 +9172,7 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>F52</t>
+          <t>F40</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
@@ -9137,26 +9182,26 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Shoe cupboard 3'-3" beside the main door (closed shutters, louvred for air)</t>
+          <t>Armchair by the north window</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E43" s="4" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>3.2</v>
+        <v>1.6</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate, 14 in deep</t>
+          <t>Cane / teak</t>
         </is>
       </c>
       <c r="I43" s="10" t="n"/>
@@ -9170,36 +9215,36 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>F41</t>
+          <t>F52</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Poomukham (verandah)</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Oonjal (swing) 3'6"</t>
+          <t>Shoe cupboard 3'-3" beside the main door (closed shutters, louvred for air)</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E44" s="4" t="n">
-        <v>3.5</v>
+        <v>1.2</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>1.5</v>
+        <v>3.2</v>
       </c>
       <c r="G44" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>Teak, chains to beam</t>
+          <t>Ply + laminate, 14 in deep</t>
         </is>
       </c>
       <c r="I44" s="10" t="n"/>
@@ -9213,7 +9258,7 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>F42</t>
+          <t>F41</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -9223,26 +9268,26 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Arugu seat (built-in, south end)</t>
+          <t>Oonjal (swing) 3'6"</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E45" s="4" t="n">
-        <v>1.2</v>
+        <v>3.5</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>2.4</v>
+        <v>1.5</v>
       </c>
       <c r="G45" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>Laterite base, teak top</t>
+          <t>Teak, chains to beam</t>
         </is>
       </c>
       <c r="I45" s="10" t="n"/>
@@ -9254,28 +9299,71 @@
       <c r="L45" s="8" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="inlineStr"/>
-      <c r="B46" s="6" t="inlineStr"/>
-      <c r="C46" s="6" t="inlineStr">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>F42</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Poomukham (verandah)</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Arugu seat (built-in, south end)</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Built-in joinery</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F46" s="4" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>Laterite base, teak top</t>
+        </is>
+      </c>
+      <c r="I46" s="10" t="n"/>
+      <c r="J46" s="11">
+        <f>G46*I46</f>
+        <v/>
+      </c>
+      <c r="K46" s="8" t="inlineStr"/>
+      <c r="L46" s="8" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr"/>
+      <c r="B47" s="6" t="inlineStr"/>
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D46" s="6" t="inlineStr"/>
-      <c r="E46" s="6" t="inlineStr"/>
-      <c r="F46" s="6" t="inlineStr"/>
-      <c r="G46" s="6">
-        <f>SUM(G2:G45)</f>
+      <c r="D47" s="6" t="inlineStr"/>
+      <c r="E47" s="6" t="inlineStr"/>
+      <c r="F47" s="6" t="inlineStr"/>
+      <c r="G47" s="6">
+        <f>SUM(G2:G46)</f>
         <v/>
       </c>
-      <c r="H46" s="6" t="inlineStr"/>
-      <c r="I46" s="12" t="inlineStr"/>
-      <c r="J46" s="12">
-        <f>SUM(J2:J45)</f>
+      <c r="H47" s="6" t="inlineStr"/>
+      <c r="I47" s="12" t="inlineStr"/>
+      <c r="J47" s="12">
+        <f>SUM(J2:J46)</f>
         <v/>
       </c>
-      <c r="K46" s="6" t="inlineStr"/>
-      <c r="L46" s="6" t="inlineStr"/>
+      <c r="K47" s="6" t="inlineStr"/>
+      <c r="L47" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10382,7 +10470,7 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>22.35</v>
+        <v>22.94</v>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
@@ -10442,7 +10530,7 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>6.02</v>
+        <v>6.18</v>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
@@ -10472,7 +10560,7 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>87.59999999999999</v>
+        <v>89.5</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
@@ -10502,7 +10590,7 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>278.7</v>
+        <v>284.9</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
@@ -10532,7 +10620,7 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>142.9</v>
+        <v>146.6</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
@@ -10562,7 +10650,7 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>44.5</v>
+        <v>47.1</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
@@ -10622,7 +10710,7 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>37.4</v>
+        <v>38.7</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
@@ -10772,7 +10860,7 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>110.5</v>
+        <v>111.7</v>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
@@ -11042,7 +11130,7 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>188.3</v>
+        <v>194.1</v>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
@@ -11072,7 +11160,7 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>39.6</v>
+        <v>40.8</v>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
@@ -11132,7 +11220,7 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>34.9</v>
+        <v>35.5</v>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
@@ -11162,7 +11250,7 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>49.9</v>
+        <v>51</v>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
@@ -11252,7 +11340,7 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>22.5</v>
+        <v>22.8</v>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
@@ -12501,7 +12589,7 @@
         </is>
       </c>
       <c r="E38" s="4" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F38" s="4" t="n">
         <v>15</v>
@@ -12530,7 +12618,7 @@
         </is>
       </c>
       <c r="E39" s="4" t="n">
-        <v>58.4</v>
+        <v>60.4</v>
       </c>
       <c r="F39" s="4" t="n">
         <v>15</v>
@@ -12563,7 +12651,7 @@
         </is>
       </c>
       <c r="E40" s="4" t="n">
-        <v>55.4</v>
+        <v>57.4</v>
       </c>
       <c r="F40" s="4" t="n">
         <v>16.6</v>
@@ -12592,7 +12680,7 @@
         </is>
       </c>
       <c r="E41" s="4" t="n">
-        <v>54.6</v>
+        <v>56.6</v>
       </c>
       <c r="F41" s="4" t="n">
         <v>16.9</v>
@@ -12625,7 +12713,7 @@
         </is>
       </c>
       <c r="E42" s="4" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F42" s="4" t="n">
         <v>6.5</v>
@@ -12654,7 +12742,7 @@
         </is>
       </c>
       <c r="E43" s="4" t="n">
-        <v>35</v>
+        <v>35.15</v>
       </c>
       <c r="F43" s="4" t="n">
         <v>3.4</v>
@@ -12687,7 +12775,7 @@
         </is>
       </c>
       <c r="E44" s="4" t="n">
-        <v>38</v>
+        <v>38.1</v>
       </c>
       <c r="F44" s="4" t="n">
         <v>3.4</v>
@@ -12720,7 +12808,7 @@
         </is>
       </c>
       <c r="E45" s="4" t="n">
-        <v>42.7</v>
+        <v>44.7</v>
       </c>
       <c r="F45" s="4" t="n">
         <v>6.2</v>
@@ -12749,7 +12837,7 @@
         </is>
       </c>
       <c r="E46" s="4" t="n">
-        <v>44.9</v>
+        <v>46.9</v>
       </c>
       <c r="F46" s="4" t="n">
         <v>3.4</v>
@@ -12782,7 +12870,7 @@
         </is>
       </c>
       <c r="E47" s="4" t="n">
-        <v>39.8</v>
+        <v>41.8</v>
       </c>
       <c r="F47" s="4" t="n">
         <v>4.5</v>
@@ -12815,7 +12903,7 @@
         </is>
       </c>
       <c r="E48" s="4" t="n">
-        <v>45.6</v>
+        <v>47.6</v>
       </c>
       <c r="F48" s="4" t="n">
         <v>6</v>
@@ -12848,7 +12936,7 @@
         </is>
       </c>
       <c r="E49" s="4" t="n">
-        <v>39.1</v>
+        <v>41.1</v>
       </c>
       <c r="F49" s="4" t="n">
         <v>9.199999999999999</v>
@@ -12881,7 +12969,7 @@
         </is>
       </c>
       <c r="E50" s="4" t="n">
-        <v>29.5</v>
+        <v>31.5</v>
       </c>
       <c r="F50" s="4" t="n">
         <v>15.5</v>
@@ -12943,7 +13031,7 @@
         </is>
       </c>
       <c r="E52" s="4" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F52" s="4" t="n">
         <v>14</v>
@@ -12972,7 +13060,7 @@
         </is>
       </c>
       <c r="E53" s="4" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F53" s="4" t="n">
         <v>20.5</v>
@@ -13001,7 +13089,7 @@
         </is>
       </c>
       <c r="E54" s="4" t="n">
-        <v>31.2</v>
+        <v>33.2</v>
       </c>
       <c r="F54" s="4" t="n">
         <v>10.9</v>
@@ -13166,7 +13254,7 @@
         </is>
       </c>
       <c r="E59" s="4" t="n">
-        <v>35.6</v>
+        <v>37.6</v>
       </c>
       <c r="F59" s="4" t="n">
         <v>15</v>
@@ -13199,7 +13287,7 @@
         </is>
       </c>
       <c r="E60" s="4" t="n">
-        <v>35.6</v>
+        <v>37.6</v>
       </c>
       <c r="F60" s="4" t="n">
         <v>15.8</v>
@@ -13232,7 +13320,7 @@
         </is>
       </c>
       <c r="E61" s="4" t="n">
-        <v>35.6</v>
+        <v>37.6</v>
       </c>
       <c r="F61" s="4" t="n">
         <v>16.6</v>
@@ -13265,7 +13353,7 @@
         </is>
       </c>
       <c r="E62" s="4" t="n">
-        <v>35.6</v>
+        <v>37.6</v>
       </c>
       <c r="F62" s="4" t="n">
         <v>17.4</v>
@@ -13298,7 +13386,7 @@
         </is>
       </c>
       <c r="E63" s="4" t="n">
-        <v>35.6</v>
+        <v>37.6</v>
       </c>
       <c r="F63" s="4" t="n">
         <v>18.6</v>
@@ -13331,14 +13419,14 @@
         </is>
       </c>
       <c r="E64" s="4" t="n">
-        <v>32.2</v>
+        <v>41.1</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>3.4</v>
+        <v>4.4</v>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>over basin</t>
+          <t>over basin, on the common bath wall</t>
         </is>
       </c>
     </row>
@@ -13364,7 +13452,7 @@
         </is>
       </c>
       <c r="E65" s="4" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F65" s="4" t="n">
         <v>25.6</v>
@@ -13397,7 +13485,7 @@
         </is>
       </c>
       <c r="E66" s="4" t="n">
-        <v>39.5</v>
+        <v>41.5</v>
       </c>
       <c r="F66" s="4" t="n">
         <v>21.5</v>
@@ -13426,7 +13514,7 @@
         </is>
       </c>
       <c r="E67" s="4" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F67" s="4" t="n">
         <v>21.5</v>
@@ -13459,7 +13547,7 @@
         </is>
       </c>
       <c r="E68" s="4" t="n">
-        <v>46.6</v>
+        <v>48.6</v>
       </c>
       <c r="F68" s="4" t="n">
         <v>24.6</v>
@@ -13488,7 +13576,7 @@
         </is>
       </c>
       <c r="E69" s="4" t="n">
-        <v>36.4</v>
+        <v>38.4</v>
       </c>
       <c r="F69" s="4" t="n">
         <v>22.4</v>
@@ -13521,7 +13609,7 @@
         </is>
       </c>
       <c r="E70" s="4" t="n">
-        <v>36.4</v>
+        <v>38.4</v>
       </c>
       <c r="F70" s="4" t="n">
         <v>21</v>
@@ -13554,7 +13642,7 @@
         </is>
       </c>
       <c r="E71" s="4" t="n">
-        <v>36.4</v>
+        <v>38.4</v>
       </c>
       <c r="F71" s="4" t="n">
         <v>20</v>
@@ -13587,7 +13675,7 @@
         </is>
       </c>
       <c r="E72" s="4" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F72" s="4" t="n">
         <v>25.6</v>
@@ -13620,7 +13708,7 @@
         </is>
       </c>
       <c r="E73" s="4" t="n">
-        <v>42.5</v>
+        <v>44.5</v>
       </c>
       <c r="F73" s="4" t="n">
         <v>15</v>
@@ -13653,7 +13741,7 @@
         </is>
       </c>
       <c r="E74" s="4" t="n">
-        <v>36.4</v>
+        <v>38.4</v>
       </c>
       <c r="F74" s="4" t="n">
         <v>17.5</v>
@@ -13682,7 +13770,7 @@
         </is>
       </c>
       <c r="E75" s="4" t="n">
-        <v>36.4</v>
+        <v>38.4</v>
       </c>
       <c r="F75" s="4" t="n">
         <v>16.2</v>
@@ -13711,7 +13799,7 @@
         </is>
       </c>
       <c r="E76" s="4" t="n">
-        <v>36.4</v>
+        <v>38.4</v>
       </c>
       <c r="F76" s="4" t="n">
         <v>13.7</v>
@@ -13744,7 +13832,7 @@
         </is>
       </c>
       <c r="E77" s="4" t="n">
-        <v>28.5</v>
+        <v>30.5</v>
       </c>
       <c r="F77" s="4" t="n">
         <v>6.75</v>
@@ -13835,7 +13923,7 @@
         </is>
       </c>
       <c r="E80" s="4" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F80" s="4" t="n">
         <v>5.5</v>
@@ -13868,7 +13956,7 @@
         </is>
       </c>
       <c r="E81" s="4" t="n">
-        <v>46.5</v>
+        <v>48.5</v>
       </c>
       <c r="F81" s="4" t="n">
         <v>8.699999999999999</v>
@@ -13901,7 +13989,7 @@
         </is>
       </c>
       <c r="E82" s="4" t="n">
-        <v>50.6</v>
+        <v>52.6</v>
       </c>
       <c r="F82" s="4" t="n">
         <v>6</v>
@@ -13934,7 +14022,7 @@
         </is>
       </c>
       <c r="E83" s="4" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F83" s="4" t="n">
         <v>8</v>
@@ -13963,7 +14051,7 @@
         </is>
       </c>
       <c r="E84" s="4" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F84" s="4" t="n">
         <v>3.5</v>
@@ -13996,7 +14084,7 @@
         </is>
       </c>
       <c r="E85" s="4" t="n">
-        <v>64.5</v>
+        <v>66.5</v>
       </c>
       <c r="F85" s="4" t="n">
         <v>9.6</v>
@@ -14029,7 +14117,7 @@
         </is>
       </c>
       <c r="E86" s="4" t="n">
-        <v>64.59999999999999</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="F86" s="4" t="n">
         <v>7.5</v>
@@ -14062,7 +14150,7 @@
         </is>
       </c>
       <c r="E87" s="4" t="n">
-        <v>56.75</v>
+        <v>58.75</v>
       </c>
       <c r="F87" s="4" t="n">
         <v>12.7</v>
@@ -14095,7 +14183,7 @@
         </is>
       </c>
       <c r="E88" s="4" t="n">
-        <v>52.5</v>
+        <v>54.5</v>
       </c>
       <c r="F88" s="4" t="n">
         <v>3.5</v>
@@ -14124,7 +14212,7 @@
         </is>
       </c>
       <c r="E89" s="4" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F89" s="4" t="n">
         <v>3.5</v>
@@ -14157,7 +14245,7 @@
         </is>
       </c>
       <c r="E90" s="4" t="n">
-        <v>61.5</v>
+        <v>63.5</v>
       </c>
       <c r="F90" s="4" t="n">
         <v>3.5</v>
@@ -14190,7 +14278,7 @@
         </is>
       </c>
       <c r="E91" s="4" t="n">
-        <v>64.59999999999999</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="F91" s="4" t="n">
         <v>5.6</v>
@@ -14219,7 +14307,7 @@
         </is>
       </c>
       <c r="E92" s="4" t="n">
-        <v>64.59999999999999</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="F92" s="4" t="n">
         <v>9.6</v>
@@ -14248,7 +14336,7 @@
         </is>
       </c>
       <c r="E93" s="4" t="n">
-        <v>57.3</v>
+        <v>59.3</v>
       </c>
       <c r="F93" s="4" t="n">
         <v>3.5</v>
@@ -14281,7 +14369,7 @@
         </is>
       </c>
       <c r="E94" s="4" t="n">
-        <v>51.4</v>
+        <v>53.4</v>
       </c>
       <c r="F94" s="4" t="n">
         <v>9</v>
@@ -14314,7 +14402,7 @@
         </is>
       </c>
       <c r="E95" s="4" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F95" s="4" t="n">
         <v>19</v>
@@ -14347,7 +14435,7 @@
         </is>
       </c>
       <c r="E96" s="4" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F96" s="4" t="n">
         <v>22.5</v>
@@ -14376,7 +14464,7 @@
         </is>
       </c>
       <c r="E97" s="4" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F97" s="4" t="n">
         <v>16</v>
@@ -14405,7 +14493,7 @@
         </is>
       </c>
       <c r="E98" s="4" t="n">
-        <v>46.2</v>
+        <v>48.2</v>
       </c>
       <c r="F98" s="4" t="n">
         <v>18.4</v>
@@ -14438,7 +14526,7 @@
         </is>
       </c>
       <c r="E99" s="4" t="n">
-        <v>50.6</v>
+        <v>52.6</v>
       </c>
       <c r="F99" s="4" t="n">
         <v>17.8</v>
@@ -14471,7 +14559,7 @@
         </is>
       </c>
       <c r="E100" s="4" t="n">
-        <v>58.6</v>
+        <v>60.6</v>
       </c>
       <c r="F100" s="4" t="n">
         <v>21</v>
@@ -14504,7 +14592,7 @@
         </is>
       </c>
       <c r="E101" s="4" t="n">
-        <v>36.4</v>
+        <v>38.4</v>
       </c>
       <c r="F101" s="4" t="n">
         <v>12.6</v>
@@ -14537,7 +14625,7 @@
         </is>
       </c>
       <c r="E102" s="4" t="n">
-        <v>36.4</v>
+        <v>38.4</v>
       </c>
       <c r="F102" s="4" t="n">
         <v>14.6</v>
@@ -14570,7 +14658,7 @@
         </is>
       </c>
       <c r="E103" s="4" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F103" s="4" t="n">
         <v>16</v>
@@ -14599,7 +14687,7 @@
         </is>
       </c>
       <c r="E104" s="4" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F104" s="4" t="n">
         <v>22</v>
@@ -14628,7 +14716,7 @@
         </is>
       </c>
       <c r="E105" s="4" t="n">
-        <v>59.4</v>
+        <v>61.4</v>
       </c>
       <c r="F105" s="4" t="n">
         <v>20.4</v>
@@ -14657,7 +14745,7 @@
         </is>
       </c>
       <c r="E106" s="4" t="n">
-        <v>64.5</v>
+        <v>66.5</v>
       </c>
       <c r="F106" s="4" t="n">
         <v>24.6</v>
@@ -14690,7 +14778,7 @@
         </is>
       </c>
       <c r="E107" s="4" t="n">
-        <v>59.4</v>
+        <v>61.4</v>
       </c>
       <c r="F107" s="4" t="n">
         <v>24</v>
@@ -14723,7 +14811,7 @@
         </is>
       </c>
       <c r="E108" s="4" t="n">
-        <v>59.4</v>
+        <v>61.4</v>
       </c>
       <c r="F108" s="4" t="n">
         <v>20.9</v>
@@ -14818,7 +14906,7 @@
         </is>
       </c>
       <c r="E111" s="4" t="n">
-        <v>66.2</v>
+        <v>68.2</v>
       </c>
       <c r="F111" s="4" t="n">
         <v>1.5</v>

</xml_diff>

<commit_message>
Bedroom 2 re-laid for 17 ft: bed head south, Bath 2 7' x 7'
Bed centred with its head on the south wall under the jali, 2 ft+ on both
sides; dresser on the west wall; door switch on the latch-side return.
Bath 2 grows to 7' x 7' with a 3' x 3'-6" wet zone and the basin in the
dry zone; door stays on its east wall.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Schedules/KH-P1_Schedules_RevB.xlsx
+++ b/03_Schedules/KH-P1_Schedules_RevB.xlsx
@@ -1107,10 +1107,10 @@
         </is>
       </c>
       <c r="D16" s="4" t="n">
-        <v>24.25</v>
+        <v>22.35</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>19.4</v>
+        <v>18.4</v>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="D18" s="4" t="n">
-        <v>26.4</v>
+        <v>26.3</v>
       </c>
       <c r="E18" s="4" t="n">
         <v>24.3</v>
@@ -1191,10 +1191,10 @@
         </is>
       </c>
       <c r="D19" s="4" t="n">
-        <v>25.5</v>
+        <v>24.6</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>20.6</v>
+        <v>19.7</v>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
@@ -4805,7 +4805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B40"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4950,7 +4950,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
+          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
         </is>
       </c>
     </row>
@@ -4960,7 +4960,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
+          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
         </is>
       </c>
     </row>
@@ -4970,7 +4970,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
+          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
         </is>
       </c>
     </row>
@@ -4980,7 +4980,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
+          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
         </is>
       </c>
     </row>
@@ -4990,7 +4990,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
+          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
         </is>
       </c>
     </row>
@@ -5000,7 +5000,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
+          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
         </is>
       </c>
     </row>
@@ -5010,7 +5010,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
+          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
+          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
         </is>
       </c>
     </row>
@@ -5030,7 +5030,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
+          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
         </is>
       </c>
     </row>
@@ -5040,7 +5040,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
+          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
         </is>
       </c>
     </row>
@@ -5050,7 +5050,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
+          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
         </is>
       </c>
     </row>
@@ -5060,7 +5060,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
+          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
+          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
         </is>
       </c>
     </row>
@@ -5080,7 +5080,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
+          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
         </is>
       </c>
     </row>
@@ -5090,7 +5090,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
+          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
         </is>
       </c>
     </row>
@@ -5100,7 +5100,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
+          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
         </is>
       </c>
     </row>
@@ -5110,7 +5110,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
+          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
         </is>
       </c>
     </row>
@@ -5120,7 +5120,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
+          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
         </is>
       </c>
     </row>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
+          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
+          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
         </is>
       </c>
     </row>
@@ -5150,7 +5150,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
+          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
         </is>
       </c>
     </row>
@@ -5160,7 +5160,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
+          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
         </is>
       </c>
     </row>
@@ -5170,7 +5170,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
+          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
         </is>
       </c>
     </row>
@@ -5180,7 +5180,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
+          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
         </is>
       </c>
     </row>
@@ -5190,7 +5190,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
         </is>
       </c>
     </row>
@@ -5200,7 +5200,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
         </is>
       </c>
     </row>
@@ -5209,6 +5209,16 @@
         <v>39</v>
       </c>
       <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>Roof: Mangalore clay tiles on steel truss over insulated cement-fibre deck; all edge tiles mechanically fixed.</t>
         </is>
@@ -5594,7 +5604,7 @@
         <v>7</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F7" s="5">
         <f>D7*E7</f>
@@ -5608,7 +5618,7 @@
         <v>6.5</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>5.33</v>
+        <v>6.33</v>
       </c>
       <c r="J7" s="5">
         <f>H7*I7</f>
@@ -7149,7 +7159,7 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>High jali vent to the sitting area (cross-ventilation with W12 and W03)</t>
+          <t>High jali vent to the sitting area, above the bed head (cross-ventilation with W12 and W03)</t>
         </is>
       </c>
       <c r="I15" s="8" t="inlineStr"/>
@@ -7327,7 +7337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8150,7 +8160,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Wash basin (south wall)</t>
+          <t>Wash basin (south wall, dry zone)</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -8193,7 +8203,7 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Fixed glass splash panel at the south edge of the 3' x 2'-9" wet zone (north-east), beside the door</t>
+          <t>Fixed glass splash panel at the south edge of the 3' x 3'-6" wet zone (north-east)</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -8236,7 +8246,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Queen bed 5' x 6'6" + headboard, head to the west wall, between the bath and the sitting area (1'-6" each side)</t>
+          <t>Queen bed 5' x 6'6" + headboard, head to the south wall, 2 ft+ free on both sides</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -8245,10 +8255,10 @@
         </is>
       </c>
       <c r="E21" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F21" s="4" t="n">
         <v>6.4</v>
-      </c>
-      <c r="F21" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8288,7 +8298,7 @@
         </is>
       </c>
       <c r="E22" s="4" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="F22" s="4" t="n">
         <v>1.1</v>
@@ -8312,7 +8322,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>F22</t>
+          <t>F57</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -8322,16 +8332,16 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Work table 4' x 2' with monitor (east wall, south of the wardrobe)</t>
+          <t>Dresser / chest of drawers with mirror (west wall)</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E23" s="4" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="F23" s="4" t="n">
         <v>4</v>
@@ -8341,7 +8351,7 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Teak / ply, cable tray, monitor arm</t>
+          <t>Teak</t>
         </is>
       </c>
       <c r="I23" s="10" t="n"/>
@@ -8355,7 +8365,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>F23</t>
+          <t>F22</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -8365,7 +8375,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Built-in wardrobe 6' (east wall, toward the house centre)</t>
+          <t>Work table 4' x 2' with monitor (east wall, south of the wardrobe)</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -8374,17 +8384,17 @@
         </is>
       </c>
       <c r="E24" s="4" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G24" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate</t>
+          <t>Teak / ply, cable tray, monitor arm</t>
         </is>
       </c>
       <c r="I24" s="10" t="n"/>
@@ -8398,36 +8408,36 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>F24</t>
+          <t>F23</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Bedroom 2</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Dining table 5' x 3', 6-seat</t>
+          <t>Built-in wardrobe 6' (east wall, toward the house centre)</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E25" s="4" t="n">
-        <v>5</v>
+        <v>1.8</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G25" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Teak or rosewood</t>
+          <t>Ply + laminate</t>
         </is>
       </c>
       <c r="I25" s="10" t="n"/>
@@ -8441,7 +8451,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F24</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -8451,7 +8461,7 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Dining chair</t>
+          <t>Dining table 5' x 3', 6-seat</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -8460,17 +8470,17 @@
         </is>
       </c>
       <c r="E26" s="4" t="n">
-        <v>1.1</v>
+        <v>5</v>
       </c>
       <c r="F26" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G26" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G26" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Teak + cane</t>
+          <t>Teak or rosewood</t>
         </is>
       </c>
       <c r="I26" s="10" t="n"/>
@@ -8484,36 +8494,36 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>F26</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Pooja</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Pooja mandapam on the east wall (idols face west; family faces east)</t>
+          <t>Dining chair</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E27" s="4" t="n">
-        <v>0.6</v>
+        <v>1.1</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Carved teak</t>
+          <t>Teak + cane</t>
         </is>
       </c>
       <c r="I27" s="10" t="n"/>
@@ -8527,36 +8537,36 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>F28</t>
+          <t>F26</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area</t>
+          <t>Pooja</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Built-in bench with storage drawers below</t>
+          <t>Pooja mandapam on the east wall (idols face west; family faces east)</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E28" s="4" t="n">
-        <v>1.5</v>
+        <v>0.6</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="G28" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Teak top, ply drawers, on legs</t>
+          <t>Carved teak</t>
         </is>
       </c>
       <c r="I28" s="10" t="n"/>
@@ -8570,36 +8580,36 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>F29</t>
+          <t>F28</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Wet area</t>
+          <t>Sitting and serving area</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Utility sink counter (on the kitchen wall)</t>
+          <t>Built-in bench with storage drawers below</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Sanitary / plumbing</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E29" s="4" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>Kadappa / granite, SS sinks</t>
+          <t>Teak top, ply drawers, on legs</t>
         </is>
       </c>
       <c r="I29" s="10" t="n"/>
@@ -8613,7 +8623,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>F30</t>
+          <t>F29</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -8623,26 +8633,26 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Washing machine bay 2' x 2' (covered back corner, 2 in clear of the bath wall)</t>
+          <t>Utility sink counter (on the kitchen wall)</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Appliance / joinery</t>
+          <t>Sanitary / plumbing</t>
         </is>
       </c>
       <c r="E30" s="4" t="n">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>1.9</v>
+        <v>2.5</v>
       </c>
       <c r="G30" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Splash-proof socket, floor drain</t>
+          <t>Kadappa / granite, SS sinks</t>
         </is>
       </c>
       <c r="I30" s="10" t="n"/>
@@ -8656,7 +8666,7 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>F31</t>
+          <t>F30</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -8666,26 +8676,26 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Fold-away clothesline in the south walkway</t>
+          <t>Washing machine bay 2' x 2' (covered back corner, 2 in clear of the bath wall)</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Appliance / joinery</t>
         </is>
       </c>
       <c r="E31" s="4" t="n">
-        <v>4</v>
+        <v>1.9</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>SS wire, wall brackets</t>
+          <t>Splash-proof socket, floor drain</t>
         </is>
       </c>
       <c r="I31" s="10" t="n"/>
@@ -8699,7 +8709,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>F44</t>
+          <t>F31</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -8709,26 +8719,26 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Tall slim utility cupboard (brooms, mops, detergents)</t>
+          <t>Fold-away clothesline in the south walkway</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E32" s="4" t="n">
-        <v>1.2</v>
+        <v>4</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="G32" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate on legs, louvred doors</t>
+          <t>SS wire, wall brackets</t>
         </is>
       </c>
       <c r="I32" s="10" t="n"/>
@@ -8742,36 +8752,36 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>F32</t>
+          <t>F44</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area</t>
+          <t>Wet area</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Hand-wash basin at the east end of the serving counter, just outside the common bath (after meals); mirror on the side wall</t>
+          <t>Tall slim utility cupboard (brooms, mops, detergents)</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Sanitary / plumbing</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
-        <v>1.9</v>
+        <v>1.2</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Ceramic basin in granite top</t>
+          <t>Ply + laminate on legs, louvred doors</t>
         </is>
       </c>
       <c r="I33" s="10" t="n"/>
@@ -8785,7 +8795,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>F33</t>
+          <t>F32</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -8795,16 +8805,16 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Serving counter with crockery cabinets above, 6 ft</t>
+          <t>Hand-wash basin at the east end of the serving counter, just outside the common bath (after meals); mirror on the side wall</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Sanitary / plumbing</t>
         </is>
       </c>
       <c r="E34" s="4" t="n">
-        <v>6</v>
+        <v>1.9</v>
       </c>
       <c r="F34" s="4" t="n">
         <v>2</v>
@@ -8814,7 +8824,7 @@
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>Granite top, teak + glass shutters</t>
+          <t>Ceramic basin in granite top</t>
         </is>
       </c>
       <c r="I34" s="10" t="n"/>
@@ -8828,7 +8838,7 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>F56</t>
+          <t>F33</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -8838,7 +8848,7 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Tall storage cupboard 5' x 2' (bedding, suitcases, festival vessels), loft above</t>
+          <t>Serving counter with crockery cabinets above, 6 ft</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -8847,7 +8857,7 @@
         </is>
       </c>
       <c r="E35" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F35" s="4" t="n">
         <v>2</v>
@@ -8857,7 +8867,7 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate, full height</t>
+          <t>Granite top, teak + glass shutters</t>
         </is>
       </c>
       <c r="I35" s="10" t="n"/>
@@ -8871,17 +8881,17 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>F34</t>
+          <t>F56</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Sitting and serving area</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>L-counter, south run</t>
+          <t>Tall storage cupboard 5' x 2' (bedding, suitcases, festival vessels), loft above</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -8890,7 +8900,7 @@
         </is>
       </c>
       <c r="E36" s="4" t="n">
-        <v>13.2</v>
+        <v>5</v>
       </c>
       <c r="F36" s="4" t="n">
         <v>2</v>
@@ -8900,7 +8910,7 @@
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>Granite top, ply carcass</t>
+          <t>Ply + laminate, full height</t>
         </is>
       </c>
       <c r="I36" s="10" t="n"/>
@@ -8914,7 +8924,7 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F34</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -8924,7 +8934,7 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>L-counter, east run (hob centred 7'-6" from the south wall face, on solid wall)</t>
+          <t>L-counter, south run</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -8933,17 +8943,17 @@
         </is>
       </c>
       <c r="E37" s="4" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="F37" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="F37" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>Granite top, cook faces east</t>
+          <t>Granite top, ply carcass</t>
         </is>
       </c>
       <c r="I37" s="10" t="n"/>
@@ -8957,7 +8967,7 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>F36</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -8967,26 +8977,26 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Refrigerator space (kitchen north wall, behind the pooja, door facing south)</t>
+          <t>L-counter, east run (hob centred 7'-6" from the south wall face, on solid wall)</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Appliance / joinery</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E38" s="4" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>2.4</v>
+        <v>7</v>
       </c>
       <c r="G38" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Double-door, 2'6" wide</t>
+          <t>Granite top, cook faces east</t>
         </is>
       </c>
       <c r="I38" s="10" t="n"/>
@@ -9000,7 +9010,7 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>F55</t>
+          <t>F36</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -9010,26 +9020,26 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Tall pantry 4'-5" x 2' on the north wall (provisions, rice, vessels)</t>
+          <t>Refrigerator space (kitchen north wall, behind the pooja, door facing south)</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Appliance / joinery</t>
         </is>
       </c>
       <c r="E39" s="4" t="n">
-        <v>4.4</v>
+        <v>2.5</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate, full height with loft</t>
+          <t>Double-door, 2'6" wide</t>
         </is>
       </c>
       <c r="I39" s="10" t="n"/>
@@ -9043,17 +9053,17 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>F38</t>
+          <t>F55</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Dining bay</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Three-seat sofa 6'6" facing west to the TV</t>
+          <t>Tall pantry 4'-5" x 2' on the north wall (provisions, rice, vessels)</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -9062,17 +9072,17 @@
         </is>
       </c>
       <c r="E40" s="4" t="n">
-        <v>2.7</v>
+        <v>4.4</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>5.9</v>
+        <v>2</v>
       </c>
       <c r="G40" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>Teak frame, cotton cushions</t>
+          <t>Ply + laminate, full height with loft</t>
         </is>
       </c>
       <c r="I40" s="10" t="n"/>
@@ -9086,7 +9096,7 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>F39</t>
+          <t>F38</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
@@ -9096,7 +9106,7 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Coffee table 3'6" x 2'</t>
+          <t>Three-seat sofa 6'6" facing west to the TV</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -9105,17 +9115,17 @@
         </is>
       </c>
       <c r="E41" s="4" t="n">
-        <v>2</v>
+        <v>2.7</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>3.5</v>
+        <v>5.9</v>
       </c>
       <c r="G41" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>Teak</t>
+          <t>Teak frame, cotton cushions</t>
         </is>
       </c>
       <c r="I41" s="10" t="n"/>
@@ -9129,7 +9139,7 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>F53</t>
+          <t>F39</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -9139,26 +9149,26 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>TV unit 4'-5" on Bedroom 2's east wall (55-65 in TV wall-mounted above)</t>
+          <t>Coffee table 3'6" x 2'</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Appliance / joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E42" s="4" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>4.4</v>
+        <v>3.5</v>
       </c>
       <c r="G42" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>Teak, low, open shelves</t>
+          <t>Teak</t>
         </is>
       </c>
       <c r="I42" s="10" t="n"/>
@@ -9172,36 +9182,36 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>F40</t>
+          <t>F53</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Dining bay</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Armchair by the north window</t>
+          <t>TV unit 4'-5" on Bedroom 2's east wall (55-65 in TV wall-mounted above)</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Appliance / joinery</t>
         </is>
       </c>
       <c r="E43" s="4" t="n">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>1.6</v>
+        <v>4.4</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>Cane / teak</t>
+          <t>Teak, low, open shelves</t>
         </is>
       </c>
       <c r="I43" s="10" t="n"/>
@@ -9215,7 +9225,7 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>F52</t>
+          <t>F40</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -9225,26 +9235,26 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Shoe cupboard 3'-3" beside the main door (closed shutters, louvred for air)</t>
+          <t>Armchair by the north window</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E44" s="4" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>3.2</v>
+        <v>1.6</v>
       </c>
       <c r="G44" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate, 14 in deep</t>
+          <t>Cane / teak</t>
         </is>
       </c>
       <c r="I44" s="10" t="n"/>
@@ -9258,36 +9268,36 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>F41</t>
+          <t>F52</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Poomukham (verandah)</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Oonjal (swing) 3'6"</t>
+          <t>Shoe cupboard 3'-3" beside the main door (closed shutters, louvred for air)</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E45" s="4" t="n">
-        <v>3.5</v>
+        <v>1.2</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>1.5</v>
+        <v>3.2</v>
       </c>
       <c r="G45" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>Teak, chains to beam</t>
+          <t>Ply + laminate, 14 in deep</t>
         </is>
       </c>
       <c r="I45" s="10" t="n"/>
@@ -9301,7 +9311,7 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>F42</t>
+          <t>F41</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -9311,26 +9321,26 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Arugu seat (built-in, south end)</t>
+          <t>Oonjal (swing) 3'6"</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E46" s="4" t="n">
-        <v>1.2</v>
+        <v>3.5</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>2.4</v>
+        <v>1.5</v>
       </c>
       <c r="G46" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>Laterite base, teak top</t>
+          <t>Teak, chains to beam</t>
         </is>
       </c>
       <c r="I46" s="10" t="n"/>
@@ -9342,28 +9352,71 @@
       <c r="L46" s="8" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="inlineStr"/>
-      <c r="B47" s="6" t="inlineStr"/>
-      <c r="C47" s="6" t="inlineStr">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>F42</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Poomukham (verandah)</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Arugu seat (built-in, south end)</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Built-in joinery</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>Laterite base, teak top</t>
+        </is>
+      </c>
+      <c r="I47" s="10" t="n"/>
+      <c r="J47" s="11">
+        <f>G47*I47</f>
+        <v/>
+      </c>
+      <c r="K47" s="8" t="inlineStr"/>
+      <c r="L47" s="8" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr"/>
+      <c r="B48" s="6" t="inlineStr"/>
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D47" s="6" t="inlineStr"/>
-      <c r="E47" s="6" t="inlineStr"/>
-      <c r="F47" s="6" t="inlineStr"/>
-      <c r="G47" s="6">
-        <f>SUM(G2:G46)</f>
+      <c r="D48" s="6" t="inlineStr"/>
+      <c r="E48" s="6" t="inlineStr"/>
+      <c r="F48" s="6" t="inlineStr"/>
+      <c r="G48" s="6">
+        <f>SUM(G2:G47)</f>
         <v/>
       </c>
-      <c r="H47" s="6" t="inlineStr"/>
-      <c r="I47" s="12" t="inlineStr"/>
-      <c r="J47" s="12">
-        <f>SUM(J2:J46)</f>
+      <c r="H48" s="6" t="inlineStr"/>
+      <c r="I48" s="12" t="inlineStr"/>
+      <c r="J48" s="12">
+        <f>SUM(J2:J47)</f>
         <v/>
       </c>
-      <c r="K47" s="6" t="inlineStr"/>
-      <c r="L47" s="6" t="inlineStr"/>
+      <c r="K48" s="6" t="inlineStr"/>
+      <c r="L48" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10500,7 +10553,7 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>3.47</v>
+        <v>3.59</v>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
@@ -10560,7 +10613,7 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>89.5</v>
+        <v>89.8</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
@@ -10590,7 +10643,7 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>284.9</v>
+        <v>286.5</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
@@ -10680,7 +10733,7 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>10.3</v>
+        <v>10.9</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
@@ -11010,7 +11063,7 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>13.8</v>
+        <v>15.1</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
@@ -11040,7 +11093,7 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>8.800000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
@@ -11382,7 +11435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G113"/>
+  <dimension ref="A1:G115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -12398,7 +12451,7 @@
         <v>24.5</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>21.8</v>
+        <v>21.2</v>
       </c>
       <c r="G32" s="4" t="inlineStr"/>
     </row>
@@ -12490,10 +12543,10 @@
         </is>
       </c>
       <c r="E35" s="4" t="n">
-        <v>25.3</v>
+        <v>23.4</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>19.4</v>
+        <v>18.4</v>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
@@ -12526,7 +12579,7 @@
         <v>28.4</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>22.2</v>
+        <v>21.3</v>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
@@ -12969,12 +13022,16 @@
         </is>
       </c>
       <c r="E50" s="4" t="n">
-        <v>31.5</v>
+        <v>29.4</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>15.5</v>
-      </c>
-      <c r="G50" s="4" t="inlineStr"/>
+        <v>15</v>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>over the bed</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -12998,10 +13055,10 @@
         </is>
       </c>
       <c r="E51" s="4" t="n">
-        <v>21.4</v>
+        <v>29.4</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>14.7</v>
+        <v>10.9</v>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
@@ -13031,7 +13088,7 @@
         </is>
       </c>
       <c r="E52" s="4" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="F52" s="4" t="n">
         <v>14</v>
@@ -13060,27 +13117,27 @@
         </is>
       </c>
       <c r="E53" s="4" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>20.5</v>
+        <v>14</v>
       </c>
       <c r="G53" s="4" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -13089,16 +13146,12 @@
         </is>
       </c>
       <c r="E54" s="4" t="n">
-        <v>33.2</v>
+        <v>33</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>10.9</v>
-      </c>
-      <c r="G54" s="4" t="inlineStr">
-        <is>
-          <t>at the door, 2-way</t>
-        </is>
-      </c>
+        <v>20.5</v>
+      </c>
+      <c r="G54" s="4" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -13122,31 +13175,31 @@
         </is>
       </c>
       <c r="E55" s="4" t="n">
-        <v>21.4</v>
+        <v>36.8</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>11.9</v>
+        <v>11.4</v>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>bedside, 2-way</t>
+          <t>at the door (latch side, on the corner return), 2-way</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -13155,14 +13208,14 @@
         </is>
       </c>
       <c r="E56" s="4" t="n">
-        <v>21.4</v>
+        <v>25.4</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>11.2</v>
+        <v>10.9</v>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>bedside</t>
+          <t>bedside, 2-way</t>
         </is>
       </c>
     </row>
@@ -13188,31 +13241,31 @@
         </is>
       </c>
       <c r="E57" s="4" t="n">
-        <v>21.4</v>
+        <v>26</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>18</v>
+        <v>10.9</v>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>bedside, north</t>
+          <t>bedside</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -13221,31 +13274,31 @@
         </is>
       </c>
       <c r="E58" s="4" t="n">
-        <v>21.4</v>
+        <v>32.4</v>
       </c>
       <c r="F58" s="4" t="n">
-        <v>18.5</v>
+        <v>10.9</v>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>bedside, north, 2-way</t>
+          <t>bedside</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -13254,26 +13307,26 @@
         </is>
       </c>
       <c r="E59" s="4" t="n">
-        <v>37.6</v>
+        <v>32.9</v>
       </c>
       <c r="F59" s="4" t="n">
-        <v>15</v>
+        <v>10.9</v>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>work table</t>
+          <t>bedside, 2-way</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Inverter (UPS) socket</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -13287,26 +13340,26 @@
         </is>
       </c>
       <c r="E60" s="4" t="n">
-        <v>37.6</v>
+        <v>21.4</v>
       </c>
       <c r="F60" s="4" t="n">
-        <v>15.8</v>
+        <v>13.5</v>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>work table, monitor</t>
+          <t>dresser</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Data point (Cat6)</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -13323,7 +13376,7 @@
         <v>37.6</v>
       </c>
       <c r="F61" s="4" t="n">
-        <v>16.6</v>
+        <v>15</v>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
@@ -13356,28 +13409,28 @@
         <v>37.6</v>
       </c>
       <c r="F62" s="4" t="n">
-        <v>17.4</v>
+        <v>15.8</v>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>work table</t>
+          <t>work table, monitor</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
+          <t>Data point (Cat6)</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>7'-6"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -13389,61 +13442,61 @@
         <v>37.6</v>
       </c>
       <c r="F63" s="4" t="n">
-        <v>18.6</v>
+        <v>16.6</v>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>east wall, not at the work table</t>
+          <t>work table</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>Inverter (UPS) socket</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area (open)</t>
+          <t>Bedroom 2</t>
         </is>
       </c>
       <c r="E64" s="4" t="n">
-        <v>41.1</v>
+        <v>37.6</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>4.4</v>
+        <v>17.4</v>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>over basin, on the common bath wall</t>
+          <t>work table</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>ODU</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>AC outdoor unit bracket</t>
+          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>7'-0" outside</t>
+          <t>7'-6"</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -13452,93 +13505,97 @@
         </is>
       </c>
       <c r="E65" s="4" t="n">
-        <v>33</v>
+        <v>37.6</v>
       </c>
       <c r="F65" s="4" t="n">
-        <v>25.6</v>
+        <v>18.6</v>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>north wall, shaded</t>
+          <t>east wall, not at the work table</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>WL</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Wall light / mirror light</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>Dining bay (north window)</t>
+          <t>Sitting and serving area (open)</t>
         </is>
       </c>
       <c r="E66" s="4" t="n">
-        <v>41.5</v>
+        <v>41.1</v>
       </c>
       <c r="F66" s="4" t="n">
-        <v>21.5</v>
-      </c>
-      <c r="G66" s="4" t="inlineStr"/>
+        <v>4.4</v>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>over basin, on the common bath wall</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>ODU</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Ceiling fan point</t>
+          <t>AC outdoor unit bracket</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>7'-0" outside</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Dining bay (north window)</t>
+          <t>Bedroom 2</t>
         </is>
       </c>
       <c r="E67" s="4" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="F67" s="4" t="n">
-        <v>21.5</v>
+        <v>25.6</v>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>long downrod, over the seating</t>
+          <t>north wall, shaded</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -13547,27 +13604,27 @@
         </is>
       </c>
       <c r="E68" s="4" t="n">
-        <v>48.6</v>
+        <v>41.5</v>
       </c>
       <c r="F68" s="4" t="n">
-        <v>24.6</v>
+        <v>21.5</v>
       </c>
       <c r="G68" s="4" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>TV</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>TV + data point</t>
+          <t>Ceiling fan point</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -13576,14 +13633,14 @@
         </is>
       </c>
       <c r="E69" s="4" t="n">
-        <v>38.4</v>
+        <v>45</v>
       </c>
       <c r="F69" s="4" t="n">
-        <v>22.4</v>
+        <v>21.5</v>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>TV wall: 2 sockets + data + HDMI conduit to the unit</t>
+          <t>long downrod, over the seating</t>
         </is>
       </c>
     </row>
@@ -13609,31 +13666,27 @@
         </is>
       </c>
       <c r="E70" s="4" t="n">
-        <v>38.4</v>
+        <v>48.6</v>
       </c>
       <c r="F70" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="G70" s="4" t="inlineStr">
-        <is>
-          <t>TV unit</t>
-        </is>
-      </c>
+        <v>24.6</v>
+      </c>
+      <c r="G70" s="4" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>TV</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
+          <t>TV + data point</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>7'-6"</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -13645,28 +13698,28 @@
         <v>38.4</v>
       </c>
       <c r="F71" s="4" t="n">
-        <v>20</v>
+        <v>22.4</v>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>above the TV unit, throws east over the seating</t>
+          <t>TV wall: 2 sockets + data + HDMI conduit to the unit</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>ODU</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>AC outdoor unit bracket</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>7'-0" outside</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
@@ -13675,93 +13728,97 @@
         </is>
       </c>
       <c r="E72" s="4" t="n">
-        <v>40</v>
+        <v>38.4</v>
       </c>
       <c r="F72" s="4" t="n">
-        <v>25.6</v>
+        <v>21</v>
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>north wall, shaded</t>
+          <t>TV unit</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>7'-6"</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Dining bay (north window)</t>
         </is>
       </c>
       <c r="E73" s="4" t="n">
-        <v>44.5</v>
+        <v>38.4</v>
       </c>
       <c r="F73" s="4" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>pendant</t>
+          <t>above the TV unit, throws east over the seating</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>ODU</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>AC outdoor unit bracket</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>7'-0" outside</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Dining bay (north window)</t>
         </is>
       </c>
       <c r="E74" s="4" t="n">
-        <v>38.4</v>
+        <v>40</v>
       </c>
       <c r="F74" s="4" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="G74" s="4" t="inlineStr"/>
+        <v>25.6</v>
+      </c>
+      <c r="G74" s="4" t="inlineStr">
+        <is>
+          <t>north wall, shaded</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -13770,27 +13827,31 @@
         </is>
       </c>
       <c r="E75" s="4" t="n">
-        <v>38.4</v>
+        <v>44.5</v>
       </c>
       <c r="F75" s="4" t="n">
-        <v>16.2</v>
-      </c>
-      <c r="G75" s="4" t="inlineStr"/>
+        <v>15</v>
+      </c>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>pendant</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>WL</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>Wall light / mirror light</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -13802,40 +13863,36 @@
         <v>38.4</v>
       </c>
       <c r="F76" s="4" t="n">
-        <v>13.7</v>
-      </c>
-      <c r="G76" s="4" t="inlineStr">
-        <is>
-          <t>dining and bay, at the passage</t>
-        </is>
-      </c>
+        <v>17.5</v>
+      </c>
+      <c r="G76" s="4" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area (open)</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E77" s="4" t="n">
-        <v>30.5</v>
+        <v>38.4</v>
       </c>
       <c r="F77" s="4" t="n">
-        <v>6.75</v>
+        <v>16.2</v>
       </c>
       <c r="G77" s="4" t="inlineStr"/>
     </row>
@@ -13857,31 +13914,35 @@
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area (open)</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E78" s="4" t="n">
-        <v>21.4</v>
+        <v>38.4</v>
       </c>
       <c r="F78" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="G78" s="4" t="inlineStr"/>
+        <v>13.7</v>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>dining and bay, at the passage</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>INV</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Inverter + battery</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>floor</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -13890,97 +13951,89 @@
         </is>
       </c>
       <c r="E79" s="4" t="n">
-        <v>22</v>
+        <v>30.5</v>
       </c>
       <c r="F79" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="G79" s="4" t="inlineStr">
-        <is>
-          <t>lithium inverter in a ventilated cabinet under the bench</t>
-        </is>
-      </c>
+        <v>6.75</v>
+      </c>
+      <c r="G79" s="4" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>Wet area (open to the walkway)</t>
+          <t>Sitting and serving area (open)</t>
         </is>
       </c>
       <c r="E80" s="4" t="n">
-        <v>50</v>
+        <v>21.4</v>
       </c>
       <c r="F80" s="4" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="G80" s="4" t="inlineStr">
-        <is>
-          <t>weatherproof</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="G80" s="4" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>INV</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>16 A power socket</t>
+          <t>Inverter + battery</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>floor</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>Wet area (open to the walkway)</t>
+          <t>Sitting and serving area (open)</t>
         </is>
       </c>
       <c r="E81" s="4" t="n">
-        <v>48.5</v>
+        <v>22</v>
       </c>
       <c r="F81" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>5</v>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>washing machine</t>
+          <t>lithium inverter in a ventilated cabinet under the bench</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -13989,93 +14042,97 @@
         </is>
       </c>
       <c r="E82" s="4" t="n">
-        <v>52.6</v>
+        <v>50</v>
       </c>
       <c r="F82" s="4" t="n">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>utility, weatherproof</t>
+          <t>weatherproof</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>16 A power socket</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>varies</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Wet area (open to the walkway)</t>
         </is>
       </c>
       <c r="E83" s="4" t="n">
-        <v>62</v>
+        <v>48.5</v>
       </c>
       <c r="F83" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="G83" s="4" t="inlineStr"/>
+        <v>8.699999999999999</v>
+      </c>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>washing machine</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Wet area (open to the walkway)</t>
         </is>
       </c>
       <c r="E84" s="4" t="n">
-        <v>61</v>
+        <v>52.6</v>
       </c>
       <c r="F84" s="4" t="n">
-        <v>3.5</v>
+        <v>6</v>
       </c>
       <c r="G84" s="4" t="inlineStr">
         <is>
-          <t>under-cabinet</t>
+          <t>utility, weatherproof</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
@@ -14084,31 +14141,27 @@
         </is>
       </c>
       <c r="E85" s="4" t="n">
-        <v>66.5</v>
+        <v>62</v>
       </c>
       <c r="F85" s="4" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="G85" s="4" t="inlineStr">
-        <is>
-          <t>under-cabinet</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="G85" s="4" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>WL</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Kitchen chimney point (16 A)</t>
+          <t>Wall light / mirror light</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>7'-0"</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -14117,31 +14170,31 @@
         </is>
       </c>
       <c r="E86" s="4" t="n">
-        <v>66.59999999999999</v>
+        <v>61</v>
       </c>
       <c r="F86" s="4" t="n">
-        <v>7.5</v>
+        <v>3.5</v>
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
-          <t>3 ft chimney on solid wall, duct out through the east wall</t>
+          <t>under-cabinet</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>WL</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>16 A power socket</t>
+          <t>Wall light / mirror light</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -14150,31 +14203,31 @@
         </is>
       </c>
       <c r="E87" s="4" t="n">
-        <v>58.75</v>
+        <v>66.5</v>
       </c>
       <c r="F87" s="4" t="n">
-        <v>12.7</v>
+        <v>9.6</v>
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>refrigerator, behind the fridge</t>
+          <t>under-cabinet</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>6 A socket at counter</t>
+          <t>Kitchen chimney point (16 A)</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>7'-0"</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -14183,27 +14236,31 @@
         </is>
       </c>
       <c r="E88" s="4" t="n">
-        <v>54.5</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="F88" s="4" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="G88" s="4" t="inlineStr"/>
+        <v>7.5</v>
+      </c>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>3 ft chimney on solid wall, duct out through the east wall</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>6 A socket at counter</t>
+          <t>16 A power socket</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>varies</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
@@ -14212,14 +14269,14 @@
         </is>
       </c>
       <c r="E89" s="4" t="n">
-        <v>58</v>
+        <v>58.75</v>
       </c>
       <c r="F89" s="4" t="n">
-        <v>3.5</v>
+        <v>12.7</v>
       </c>
       <c r="G89" s="4" t="inlineStr">
         <is>
-          <t>microwave / OTG</t>
+          <t>refrigerator, behind the fridge</t>
         </is>
       </c>
     </row>
@@ -14245,16 +14302,12 @@
         </is>
       </c>
       <c r="E90" s="4" t="n">
-        <v>63.5</v>
+        <v>54.5</v>
       </c>
       <c r="F90" s="4" t="n">
         <v>3.5</v>
       </c>
-      <c r="G90" s="4" t="inlineStr">
-        <is>
-          <t>mixer</t>
-        </is>
-      </c>
+      <c r="G90" s="4" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
@@ -14278,12 +14331,16 @@
         </is>
       </c>
       <c r="E91" s="4" t="n">
-        <v>66.59999999999999</v>
+        <v>58</v>
       </c>
       <c r="F91" s="4" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="G91" s="4" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>microwave / OTG</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
@@ -14307,12 +14364,16 @@
         </is>
       </c>
       <c r="E92" s="4" t="n">
-        <v>66.59999999999999</v>
+        <v>63.5</v>
       </c>
       <c r="F92" s="4" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="G92" s="4" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
+          <t>mixer</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
@@ -14336,31 +14397,27 @@
         </is>
       </c>
       <c r="E93" s="4" t="n">
-        <v>59.3</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="F93" s="4" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="G93" s="4" t="inlineStr">
-        <is>
-          <t>RO purifier, by sink</t>
-        </is>
-      </c>
+        <v>5.6</v>
+      </c>
+      <c r="G93" s="4" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>6 A socket at counter</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
@@ -14369,88 +14426,88 @@
         </is>
       </c>
       <c r="E94" s="4" t="n">
-        <v>53.4</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="F94" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="G94" s="4" t="inlineStr">
-        <is>
-          <t>beside the entry, latch side</t>
-        </is>
-      </c>
+        <v>9.6</v>
+      </c>
+      <c r="G94" s="4" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>Ceiling fan point</t>
+          <t>6 A socket at counter</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="E95" s="4" t="n">
-        <v>55</v>
+        <v>59.3</v>
       </c>
       <c r="F95" s="4" t="n">
-        <v>19</v>
+        <v>3.5</v>
       </c>
       <c r="G95" s="4" t="inlineStr">
         <is>
-          <t>long downrod</t>
+          <t>RO purifier, by sink</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="E96" s="4" t="n">
-        <v>52</v>
+        <v>53.4</v>
       </c>
       <c r="F96" s="4" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="G96" s="4" t="inlineStr"/>
+        <v>9</v>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>beside the entry, latch side</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Ceiling fan point</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
@@ -14467,57 +14524,57 @@
         <v>55</v>
       </c>
       <c r="F97" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="G97" s="4" t="inlineStr"/>
+        <v>19</v>
+      </c>
+      <c r="G97" s="4" t="inlineStr">
+        <is>
+          <t>long downrod</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>Dining bay (north window)</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="E98" s="4" t="n">
-        <v>48.2</v>
+        <v>52</v>
       </c>
       <c r="F98" s="4" t="n">
-        <v>18.4</v>
-      </c>
-      <c r="G98" s="4" t="inlineStr">
-        <is>
-          <t>floor socket, sofa end</t>
-        </is>
-      </c>
+        <v>22.5</v>
+      </c>
+      <c r="G98" s="4" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
@@ -14526,188 +14583,192 @@
         </is>
       </c>
       <c r="E99" s="4" t="n">
-        <v>52.6</v>
+        <v>55</v>
       </c>
       <c r="F99" s="4" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="G99" s="4" t="inlineStr">
-        <is>
-          <t>floor socket, armchair</t>
-        </is>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="G99" s="4" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Dining bay (north window)</t>
         </is>
       </c>
       <c r="E100" s="4" t="n">
-        <v>60.6</v>
+        <v>48.2</v>
       </c>
       <c r="F100" s="4" t="n">
-        <v>21</v>
+        <v>18.4</v>
       </c>
       <c r="G100" s="4" t="inlineStr">
         <is>
-          <t>main switch at door</t>
+          <t>floor socket, sofa end</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>Distribution board</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>5'-0" to top</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="E101" s="4" t="n">
-        <v>38.4</v>
+        <v>52.6</v>
       </c>
       <c r="F101" s="4" t="n">
-        <v>12.6</v>
+        <v>17.8</v>
       </c>
       <c r="G101" s="4" t="inlineStr">
         <is>
-          <t>dining face of Bedroom 2's east wall, by the passage; dry wall away from the pooja and wet area</t>
+          <t>floor socket, armchair</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Inverter (UPS) socket</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="E102" s="4" t="n">
-        <v>38.4</v>
+        <v>60.6</v>
       </c>
       <c r="F102" s="4" t="n">
-        <v>14.6</v>
+        <v>21</v>
       </c>
       <c r="G102" s="4" t="inlineStr">
         <is>
-          <t>router (central)</t>
+          <t>main switch at door</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Distribution board</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>5'-0" to top</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>Poomukham (verandah)</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E103" s="4" t="n">
-        <v>64</v>
+        <v>38.4</v>
       </c>
       <c r="F103" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="G103" s="4" t="inlineStr"/>
+        <v>12.6</v>
+      </c>
+      <c r="G103" s="4" t="inlineStr">
+        <is>
+          <t>dining face of Bedroom 2's east wall, by the passage; dry wall away from the pooja and wet area</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Inverter (UPS) socket</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>Poomukham (verandah)</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E104" s="4" t="n">
-        <v>64</v>
+        <v>38.4</v>
       </c>
       <c r="F104" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="G104" s="4" t="inlineStr"/>
+        <v>14.6</v>
+      </c>
+      <c r="G104" s="4" t="inlineStr">
+        <is>
+          <t>router (central)</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>BELL</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>Bell push</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>4'-6"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
@@ -14716,27 +14777,27 @@
         </is>
       </c>
       <c r="E105" s="4" t="n">
-        <v>61.4</v>
+        <v>64</v>
       </c>
       <c r="F105" s="4" t="n">
-        <v>20.4</v>
+        <v>16</v>
       </c>
       <c r="G105" s="4" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>CAM</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>CCTV point</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>8'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
@@ -14745,31 +14806,27 @@
         </is>
       </c>
       <c r="E106" s="4" t="n">
-        <v>66.5</v>
+        <v>64</v>
       </c>
       <c r="F106" s="4" t="n">
-        <v>24.6</v>
-      </c>
-      <c r="G106" s="4" t="inlineStr">
-        <is>
-          <t>covers gate and door</t>
-        </is>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="G106" s="4" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>BELL</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Bell push</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>4'-6"</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
@@ -14781,28 +14838,24 @@
         <v>61.4</v>
       </c>
       <c r="F107" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="G107" s="4" t="inlineStr">
-        <is>
-          <t>outdoor, weatherproof</t>
-        </is>
-      </c>
+        <v>20.4</v>
+      </c>
+      <c r="G107" s="4" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>CAM</t>
         </is>
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>CCTV point</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>8'-0"</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
@@ -14811,93 +14864,93 @@
         </is>
       </c>
       <c r="E108" s="4" t="n">
-        <v>61.4</v>
+        <v>66.5</v>
       </c>
       <c r="F108" s="4" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="G108" s="4" t="inlineStr"/>
+        <v>24.6</v>
+      </c>
+      <c r="G108" s="4" t="inlineStr">
+        <is>
+          <t>covers gate and door</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>MTR</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>Meter at gate</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>5'-0"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>Site</t>
+          <t>Poomukham (verandah)</t>
         </is>
       </c>
       <c r="E109" s="4" t="n">
-        <v>74.59999999999999</v>
+        <v>61.4</v>
       </c>
       <c r="F109" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G109" s="4" t="inlineStr">
         <is>
-          <t>meter in compound wall by gate</t>
+          <t>outdoor, weatherproof</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>GL</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>Outdoor / gate light</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>7'-0"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>Site</t>
+          <t>Poomukham (verandah)</t>
         </is>
       </c>
       <c r="E110" s="4" t="n">
-        <v>74.59999999999999</v>
+        <v>61.4</v>
       </c>
       <c r="F110" s="4" t="n">
-        <v>14.5</v>
-      </c>
-      <c r="G110" s="4" t="inlineStr">
-        <is>
-          <t>gate light</t>
-        </is>
-      </c>
+        <v>20.9</v>
+      </c>
+      <c r="G110" s="4" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>EP</t>
+          <t>MTR</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>Earth pit</t>
+          <t>Meter at gate</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>ground</t>
+          <t>5'-0"</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
@@ -14906,31 +14959,31 @@
         </is>
       </c>
       <c r="E111" s="4" t="n">
-        <v>68.2</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="F111" s="4" t="n">
-        <v>1.5</v>
+        <v>23</v>
       </c>
       <c r="G111" s="4" t="inlineStr">
         <is>
-          <t>earth pit 1</t>
+          <t>meter in compound wall by gate</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>EP</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>Earth pit</t>
+          <t>Outdoor / gate light</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>ground</t>
+          <t>7'-0"</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
@@ -14939,45 +14992,111 @@
         </is>
       </c>
       <c r="E112" s="4" t="n">
-        <v>73.5</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="F112" s="4" t="n">
-        <v>1.5</v>
+        <v>14.5</v>
       </c>
       <c r="G112" s="4" t="inlineStr">
         <is>
-          <t>earth pit 2</t>
+          <t>gate light</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
+          <t>EP</t>
+        </is>
+      </c>
+      <c r="B113" s="4" t="inlineStr">
+        <is>
+          <t>Earth pit</t>
+        </is>
+      </c>
+      <c r="C113" s="4" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="D113" s="4" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="E113" s="4" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="F113" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G113" s="4" t="inlineStr">
+        <is>
+          <t>earth pit 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="4" t="inlineStr">
+        <is>
+          <t>EP</t>
+        </is>
+      </c>
+      <c r="B114" s="4" t="inlineStr">
+        <is>
+          <t>Earth pit</t>
+        </is>
+      </c>
+      <c r="C114" s="4" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="D114" s="4" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="E114" s="4" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="F114" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G114" s="4" t="inlineStr">
+        <is>
+          <t>earth pit 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr">
+        <is>
           <t>GL</t>
         </is>
       </c>
-      <c r="B113" s="4" t="inlineStr">
+      <c r="B115" s="4" t="inlineStr">
         <is>
           <t>Outdoor / gate light</t>
         </is>
       </c>
-      <c r="C113" s="4" t="inlineStr">
+      <c r="C115" s="4" t="inlineStr">
         <is>
           <t>7'-0"</t>
         </is>
       </c>
-      <c r="D113" s="4" t="inlineStr">
+      <c r="D115" s="4" t="inlineStr">
         <is>
           <t>Site</t>
         </is>
       </c>
-      <c r="E113" s="4" t="n">
+      <c r="E115" s="4" t="n">
         <v>2.5</v>
       </c>
-      <c r="F113" s="4" t="n">
+      <c r="F115" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="G113" s="4" t="inlineStr">
+      <c r="G115" s="4" t="inlineStr">
         <is>
           <t>rear garden</t>
         </is>

</xml_diff>

<commit_message>
Bedroom 2: bed on the east wall, wardrobe to the west wall
Bed head east with bedsides both sides, clear of the entrance door;
work table north of the bed with its points; 6 ft wardrobe with a mirror
door on the wall shared with the master (dresser dropped); AC moved to the
bath's outer wall near the north corner. Leaves an open floor from the
door to the bath and window.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Schedules/KH-P1_Schedules_RevB.xlsx
+++ b/03_Schedules/KH-P1_Schedules_RevB.xlsx
@@ -4805,7 +4805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4950,7 +4950,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
+          <t>Twentieth review: Bedroom 2's bed moves to the east wall, head east, leaving an 8 x 14 ft open floor from the door to the bath and window; wardrobe to the west wall (sound buffer to the master), work table north of the bed, AC on the bath's outer wall; dresser dropped (mirror on the wardrobe).</t>
         </is>
       </c>
     </row>
@@ -4960,7 +4960,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
+          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
         </is>
       </c>
     </row>
@@ -4970,7 +4970,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
+          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
         </is>
       </c>
     </row>
@@ -4980,7 +4980,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
+          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
         </is>
       </c>
     </row>
@@ -4990,7 +4990,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
+          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
         </is>
       </c>
     </row>
@@ -5000,7 +5000,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
+          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
         </is>
       </c>
     </row>
@@ -5010,7 +5010,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
+          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
+          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
         </is>
       </c>
     </row>
@@ -5030,7 +5030,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
+          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
         </is>
       </c>
     </row>
@@ -5040,7 +5040,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
+          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
         </is>
       </c>
     </row>
@@ -5050,7 +5050,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
+          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
         </is>
       </c>
     </row>
@@ -5060,7 +5060,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
+          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
+          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
         </is>
       </c>
     </row>
@@ -5080,7 +5080,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
+          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
         </is>
       </c>
     </row>
@@ -5090,7 +5090,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
+          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
         </is>
       </c>
     </row>
@@ -5100,7 +5100,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
+          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
         </is>
       </c>
     </row>
@@ -5110,7 +5110,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
+          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
         </is>
       </c>
     </row>
@@ -5120,7 +5120,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
+          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
         </is>
       </c>
     </row>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
+          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
+          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
         </is>
       </c>
     </row>
@@ -5150,7 +5150,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
+          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
         </is>
       </c>
     </row>
@@ -5160,7 +5160,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
+          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
         </is>
       </c>
     </row>
@@ -5170,7 +5170,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
+          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
         </is>
       </c>
     </row>
@@ -5180,7 +5180,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
+          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
         </is>
       </c>
     </row>
@@ -5190,7 +5190,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
+          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
         </is>
       </c>
     </row>
@@ -5200,7 +5200,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
         </is>
       </c>
     </row>
@@ -5210,7 +5210,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
         </is>
       </c>
     </row>
@@ -5219,6 +5219,16 @@
         <v>40</v>
       </c>
       <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>Roof: Mangalore clay tiles on steel truss over insulated cement-fibre deck; all edge tiles mechanically fixed.</t>
         </is>
@@ -6390,7 +6400,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Bedroom 2 (from the sitting area, east end; open leaf screens the bed)</t>
+          <t>Bedroom 2 (from the sitting area, east end)</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
@@ -7337,7 +7347,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8246,7 +8256,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Queen bed 5' x 6'6" + headboard, head to the south wall, 2 ft+ free on both sides</t>
+          <t>Queen bed 5' x 6'6" + headboard, head to the east wall (padded headboard: TV on the other side)</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -8255,10 +8265,10 @@
         </is>
       </c>
       <c r="E21" s="4" t="n">
+        <v>6.35</v>
+      </c>
+      <c r="F21" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="F21" s="4" t="n">
-        <v>6.4</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8301,7 +8311,7 @@
         <v>1</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="G22" s="4" t="n">
         <v>2</v>
@@ -8322,7 +8332,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>F57</t>
+          <t>F22</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -8332,7 +8342,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Dresser / chest of drawers with mirror (west wall)</t>
+          <t>Work table 4' x 2' with monitor (east wall, north of the bed; north window to the side)</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -8341,7 +8351,7 @@
         </is>
       </c>
       <c r="E23" s="4" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="F23" s="4" t="n">
         <v>4</v>
@@ -8351,7 +8361,7 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Teak</t>
+          <t>Teak / ply, cable tray, monitor arm</t>
         </is>
       </c>
       <c r="I23" s="10" t="n"/>
@@ -8365,7 +8375,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>F22</t>
+          <t>F23</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -8375,7 +8385,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Work table 4' x 2' with monitor (east wall, south of the wardrobe)</t>
+          <t>Built-in wardrobe 6' with a mirror door (west wall, shared with the master: also a sound buffer)</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -8387,14 +8397,14 @@
         <v>2</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G24" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Teak / ply, cable tray, monitor arm</t>
+          <t>Ply + laminate</t>
         </is>
       </c>
       <c r="I24" s="10" t="n"/>
@@ -8408,36 +8418,36 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>F23</t>
+          <t>F24</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Bedroom 2</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Built-in wardrobe 6' (east wall, toward the house centre)</t>
+          <t>Dining table 5' x 3', 6-seat</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E25" s="4" t="n">
-        <v>1.8</v>
+        <v>5</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G25" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate</t>
+          <t>Teak or rosewood</t>
         </is>
       </c>
       <c r="I25" s="10" t="n"/>
@@ -8451,7 +8461,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>F24</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -8461,7 +8471,7 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Dining table 5' x 3', 6-seat</t>
+          <t>Dining chair</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -8470,17 +8480,17 @@
         </is>
       </c>
       <c r="E26" s="4" t="n">
-        <v>5</v>
+        <v>1.1</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Teak or rosewood</t>
+          <t>Teak + cane</t>
         </is>
       </c>
       <c r="I26" s="10" t="n"/>
@@ -8494,36 +8504,36 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F26</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Pooja</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Dining chair</t>
+          <t>Pooja mandapam on the east wall (idols face west; family faces east)</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E27" s="4" t="n">
-        <v>1.1</v>
+        <v>0.6</v>
       </c>
       <c r="F27" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G27" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G27" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Teak + cane</t>
+          <t>Carved teak</t>
         </is>
       </c>
       <c r="I27" s="10" t="n"/>
@@ -8537,36 +8547,36 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>F26</t>
+          <t>F28</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Pooja</t>
+          <t>Sitting and serving area</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Pooja mandapam on the east wall (idols face west; family faces east)</t>
+          <t>Built-in bench with storage drawers below</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E28" s="4" t="n">
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="G28" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Carved teak</t>
+          <t>Teak top, ply drawers, on legs</t>
         </is>
       </c>
       <c r="I28" s="10" t="n"/>
@@ -8580,36 +8590,36 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>F28</t>
+          <t>F29</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area</t>
+          <t>Wet area</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Built-in bench with storage drawers below</t>
+          <t>Utility sink counter (on the kitchen wall)</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Sanitary / plumbing</t>
         </is>
       </c>
       <c r="E29" s="4" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>2.8</v>
+        <v>2.5</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>Teak top, ply drawers, on legs</t>
+          <t>Kadappa / granite, SS sinks</t>
         </is>
       </c>
       <c r="I29" s="10" t="n"/>
@@ -8623,7 +8633,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>F29</t>
+          <t>F30</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -8633,26 +8643,26 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Utility sink counter (on the kitchen wall)</t>
+          <t>Washing machine bay 2' x 2' (covered back corner, 2 in clear of the bath wall)</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Sanitary / plumbing</t>
+          <t>Appliance / joinery</t>
         </is>
       </c>
       <c r="E30" s="4" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>2.5</v>
+        <v>1.9</v>
       </c>
       <c r="G30" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Kadappa / granite, SS sinks</t>
+          <t>Splash-proof socket, floor drain</t>
         </is>
       </c>
       <c r="I30" s="10" t="n"/>
@@ -8666,7 +8676,7 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>F30</t>
+          <t>F31</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -8676,26 +8686,26 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Washing machine bay 2' x 2' (covered back corner, 2 in clear of the bath wall)</t>
+          <t>Fold-away clothesline in the south walkway</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Appliance / joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E31" s="4" t="n">
-        <v>1.9</v>
+        <v>4</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>Splash-proof socket, floor drain</t>
+          <t>SS wire, wall brackets</t>
         </is>
       </c>
       <c r="I31" s="10" t="n"/>
@@ -8709,7 +8719,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>F31</t>
+          <t>F44</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -8719,26 +8729,26 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Fold-away clothesline in the south walkway</t>
+          <t>Tall slim utility cupboard (brooms, mops, detergents)</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E32" s="4" t="n">
-        <v>4</v>
+        <v>1.2</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
       <c r="G32" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>SS wire, wall brackets</t>
+          <t>Ply + laminate on legs, louvred doors</t>
         </is>
       </c>
       <c r="I32" s="10" t="n"/>
@@ -8752,36 +8762,36 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>F44</t>
+          <t>F32</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Wet area</t>
+          <t>Sitting and serving area</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Tall slim utility cupboard (brooms, mops, detergents)</t>
+          <t>Hand-wash basin at the east end of the serving counter, just outside the common bath (after meals); mirror on the side wall</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Sanitary / plumbing</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
-        <v>1.2</v>
+        <v>1.9</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate on legs, louvred doors</t>
+          <t>Ceramic basin in granite top</t>
         </is>
       </c>
       <c r="I33" s="10" t="n"/>
@@ -8795,7 +8805,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>F32</t>
+          <t>F33</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -8805,16 +8815,16 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Hand-wash basin at the east end of the serving counter, just outside the common bath (after meals); mirror on the side wall</t>
+          <t>Serving counter with crockery cabinets above, 6 ft</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Sanitary / plumbing</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E34" s="4" t="n">
-        <v>1.9</v>
+        <v>6</v>
       </c>
       <c r="F34" s="4" t="n">
         <v>2</v>
@@ -8824,7 +8834,7 @@
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>Ceramic basin in granite top</t>
+          <t>Granite top, teak + glass shutters</t>
         </is>
       </c>
       <c r="I34" s="10" t="n"/>
@@ -8838,7 +8848,7 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>F33</t>
+          <t>F56</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -8848,7 +8858,7 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Serving counter with crockery cabinets above, 6 ft</t>
+          <t>Tall storage cupboard 5' x 2' (bedding, suitcases, festival vessels), loft above</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -8857,7 +8867,7 @@
         </is>
       </c>
       <c r="E35" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F35" s="4" t="n">
         <v>2</v>
@@ -8867,7 +8877,7 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>Granite top, teak + glass shutters</t>
+          <t>Ply + laminate, full height</t>
         </is>
       </c>
       <c r="I35" s="10" t="n"/>
@@ -8881,17 +8891,17 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>F56</t>
+          <t>F34</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Tall storage cupboard 5' x 2' (bedding, suitcases, festival vessels), loft above</t>
+          <t>L-counter, south run</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -8900,7 +8910,7 @@
         </is>
       </c>
       <c r="E36" s="4" t="n">
-        <v>5</v>
+        <v>13.2</v>
       </c>
       <c r="F36" s="4" t="n">
         <v>2</v>
@@ -8910,7 +8920,7 @@
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate, full height</t>
+          <t>Granite top, ply carcass</t>
         </is>
       </c>
       <c r="I36" s="10" t="n"/>
@@ -8924,7 +8934,7 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>F34</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -8934,7 +8944,7 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>L-counter, south run</t>
+          <t>L-counter, east run (hob centred 7'-6" from the south wall face, on solid wall)</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -8943,17 +8953,17 @@
         </is>
       </c>
       <c r="E37" s="4" t="n">
-        <v>13.2</v>
+        <v>2</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>Granite top, ply carcass</t>
+          <t>Granite top, cook faces east</t>
         </is>
       </c>
       <c r="I37" s="10" t="n"/>
@@ -8967,7 +8977,7 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F36</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -8977,26 +8987,26 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>L-counter, east run (hob centred 7'-6" from the south wall face, on solid wall)</t>
+          <t>Refrigerator space (kitchen north wall, behind the pooja, door facing south)</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Appliance / joinery</t>
         </is>
       </c>
       <c r="E38" s="4" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>7</v>
+        <v>2.4</v>
       </c>
       <c r="G38" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Granite top, cook faces east</t>
+          <t>Double-door, 2'6" wide</t>
         </is>
       </c>
       <c r="I38" s="10" t="n"/>
@@ -9010,7 +9020,7 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>F36</t>
+          <t>F55</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -9020,26 +9030,26 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Refrigerator space (kitchen north wall, behind the pooja, door facing south)</t>
+          <t>Tall pantry 4'-5" x 2' on the north wall (provisions, rice, vessels)</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Appliance / joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E39" s="4" t="n">
-        <v>2.5</v>
+        <v>4.4</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Double-door, 2'6" wide</t>
+          <t>Ply + laminate, full height with loft</t>
         </is>
       </c>
       <c r="I39" s="10" t="n"/>
@@ -9053,17 +9063,17 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>F55</t>
+          <t>F38</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Dining bay</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Tall pantry 4'-5" x 2' on the north wall (provisions, rice, vessels)</t>
+          <t>Three-seat sofa 6'6" facing west to the TV</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -9072,17 +9082,17 @@
         </is>
       </c>
       <c r="E40" s="4" t="n">
-        <v>4.4</v>
+        <v>2.7</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>2</v>
+        <v>5.9</v>
       </c>
       <c r="G40" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate, full height with loft</t>
+          <t>Teak frame, cotton cushions</t>
         </is>
       </c>
       <c r="I40" s="10" t="n"/>
@@ -9096,7 +9106,7 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>F38</t>
+          <t>F39</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
@@ -9106,7 +9116,7 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Three-seat sofa 6'6" facing west to the TV</t>
+          <t>Coffee table 3'6" x 2'</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -9115,17 +9125,17 @@
         </is>
       </c>
       <c r="E41" s="4" t="n">
-        <v>2.7</v>
+        <v>2</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>5.9</v>
+        <v>3.5</v>
       </c>
       <c r="G41" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>Teak frame, cotton cushions</t>
+          <t>Teak</t>
         </is>
       </c>
       <c r="I41" s="10" t="n"/>
@@ -9139,7 +9149,7 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>F39</t>
+          <t>F53</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -9149,26 +9159,26 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Coffee table 3'6" x 2'</t>
+          <t>TV unit 4'-5" on Bedroom 2's east wall (55-65 in TV wall-mounted above)</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Appliance / joinery</t>
         </is>
       </c>
       <c r="E42" s="4" t="n">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>3.5</v>
+        <v>4.4</v>
       </c>
       <c r="G42" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>Teak</t>
+          <t>Teak, low, open shelves</t>
         </is>
       </c>
       <c r="I42" s="10" t="n"/>
@@ -9182,36 +9192,36 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>F53</t>
+          <t>F40</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Dining bay</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>TV unit 4'-5" on Bedroom 2's east wall (55-65 in TV wall-mounted above)</t>
+          <t>Armchair by the north window</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Appliance / joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E43" s="4" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>4.4</v>
+        <v>1.6</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>Teak, low, open shelves</t>
+          <t>Cane / teak</t>
         </is>
       </c>
       <c r="I43" s="10" t="n"/>
@@ -9225,7 +9235,7 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>F40</t>
+          <t>F52</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -9235,26 +9245,26 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Armchair by the north window</t>
+          <t>Shoe cupboard 3'-3" beside the main door (closed shutters, louvred for air)</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E44" s="4" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>1.6</v>
+        <v>3.2</v>
       </c>
       <c r="G44" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>Cane / teak</t>
+          <t>Ply + laminate, 14 in deep</t>
         </is>
       </c>
       <c r="I44" s="10" t="n"/>
@@ -9268,36 +9278,36 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>F52</t>
+          <t>F41</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Poomukham (verandah)</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Shoe cupboard 3'-3" beside the main door (closed shutters, louvred for air)</t>
+          <t>Oonjal (swing) 3'6"</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E45" s="4" t="n">
-        <v>1.2</v>
+        <v>3.5</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>3.2</v>
+        <v>1.5</v>
       </c>
       <c r="G45" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate, 14 in deep</t>
+          <t>Teak, chains to beam</t>
         </is>
       </c>
       <c r="I45" s="10" t="n"/>
@@ -9311,7 +9321,7 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>F41</t>
+          <t>F42</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -9321,26 +9331,26 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Oonjal (swing) 3'6"</t>
+          <t>Arugu seat (built-in, south end)</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E46" s="4" t="n">
-        <v>3.5</v>
+        <v>1.2</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>1.5</v>
+        <v>2.4</v>
       </c>
       <c r="G46" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>Teak, chains to beam</t>
+          <t>Laterite base, teak top</t>
         </is>
       </c>
       <c r="I46" s="10" t="n"/>
@@ -9352,71 +9362,28 @@
       <c r="L46" s="8" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>F42</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>Poomukham (verandah)</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>Arugu seat (built-in, south end)</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>Built-in joinery</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="F47" s="4" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="G47" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H47" s="4" t="inlineStr">
-        <is>
-          <t>Laterite base, teak top</t>
-        </is>
-      </c>
-      <c r="I47" s="10" t="n"/>
-      <c r="J47" s="11">
-        <f>G47*I47</f>
+      <c r="A47" s="6" t="inlineStr"/>
+      <c r="B47" s="6" t="inlineStr"/>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr"/>
+      <c r="E47" s="6" t="inlineStr"/>
+      <c r="F47" s="6" t="inlineStr"/>
+      <c r="G47" s="6">
+        <f>SUM(G2:G46)</f>
         <v/>
       </c>
-      <c r="K47" s="8" t="inlineStr"/>
-      <c r="L47" s="8" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="6" t="inlineStr"/>
-      <c r="B48" s="6" t="inlineStr"/>
-      <c r="C48" s="6" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="D48" s="6" t="inlineStr"/>
-      <c r="E48" s="6" t="inlineStr"/>
-      <c r="F48" s="6" t="inlineStr"/>
-      <c r="G48" s="6">
-        <f>SUM(G2:G47)</f>
+      <c r="H47" s="6" t="inlineStr"/>
+      <c r="I47" s="12" t="inlineStr"/>
+      <c r="J47" s="12">
+        <f>SUM(J2:J46)</f>
         <v/>
       </c>
-      <c r="H48" s="6" t="inlineStr"/>
-      <c r="I48" s="12" t="inlineStr"/>
-      <c r="J48" s="12">
-        <f>SUM(J2:J47)</f>
-        <v/>
-      </c>
-      <c r="K48" s="6" t="inlineStr"/>
-      <c r="L48" s="6" t="inlineStr"/>
+      <c r="K47" s="6" t="inlineStr"/>
+      <c r="L47" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11435,7 +11402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G115"/>
+  <dimension ref="A1:G114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -13022,10 +12989,10 @@
         </is>
       </c>
       <c r="E50" s="4" t="n">
-        <v>29.4</v>
+        <v>34.6</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>15</v>
+        <v>16.5</v>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
@@ -13055,10 +13022,10 @@
         </is>
       </c>
       <c r="E51" s="4" t="n">
-        <v>29.4</v>
+        <v>37.6</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>10.9</v>
+        <v>16.5</v>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
@@ -13208,10 +13175,10 @@
         </is>
       </c>
       <c r="E56" s="4" t="n">
-        <v>25.4</v>
+        <v>37.6</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>10.9</v>
+        <v>13</v>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
@@ -13241,10 +13208,10 @@
         </is>
       </c>
       <c r="E57" s="4" t="n">
-        <v>26</v>
+        <v>37.6</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>10.9</v>
+        <v>13.5</v>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
@@ -13274,10 +13241,10 @@
         </is>
       </c>
       <c r="E58" s="4" t="n">
-        <v>32.4</v>
+        <v>37.6</v>
       </c>
       <c r="F58" s="4" t="n">
-        <v>10.9</v>
+        <v>19.5</v>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
@@ -13307,10 +13274,10 @@
         </is>
       </c>
       <c r="E59" s="4" t="n">
-        <v>32.9</v>
+        <v>37.6</v>
       </c>
       <c r="F59" s="4" t="n">
-        <v>10.9</v>
+        <v>19.9</v>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
@@ -13340,26 +13307,26 @@
         </is>
       </c>
       <c r="E60" s="4" t="n">
-        <v>21.4</v>
+        <v>37.6</v>
       </c>
       <c r="F60" s="4" t="n">
-        <v>13.5</v>
+        <v>20.8</v>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>dresser</t>
+          <t>work table</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Inverter (UPS) socket</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -13376,23 +13343,23 @@
         <v>37.6</v>
       </c>
       <c r="F61" s="4" t="n">
-        <v>15</v>
+        <v>21.6</v>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>work table</t>
+          <t>work table, monitor</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Inverter (UPS) socket</t>
+          <t>Data point (Cat6)</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -13409,23 +13376,23 @@
         <v>37.6</v>
       </c>
       <c r="F62" s="4" t="n">
-        <v>15.8</v>
+        <v>22.4</v>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>work table, monitor</t>
+          <t>work table</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Data point (Cat6)</t>
+          <t>Inverter (UPS) socket</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
@@ -13442,7 +13409,7 @@
         <v>37.6</v>
       </c>
       <c r="F63" s="4" t="n">
-        <v>16.6</v>
+        <v>23.2</v>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
@@ -13453,17 +13420,17 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Inverter (UPS) socket</t>
+          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>7'-6"</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -13472,125 +13439,121 @@
         </is>
       </c>
       <c r="E64" s="4" t="n">
-        <v>37.6</v>
+        <v>28.4</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>17.4</v>
+        <v>24</v>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>work table</t>
+          <t>high on the bath's east wall near the north corner, throws east toward the bed foot</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>WL</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
+          <t>Wall light / mirror light</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>7'-6"</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Bedroom 2</t>
+          <t>Sitting and serving area (open)</t>
         </is>
       </c>
       <c r="E65" s="4" t="n">
-        <v>37.6</v>
+        <v>41.1</v>
       </c>
       <c r="F65" s="4" t="n">
-        <v>18.6</v>
+        <v>4.4</v>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>east wall, not at the work table</t>
+          <t>over basin, on the common bath wall</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>ODU</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>AC outdoor unit bracket</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>7'-0" outside</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area (open)</t>
+          <t>Bedroom 2</t>
         </is>
       </c>
       <c r="E66" s="4" t="n">
-        <v>41.1</v>
+        <v>29.5</v>
       </c>
       <c r="F66" s="4" t="n">
-        <v>4.4</v>
+        <v>25.6</v>
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>over basin, on the common bath wall</t>
+          <t>north wall, shaded</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>ODU</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>AC outdoor unit bracket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>7'-0" outside</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Bedroom 2</t>
+          <t>Dining bay (north window)</t>
         </is>
       </c>
       <c r="E67" s="4" t="n">
-        <v>33</v>
+        <v>41.5</v>
       </c>
       <c r="F67" s="4" t="n">
-        <v>25.6</v>
-      </c>
-      <c r="G67" s="4" t="inlineStr">
-        <is>
-          <t>north wall, shaded</t>
-        </is>
-      </c>
+        <v>21.5</v>
+      </c>
+      <c r="G67" s="4" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Ceiling fan point</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
@@ -13604,27 +13567,31 @@
         </is>
       </c>
       <c r="E68" s="4" t="n">
-        <v>41.5</v>
+        <v>45</v>
       </c>
       <c r="F68" s="4" t="n">
         <v>21.5</v>
       </c>
-      <c r="G68" s="4" t="inlineStr"/>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t>long downrod, over the seating</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Ceiling fan point</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -13633,31 +13600,27 @@
         </is>
       </c>
       <c r="E69" s="4" t="n">
-        <v>45</v>
+        <v>48.6</v>
       </c>
       <c r="F69" s="4" t="n">
-        <v>21.5</v>
-      </c>
-      <c r="G69" s="4" t="inlineStr">
-        <is>
-          <t>long downrod, over the seating</t>
-        </is>
-      </c>
+        <v>24.6</v>
+      </c>
+      <c r="G69" s="4" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>TV</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>TV + data point</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -13666,27 +13629,31 @@
         </is>
       </c>
       <c r="E70" s="4" t="n">
-        <v>48.6</v>
+        <v>38.4</v>
       </c>
       <c r="F70" s="4" t="n">
-        <v>24.6</v>
-      </c>
-      <c r="G70" s="4" t="inlineStr"/>
+        <v>22.4</v>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t>TV wall: 2 sockets + data + HDMI conduit to the unit</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>TV</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>TV + data point</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -13698,28 +13665,28 @@
         <v>38.4</v>
       </c>
       <c r="F71" s="4" t="n">
-        <v>22.4</v>
+        <v>21</v>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>TV wall: 2 sockets + data + HDMI conduit to the unit</t>
+          <t>TV unit</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>7'-6"</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
@@ -13731,28 +13698,28 @@
         <v>38.4</v>
       </c>
       <c r="F72" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>TV unit</t>
+          <t>above the TV unit, throws east over the seating</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>ODU</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
+          <t>AC outdoor unit bracket</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>7'-6"</t>
+          <t>7'-0" outside</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
@@ -13761,64 +13728,64 @@
         </is>
       </c>
       <c r="E73" s="4" t="n">
-        <v>38.4</v>
+        <v>40</v>
       </c>
       <c r="F73" s="4" t="n">
-        <v>20</v>
+        <v>25.6</v>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>above the TV unit, throws east over the seating</t>
+          <t>north wall, shaded</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>ODU</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>AC outdoor unit bracket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>7'-0" outside</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>Dining bay (north window)</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E74" s="4" t="n">
-        <v>40</v>
+        <v>44.5</v>
       </c>
       <c r="F74" s="4" t="n">
-        <v>25.6</v>
+        <v>15</v>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>north wall, shaded</t>
+          <t>pendant</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>WL</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Wall light / mirror light</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -13827,31 +13794,27 @@
         </is>
       </c>
       <c r="E75" s="4" t="n">
-        <v>44.5</v>
+        <v>38.4</v>
       </c>
       <c r="F75" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G75" s="4" t="inlineStr">
-        <is>
-          <t>pendant</t>
-        </is>
-      </c>
+        <v>17.5</v>
+      </c>
+      <c r="G75" s="4" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -13863,24 +13826,24 @@
         <v>38.4</v>
       </c>
       <c r="F76" s="4" t="n">
-        <v>17.5</v>
+        <v>16.2</v>
       </c>
       <c r="G76" s="4" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
@@ -13892,57 +13855,57 @@
         <v>38.4</v>
       </c>
       <c r="F77" s="4" t="n">
-        <v>16.2</v>
-      </c>
-      <c r="G77" s="4" t="inlineStr"/>
+        <v>13.7</v>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>dining and bay, at the passage</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Sitting and serving area (open)</t>
         </is>
       </c>
       <c r="E78" s="4" t="n">
-        <v>38.4</v>
+        <v>30.5</v>
       </c>
       <c r="F78" s="4" t="n">
-        <v>13.7</v>
-      </c>
-      <c r="G78" s="4" t="inlineStr">
-        <is>
-          <t>dining and bay, at the passage</t>
-        </is>
-      </c>
+        <v>6.75</v>
+      </c>
+      <c r="G78" s="4" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -13951,27 +13914,27 @@
         </is>
       </c>
       <c r="E79" s="4" t="n">
-        <v>30.5</v>
+        <v>21.4</v>
       </c>
       <c r="F79" s="4" t="n">
-        <v>6.75</v>
+        <v>6</v>
       </c>
       <c r="G79" s="4" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>INV</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>Inverter + battery</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>floor</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -13980,60 +13943,64 @@
         </is>
       </c>
       <c r="E80" s="4" t="n">
-        <v>21.4</v>
+        <v>22</v>
       </c>
       <c r="F80" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="G80" s="4" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>lithium inverter in a ventilated cabinet under the bench</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>INV</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Inverter + battery</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>floor</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area (open)</t>
+          <t>Wet area (open to the walkway)</t>
         </is>
       </c>
       <c r="E81" s="4" t="n">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="F81" s="4" t="n">
-        <v>5</v>
+        <v>5.5</v>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>lithium inverter in a ventilated cabinet under the bench</t>
+          <t>weatherproof</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>16 A power socket</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>varies</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -14042,31 +14009,31 @@
         </is>
       </c>
       <c r="E82" s="4" t="n">
-        <v>50</v>
+        <v>48.5</v>
       </c>
       <c r="F82" s="4" t="n">
-        <v>5.5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>weatherproof</t>
+          <t>washing machine</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>16 A power socket</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
@@ -14075,64 +14042,60 @@
         </is>
       </c>
       <c r="E83" s="4" t="n">
-        <v>48.5</v>
+        <v>52.6</v>
       </c>
       <c r="F83" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>6</v>
       </c>
       <c r="G83" s="4" t="inlineStr">
         <is>
-          <t>washing machine</t>
+          <t>utility, weatherproof</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>Wet area (open to the walkway)</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="E84" s="4" t="n">
-        <v>52.6</v>
+        <v>62</v>
       </c>
       <c r="F84" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="G84" s="4" t="inlineStr">
-        <is>
-          <t>utility, weatherproof</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="G84" s="4" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>WL</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Wall light / mirror light</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
@@ -14141,12 +14104,16 @@
         </is>
       </c>
       <c r="E85" s="4" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F85" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="G85" s="4" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>under-cabinet</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
@@ -14170,10 +14137,10 @@
         </is>
       </c>
       <c r="E86" s="4" t="n">
-        <v>61</v>
+        <v>66.5</v>
       </c>
       <c r="F86" s="4" t="n">
-        <v>3.5</v>
+        <v>9.6</v>
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
@@ -14184,17 +14151,17 @@
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>Kitchen chimney point (16 A)</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>7'-0"</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -14203,31 +14170,31 @@
         </is>
       </c>
       <c r="E87" s="4" t="n">
-        <v>66.5</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="F87" s="4" t="n">
-        <v>9.6</v>
+        <v>7.5</v>
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>under-cabinet</t>
+          <t>3 ft chimney on solid wall, duct out through the east wall</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Kitchen chimney point (16 A)</t>
+          <t>16 A power socket</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>7'-0"</t>
+          <t>varies</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -14236,31 +14203,31 @@
         </is>
       </c>
       <c r="E88" s="4" t="n">
-        <v>66.59999999999999</v>
+        <v>58.75</v>
       </c>
       <c r="F88" s="4" t="n">
-        <v>7.5</v>
+        <v>12.7</v>
       </c>
       <c r="G88" s="4" t="inlineStr">
         <is>
-          <t>3 ft chimney on solid wall, duct out through the east wall</t>
+          <t>refrigerator, behind the fridge</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>16 A power socket</t>
+          <t>6 A socket at counter</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
@@ -14269,16 +14236,12 @@
         </is>
       </c>
       <c r="E89" s="4" t="n">
-        <v>58.75</v>
+        <v>54.5</v>
       </c>
       <c r="F89" s="4" t="n">
-        <v>12.7</v>
-      </c>
-      <c r="G89" s="4" t="inlineStr">
-        <is>
-          <t>refrigerator, behind the fridge</t>
-        </is>
-      </c>
+        <v>3.5</v>
+      </c>
+      <c r="G89" s="4" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
@@ -14302,12 +14265,16 @@
         </is>
       </c>
       <c r="E90" s="4" t="n">
-        <v>54.5</v>
+        <v>58</v>
       </c>
       <c r="F90" s="4" t="n">
         <v>3.5</v>
       </c>
-      <c r="G90" s="4" t="inlineStr"/>
+      <c r="G90" s="4" t="inlineStr">
+        <is>
+          <t>microwave / OTG</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
@@ -14331,14 +14298,14 @@
         </is>
       </c>
       <c r="E91" s="4" t="n">
-        <v>58</v>
+        <v>63.5</v>
       </c>
       <c r="F91" s="4" t="n">
         <v>3.5</v>
       </c>
       <c r="G91" s="4" t="inlineStr">
         <is>
-          <t>microwave / OTG</t>
+          <t>mixer</t>
         </is>
       </c>
     </row>
@@ -14364,16 +14331,12 @@
         </is>
       </c>
       <c r="E92" s="4" t="n">
-        <v>63.5</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="F92" s="4" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="G92" s="4" t="inlineStr">
-        <is>
-          <t>mixer</t>
-        </is>
-      </c>
+        <v>5.6</v>
+      </c>
+      <c r="G92" s="4" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
@@ -14400,7 +14363,7 @@
         <v>66.59999999999999</v>
       </c>
       <c r="F93" s="4" t="n">
-        <v>5.6</v>
+        <v>9.6</v>
       </c>
       <c r="G93" s="4" t="inlineStr"/>
     </row>
@@ -14426,27 +14389,31 @@
         </is>
       </c>
       <c r="E94" s="4" t="n">
-        <v>66.59999999999999</v>
+        <v>59.3</v>
       </c>
       <c r="F94" s="4" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="G94" s="4" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="G94" s="4" t="inlineStr">
+        <is>
+          <t>RO purifier, by sink</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>6 A socket at counter</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
@@ -14455,59 +14422,59 @@
         </is>
       </c>
       <c r="E95" s="4" t="n">
-        <v>59.3</v>
+        <v>53.4</v>
       </c>
       <c r="F95" s="4" t="n">
-        <v>3.5</v>
+        <v>9</v>
       </c>
       <c r="G95" s="4" t="inlineStr">
         <is>
-          <t>RO purifier, by sink</t>
+          <t>beside the entry, latch side</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>Ceiling fan point</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="E96" s="4" t="n">
-        <v>53.4</v>
+        <v>55</v>
       </c>
       <c r="F96" s="4" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="G96" s="4" t="inlineStr">
         <is>
-          <t>beside the entry, latch side</t>
+          <t>long downrod</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>Ceiling fan point</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
@@ -14521,16 +14488,12 @@
         </is>
       </c>
       <c r="E97" s="4" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F97" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="G97" s="4" t="inlineStr">
-        <is>
-          <t>long downrod</t>
-        </is>
-      </c>
+        <v>22.5</v>
+      </c>
+      <c r="G97" s="4" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
@@ -14554,41 +14517,45 @@
         </is>
       </c>
       <c r="E98" s="4" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F98" s="4" t="n">
-        <v>22.5</v>
+        <v>16</v>
       </c>
       <c r="G98" s="4" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Dining bay (north window)</t>
         </is>
       </c>
       <c r="E99" s="4" t="n">
-        <v>55</v>
+        <v>48.2</v>
       </c>
       <c r="F99" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="G99" s="4" t="inlineStr"/>
+        <v>18.4</v>
+      </c>
+      <c r="G99" s="4" t="inlineStr">
+        <is>
+          <t>floor socket, sofa end</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
@@ -14608,35 +14575,35 @@
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>Dining bay (north window)</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="E100" s="4" t="n">
-        <v>48.2</v>
+        <v>52.6</v>
       </c>
       <c r="F100" s="4" t="n">
-        <v>18.4</v>
+        <v>17.8</v>
       </c>
       <c r="G100" s="4" t="inlineStr">
         <is>
-          <t>floor socket, sofa end</t>
+          <t>floor socket, armchair</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
@@ -14645,64 +14612,64 @@
         </is>
       </c>
       <c r="E101" s="4" t="n">
-        <v>52.6</v>
+        <v>60.6</v>
       </c>
       <c r="F101" s="4" t="n">
-        <v>17.8</v>
+        <v>21</v>
       </c>
       <c r="G101" s="4" t="inlineStr">
         <is>
-          <t>floor socket, armchair</t>
+          <t>main switch at door</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>Distribution board</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>5'-0" to top</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E102" s="4" t="n">
-        <v>60.6</v>
+        <v>38.4</v>
       </c>
       <c r="F102" s="4" t="n">
-        <v>21</v>
+        <v>12.6</v>
       </c>
       <c r="G102" s="4" t="inlineStr">
         <is>
-          <t>main switch at door</t>
+          <t>dining face of Bedroom 2's east wall, by the passage; dry wall away from the pooja and wet area</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>Distribution board</t>
+          <t>Inverter (UPS) socket</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>5'-0" to top</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
@@ -14714,46 +14681,42 @@
         <v>38.4</v>
       </c>
       <c r="F103" s="4" t="n">
-        <v>12.6</v>
+        <v>14.6</v>
       </c>
       <c r="G103" s="4" t="inlineStr">
         <is>
-          <t>dining face of Bedroom 2's east wall, by the passage; dry wall away from the pooja and wet area</t>
+          <t>router (central)</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>Inverter (UPS) socket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Poomukham (verandah)</t>
         </is>
       </c>
       <c r="E104" s="4" t="n">
-        <v>38.4</v>
+        <v>64</v>
       </c>
       <c r="F104" s="4" t="n">
-        <v>14.6</v>
-      </c>
-      <c r="G104" s="4" t="inlineStr">
-        <is>
-          <t>router (central)</t>
-        </is>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="G104" s="4" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -14780,24 +14743,24 @@
         <v>64</v>
       </c>
       <c r="F105" s="4" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="G105" s="4" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>BELL</t>
         </is>
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Bell push</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>4'-6"</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
@@ -14806,27 +14769,27 @@
         </is>
       </c>
       <c r="E106" s="4" t="n">
-        <v>64</v>
+        <v>61.4</v>
       </c>
       <c r="F106" s="4" t="n">
-        <v>22</v>
+        <v>20.4</v>
       </c>
       <c r="G106" s="4" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>BELL</t>
+          <t>CAM</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>Bell push</t>
+          <t>CCTV point</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>4'-6"</t>
+          <t>8'-0"</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
@@ -14835,27 +14798,31 @@
         </is>
       </c>
       <c r="E107" s="4" t="n">
-        <v>61.4</v>
+        <v>66.5</v>
       </c>
       <c r="F107" s="4" t="n">
-        <v>20.4</v>
-      </c>
-      <c r="G107" s="4" t="inlineStr"/>
+        <v>24.6</v>
+      </c>
+      <c r="G107" s="4" t="inlineStr">
+        <is>
+          <t>covers gate and door</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>CAM</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>CCTV point</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>8'-0"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
@@ -14864,31 +14831,31 @@
         </is>
       </c>
       <c r="E108" s="4" t="n">
-        <v>66.5</v>
+        <v>61.4</v>
       </c>
       <c r="F108" s="4" t="n">
-        <v>24.6</v>
+        <v>24</v>
       </c>
       <c r="G108" s="4" t="inlineStr">
         <is>
-          <t>covers gate and door</t>
+          <t>outdoor, weatherproof</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
@@ -14900,57 +14867,57 @@
         <v>61.4</v>
       </c>
       <c r="F109" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="G109" s="4" t="inlineStr">
-        <is>
-          <t>outdoor, weatherproof</t>
-        </is>
-      </c>
+        <v>20.9</v>
+      </c>
+      <c r="G109" s="4" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>MTR</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>Meter at gate</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>5'-0"</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>Poomukham (verandah)</t>
+          <t>Site</t>
         </is>
       </c>
       <c r="E110" s="4" t="n">
-        <v>61.4</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="F110" s="4" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="G110" s="4" t="inlineStr"/>
+        <v>23</v>
+      </c>
+      <c r="G110" s="4" t="inlineStr">
+        <is>
+          <t>meter in compound wall by gate</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>MTR</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>Meter at gate</t>
+          <t>Outdoor / gate light</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>5'-0"</t>
+          <t>7'-0"</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
@@ -14962,28 +14929,28 @@
         <v>74.59999999999999</v>
       </c>
       <c r="F111" s="4" t="n">
-        <v>23</v>
+        <v>14.5</v>
       </c>
       <c r="G111" s="4" t="inlineStr">
         <is>
-          <t>meter in compound wall by gate</t>
+          <t>gate light</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>GL</t>
+          <t>EP</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>Outdoor / gate light</t>
+          <t>Earth pit</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>7'-0"</t>
+          <t>ground</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
@@ -14992,14 +14959,14 @@
         </is>
       </c>
       <c r="E112" s="4" t="n">
-        <v>74.59999999999999</v>
+        <v>68.2</v>
       </c>
       <c r="F112" s="4" t="n">
-        <v>14.5</v>
+        <v>1.5</v>
       </c>
       <c r="G112" s="4" t="inlineStr">
         <is>
-          <t>gate light</t>
+          <t>earth pit 1</t>
         </is>
       </c>
     </row>
@@ -15025,31 +14992,31 @@
         </is>
       </c>
       <c r="E113" s="4" t="n">
-        <v>68.2</v>
+        <v>73.5</v>
       </c>
       <c r="F113" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="G113" s="4" t="inlineStr">
         <is>
-          <t>earth pit 1</t>
+          <t>earth pit 2</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>EP</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>Earth pit</t>
+          <t>Outdoor / gate light</t>
         </is>
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>ground</t>
+          <t>7'-0"</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
@@ -15058,45 +15025,12 @@
         </is>
       </c>
       <c r="E114" s="4" t="n">
-        <v>73.5</v>
+        <v>2.5</v>
       </c>
       <c r="F114" s="4" t="n">
-        <v>1.5</v>
+        <v>8</v>
       </c>
       <c r="G114" s="4" t="inlineStr">
-        <is>
-          <t>earth pit 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="4" t="inlineStr">
-        <is>
-          <t>GL</t>
-        </is>
-      </c>
-      <c r="B115" s="4" t="inlineStr">
-        <is>
-          <t>Outdoor / gate light</t>
-        </is>
-      </c>
-      <c r="C115" s="4" t="inlineStr">
-        <is>
-          <t>7'-0"</t>
-        </is>
-      </c>
-      <c r="D115" s="4" t="inlineStr">
-        <is>
-          <t>Site</t>
-        </is>
-      </c>
-      <c r="E115" s="4" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="F115" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="G115" s="4" t="inlineStr">
         <is>
           <t>rear garden</t>
         </is>

</xml_diff>

<commit_message>
Open hall in three zones: TV lounge, dining, guest sitting by the door
5'-6" sofa facing the TV in the dining bay; dining table moved 9 in south
under the ventilator so chairs clear the sofa; 6 ft window diwan with
drawers and the armchair under the living's north window for guests, with
a light and floor socket; clear walk from the main door to the dining.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Schedules/KH-P1_Schedules_RevB.xlsx
+++ b/03_Schedules/KH-P1_Schedules_RevB.xlsx
@@ -4805,7 +4805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4950,7 +4950,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Twentieth review: Bedroom 2's bed moves to the east wall, head east, leaving an 8 x 14 ft open floor from the door to the bath and window; wardrobe to the west wall (sound buffer to the master), work table north of the bed, AC on the bath's outer wall; dresser dropped (mirror on the wardrobe).</t>
+          <t>Twenty-first review: the open hall becomes three zones: family TV lounge in the dining bay (5'-6" sofa facing the TV), dining under the ventilator moved 9 in south (about 2 ft behind the chairs on both sides), and guest sitting by the main door with a 6 ft window diwan and an armchair under the living's north window; a clear walk of about 4'-11" from the main door to the dining and kitchen, pooja front kept clear.</t>
         </is>
       </c>
     </row>
@@ -4960,7 +4960,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
+          <t>Twentieth review: Bedroom 2's bed moves to the east wall, head east, leaving an 8 x 14 ft open floor from the door to the bath and window; wardrobe to the west wall (sound buffer to the master), work table north of the bed, AC on the bath's outer wall; dresser dropped (mirror on the wardrobe).</t>
         </is>
       </c>
     </row>
@@ -4970,7 +4970,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
+          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
         </is>
       </c>
     </row>
@@ -4980,7 +4980,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
+          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
         </is>
       </c>
     </row>
@@ -4990,7 +4990,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
+          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
         </is>
       </c>
     </row>
@@ -5000,7 +5000,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
+          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
         </is>
       </c>
     </row>
@@ -5010,7 +5010,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
+          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
+          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
         </is>
       </c>
     </row>
@@ -5030,7 +5030,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
+          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
         </is>
       </c>
     </row>
@@ -5040,7 +5040,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
+          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
         </is>
       </c>
     </row>
@@ -5050,7 +5050,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
+          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
         </is>
       </c>
     </row>
@@ -5060,7 +5060,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
+          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
+          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
         </is>
       </c>
     </row>
@@ -5080,7 +5080,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
+          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
         </is>
       </c>
     </row>
@@ -5090,7 +5090,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
+          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
         </is>
       </c>
     </row>
@@ -5100,7 +5100,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
+          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
         </is>
       </c>
     </row>
@@ -5110,7 +5110,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
+          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
         </is>
       </c>
     </row>
@@ -5120,7 +5120,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
+          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
         </is>
       </c>
     </row>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
+          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
+          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
         </is>
       </c>
     </row>
@@ -5150,7 +5150,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
+          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
         </is>
       </c>
     </row>
@@ -5160,7 +5160,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
+          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
         </is>
       </c>
     </row>
@@ -5170,7 +5170,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
+          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
         </is>
       </c>
     </row>
@@ -5180,7 +5180,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
+          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
         </is>
       </c>
     </row>
@@ -5190,7 +5190,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
+          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
         </is>
       </c>
     </row>
@@ -5200,7 +5200,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
+          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
         </is>
       </c>
     </row>
@@ -5210,7 +5210,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
         </is>
       </c>
     </row>
@@ -5229,6 +5229,16 @@
         <v>41</v>
       </c>
       <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>Roof: Mangalore clay tiles on steel truss over insulated cement-fibre deck; all edge tiles mechanically fixed.</t>
         </is>
@@ -7347,7 +7357,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8428,7 +8438,7 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Dining table 5' x 3', 6-seat</t>
+          <t>Dining table 5' x 3', 6-seat (under the ventilator)</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -9073,7 +9083,7 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Three-seat sofa 6'6" facing west to the TV</t>
+          <t>Sofa 5'-6" (2-3 seats) facing west to the TV</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -9085,7 +9095,7 @@
         <v>2.7</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>5.9</v>
+        <v>5.5</v>
       </c>
       <c r="G40" s="4" t="n">
         <v>1</v>
@@ -9202,7 +9212,7 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Armchair by the north window</t>
+          <t>Armchair at the west end of the window diwan</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -9211,10 +9221,10 @@
         </is>
       </c>
       <c r="E43" s="4" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>1</v>
@@ -9235,7 +9245,7 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>F52</t>
+          <t>F58</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -9245,26 +9255,26 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Shoe cupboard 3'-3" beside the main door (closed shutters, louvred for air)</t>
+          <t>Window diwan 6' x 2'-6" under the north window, drawers below (guest seating, extra bed at festivals)</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E44" s="4" t="n">
-        <v>1.2</v>
+        <v>6</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>3.2</v>
+        <v>2.6</v>
       </c>
       <c r="G44" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate, 14 in deep</t>
+          <t>Teak frame, cotton mattress and bolsters</t>
         </is>
       </c>
       <c r="I44" s="10" t="n"/>
@@ -9278,36 +9288,36 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>F41</t>
+          <t>F52</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Poomukham (verandah)</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Oonjal (swing) 3'6"</t>
+          <t>Shoe cupboard 3'-3" beside the main door (closed shutters, louvred for air)</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E45" s="4" t="n">
-        <v>3.5</v>
+        <v>1.2</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>1.5</v>
+        <v>3.2</v>
       </c>
       <c r="G45" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>Teak, chains to beam</t>
+          <t>Ply + laminate, 14 in deep</t>
         </is>
       </c>
       <c r="I45" s="10" t="n"/>
@@ -9321,7 +9331,7 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>F42</t>
+          <t>F41</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -9331,26 +9341,26 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Arugu seat (built-in, south end)</t>
+          <t>Oonjal (swing) 3'6"</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E46" s="4" t="n">
-        <v>1.2</v>
+        <v>3.5</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>2.4</v>
+        <v>1.5</v>
       </c>
       <c r="G46" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>Laterite base, teak top</t>
+          <t>Teak, chains to beam</t>
         </is>
       </c>
       <c r="I46" s="10" t="n"/>
@@ -9362,28 +9372,71 @@
       <c r="L46" s="8" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="inlineStr"/>
-      <c r="B47" s="6" t="inlineStr"/>
-      <c r="C47" s="6" t="inlineStr">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>F42</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Poomukham (verandah)</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Arugu seat (built-in, south end)</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Built-in joinery</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>Laterite base, teak top</t>
+        </is>
+      </c>
+      <c r="I47" s="10" t="n"/>
+      <c r="J47" s="11">
+        <f>G47*I47</f>
+        <v/>
+      </c>
+      <c r="K47" s="8" t="inlineStr"/>
+      <c r="L47" s="8" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr"/>
+      <c r="B48" s="6" t="inlineStr"/>
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D47" s="6" t="inlineStr"/>
-      <c r="E47" s="6" t="inlineStr"/>
-      <c r="F47" s="6" t="inlineStr"/>
-      <c r="G47" s="6">
-        <f>SUM(G2:G46)</f>
+      <c r="D48" s="6" t="inlineStr"/>
+      <c r="E48" s="6" t="inlineStr"/>
+      <c r="F48" s="6" t="inlineStr"/>
+      <c r="G48" s="6">
+        <f>SUM(G2:G47)</f>
         <v/>
       </c>
-      <c r="H47" s="6" t="inlineStr"/>
-      <c r="I47" s="12" t="inlineStr"/>
-      <c r="J47" s="12">
-        <f>SUM(J2:J46)</f>
+      <c r="H48" s="6" t="inlineStr"/>
+      <c r="I48" s="12" t="inlineStr"/>
+      <c r="J48" s="12">
+        <f>SUM(J2:J47)</f>
         <v/>
       </c>
-      <c r="K47" s="6" t="inlineStr"/>
-      <c r="L47" s="6" t="inlineStr"/>
+      <c r="K48" s="6" t="inlineStr"/>
+      <c r="L48" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14488,12 +14541,16 @@
         </is>
       </c>
       <c r="E97" s="4" t="n">
-        <v>52</v>
+        <v>54.9</v>
       </c>
       <c r="F97" s="4" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="G97" s="4" t="inlineStr"/>
+        <v>22.8</v>
+      </c>
+      <c r="G97" s="4" t="inlineStr">
+        <is>
+          <t>over the diwan</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
@@ -14549,7 +14606,7 @@
         <v>48.2</v>
       </c>
       <c r="F99" s="4" t="n">
-        <v>18.4</v>
+        <v>18.8</v>
       </c>
       <c r="G99" s="4" t="inlineStr">
         <is>
@@ -14579,14 +14636,14 @@
         </is>
       </c>
       <c r="E100" s="4" t="n">
-        <v>52.6</v>
+        <v>51</v>
       </c>
       <c r="F100" s="4" t="n">
-        <v>17.8</v>
+        <v>20.3</v>
       </c>
       <c r="G100" s="4" t="inlineStr">
         <is>
-          <t>floor socket, armchair</t>
+          <t>floor socket, armchair and diwan (lamp, charger)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
3D model: walk-in mode, window light and detailed interiors
Windows are real openings (jali and glazed teak frames) with a time-of-day
sun slider; first-person walk-in from the gate with collision, floor levels
and a tap-to-jump plan map. Detailed finishes from the room schedule
(red oxide, vitrified, anti-skid, marble, granite floors; plaster walls and
skirting; bath tiling; false ceilings and a timber roof soffit), framed doors
open on their hinges, turned teak pillars, laterite plinth and compound wall,
gate, and furniture and fixtures built to plan size. Room lights glow at dusk.
Window diwan shortened to keep 3 ft clear inside the main door.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Schedules/KH-P1_Schedules_RevB.xlsx
+++ b/03_Schedules/KH-P1_Schedules_RevB.xlsx
@@ -4950,7 +4950,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Twenty-first review: the open hall becomes three zones: family TV lounge in the dining bay (5'-6" sofa facing the TV), dining under the ventilator moved 9 in south (about 2 ft behind the chairs on both sides), and guest sitting by the main door with a 6 ft window diwan and an armchair under the living's north window; a clear walk of about 4'-11" from the main door to the dining and kitchen, pooja front kept clear.</t>
+          <t>Twenty-first review: the open hall becomes three zones: family TV lounge in the dining bay (5'-6" sofa facing the TV), dining under the ventilator moved 9 in south (about 2 ft behind the chairs on both sides), and guest sitting by the main door with a 4'-6" window diwan (shortened after the walk-through showed a 1'-6" pinch at the shoe cupboard) and an armchair under the living's north window; a clear walk of about 4'-11" from the main door to the dining and kitchen, pooja front kept clear.</t>
         </is>
       </c>
     </row>
@@ -9255,16 +9255,16 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Window diwan 6' x 2'-6" under the north window, drawers below (guest seating, extra bed at festivals)</t>
+          <t>Window diwan 4'-6" x 2'-6" under the north window, drawers below (guest seating, day bed); stops 3 ft short of the shoe cupboard so the way in from the main door stays clear</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E44" s="4" t="n">
-        <v>6</v>
+        <v>4.5</v>
       </c>
       <c r="F44" s="4" t="n">
         <v>2.6</v>
@@ -14541,7 +14541,7 @@
         </is>
       </c>
       <c r="E97" s="4" t="n">
-        <v>54.9</v>
+        <v>54.2</v>
       </c>
       <c r="F97" s="4" t="n">
         <v>22.8</v>

</xml_diff>

<commit_message>
27 ft plot only; fridge out of the kitchen; look selector
Planned without the north strip: roof eaves cut to 2 ft so the north eave
stays inside the plot, sealed septic tank under the two-wheeler bay with a
lined soak pit in the front yard, drains rerouted along the south walkway,
rainwater to the sump with overflow to the road. Fridge moves to the dining
alcove beside the kitchen door; pantry and dining set removed. The 3D model
gets a Look selector with five colour and material schemes; the choice is
logged as an open decision.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Schedules/KH-P1_Schedules_RevB.xlsx
+++ b/03_Schedules/KH-P1_Schedules_RevB.xlsx
@@ -671,7 +671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1715,14 +1715,14 @@
         </is>
       </c>
       <c r="D38" s="4" t="n">
-        <v>4.2</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>IC-7 grey</t>
+          <t>IC-12 soil, to the septic tank</t>
         </is>
       </c>
     </row>
@@ -1743,14 +1743,14 @@
         </is>
       </c>
       <c r="D39" s="4" t="n">
-        <v>4.2</v>
+        <v>73.2</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>IC-8 grey</t>
+          <t>IC-13 grey, to the soak pit</t>
         </is>
       </c>
     </row>
@@ -1771,14 +1771,14 @@
         </is>
       </c>
       <c r="D40" s="4" t="n">
-        <v>9.6</v>
+        <v>4.2</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>IC-9 ensuite grey</t>
+          <t>IC-7 grey</t>
         </is>
       </c>
     </row>
@@ -1799,14 +1799,14 @@
         </is>
       </c>
       <c r="D41" s="4" t="n">
-        <v>22.5</v>
+        <v>4.2</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>26.6</v>
+        <v>26</v>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>IC-10 Bath 2 soil</t>
+          <t>IC-8 grey</t>
         </is>
       </c>
     </row>
@@ -1827,12 +1827,68 @@
         </is>
       </c>
       <c r="D42" s="4" t="n">
-        <v>26.4</v>
+        <v>9.6</v>
       </c>
       <c r="E42" s="4" t="n">
         <v>26</v>
       </c>
       <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>IC-9 ensuite grey</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>IC</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Inspection chamber</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>IC-10 Bath 2 soil</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>IC</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Inspection chamber</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
         <is>
           <t>IC-11 Bath 2 grey</t>
         </is>
@@ -1945,7 +2001,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Lay a 3 ft paved apron sloping away, run gutters to the sump, and keep soak pits and septic 6 ft+ away (here they are in the north strip).</t>
+          <t>Lay a 3 ft paved apron sloping away, run gutters to the sump, and keep soak pits and septic 6 ft+ away where the plot allows (here a sealed septic tank and lined soak pit sit in the front yard; a road-drain outflow is better if available).</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -2520,7 +2576,7 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Clear size is about 8'9" x 7'6". A 6-seat 5 x 3 ft table leaves about 2'3" each side, so use a 4-seat or round table, or let it spill into the hall.</t>
+          <t>No table is drawn for now. If one is added later, the open space under the ventilator takes a 6-seat 5 x 3 ft table with about 2 ft behind the chairs; a 4-seat or round table is easier.</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -2773,7 +2829,7 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Fridge on the kitchen's north wall behind the pooja, beside the tall pantry and well away from the hob; nothing blocks the counter.</t>
+          <t>Fridge just outside the kitchen in the dining alcove, beside the kitchen door: reachable from the dining without crossing the cooking area, and well away from the hob.</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -3785,7 +3841,7 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Gutters on both long eaves, downpipes into the sump filter and recharge pit.</t>
+          <t>Gutters on both long eaves, downpipes into the sump filter; overflow to the road drain (no recharge pit near the walls on this narrow plot).</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -4015,7 +4071,7 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>Keep soil and grey water separate: soil to the septic, grey to a soak trench, with inspection chambers at every bend.</t>
+          <t>Keep soil and grey water separate: soil to the septic, grey to the soak pit or a road drain, with inspection chambers at every bend.</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
@@ -4382,7 +4438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4425,17 +4481,17 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Land</t>
+          <t>Finishes</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Front yard is now 8 ft (house 62 ft long): confirm the front setback allowed for this plot and road width before finalising; fall back to a 60 ft house if 10 ft is required</t>
+          <t>Colour and material scheme to choose: five looks to compare in the 3D model (As drawn, Classic Kerala refined, Chettinad ochre, Modern tropical, Lime and green); decide before ordering floor tiles, paint and door finishes</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
@@ -4450,17 +4506,17 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Layout</t>
+          <t>Land</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>TV on Bedroom 2's east wall facing the dining bay: confirm screen size (55-65 in at about 9 ft) and a concealed HDMI/data conduit from the unit</t>
+          <t>Front yard is now 8 ft (house 62 ft long): confirm the front setback allowed for this plot and road width before finalising; fall back to a 60 ft house if 10 ft is required</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Architect</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
@@ -4475,17 +4531,17 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Land</t>
+          <t>Layout</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Agricultural land: confirm conversion to non-agricultural use with the gram panchayat / collector (AP repealed the NALA Act in 2025; new process to be confirmed)</t>
+          <t>TV on Bedroom 2's east wall facing the dining bay: confirm screen size (55-65 in at about 9 ft) and a concealed HDMI/data conduit from the unit</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Owner / surveyor</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
@@ -4505,12 +4561,12 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Building permission route (panchayat vs DTCP / APCRDA via APDPMS) and setbacks under AP Building Rules 2017</t>
+          <t>Agricultural land: confirm conversion to non-agricultural use with the gram panchayat / collector (AP repealed the NALA Act in 2025; new process to be confirmed)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Owner / surveyor</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -4530,7 +4586,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Plot 27 ft x 75 ft (length to confirm by survey): north wall is 2 ft from the plot line and eaves overhang the owned north strip; septic and soak trench sit in the strip</t>
+          <t>Building permission route (panchayat vs DTCP / APCRDA via APDPMS) and setbacks under AP Building Rules 2017</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -4550,17 +4606,17 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Soil</t>
+          <t>Land</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Soil test (bore holes to 3 m min): black cotton soil is common in Guntur. Foundation type (isolated footings below active zone, under-reamed piles, or soil replacement) depends on it</t>
+          <t>Plot 27 ft x 75 ft (length to confirm by survey), planned without the north strip: north wall 2 ft from the plot line, eaves cut to 2 ft so they stay inside the plot (gutters both sides); septic tank and soak pit in the front yard</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Structural engineer</t>
+          <t>Architect</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -4575,12 +4631,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>Soil</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>RCC frame with AAC infill: columns, plinth beam, lintel band, ring beam; steel truss with cyclone tie-downs</t>
+          <t>Soil test (bore holes to 3 m min): black cotton soil is common in Guntur. Foundation type (isolated footings below active zone, under-reamed piles, or soil replacement) depends on it</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -4600,17 +4656,17 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Structure</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Wet area is open to the walkway: lockable steel/WPC kitchen-to-wet-area door, compound wall and gate at the back; optional MS grille shutter across the wet area opening</t>
+          <t>RCC frame with AAC infill: columns, plinth beam, lintel band, ring beam; steel truss with cyclone tie-downs</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Owner / architect</t>
+          <t>Structural engineer</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -4625,17 +4681,17 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Services</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Groundwater: test TDS, hardness, fluoride. Plan RO for drinking and a softener for bathrooms if hardness is high</t>
+          <t>Wet area is open to the walkway: lockable steel/WPC kitchen-to-wet-area door, compound wall and gate at the back; optional MS grille shutter across the wet area opening</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Plumber / owner</t>
+          <t>Owner / architect</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -4655,12 +4711,12 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Septic tank size and soak trench length (percolation test); keep soak trenches and gardens 6 ft+ from foundations in expansive soil</t>
+          <t>Groundwater: test TDS, hardness, fluoride. Plan RO for drinking and a softener for bathrooms if hardness is high</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Plumber / owner</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -4680,12 +4736,12 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Electrical load (with ACs), service connection size, earthing, inverter / solar PV</t>
+          <t>Septic tank size and soak pit size (percolation test); keep soak pits and gardens as far from foundations as the plot allows in expansive soil</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Electrical engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -4700,22 +4756,22 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Services</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Phase 2 on the north strip will block north light and sits on the septic: plan the split now</t>
+          <t>Electrical load (with ACs), service connection size, earthing, inverter / solar PV</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Electrical engineer</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Deferred by owner</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -4725,22 +4781,22 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Vastu</t>
+          <t>Future land</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Bed head east (master), NW ensuite, Bedroom 2's attached bath in its north-west corner on the north wall (north-west of the plot centre), common bath south of the plot centre beside the wet area (outside the central zone), dining at the plot centre, pooja in the living's south-east corner back to back with the kitchen, opening west (devotees face east), shoe cupboard between the pooja and the main door (behind the pooja's solid north wall), DB on the dining face of Bedroom 2's east wall</t>
+          <t>If the 10 ft north strip is bought later: move the soak pit there (6 ft+ from the house), and plan any Phase 2 so the north windows keep their light</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Vastu consultant</t>
+          <t>Owner / architect</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>To confirm</t>
+          <t>Deferred by owner</t>
         </is>
       </c>
     </row>
@@ -4750,17 +4806,17 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Climate</t>
+          <t>Services</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Roof heat: insulation, ventilated attic, ventilator lantern louvres and shutters; ODU positions on shaded walls</t>
+          <t>Soak pit in the front yard is only about 5 ft from the house and 13 ft from the sump in black cotton soil: prefer a sealed septic tank with treated outflow to a road or panchayat drain, or a bio-digester tank; confirm with the engineer and the panchayat</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Engineer / panchayat</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -4775,20 +4831,70 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
+          <t>Vastu</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Bed head east (master), NW ensuite, Bedroom 2's attached bath in its north-west corner on the north wall (north-west of the plot centre), common bath south of the plot centre beside the wet area (outside the central zone), dining at the plot centre, pooja in the living's south-east corner back to back with the kitchen, opening west (devotees face east), shoe cupboard between the pooja and the main door (behind the pooja's solid north wall), DB on the dining face of Bedroom 2's east wall</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Vastu consultant</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Climate</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Roof heat: insulation, ventilated attic, ventilator lantern louvres and shutters; ODU positions on shaded walls</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
           <t>Levels</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Survey road and field levels; plinth at 2 ft above finished ground (raise if site floods)</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Surveyor / architect</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -4805,7 +4911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4950,7 +5056,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Twenty-first review: the open hall becomes three zones: family TV lounge in the dining bay (5'-6" sofa facing the TV), dining under the ventilator moved 9 in south (about 2 ft behind the chairs on both sides), and guest sitting by the main door with a 4'-6" window diwan (shortened after the walk-through showed a 1'-6" pinch at the shoe cupboard) and an armchair under the living's north window; a clear walk of about 4'-11" from the main door to the dining and kitchen, pooja front kept clear.</t>
+          <t>Twenty-fourth review: planned on the 27 ft plot alone (north strip dropped for now): roof eaves cut from 2'-6" to 2'-0" so the north eave stays inside the plot line, septic tank moved under the two-wheeler bay in the front yard with a lined soak pit beside it, all drains rerouted along the south walkway to the front, rainwater to the sump with overflow to the road; north-strip trees and recharge pit removed.</t>
         </is>
       </c>
     </row>
@@ -4960,7 +5066,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Twentieth review: Bedroom 2's bed moves to the east wall, head east, leaving an 8 x 14 ft open floor from the door to the bath and window; wardrobe to the west wall (sound buffer to the master), work table north of the bed, AC on the bath's outer wall; dresser dropped (mirror on the wardrobe).</t>
+          <t>Twenty-third review: the fridge moves out of the kitchen into the dining alcove beside the kitchen door, against the wet-area wall; the kitchen's north wall is now free.</t>
         </is>
       </c>
     </row>
@@ -4970,7 +5076,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
+          <t>Twenty-second review: the kitchen's tall pantry and the dining table and chairs are removed at the owner's request; the dining space under the ventilator stays open (the pendant light and points stay for a table later).</t>
         </is>
       </c>
     </row>
@@ -4980,7 +5086,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
+          <t>Twenty-first review: the open hall becomes three zones: family TV lounge in the dining bay (5'-6" sofa facing the TV), dining under the ventilator moved 9 in south (about 2 ft behind the chairs on both sides), and guest sitting by the main door with a 4'-6" window diwan (shortened after the walk-through showed a 1'-6" pinch at the shoe cupboard) and an armchair under the living's north window; a clear walk of about 4'-11" from the main door to the dining and kitchen, pooja front kept clear.</t>
         </is>
       </c>
     </row>
@@ -4990,7 +5096,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
+          <t>Twentieth review: Bedroom 2's bed moves to the east wall, head east, leaving an 8 x 14 ft open floor from the door to the bath and window; wardrobe to the west wall (sound buffer to the master), work table north of the bed, AC on the bath's outer wall; dresser dropped (mirror on the wardrobe).</t>
         </is>
       </c>
     </row>
@@ -5000,7 +5106,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
+          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
         </is>
       </c>
     </row>
@@ -5010,7 +5116,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
+          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5126,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
+          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
         </is>
       </c>
     </row>
@@ -5030,7 +5136,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
+          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
         </is>
       </c>
     </row>
@@ -5040,7 +5146,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
+          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
         </is>
       </c>
     </row>
@@ -5050,7 +5156,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
+          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
         </is>
       </c>
     </row>
@@ -5060,7 +5166,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
+          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5176,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
+          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
         </is>
       </c>
     </row>
@@ -5080,7 +5186,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
+          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
         </is>
       </c>
     </row>
@@ -5090,7 +5196,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
+          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
         </is>
       </c>
     </row>
@@ -5100,7 +5206,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
+          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
         </is>
       </c>
     </row>
@@ -5110,7 +5216,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
+          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
         </is>
       </c>
     </row>
@@ -5120,7 +5226,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
+          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
         </is>
       </c>
     </row>
@@ -5130,7 +5236,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
+          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5246,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
+          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
         </is>
       </c>
     </row>
@@ -5150,7 +5256,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
+          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
         </is>
       </c>
     </row>
@@ -5160,7 +5266,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
+          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
         </is>
       </c>
     </row>
@@ -5170,7 +5276,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
+          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
         </is>
       </c>
     </row>
@@ -5180,7 +5286,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
+          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
         </is>
       </c>
     </row>
@@ -5190,7 +5296,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
+          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
         </is>
       </c>
     </row>
@@ -5200,7 +5306,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
+          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
         </is>
       </c>
     </row>
@@ -5210,7 +5316,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
+          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5326,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
         </is>
       </c>
     </row>
@@ -5230,7 +5336,7 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
         </is>
       </c>
     </row>
@@ -5239,6 +5345,36 @@
         <v>42</v>
       </c>
       <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>Roof: Mangalore clay tiles on steel truss over insulated cement-fibre deck; all edge tiles mechanically fixed.</t>
         </is>
@@ -7357,7 +7493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8428,26 +8564,26 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>F24</t>
+          <t>F26</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Pooja</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Dining table 5' x 3', 6-seat (under the ventilator)</t>
+          <t>Pooja mandapam on the east wall (idols face west; family faces east)</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E25" s="4" t="n">
-        <v>5</v>
+        <v>0.6</v>
       </c>
       <c r="F25" s="4" t="n">
         <v>3</v>
@@ -8457,7 +8593,7 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Teak or rosewood</t>
+          <t>Carved teak</t>
         </is>
       </c>
       <c r="I25" s="10" t="n"/>
@@ -8471,17 +8607,17 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F28</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Sitting and serving area</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Dining chair</t>
+          <t>Built-in bench with storage drawers below</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -8490,17 +8626,17 @@
         </is>
       </c>
       <c r="E26" s="4" t="n">
-        <v>1.1</v>
+        <v>1.5</v>
       </c>
       <c r="F26" s="4" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="G26" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G26" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Teak + cane</t>
+          <t>Teak top, ply drawers, on legs</t>
         </is>
       </c>
       <c r="I26" s="10" t="n"/>
@@ -8514,36 +8650,36 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>F26</t>
+          <t>F29</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Pooja</t>
+          <t>Wet area</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Pooja mandapam on the east wall (idols face west; family faces east)</t>
+          <t>Utility sink counter (on the kitchen wall)</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Sanitary / plumbing</t>
         </is>
       </c>
       <c r="E27" s="4" t="n">
-        <v>0.6</v>
+        <v>1.7</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="G27" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Carved teak</t>
+          <t>Kadappa / granite, SS sinks</t>
         </is>
       </c>
       <c r="I27" s="10" t="n"/>
@@ -8557,36 +8693,36 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>F28</t>
+          <t>F30</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area</t>
+          <t>Wet area</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Built-in bench with storage drawers below</t>
+          <t>Washing machine bay 2' x 2' (covered back corner, 2 in clear of the bath wall)</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Appliance / joinery</t>
         </is>
       </c>
       <c r="E28" s="4" t="n">
-        <v>1.5</v>
+        <v>1.9</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>2.8</v>
+        <v>1.9</v>
       </c>
       <c r="G28" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Teak top, ply drawers, on legs</t>
+          <t>Splash-proof socket, floor drain</t>
         </is>
       </c>
       <c r="I28" s="10" t="n"/>
@@ -8600,7 +8736,7 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>F29</t>
+          <t>F31</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -8610,26 +8746,26 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Utility sink counter (on the kitchen wall)</t>
+          <t>Fold-away clothesline in the south walkway</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Sanitary / plumbing</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E29" s="4" t="n">
-        <v>1.7</v>
+        <v>4</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>Kadappa / granite, SS sinks</t>
+          <t>SS wire, wall brackets</t>
         </is>
       </c>
       <c r="I29" s="10" t="n"/>
@@ -8643,7 +8779,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>F30</t>
+          <t>F44</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -8653,26 +8789,26 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Washing machine bay 2' x 2' (covered back corner, 2 in clear of the bath wall)</t>
+          <t>Tall slim utility cupboard (brooms, mops, detergents)</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Appliance / joinery</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E30" s="4" t="n">
-        <v>1.9</v>
+        <v>1.2</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>1.9</v>
+        <v>1.2</v>
       </c>
       <c r="G30" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Splash-proof socket, floor drain</t>
+          <t>Ply + laminate on legs, louvred doors</t>
         </is>
       </c>
       <c r="I30" s="10" t="n"/>
@@ -8686,36 +8822,36 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>F31</t>
+          <t>F32</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Wet area</t>
+          <t>Sitting and serving area</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Fold-away clothesline in the south walkway</t>
+          <t>Hand-wash basin at the east end of the serving counter, just outside the common bath (after meals); mirror on the side wall</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Sanitary / plumbing</t>
         </is>
       </c>
       <c r="E31" s="4" t="n">
-        <v>4</v>
+        <v>1.9</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>SS wire, wall brackets</t>
+          <t>Ceramic basin in granite top</t>
         </is>
       </c>
       <c r="I31" s="10" t="n"/>
@@ -8729,17 +8865,17 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>F44</t>
+          <t>F33</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Wet area</t>
+          <t>Sitting and serving area</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Tall slim utility cupboard (brooms, mops, detergents)</t>
+          <t>Serving counter with crockery cabinets above, 6 ft</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -8748,17 +8884,17 @@
         </is>
       </c>
       <c r="E32" s="4" t="n">
-        <v>1.2</v>
+        <v>6</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="G32" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate on legs, louvred doors</t>
+          <t>Granite top, teak + glass shutters</t>
         </is>
       </c>
       <c r="I32" s="10" t="n"/>
@@ -8772,7 +8908,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>F32</t>
+          <t>F56</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -8782,16 +8918,16 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Hand-wash basin at the east end of the serving counter, just outside the common bath (after meals); mirror on the side wall</t>
+          <t>Tall storage cupboard 5' x 2' (bedding, suitcases, festival vessels), loft above</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Sanitary / plumbing</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
-        <v>1.9</v>
+        <v>5</v>
       </c>
       <c r="F33" s="4" t="n">
         <v>2</v>
@@ -8801,7 +8937,7 @@
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Ceramic basin in granite top</t>
+          <t>Ply + laminate, full height</t>
         </is>
       </c>
       <c r="I33" s="10" t="n"/>
@@ -8815,17 +8951,17 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>F33</t>
+          <t>F34</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Serving counter with crockery cabinets above, 6 ft</t>
+          <t>L-counter, south run</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -8834,7 +8970,7 @@
         </is>
       </c>
       <c r="E34" s="4" t="n">
-        <v>6</v>
+        <v>13.2</v>
       </c>
       <c r="F34" s="4" t="n">
         <v>2</v>
@@ -8844,7 +8980,7 @@
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>Granite top, teak + glass shutters</t>
+          <t>Granite top, ply carcass</t>
         </is>
       </c>
       <c r="I34" s="10" t="n"/>
@@ -8858,17 +8994,17 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>F56</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Tall storage cupboard 5' x 2' (bedding, suitcases, festival vessels), loft above</t>
+          <t>L-counter, east run (hob centred 7'-6" from the south wall face, on solid wall)</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -8877,17 +9013,17 @@
         </is>
       </c>
       <c r="E35" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate, full height</t>
+          <t>Granite top, cook faces east</t>
         </is>
       </c>
       <c r="I35" s="10" t="n"/>
@@ -8901,36 +9037,36 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>F34</t>
+          <t>F36</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>L-counter, south run</t>
+          <t>Refrigerator space (dining alcove beside the kitchen door, against the wet-area wall, door facing north)</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Appliance / joinery</t>
         </is>
       </c>
       <c r="E36" s="4" t="n">
-        <v>13.2</v>
+        <v>2.5</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="G36" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>Granite top, ply carcass</t>
+          <t>Double-door, 2'6" wide</t>
         </is>
       </c>
       <c r="I36" s="10" t="n"/>
@@ -8944,36 +9080,36 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F38</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Dining bay</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>L-counter, east run (hob centred 7'-6" from the south wall face, on solid wall)</t>
+          <t>Sofa 5'-6" (2-3 seats) facing west to the TV</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E37" s="4" t="n">
-        <v>2</v>
+        <v>2.7</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>Granite top, cook faces east</t>
+          <t>Teak frame, cotton cushions</t>
         </is>
       </c>
       <c r="I37" s="10" t="n"/>
@@ -8987,36 +9123,36 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>F36</t>
+          <t>F39</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Dining bay</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Refrigerator space (kitchen north wall, behind the pooja, door facing south)</t>
+          <t>Coffee table 3'6" x 2'</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Appliance / joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E38" s="4" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="G38" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Double-door, 2'6" wide</t>
+          <t>Teak</t>
         </is>
       </c>
       <c r="I38" s="10" t="n"/>
@@ -9030,36 +9166,36 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>F55</t>
+          <t>F53</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Dining bay</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Tall pantry 4'-5" x 2' on the north wall (provisions, rice, vessels)</t>
+          <t>TV unit 4'-5" on Bedroom 2's east wall (55-65 in TV wall-mounted above)</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Appliance / joinery</t>
         </is>
       </c>
       <c r="E39" s="4" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F39" s="4" t="n">
         <v>4.4</v>
-      </c>
-      <c r="F39" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate, full height with loft</t>
+          <t>Teak, low, open shelves</t>
         </is>
       </c>
       <c r="I39" s="10" t="n"/>
@@ -9073,17 +9209,17 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>F38</t>
+          <t>F40</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Dining bay</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Sofa 5'-6" (2-3 seats) facing west to the TV</t>
+          <t>Armchair at the west end of the window diwan</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -9092,17 +9228,17 @@
         </is>
       </c>
       <c r="E40" s="4" t="n">
-        <v>2.7</v>
+        <v>1.8</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>5.5</v>
+        <v>1.8</v>
       </c>
       <c r="G40" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>Teak frame, cotton cushions</t>
+          <t>Cane / teak</t>
         </is>
       </c>
       <c r="I40" s="10" t="n"/>
@@ -9116,36 +9252,36 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>F39</t>
+          <t>F58</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Dining bay</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Coffee table 3'6" x 2'</t>
+          <t>Window diwan 4'-6" x 2'-6" under the north window, drawers below (guest seating, day bed); stops 3 ft short of the shoe cupboard so the way in from the main door stays clear</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E41" s="4" t="n">
-        <v>2</v>
+        <v>4.5</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>3.5</v>
+        <v>2.6</v>
       </c>
       <c r="G41" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>Teak</t>
+          <t>Teak frame, cotton mattress and bolsters</t>
         </is>
       </c>
       <c r="I41" s="10" t="n"/>
@@ -9159,36 +9295,36 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>F53</t>
+          <t>F52</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Dining bay</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>TV unit 4'-5" on Bedroom 2's east wall (55-65 in TV wall-mounted above)</t>
+          <t>Shoe cupboard 3'-3" beside the main door (closed shutters, louvred for air)</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Appliance / joinery</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E42" s="4" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>4.4</v>
+        <v>3.2</v>
       </c>
       <c r="G42" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>Teak, low, open shelves</t>
+          <t>Ply + laminate, 14 in deep</t>
         </is>
       </c>
       <c r="I42" s="10" t="n"/>
@@ -9202,17 +9338,17 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>F40</t>
+          <t>F41</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Poomukham (verandah)</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Armchair at the west end of the window diwan</t>
+          <t>Oonjal (swing) 3'6"</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -9221,17 +9357,17 @@
         </is>
       </c>
       <c r="E43" s="4" t="n">
-        <v>1.8</v>
+        <v>3.5</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>Cane / teak</t>
+          <t>Teak, chains to beam</t>
         </is>
       </c>
       <c r="I43" s="10" t="n"/>
@@ -9245,17 +9381,17 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>F58</t>
+          <t>F42</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Poomukham (verandah)</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Window diwan 4'-6" x 2'-6" under the north window, drawers below (guest seating, day bed); stops 3 ft short of the shoe cupboard so the way in from the main door stays clear</t>
+          <t>Arugu seat (built-in, south end)</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
@@ -9264,17 +9400,17 @@
         </is>
       </c>
       <c r="E44" s="4" t="n">
-        <v>4.5</v>
+        <v>1.2</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="G44" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>Teak frame, cotton mattress and bolsters</t>
+          <t>Laterite base, teak top</t>
         </is>
       </c>
       <c r="I44" s="10" t="n"/>
@@ -9286,157 +9422,28 @@
       <c r="L44" s="8" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>F52</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>Living</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>Shoe cupboard 3'-3" beside the main door (closed shutters, louvred for air)</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>Built-in joinery</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="F45" s="4" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="G45" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H45" s="4" t="inlineStr">
-        <is>
-          <t>Ply + laminate, 14 in deep</t>
-        </is>
-      </c>
-      <c r="I45" s="10" t="n"/>
-      <c r="J45" s="11">
-        <f>G45*I45</f>
+      <c r="A45" s="6" t="inlineStr"/>
+      <c r="B45" s="6" t="inlineStr"/>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr"/>
+      <c r="E45" s="6" t="inlineStr"/>
+      <c r="F45" s="6" t="inlineStr"/>
+      <c r="G45" s="6">
+        <f>SUM(G2:G44)</f>
         <v/>
       </c>
-      <c r="K45" s="8" t="inlineStr"/>
-      <c r="L45" s="8" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>F41</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>Poomukham (verandah)</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>Oonjal (swing) 3'6"</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>Loose furniture</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="F46" s="4" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G46" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H46" s="4" t="inlineStr">
-        <is>
-          <t>Teak, chains to beam</t>
-        </is>
-      </c>
-      <c r="I46" s="10" t="n"/>
-      <c r="J46" s="11">
-        <f>G46*I46</f>
+      <c r="H45" s="6" t="inlineStr"/>
+      <c r="I45" s="12" t="inlineStr"/>
+      <c r="J45" s="12">
+        <f>SUM(J2:J44)</f>
         <v/>
       </c>
-      <c r="K46" s="8" t="inlineStr"/>
-      <c r="L46" s="8" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>F42</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>Poomukham (verandah)</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>Arugu seat (built-in, south end)</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>Built-in joinery</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="F47" s="4" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="G47" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H47" s="4" t="inlineStr">
-        <is>
-          <t>Laterite base, teak top</t>
-        </is>
-      </c>
-      <c r="I47" s="10" t="n"/>
-      <c r="J47" s="11">
-        <f>G47*I47</f>
-        <v/>
-      </c>
-      <c r="K47" s="8" t="inlineStr"/>
-      <c r="L47" s="8" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="6" t="inlineStr"/>
-      <c r="B48" s="6" t="inlineStr"/>
-      <c r="C48" s="6" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="D48" s="6" t="inlineStr"/>
-      <c r="E48" s="6" t="inlineStr"/>
-      <c r="F48" s="6" t="inlineStr"/>
-      <c r="G48" s="6">
-        <f>SUM(G2:G47)</f>
-        <v/>
-      </c>
-      <c r="H48" s="6" t="inlineStr"/>
-      <c r="I48" s="12" t="inlineStr"/>
-      <c r="J48" s="12">
-        <f>SUM(J2:J47)</f>
-        <v/>
-      </c>
-      <c r="K48" s="6" t="inlineStr"/>
-      <c r="L48" s="6" t="inlineStr"/>
+      <c r="K45" s="6" t="inlineStr"/>
+      <c r="L45" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10176,7 +10183,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>150 mm half-round gutters with leaf guard, 100 mm downpipes at 8 points, to sump filter and recharge pit</t>
+          <t>150 mm half-round gutters with leaf guard, 100 mm downpipes at 8 points, to the sump filter, overflow to the road drain</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -11203,7 +11210,7 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>194.1</v>
+        <v>184.1</v>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
@@ -11233,7 +11240,7 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>40.8</v>
+        <v>40.2</v>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
@@ -11293,7 +11300,7 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>35.5</v>
+        <v>34.6</v>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
@@ -14237,17 +14244,17 @@
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>16 A power socket</t>
+          <t>6 A socket at counter</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -14256,16 +14263,12 @@
         </is>
       </c>
       <c r="E88" s="4" t="n">
-        <v>58.75</v>
+        <v>54.5</v>
       </c>
       <c r="F88" s="4" t="n">
-        <v>12.7</v>
-      </c>
-      <c r="G88" s="4" t="inlineStr">
-        <is>
-          <t>refrigerator, behind the fridge</t>
-        </is>
-      </c>
+        <v>3.5</v>
+      </c>
+      <c r="G88" s="4" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -14289,12 +14292,16 @@
         </is>
       </c>
       <c r="E89" s="4" t="n">
-        <v>54.5</v>
+        <v>58</v>
       </c>
       <c r="F89" s="4" t="n">
         <v>3.5</v>
       </c>
-      <c r="G89" s="4" t="inlineStr"/>
+      <c r="G89" s="4" t="inlineStr">
+        <is>
+          <t>microwave / OTG</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
@@ -14318,14 +14325,14 @@
         </is>
       </c>
       <c r="E90" s="4" t="n">
-        <v>58</v>
+        <v>63.5</v>
       </c>
       <c r="F90" s="4" t="n">
         <v>3.5</v>
       </c>
       <c r="G90" s="4" t="inlineStr">
         <is>
-          <t>microwave / OTG</t>
+          <t>mixer</t>
         </is>
       </c>
     </row>
@@ -14351,16 +14358,12 @@
         </is>
       </c>
       <c r="E91" s="4" t="n">
-        <v>63.5</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="F91" s="4" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="G91" s="4" t="inlineStr">
-        <is>
-          <t>mixer</t>
-        </is>
-      </c>
+        <v>5.6</v>
+      </c>
+      <c r="G91" s="4" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
@@ -14387,7 +14390,7 @@
         <v>66.59999999999999</v>
       </c>
       <c r="F92" s="4" t="n">
-        <v>5.6</v>
+        <v>9.6</v>
       </c>
       <c r="G92" s="4" t="inlineStr"/>
     </row>
@@ -14413,27 +14416,31 @@
         </is>
       </c>
       <c r="E93" s="4" t="n">
-        <v>66.59999999999999</v>
+        <v>59.3</v>
       </c>
       <c r="F93" s="4" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="G93" s="4" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="G93" s="4" t="inlineStr">
+        <is>
+          <t>RO purifier, by sink</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>6 A socket at counter</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
@@ -14442,59 +14449,59 @@
         </is>
       </c>
       <c r="E94" s="4" t="n">
-        <v>59.3</v>
+        <v>53.4</v>
       </c>
       <c r="F94" s="4" t="n">
-        <v>3.5</v>
+        <v>9</v>
       </c>
       <c r="G94" s="4" t="inlineStr">
         <is>
-          <t>RO purifier, by sink</t>
+          <t>beside the entry, latch side</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>Ceiling fan point</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="E95" s="4" t="n">
-        <v>53.4</v>
+        <v>55</v>
       </c>
       <c r="F95" s="4" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="G95" s="4" t="inlineStr">
         <is>
-          <t>beside the entry, latch side</t>
+          <t>long downrod</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Ceiling fan point</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
@@ -14508,14 +14515,14 @@
         </is>
       </c>
       <c r="E96" s="4" t="n">
-        <v>55</v>
+        <v>54.2</v>
       </c>
       <c r="F96" s="4" t="n">
-        <v>19</v>
+        <v>22.8</v>
       </c>
       <c r="G96" s="4" t="inlineStr">
         <is>
-          <t>long downrod</t>
+          <t>over the diwan</t>
         </is>
       </c>
     </row>
@@ -14541,45 +14548,45 @@
         </is>
       </c>
       <c r="E97" s="4" t="n">
-        <v>54.2</v>
+        <v>55</v>
       </c>
       <c r="F97" s="4" t="n">
-        <v>22.8</v>
-      </c>
-      <c r="G97" s="4" t="inlineStr">
-        <is>
-          <t>over the diwan</t>
-        </is>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="G97" s="4" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Dining bay (north window)</t>
         </is>
       </c>
       <c r="E98" s="4" t="n">
-        <v>55</v>
+        <v>48.2</v>
       </c>
       <c r="F98" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="G98" s="4" t="inlineStr"/>
+        <v>18.8</v>
+      </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t>floor socket, sofa end</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
@@ -14599,35 +14606,35 @@
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>Dining bay (north window)</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="E99" s="4" t="n">
-        <v>48.2</v>
+        <v>51</v>
       </c>
       <c r="F99" s="4" t="n">
-        <v>18.8</v>
+        <v>20.3</v>
       </c>
       <c r="G99" s="4" t="inlineStr">
         <is>
-          <t>floor socket, sofa end</t>
+          <t>floor socket, armchair and diwan (lamp, charger)</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
@@ -14636,64 +14643,64 @@
         </is>
       </c>
       <c r="E100" s="4" t="n">
-        <v>51</v>
+        <v>60.6</v>
       </c>
       <c r="F100" s="4" t="n">
-        <v>20.3</v>
+        <v>21</v>
       </c>
       <c r="G100" s="4" t="inlineStr">
         <is>
-          <t>floor socket, armchair and diwan (lamp, charger)</t>
+          <t>main switch at door</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>Distribution board</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>5'-0" to top</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E101" s="4" t="n">
-        <v>60.6</v>
+        <v>38.4</v>
       </c>
       <c r="F101" s="4" t="n">
-        <v>21</v>
+        <v>12.6</v>
       </c>
       <c r="G101" s="4" t="inlineStr">
         <is>
-          <t>main switch at door</t>
+          <t>dining face of Bedroom 2's east wall, by the passage; dry wall away from the pooja and wet area</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Distribution board</t>
+          <t>16 A power socket</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>5'-0" to top</t>
+          <t>varies</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
@@ -14702,14 +14709,14 @@
         </is>
       </c>
       <c r="E102" s="4" t="n">
-        <v>38.4</v>
+        <v>49.55</v>
       </c>
       <c r="F102" s="4" t="n">
-        <v>12.6</v>
+        <v>9.4</v>
       </c>
       <c r="G102" s="4" t="inlineStr">
         <is>
-          <t>dining face of Bedroom 2's east wall, by the passage; dry wall away from the pooja and wet area</t>
+          <t>refrigerator, behind the fridge (dining alcove)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Main door moved south, centred under the front gable
Door opens straight onto the walk between the pooja and the diwan; shoe
cupboard on the east wall north of the door; 6 ft window diwan out of the
door's line; entrance steps, middle verandah pillars, swing, bell and
switch realigned.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Schedules/KH-P1_Schedules_RevB.xlsx
+++ b/03_Schedules/KH-P1_Schedules_RevB.xlsx
@@ -4836,7 +4836,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Bed head east (master), NW ensuite, Bedroom 2's attached bath in its north-west corner on the north wall (north-west of the plot centre), common bath south of the plot centre beside the wet area (outside the central zone), dining at the plot centre, pooja in the living's south-east corner back to back with the kitchen, opening west (devotees face east), shoe cupboard between the pooja and the main door (behind the pooja's solid north wall), DB on the dining face of Bedroom 2's east wall</t>
+          <t>Bed head east (master), NW ensuite, Bedroom 2's attached bath in its north-west corner on the north wall (north-west of the plot centre), common bath south of the plot centre beside the wet area (outside the central zone), dining at the plot centre, pooja in the living's south-east corner back to back with the kitchen, opening west (devotees face east), shoe cupboard on the east wall north of the main door, DB on the dining face of Bedroom 2's east wall</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -4911,7 +4911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B46"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5056,7 +5056,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Twenty-fourth review: planned on the 27 ft plot alone (north strip dropped for now): roof eaves cut from 2'-6" to 2'-0" so the north eave stays inside the plot line, septic tank moved under the two-wheeler bay in the front yard with a lined soak pit beside it, all drains rerouted along the south walkway to the front, rainwater to the sump with overflow to the road; north-strip trees and recharge pit removed.</t>
+          <t>Twenty-fifth review: main door moved 3'-4" south (y 17'-7" to 20'-7"), centred under the front gable and opening straight onto the 5 ft walk between the pooja and the diwan; shoe cupboard to its north on the east wall; window diwan back to 6 ft along the north window, out of the door's line; steps, middle verandah pillars and the swing realigned.</t>
         </is>
       </c>
     </row>
@@ -5066,7 +5066,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Twenty-third review: the fridge moves out of the kitchen into the dining alcove beside the kitchen door, against the wet-area wall; the kitchen's north wall is now free.</t>
+          <t>Twenty-fourth review: planned on the 27 ft plot alone (north strip dropped for now): roof eaves cut from 2'-6" to 2'-0" so the north eave stays inside the plot line, septic tank moved under the two-wheeler bay in the front yard with a lined soak pit beside it, all drains rerouted along the south walkway to the front, rainwater to the sump with overflow to the road; north-strip trees and recharge pit removed.</t>
         </is>
       </c>
     </row>
@@ -5076,7 +5076,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Twenty-second review: the kitchen's tall pantry and the dining table and chairs are removed at the owner's request; the dining space under the ventilator stays open (the pendant light and points stay for a table later).</t>
+          <t>Twenty-third review: the fridge moves out of the kitchen into the dining alcove beside the kitchen door, against the wet-area wall; the kitchen's north wall is now free.</t>
         </is>
       </c>
     </row>
@@ -5086,7 +5086,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Twenty-first review: the open hall becomes three zones: family TV lounge in the dining bay (5'-6" sofa facing the TV), dining under the ventilator moved 9 in south (about 2 ft behind the chairs on both sides), and guest sitting by the main door with a 4'-6" window diwan (shortened after the walk-through showed a 1'-6" pinch at the shoe cupboard) and an armchair under the living's north window; a clear walk of about 4'-11" from the main door to the dining and kitchen, pooja front kept clear.</t>
+          <t>Twenty-second review: the kitchen's tall pantry and the dining table and chairs are removed at the owner's request; the dining space under the ventilator stays open (the pendant light and points stay for a table later).</t>
         </is>
       </c>
     </row>
@@ -5096,7 +5096,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Twentieth review: Bedroom 2's bed moves to the east wall, head east, leaving an 8 x 14 ft open floor from the door to the bath and window; wardrobe to the west wall (sound buffer to the master), work table north of the bed, AC on the bath's outer wall; dresser dropped (mirror on the wardrobe).</t>
+          <t>Twenty-first review: the open hall becomes three zones: family TV lounge in the dining bay (5'-6" sofa facing the TV), dining under the ventilator moved 9 in south (about 2 ft behind the chairs on both sides), and guest sitting by the main door with a 4'-6" window diwan (shortened after the walk-through showed a 1'-6" pinch at the shoe cupboard) and an armchair under the living's north window; a clear walk of about 4'-11" from the main door to the dining and kitchen, pooja front kept clear.</t>
         </is>
       </c>
     </row>
@@ -5106,7 +5106,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
+          <t>Twentieth review: Bedroom 2's bed moves to the east wall, head east, leaving an 8 x 14 ft open floor from the door to the bath and window; wardrobe to the west wall (sound buffer to the master), work table north of the bed, AC on the bath's outer wall; dresser dropped (mirror on the wardrobe).</t>
         </is>
       </c>
     </row>
@@ -5116,7 +5116,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
+          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
+          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
         </is>
       </c>
     </row>
@@ -5136,7 +5136,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
+          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
         </is>
       </c>
     </row>
@@ -5146,7 +5146,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
+          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
         </is>
       </c>
     </row>
@@ -5156,7 +5156,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
+          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
         </is>
       </c>
     </row>
@@ -5166,7 +5166,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
+          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
+          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
         </is>
       </c>
     </row>
@@ -5186,7 +5186,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
+          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
+          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
         </is>
       </c>
     </row>
@@ -5206,7 +5206,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
+          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
         </is>
       </c>
     </row>
@@ -5216,7 +5216,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
+          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
         </is>
       </c>
     </row>
@@ -5226,7 +5226,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
+          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
         </is>
       </c>
     </row>
@@ -5236,7 +5236,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
+          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
         </is>
       </c>
     </row>
@@ -5246,7 +5246,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
+          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
         </is>
       </c>
     </row>
@@ -5256,7 +5256,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
+          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5266,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
+          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
         </is>
       </c>
     </row>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
+          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
         </is>
       </c>
     </row>
@@ -5286,7 +5286,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
+          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
         </is>
       </c>
     </row>
@@ -5296,7 +5296,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
+          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
         </is>
       </c>
     </row>
@@ -5306,7 +5306,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
+          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
         </is>
       </c>
     </row>
@@ -5316,7 +5316,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
+          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
         </is>
       </c>
     </row>
@@ -5326,7 +5326,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
+          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
         </is>
       </c>
     </row>
@@ -5336,7 +5336,7 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
+          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
         </is>
       </c>
     </row>
@@ -5346,7 +5346,7 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
+          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
         </is>
       </c>
     </row>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
         </is>
       </c>
     </row>
@@ -5375,6 +5375,16 @@
         <v>45</v>
       </c>
       <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>Roof: Mangalore clay tiles on steel truss over insulated cement-fibre deck; all edge tiles mechanically fixed.</t>
         </is>
@@ -6441,7 +6451,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Main entrance</t>
+          <t>Main entrance (centred under the front gable)</t>
         </is>
       </c>
       <c r="C2" s="4" t="n">
@@ -9262,16 +9272,16 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Window diwan 4'-6" x 2'-6" under the north window, drawers below (guest seating, day bed); stops 3 ft short of the shoe cupboard so the way in from the main door stays clear</t>
+          <t>Window diwan 6' x 2'-6" under the north window, drawers below (guest seating, day bed); out of the line of the main door</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E41" s="4" t="n">
-        <v>4.5</v>
+        <v>6</v>
       </c>
       <c r="F41" s="4" t="n">
         <v>2.6</v>
@@ -9305,7 +9315,7 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Shoe cupboard 3'-3" beside the main door (closed shutters, louvred for air)</t>
+          <t>Shoe cupboard 3'-3" on the east wall just north of the main door (closed shutters, louvred for air)</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -9348,7 +9358,7 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Oonjal (swing) 3'6"</t>
+          <t>Oonjal (swing) 3'6", north side of the verandah, clear of the entrance</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -14515,7 +14525,7 @@
         </is>
       </c>
       <c r="E96" s="4" t="n">
-        <v>54.2</v>
+        <v>54.9</v>
       </c>
       <c r="F96" s="4" t="n">
         <v>22.8</v>
@@ -14836,7 +14846,7 @@
         <v>61.4</v>
       </c>
       <c r="F106" s="4" t="n">
-        <v>20.4</v>
+        <v>21</v>
       </c>
       <c r="G106" s="4" t="inlineStr"/>
     </row>
@@ -14931,7 +14941,7 @@
         <v>61.4</v>
       </c>
       <c r="F109" s="4" t="n">
-        <v>20.9</v>
+        <v>21.5</v>
       </c>
       <c r="G109" s="4" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Built-in ideas borrowed and adapted: niches, shoe bench, lamp niche, racks
Recessed tiled shower niches in all three baths, mirror cabinets over the
basins, genkan-style shoe bench with hooks and a granite threshold band,
carved teak vilakku madam facing the main door, floating bedside shelves,
drawers-first kitchen with a masala pull-out and utensil rail, dish-drying
rack over the utility sink and a ceiling clothes airer in the wet area.
Furniture key on A-103 shortened to item names.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Schedules/KH-P1_Schedules_RevB.xlsx
+++ b/03_Schedules/KH-P1_Schedules_RevB.xlsx
@@ -4911,7 +4911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:B48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5056,7 +5056,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Twenty-fifth review: main door moved 3'-4" south (y 17'-7" to 20'-7"), centred under the front gable and opening straight onto the 5 ft walk between the pooja and the diwan; shoe cupboard to its north on the east wall; window diwan back to 6 ft along the north window, out of the door's line; steps, middle verandah pillars and the swing realigned.</t>
+          <t>Twenty-sixth review: built-in ideas borrowed and adapted (function, not style, in Kerala materials): recessed shower niches, mirror cabinets over basins, genkan-style shoe bench with hooks and a granite threshold band, vilakku madam lamp niche facing the main door, floating bedside shelves (walls too thin for recesses), drawers-first kitchen with a masala pull-out and utensil rail, dish-drying rack over the utility sink, ceiling clothes airer in the wet area.</t>
         </is>
       </c>
     </row>
@@ -5066,7 +5066,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Twenty-fourth review: planned on the 27 ft plot alone (north strip dropped for now): roof eaves cut from 2'-6" to 2'-0" so the north eave stays inside the plot line, septic tank moved under the two-wheeler bay in the front yard with a lined soak pit beside it, all drains rerouted along the south walkway to the front, rainwater to the sump with overflow to the road; north-strip trees and recharge pit removed.</t>
+          <t>Twenty-fifth review: main door moved 3'-4" south (y 17'-7" to 20'-7"), centred under the front gable and opening straight onto the 5 ft walk between the pooja and the diwan; shoe cupboard to its north on the east wall; window diwan back to 6 ft along the north window, out of the door's line; steps, middle verandah pillars and the swing realigned.</t>
         </is>
       </c>
     </row>
@@ -5076,7 +5076,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Twenty-third review: the fridge moves out of the kitchen into the dining alcove beside the kitchen door, against the wet-area wall; the kitchen's north wall is now free.</t>
+          <t>Twenty-fourth review: planned on the 27 ft plot alone (north strip dropped for now): roof eaves cut from 2'-6" to 2'-0" so the north eave stays inside the plot line, septic tank moved under the two-wheeler bay in the front yard with a lined soak pit beside it, all drains rerouted along the south walkway to the front, rainwater to the sump with overflow to the road; north-strip trees and recharge pit removed.</t>
         </is>
       </c>
     </row>
@@ -5086,7 +5086,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Twenty-second review: the kitchen's tall pantry and the dining table and chairs are removed at the owner's request; the dining space under the ventilator stays open (the pendant light and points stay for a table later).</t>
+          <t>Twenty-third review: the fridge moves out of the kitchen into the dining alcove beside the kitchen door, against the wet-area wall; the kitchen's north wall is now free.</t>
         </is>
       </c>
     </row>
@@ -5096,7 +5096,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Twenty-first review: the open hall becomes three zones: family TV lounge in the dining bay (5'-6" sofa facing the TV), dining under the ventilator moved 9 in south (about 2 ft behind the chairs on both sides), and guest sitting by the main door with a 4'-6" window diwan (shortened after the walk-through showed a 1'-6" pinch at the shoe cupboard) and an armchair under the living's north window; a clear walk of about 4'-11" from the main door to the dining and kitchen, pooja front kept clear.</t>
+          <t>Twenty-second review: the kitchen's tall pantry and the dining table and chairs are removed at the owner's request; the dining space under the ventilator stays open (the pendant light and points stay for a table later).</t>
         </is>
       </c>
     </row>
@@ -5106,7 +5106,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Twentieth review: Bedroom 2's bed moves to the east wall, head east, leaving an 8 x 14 ft open floor from the door to the bath and window; wardrobe to the west wall (sound buffer to the master), work table north of the bed, AC on the bath's outer wall; dresser dropped (mirror on the wardrobe).</t>
+          <t>Twenty-first review: the open hall becomes three zones: family TV lounge in the dining bay (5'-6" sofa facing the TV), dining under the ventilator moved 9 in south (about 2 ft behind the chairs on both sides), and guest sitting by the main door with a 4'-6" window diwan (shortened after the walk-through showed a 1'-6" pinch at the shoe cupboard) and an armchair under the living's north window; a clear walk of about 4'-11" from the main door to the dining and kitchen, pooja front kept clear.</t>
         </is>
       </c>
     </row>
@@ -5116,7 +5116,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
+          <t>Twentieth review: Bedroom 2's bed moves to the east wall, head east, leaving an 8 x 14 ft open floor from the door to the bath and window; wardrobe to the west wall (sound buffer to the master), work table north of the bed, AC on the bath's outer wall; dresser dropped (mirror on the wardrobe).</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
+          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
         </is>
       </c>
     </row>
@@ -5136,7 +5136,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
+          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
         </is>
       </c>
     </row>
@@ -5146,7 +5146,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
+          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
         </is>
       </c>
     </row>
@@ -5156,7 +5156,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
+          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
         </is>
       </c>
     </row>
@@ -5166,7 +5166,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
+          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
+          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
         </is>
       </c>
     </row>
@@ -5186,7 +5186,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
+          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
+          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
         </is>
       </c>
     </row>
@@ -5206,7 +5206,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
+          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
         </is>
       </c>
     </row>
@@ -5216,7 +5216,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
+          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
         </is>
       </c>
     </row>
@@ -5226,7 +5226,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
+          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
         </is>
       </c>
     </row>
@@ -5236,7 +5236,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
+          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
         </is>
       </c>
     </row>
@@ -5246,7 +5246,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
+          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
         </is>
       </c>
     </row>
@@ -5256,7 +5256,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
+          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5266,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
+          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
         </is>
       </c>
     </row>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
+          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
         </is>
       </c>
     </row>
@@ -5286,7 +5286,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
+          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
         </is>
       </c>
     </row>
@@ -5296,7 +5296,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
+          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
         </is>
       </c>
     </row>
@@ -5306,7 +5306,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
+          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
         </is>
       </c>
     </row>
@@ -5316,7 +5316,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
+          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
         </is>
       </c>
     </row>
@@ -5326,7 +5326,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
+          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
         </is>
       </c>
     </row>
@@ -5336,7 +5336,7 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
+          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
         </is>
       </c>
     </row>
@@ -5346,7 +5346,7 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
+          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
+          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
         </is>
       </c>
     </row>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
         </is>
       </c>
     </row>
@@ -5376,7 +5376,7 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
         </is>
       </c>
     </row>
@@ -5385,6 +5385,16 @@
         <v>46</v>
       </c>
       <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>Roof: Mangalore clay tiles on steel truss over insulated cement-fibre deck; all edge tiles mechanically fixed.</t>
         </is>
@@ -7503,7 +7513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -7853,7 +7863,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Vanity basin counter 3'-6"</t>
+          <t>Vanity basin counter 3'-6" with a mirror cabinet above (toothbrushes, medicines)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -8025,7 +8035,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Bedside table</t>
+          <t>Floating bedside shelf with a drawer, reading light and charging point above (5 in walls are too thin for recessed niches)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -8044,7 +8054,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Teak</t>
+          <t>Teak, wall-hung</t>
         </is>
       </c>
       <c r="I12" s="10" t="n"/>
@@ -8197,7 +8207,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Wash basin</t>
+          <t>Wash basin with a mirror cabinet above</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -8326,7 +8336,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Wash basin (south wall, dry zone)</t>
+          <t>Wash basin (south wall, dry zone) with a mirror cabinet above</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -8359,36 +8369,36 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>F50</t>
+          <t>F63</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Bath 2</t>
+          <t>Ensuite</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Fixed glass splash panel at the south edge of the 3' x 3'-6" wet zone (north-east)</t>
+          <t>Recessed shower niche 1' x 1'-7" x 3 in deep, tiled, sloped sill (north wall below the window)</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Sanitary / plumbing</t>
         </is>
       </c>
       <c r="E20" s="4" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>0.15</v>
+        <v>0.22</v>
       </c>
       <c r="G20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>8 mm toughened glass</t>
+          <t>Tile lined, waterproofed</t>
         </is>
       </c>
       <c r="I20" s="10" t="n"/>
@@ -8402,36 +8412,36 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>F20</t>
+          <t>F64</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Bedroom 2</t>
+          <t>Common bath</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Queen bed 5' x 6'6" + headboard, head to the east wall (padded headboard: TV on the other side)</t>
+          <t>Recessed shower niche 1' x 1'-7" x 3 in deep, tiled, sloped sill (south wall below the window)</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Sanitary / plumbing</t>
         </is>
       </c>
       <c r="E21" s="4" t="n">
-        <v>6.35</v>
+        <v>1</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>5</v>
+        <v>0.22</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Teak</t>
+          <t>Tile lined, waterproofed</t>
         </is>
       </c>
       <c r="I21" s="10" t="n"/>
@@ -8445,36 +8455,36 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>F51</t>
+          <t>F65</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Bedroom 2</t>
+          <t>Bath 2</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Bedside table</t>
+          <t>Recessed shower niche 1' x 1'-10" x 3 in deep in the 7 in wet wall, tiled, sloped sill</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Sanitary / plumbing</t>
         </is>
       </c>
       <c r="E22" s="4" t="n">
-        <v>1</v>
+        <v>0.23</v>
       </c>
       <c r="F22" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Teak</t>
+          <t>Tile lined, waterproofed</t>
         </is>
       </c>
       <c r="I22" s="10" t="n"/>
@@ -8488,17 +8498,17 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>F22</t>
+          <t>F50</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Bedroom 2</t>
+          <t>Bath 2</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Work table 4' x 2' with monitor (east wall, north of the bed; north window to the side)</t>
+          <t>Fixed glass splash panel at the south edge of the 3' x 3'-6" wet zone (north-east)</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -8507,17 +8517,17 @@
         </is>
       </c>
       <c r="E23" s="4" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>4</v>
+        <v>0.15</v>
       </c>
       <c r="G23" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Teak / ply, cable tray, monitor arm</t>
+          <t>8 mm toughened glass</t>
         </is>
       </c>
       <c r="I23" s="10" t="n"/>
@@ -8531,7 +8541,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>F23</t>
+          <t>F20</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -8541,26 +8551,26 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Built-in wardrobe 6' with a mirror door (west wall, shared with the master: also a sound buffer)</t>
+          <t>Queen bed 5' x 6'6" + headboard, head to the east wall (padded headboard: TV on the other side)</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E24" s="4" t="n">
-        <v>2</v>
+        <v>6.35</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G24" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate</t>
+          <t>Teak</t>
         </is>
       </c>
       <c r="I24" s="10" t="n"/>
@@ -8574,36 +8584,36 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>F26</t>
+          <t>F51</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Pooja</t>
+          <t>Bedroom 2</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Pooja mandapam on the east wall (idols face west; family faces east)</t>
+          <t>Floating bedside shelf with a drawer, reading light and charging point above</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E25" s="4" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Carved teak</t>
+          <t>Teak, wall-hung</t>
         </is>
       </c>
       <c r="I25" s="10" t="n"/>
@@ -8617,17 +8627,17 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>F28</t>
+          <t>F22</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area</t>
+          <t>Bedroom 2</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Built-in bench with storage drawers below</t>
+          <t>Work table 4' x 2' with monitor (east wall, north of the bed; north window to the side)</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -8636,17 +8646,17 @@
         </is>
       </c>
       <c r="E26" s="4" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="G26" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Teak top, ply drawers, on legs</t>
+          <t>Teak / ply, cable tray, monitor arm</t>
         </is>
       </c>
       <c r="I26" s="10" t="n"/>
@@ -8660,36 +8670,36 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>F29</t>
+          <t>F23</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Wet area</t>
+          <t>Bedroom 2</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Utility sink counter (on the kitchen wall)</t>
+          <t>Built-in wardrobe 6' with a mirror door (west wall, shared with the master: also a sound buffer)</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Sanitary / plumbing</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E27" s="4" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="G27" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Kadappa / granite, SS sinks</t>
+          <t>Ply + laminate</t>
         </is>
       </c>
       <c r="I27" s="10" t="n"/>
@@ -8703,36 +8713,36 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>F30</t>
+          <t>F26</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Wet area</t>
+          <t>Pooja</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Washing machine bay 2' x 2' (covered back corner, 2 in clear of the bath wall)</t>
+          <t>Pooja mandapam on the east wall (idols face west; family faces east)</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Appliance / joinery</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E28" s="4" t="n">
-        <v>1.9</v>
+        <v>0.6</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>1.9</v>
+        <v>3</v>
       </c>
       <c r="G28" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Splash-proof socket, floor drain</t>
+          <t>Carved teak</t>
         </is>
       </c>
       <c r="I28" s="10" t="n"/>
@@ -8746,17 +8756,17 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>F31</t>
+          <t>F28</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Wet area</t>
+          <t>Sitting and serving area</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Fold-away clothesline in the south walkway</t>
+          <t>Built-in bench with storage drawers below</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -8765,17 +8775,17 @@
         </is>
       </c>
       <c r="E29" s="4" t="n">
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>1.8</v>
+        <v>2.8</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>SS wire, wall brackets</t>
+          <t>Teak top, ply drawers, on legs</t>
         </is>
       </c>
       <c r="I29" s="10" t="n"/>
@@ -8789,7 +8799,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>F44</t>
+          <t>F29</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -8799,26 +8809,26 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Tall slim utility cupboard (brooms, mops, detergents)</t>
+          <t>Utility sink counter (on the kitchen wall), where vessels are washed</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Sanitary / plumbing</t>
         </is>
       </c>
       <c r="E30" s="4" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>1.2</v>
+        <v>2.5</v>
       </c>
       <c r="G30" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate on legs, louvred doors</t>
+          <t>Kadappa / granite, SS sinks</t>
         </is>
       </c>
       <c r="I30" s="10" t="n"/>
@@ -8832,17 +8842,17 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>F32</t>
+          <t>F62</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area</t>
+          <t>Wet area</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Hand-wash basin at the east end of the serving counter, just outside the common bath (after meals); mirror on the side wall</t>
+          <t>Dish-drying rack over the utility sink (Swedish diskskap idea): steel rods, drip tray draining into the sink</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -8851,17 +8861,17 @@
         </is>
       </c>
       <c r="E31" s="4" t="n">
-        <v>1.9</v>
+        <v>0.8</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>Ceramic basin in granite top</t>
+          <t>SS 304</t>
         </is>
       </c>
       <c r="I31" s="10" t="n"/>
@@ -8875,17 +8885,17 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>F33</t>
+          <t>F61</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area</t>
+          <t>Wet area</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Serving counter with crockery cabinets above, 6 ft</t>
+          <t>Ceiling clothes airer on pulleys (lower to load, raise to dry), fixed to the roof truss</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -8894,17 +8904,17 @@
         </is>
       </c>
       <c r="E32" s="4" t="n">
-        <v>6</v>
+        <v>3.8</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="G32" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>Granite top, teak + glass shutters</t>
+          <t>Aluminium rails, nylon rope, cleat on the wall</t>
         </is>
       </c>
       <c r="I32" s="10" t="n"/>
@@ -8918,36 +8928,36 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>F56</t>
+          <t>F30</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area</t>
+          <t>Wet area</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Tall storage cupboard 5' x 2' (bedding, suitcases, festival vessels), loft above</t>
+          <t>Washing machine bay 2' x 2' (covered back corner, 2 in clear of the bath wall)</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Appliance / joinery</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
-        <v>5</v>
+        <v>1.9</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate, full height</t>
+          <t>Splash-proof socket, floor drain</t>
         </is>
       </c>
       <c r="I33" s="10" t="n"/>
@@ -8961,36 +8971,36 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>F34</t>
+          <t>F31</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Wet area</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>L-counter, south run</t>
+          <t>Fold-away clothesline in the south walkway</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E34" s="4" t="n">
-        <v>13.2</v>
+        <v>4</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="G34" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>Granite top, ply carcass</t>
+          <t>SS wire, wall brackets</t>
         </is>
       </c>
       <c r="I34" s="10" t="n"/>
@@ -9004,17 +9014,17 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>F35</t>
+          <t>F44</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Wet area</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>L-counter, east run (hob centred 7'-6" from the south wall face, on solid wall)</t>
+          <t>Tall slim utility cupboard (brooms, mops, detergents)</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -9023,17 +9033,17 @@
         </is>
       </c>
       <c r="E35" s="4" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>7</v>
+        <v>1.2</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>Granite top, cook faces east</t>
+          <t>Ply + laminate on legs, louvred doors</t>
         </is>
       </c>
       <c r="I35" s="10" t="n"/>
@@ -9047,36 +9057,36 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>F36</t>
+          <t>F32</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Sitting and serving area</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Refrigerator space (dining alcove beside the kitchen door, against the wet-area wall, door facing north)</t>
+          <t>Hand-wash basin at the east end of the serving counter, just outside the common bath (after meals); mirror on the side wall</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Appliance / joinery</t>
+          <t>Sanitary / plumbing</t>
         </is>
       </c>
       <c r="E36" s="4" t="n">
-        <v>2.5</v>
+        <v>1.9</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="G36" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>Double-door, 2'6" wide</t>
+          <t>Ceramic basin in granite top</t>
         </is>
       </c>
       <c r="I36" s="10" t="n"/>
@@ -9090,36 +9100,36 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>F38</t>
+          <t>F33</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Dining bay</t>
+          <t>Sitting and serving area</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Sofa 5'-6" (2-3 seats) facing west to the TV</t>
+          <t>Serving counter with crockery cabinets above, 6 ft</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E37" s="4" t="n">
-        <v>2.7</v>
+        <v>6</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>5.5</v>
+        <v>2</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>Teak frame, cotton cushions</t>
+          <t>Granite top, teak + glass shutters</t>
         </is>
       </c>
       <c r="I37" s="10" t="n"/>
@@ -9133,36 +9143,36 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>F39</t>
+          <t>F56</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Dining bay</t>
+          <t>Sitting and serving area</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Coffee table 3'6" x 2'</t>
+          <t>Tall storage cupboard 5' x 2' (bedding, suitcases, festival vessels), loft above</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E38" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F38" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="F38" s="4" t="n">
-        <v>3.5</v>
       </c>
       <c r="G38" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Teak</t>
+          <t>Ply + laminate, full height</t>
         </is>
       </c>
       <c r="I38" s="10" t="n"/>
@@ -9176,36 +9186,36 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>F53</t>
+          <t>F34</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Dining bay</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>TV unit 4'-5" on Bedroom 2's east wall (55-65 in TV wall-mounted above)</t>
+          <t>L-counter, south run: deep drawers for vessels instead of shutters</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Appliance / joinery</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E39" s="4" t="n">
-        <v>1.3</v>
+        <v>13.2</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>4.4</v>
+        <v>2</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Teak, low, open shelves</t>
+          <t>Granite top, ply carcass</t>
         </is>
       </c>
       <c r="I39" s="10" t="n"/>
@@ -9219,17 +9229,17 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>F40</t>
+          <t>F60</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Armchair at the west end of the window diwan</t>
+          <t>Utensil rail with hooks beside the hob (ladles, tongs, strainers)</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -9238,17 +9248,17 @@
         </is>
       </c>
       <c r="E40" s="4" t="n">
-        <v>1.8</v>
+        <v>2.2</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>1.8</v>
+        <v>0.15</v>
       </c>
       <c r="G40" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>Cane / teak</t>
+          <t>SS rail and S-hooks</t>
         </is>
       </c>
       <c r="I40" s="10" t="n"/>
@@ -9262,36 +9272,36 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>F58</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Window diwan 6' x 2'-6" under the north window, drawers below (guest seating, day bed); out of the line of the main door</t>
+          <t>L-counter, east run (hob centred 7'-6" from the south wall face, on solid wall; pull-out masala drawer beside the hob)</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E41" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>2.6</v>
+        <v>7</v>
       </c>
       <c r="G41" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>Teak frame, cotton mattress and bolsters</t>
+          <t>Granite top, cook faces east</t>
         </is>
       </c>
       <c r="I41" s="10" t="n"/>
@@ -9305,36 +9315,36 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>F52</t>
+          <t>F36</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Shoe cupboard 3'-3" on the east wall just north of the main door (closed shutters, louvred for air)</t>
+          <t>Refrigerator space (dining alcove beside the kitchen door, against the wet-area wall, door facing north)</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Appliance / joinery</t>
         </is>
       </c>
       <c r="E42" s="4" t="n">
-        <v>1.2</v>
+        <v>2.5</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>3.2</v>
+        <v>2.4</v>
       </c>
       <c r="G42" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>Ply + laminate, 14 in deep</t>
+          <t>Double-door, 2'6" wide</t>
         </is>
       </c>
       <c r="I42" s="10" t="n"/>
@@ -9348,17 +9358,17 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>F41</t>
+          <t>F38</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Poomukham (verandah)</t>
+          <t>Dining bay</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Oonjal (swing) 3'6", north side of the verandah, clear of the entrance</t>
+          <t>Sofa 5'-6" (2-3 seats) facing west to the TV</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -9367,17 +9377,17 @@
         </is>
       </c>
       <c r="E43" s="4" t="n">
-        <v>3.5</v>
+        <v>2.7</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>1.5</v>
+        <v>5.5</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>Teak, chains to beam</t>
+          <t>Teak frame, cotton cushions</t>
         </is>
       </c>
       <c r="I43" s="10" t="n"/>
@@ -9391,36 +9401,36 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>F42</t>
+          <t>F39</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Poomukham (verandah)</t>
+          <t>Dining bay</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Arugu seat (built-in, south end)</t>
+          <t>Coffee table 3'6" x 2'</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E44" s="4" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>2.4</v>
+        <v>3.5</v>
       </c>
       <c r="G44" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>Laterite base, teak top</t>
+          <t>Teak</t>
         </is>
       </c>
       <c r="I44" s="10" t="n"/>
@@ -9432,28 +9442,329 @@
       <c r="L44" s="8" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="6" t="inlineStr"/>
-      <c r="B45" s="6" t="inlineStr"/>
-      <c r="C45" s="6" t="inlineStr">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>F53</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Dining bay</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>TV unit 4'-5" on Bedroom 2's east wall (55-65 in TV wall-mounted above)</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Appliance / joinery</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F45" s="4" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>Teak, low, open shelves</t>
+        </is>
+      </c>
+      <c r="I45" s="10" t="n"/>
+      <c r="J45" s="11">
+        <f>G45*I45</f>
+        <v/>
+      </c>
+      <c r="K45" s="8" t="inlineStr"/>
+      <c r="L45" s="8" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>F40</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Living</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Armchair at the west end of the window diwan</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Loose furniture</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F46" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>Cane / teak</t>
+        </is>
+      </c>
+      <c r="I46" s="10" t="n"/>
+      <c r="J46" s="11">
+        <f>G46*I46</f>
+        <v/>
+      </c>
+      <c r="K46" s="8" t="inlineStr"/>
+      <c r="L46" s="8" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>F58</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Living</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Window diwan 6' x 2'-6" under the north window, drawers below (guest seating, day bed); out of the line of the main door</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Loose furniture</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>Teak frame, cotton mattress and bolsters</t>
+        </is>
+      </c>
+      <c r="I47" s="10" t="n"/>
+      <c r="J47" s="11">
+        <f>G47*I47</f>
+        <v/>
+      </c>
+      <c r="K47" s="8" t="inlineStr"/>
+      <c r="L47" s="8" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>F52</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Living</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Shoe bench 3'-3" (Japanese genkan idea): sit to take shoes off, louvred shoe shelves below, hooks and a keys niche above, small cabinet over</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Loose furniture</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F48" s="4" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="G48" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>Teak top, ply + laminate, 14 in deep</t>
+        </is>
+      </c>
+      <c r="I48" s="10" t="n"/>
+      <c r="J48" s="11">
+        <f>G48*I48</f>
+        <v/>
+      </c>
+      <c r="K48" s="8" t="inlineStr"/>
+      <c r="L48" s="8" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>F59</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Living</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Vilakku madam: carved teak lamp niche with a light inside, on the wall facing the main door</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Loose furniture</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="F49" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G49" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>Carved teak, brass lamp</t>
+        </is>
+      </c>
+      <c r="I49" s="10" t="n"/>
+      <c r="J49" s="11">
+        <f>G49*I49</f>
+        <v/>
+      </c>
+      <c r="K49" s="8" t="inlineStr"/>
+      <c r="L49" s="8" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>F41</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Poomukham (verandah)</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Oonjal (swing) 3'6", north side of the verandah, clear of the entrance</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Loose furniture</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F50" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G50" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>Teak, chains to beam</t>
+        </is>
+      </c>
+      <c r="I50" s="10" t="n"/>
+      <c r="J50" s="11">
+        <f>G50*I50</f>
+        <v/>
+      </c>
+      <c r="K50" s="8" t="inlineStr"/>
+      <c r="L50" s="8" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>F42</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Poomukham (verandah)</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Arugu seat (built-in, south end)</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>Built-in joinery</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F51" s="4" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G51" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>Laterite base, teak top</t>
+        </is>
+      </c>
+      <c r="I51" s="10" t="n"/>
+      <c r="J51" s="11">
+        <f>G51*I51</f>
+        <v/>
+      </c>
+      <c r="K51" s="8" t="inlineStr"/>
+      <c r="L51" s="8" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr"/>
+      <c r="B52" s="6" t="inlineStr"/>
+      <c r="C52" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D45" s="6" t="inlineStr"/>
-      <c r="E45" s="6" t="inlineStr"/>
-      <c r="F45" s="6" t="inlineStr"/>
-      <c r="G45" s="6">
-        <f>SUM(G2:G44)</f>
+      <c r="D52" s="6" t="inlineStr"/>
+      <c r="E52" s="6" t="inlineStr"/>
+      <c r="F52" s="6" t="inlineStr"/>
+      <c r="G52" s="6">
+        <f>SUM(G2:G51)</f>
         <v/>
       </c>
-      <c r="H45" s="6" t="inlineStr"/>
-      <c r="I45" s="12" t="inlineStr"/>
-      <c r="J45" s="12">
-        <f>SUM(J2:J44)</f>
+      <c r="H52" s="6" t="inlineStr"/>
+      <c r="I52" s="12" t="inlineStr"/>
+      <c r="J52" s="12">
+        <f>SUM(J2:J51)</f>
         <v/>
       </c>
-      <c r="K45" s="6" t="inlineStr"/>
-      <c r="L45" s="6" t="inlineStr"/>
+      <c r="K52" s="6" t="inlineStr"/>
+      <c r="L52" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9617,7 +9928,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Counter granite (local Ongole / Chimakurthy), 2 ft deep</t>
+          <t>Counter granite (local Ongole / Chimakurthy), 2 ft deep; deep drawers for vessels, pull-out masala drawer by the hob, utensil rail on the wall beside it</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr"/>
@@ -9645,7 +9956,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>12 mm step down, no raised threshold; doors open outward; SS grab bars by the WC and in the shower</t>
+          <t>Recessed tiled shower niche with a sloped sill; mirror cabinet over the basin; towel and clothes hooks at the dry end; 12 mm step down, no raised threshold; doors open outward; SS grab bars by the WC and in the shower</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr"/>
@@ -13867,9 +14178,13 @@
         <v>38.4</v>
       </c>
       <c r="F75" s="4" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="G75" s="4" t="inlineStr"/>
+        <v>17.3</v>
+      </c>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>inside the lamp niche</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">

</xml_diff>

<commit_message>
TV lounge in the centre with a window-seat enclave behind the sofa
TV moves to the north face of the common-bath wall; sofa faces south about
8 ft from it, main door in side view, TV no longer facing the door. Behind
the sofa a 3 ft walk and a built-in window seat (charupadi-style) under the
dining-bay window; reading chair in the corner; coffee table, rug and
points moved to suit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Schedules/KH-P1_Schedules_RevB.xlsx
+++ b/03_Schedules/KH-P1_Schedules_RevB.xlsx
@@ -4536,7 +4536,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>TV on Bedroom 2's east wall facing the dining bay: confirm screen size (55-65 in at about 9 ft) and a concealed HDMI/data conduit from the unit</t>
+          <t>TV on the north face of the common-bath wall in the dining space, sofa facing south: confirm screen size (55-65 in at about 8 ft from the sofa) and a concealed HDMI/data conduit; the north window behind the sofa may reflect on the screen (matt screen or sheer blind)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -4911,7 +4911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B48"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5056,7 +5056,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Twenty-sixth review: built-in ideas borrowed and adapted (function, not style, in Kerala materials): recessed shower niches, mirror cabinets over basins, genkan-style shoe bench with hooks and a granite threshold band, vilakku madam lamp niche facing the main door, floating bedside shelves (walls too thin for recesses), drawers-first kitchen with a masala pull-out and utensil rail, dish-drying rack over the utility sink, ceiling clothes airer in the wet area.</t>
+          <t>Twenty-eighth review: TV lounge reworked: sofa brought forward to about 8 ft from the TV, a 3 ft walk behind it, and a built-in window seat (charupadi-style enclave) under the dining-bay window, so the sofa backs onto a quiet seating nook rather than the entrance and nobody walks in front of the TV.</t>
         </is>
       </c>
     </row>
@@ -5066,7 +5066,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Twenty-fifth review: main door moved 3'-4" south (y 17'-7" to 20'-7"), centred under the front gable and opening straight onto the 5 ft walk between the pooja and the diwan; shoe cupboard to its north on the east wall; window diwan back to 6 ft along the north window, out of the door's line; steps, middle verandah pillars and the swing realigned.</t>
+          <t>Twenty-seventh review: TV lounge moves to the open dining space under the ventilator: TV on the north face of the common-bath wall, sofa facing south with its back to the north window, so the main door is in side view, not behind (commanding position) and the TV no longer faces the main door; the dining bay becomes a reading / dining nook with a chair by the window.</t>
         </is>
       </c>
     </row>
@@ -5076,7 +5076,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Twenty-fourth review: planned on the 27 ft plot alone (north strip dropped for now): roof eaves cut from 2'-6" to 2'-0" so the north eave stays inside the plot line, septic tank moved under the two-wheeler bay in the front yard with a lined soak pit beside it, all drains rerouted along the south walkway to the front, rainwater to the sump with overflow to the road; north-strip trees and recharge pit removed.</t>
+          <t>Twenty-sixth review: built-in ideas borrowed and adapted (function, not style, in Kerala materials): recessed shower niches, mirror cabinets over basins, genkan-style shoe bench with hooks and a granite threshold band, vilakku madam lamp niche facing the main door, floating bedside shelves (walls too thin for recesses), drawers-first kitchen with a masala pull-out and utensil rail, dish-drying rack over the utility sink, ceiling clothes airer in the wet area.</t>
         </is>
       </c>
     </row>
@@ -5086,7 +5086,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Twenty-third review: the fridge moves out of the kitchen into the dining alcove beside the kitchen door, against the wet-area wall; the kitchen's north wall is now free.</t>
+          <t>Twenty-fifth review: main door moved 3'-4" south (y 17'-7" to 20'-7"), centred under the front gable and opening straight onto the 5 ft walk between the pooja and the diwan; shoe cupboard to its north on the east wall; window diwan back to 6 ft along the north window, out of the door's line; steps, middle verandah pillars and the swing realigned.</t>
         </is>
       </c>
     </row>
@@ -5096,7 +5096,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Twenty-second review: the kitchen's tall pantry and the dining table and chairs are removed at the owner's request; the dining space under the ventilator stays open (the pendant light and points stay for a table later).</t>
+          <t>Twenty-fourth review: planned on the 27 ft plot alone (north strip dropped for now): roof eaves cut from 2'-6" to 2'-0" so the north eave stays inside the plot line, septic tank moved under the two-wheeler bay in the front yard with a lined soak pit beside it, all drains rerouted along the south walkway to the front, rainwater to the sump with overflow to the road; north-strip trees and recharge pit removed.</t>
         </is>
       </c>
     </row>
@@ -5106,7 +5106,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Twenty-first review: the open hall becomes three zones: family TV lounge in the dining bay (5'-6" sofa facing the TV), dining under the ventilator moved 9 in south (about 2 ft behind the chairs on both sides), and guest sitting by the main door with a 4'-6" window diwan (shortened after the walk-through showed a 1'-6" pinch at the shoe cupboard) and an armchair under the living's north window; a clear walk of about 4'-11" from the main door to the dining and kitchen, pooja front kept clear.</t>
+          <t>Twenty-third review: the fridge moves out of the kitchen into the dining alcove beside the kitchen door, against the wet-area wall; the kitchen's north wall is now free.</t>
         </is>
       </c>
     </row>
@@ -5116,7 +5116,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Twentieth review: Bedroom 2's bed moves to the east wall, head east, leaving an 8 x 14 ft open floor from the door to the bath and window; wardrobe to the west wall (sound buffer to the master), work table north of the bed, AC on the bath's outer wall; dresser dropped (mirror on the wardrobe).</t>
+          <t>Twenty-second review: the kitchen's tall pantry and the dining table and chairs are removed at the owner's request; the dining space under the ventilator stays open (the pendant light and points stay for a table later).</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
+          <t>Twenty-first review: the open hall becomes three zones: family TV lounge in the dining bay (5'-6" sofa facing the TV), dining under the ventilator moved 9 in south (about 2 ft behind the chairs on both sides), and guest sitting by the main door with a 4'-6" window diwan (shortened after the walk-through showed a 1'-6" pinch at the shoe cupboard) and an armchair under the living's north window; a clear walk of about 4'-11" from the main door to the dining and kitchen, pooja front kept clear.</t>
         </is>
       </c>
     </row>
@@ -5136,7 +5136,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
+          <t>Twentieth review: Bedroom 2's bed moves to the east wall, head east, leaving an 8 x 14 ft open floor from the door to the bath and window; wardrobe to the west wall (sound buffer to the master), work table north of the bed, AC on the bath's outer wall; dresser dropped (mirror on the wardrobe).</t>
         </is>
       </c>
     </row>
@@ -5146,7 +5146,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
+          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
         </is>
       </c>
     </row>
@@ -5156,7 +5156,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
+          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
         </is>
       </c>
     </row>
@@ -5166,7 +5166,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
+          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
+          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
         </is>
       </c>
     </row>
@@ -5186,7 +5186,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
+          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
+          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
         </is>
       </c>
     </row>
@@ -5206,7 +5206,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
+          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
         </is>
       </c>
     </row>
@@ -5216,7 +5216,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
+          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
         </is>
       </c>
     </row>
@@ -5226,7 +5226,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
+          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
         </is>
       </c>
     </row>
@@ -5236,7 +5236,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
+          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
         </is>
       </c>
     </row>
@@ -5246,7 +5246,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
+          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
         </is>
       </c>
     </row>
@@ -5256,7 +5256,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
+          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5266,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
+          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
         </is>
       </c>
     </row>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
+          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
         </is>
       </c>
     </row>
@@ -5286,7 +5286,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
+          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
         </is>
       </c>
     </row>
@@ -5296,7 +5296,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
+          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
         </is>
       </c>
     </row>
@@ -5306,7 +5306,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
+          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
         </is>
       </c>
     </row>
@@ -5316,7 +5316,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
+          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
         </is>
       </c>
     </row>
@@ -5326,7 +5326,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
+          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
         </is>
       </c>
     </row>
@@ -5336,7 +5336,7 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
+          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
         </is>
       </c>
     </row>
@@ -5346,7 +5346,7 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
+          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
+          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
         </is>
       </c>
     </row>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
+          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
         </is>
       </c>
     </row>
@@ -5376,7 +5376,7 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
         </is>
       </c>
     </row>
@@ -5395,6 +5395,26 @@
         <v>47</v>
       </c>
       <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>Roof: Mangalore clay tiles on steel truss over insulated cement-fibre deck; all edge tiles mechanically fixed.</t>
         </is>
@@ -7513,7 +7533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -9363,12 +9383,12 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Dining bay</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Sofa 5'-6" (2-3 seats) facing west to the TV</t>
+          <t>Sofa 5'-6" (2-3 seats) facing south to the TV about 8 ft away; behind it a 3 ft walk and the window-seat enclave; main door in side view</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -9377,10 +9397,10 @@
         </is>
       </c>
       <c r="E43" s="4" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="F43" s="4" t="n">
         <v>2.7</v>
-      </c>
-      <c r="F43" s="4" t="n">
-        <v>5.5</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>1</v>
@@ -9406,7 +9426,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Dining bay</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -9420,10 +9440,10 @@
         </is>
       </c>
       <c r="E44" s="4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F44" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="F44" s="4" t="n">
-        <v>3.5</v>
       </c>
       <c r="G44" s="4" t="n">
         <v>1</v>
@@ -9449,12 +9469,12 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Dining bay</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>TV unit 4'-5" on Bedroom 2's east wall (55-65 in TV wall-mounted above)</t>
+          <t>TV unit 4'-5" on the north face of the common-bath wall (55-65 in TV wall-mounted above)</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -9463,10 +9483,10 @@
         </is>
       </c>
       <c r="E45" s="4" t="n">
-        <v>1.3</v>
+        <v>4.4</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>4.4</v>
+        <v>1.25</v>
       </c>
       <c r="G45" s="4" t="n">
         <v>1</v>
@@ -9487,17 +9507,17 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>F40</t>
+          <t>F68</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Dining bay</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Armchair at the west end of the window diwan</t>
+          <t>Built-in window seat 6'-5" x 2' under the north window (charupadi-style enclave: cushions, bolsters, drawers below)</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -9506,17 +9526,17 @@
         </is>
       </c>
       <c r="E46" s="4" t="n">
-        <v>1.8</v>
+        <v>6.4</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="G46" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>Cane / teak</t>
+          <t>Teak, cotton cushions</t>
         </is>
       </c>
       <c r="I46" s="10" t="n"/>
@@ -9530,17 +9550,17 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>F58</t>
+          <t>F66</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Dining bay</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Window diwan 6' x 2'-6" under the north window, drawers below (guest seating, day bed); out of the line of the main door</t>
+          <t>Reading chair in the north-west corner of the bay</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -9549,17 +9569,17 @@
         </is>
       </c>
       <c r="E47" s="4" t="n">
-        <v>6</v>
+        <v>1.8</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>2.6</v>
+        <v>1.8</v>
       </c>
       <c r="G47" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>Teak frame, cotton mattress and bolsters</t>
+          <t>Cane / teak</t>
         </is>
       </c>
       <c r="I47" s="10" t="n"/>
@@ -9573,7 +9593,7 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>F52</t>
+          <t>F40</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -9583,7 +9603,7 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Shoe bench 3'-3" (Japanese genkan idea): sit to take shoes off, louvred shoe shelves below, hooks and a keys niche above, small cabinet over</t>
+          <t>Armchair at the west end of the window diwan</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -9592,17 +9612,17 @@
         </is>
       </c>
       <c r="E48" s="4" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>3.2</v>
+        <v>1.8</v>
       </c>
       <c r="G48" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>Teak top, ply + laminate, 14 in deep</t>
+          <t>Cane / teak</t>
         </is>
       </c>
       <c r="I48" s="10" t="n"/>
@@ -9616,7 +9636,7 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>F59</t>
+          <t>F58</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -9626,7 +9646,7 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Vilakku madam: carved teak lamp niche with a light inside, on the wall facing the main door</t>
+          <t>Window diwan 6' x 2'-6" under the north window, drawers below (guest seating, day bed); out of the line of the main door</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -9635,17 +9655,17 @@
         </is>
       </c>
       <c r="E49" s="4" t="n">
-        <v>0.34</v>
+        <v>6</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>1.8</v>
+        <v>2.6</v>
       </c>
       <c r="G49" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>Carved teak, brass lamp</t>
+          <t>Teak frame, cotton mattress and bolsters</t>
         </is>
       </c>
       <c r="I49" s="10" t="n"/>
@@ -9659,17 +9679,17 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>F41</t>
+          <t>F52</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Poomukham (verandah)</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Oonjal (swing) 3'6", north side of the verandah, clear of the entrance</t>
+          <t>Shoe bench 3'-3" (Japanese genkan idea): sit to take shoes off, louvred shoe shelves below, hooks and a keys niche above, small cabinet over</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -9678,17 +9698,17 @@
         </is>
       </c>
       <c r="E50" s="4" t="n">
-        <v>3.5</v>
+        <v>1.2</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>1.5</v>
+        <v>3.2</v>
       </c>
       <c r="G50" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H50" s="4" t="inlineStr">
         <is>
-          <t>Teak, chains to beam</t>
+          <t>Teak top, ply + laminate, 14 in deep</t>
         </is>
       </c>
       <c r="I50" s="10" t="n"/>
@@ -9702,36 +9722,36 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>F42</t>
+          <t>F59</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Poomukham (verandah)</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Arugu seat (built-in, south end)</t>
+          <t>Vilakku madam: carved teak lamp niche with a light inside, on the wall facing the main door</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E51" s="4" t="n">
-        <v>1.2</v>
+        <v>0.34</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>2.4</v>
+        <v>1.8</v>
       </c>
       <c r="G51" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>Laterite base, teak top</t>
+          <t>Carved teak, brass lamp</t>
         </is>
       </c>
       <c r="I51" s="10" t="n"/>
@@ -9743,28 +9763,114 @@
       <c r="L51" s="8" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="6" t="inlineStr"/>
-      <c r="B52" s="6" t="inlineStr"/>
-      <c r="C52" s="6" t="inlineStr">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>F41</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Poomukham (verandah)</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Oonjal (swing) 3'6", north side of the verandah, clear of the entrance</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>Loose furniture</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F52" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G52" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H52" s="4" t="inlineStr">
+        <is>
+          <t>Teak, chains to beam</t>
+        </is>
+      </c>
+      <c r="I52" s="10" t="n"/>
+      <c r="J52" s="11">
+        <f>G52*I52</f>
+        <v/>
+      </c>
+      <c r="K52" s="8" t="inlineStr"/>
+      <c r="L52" s="8" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>F42</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Poomukham (verandah)</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>Arugu seat (built-in, south end)</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>Built-in joinery</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F53" s="4" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G53" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>Laterite base, teak top</t>
+        </is>
+      </c>
+      <c r="I53" s="10" t="n"/>
+      <c r="J53" s="11">
+        <f>G53*I53</f>
+        <v/>
+      </c>
+      <c r="K53" s="8" t="inlineStr"/>
+      <c r="L53" s="8" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr"/>
+      <c r="B54" s="6" t="inlineStr"/>
+      <c r="C54" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D52" s="6" t="inlineStr"/>
-      <c r="E52" s="6" t="inlineStr"/>
-      <c r="F52" s="6" t="inlineStr"/>
-      <c r="G52" s="6">
-        <f>SUM(G2:G51)</f>
+      <c r="D54" s="6" t="inlineStr"/>
+      <c r="E54" s="6" t="inlineStr"/>
+      <c r="F54" s="6" t="inlineStr"/>
+      <c r="G54" s="6">
+        <f>SUM(G2:G53)</f>
         <v/>
       </c>
-      <c r="H52" s="6" t="inlineStr"/>
-      <c r="I52" s="12" t="inlineStr"/>
-      <c r="J52" s="12">
-        <f>SUM(J2:J51)</f>
+      <c r="H54" s="6" t="inlineStr"/>
+      <c r="I54" s="12" t="inlineStr"/>
+      <c r="J54" s="12">
+        <f>SUM(J2:J53)</f>
         <v/>
       </c>
-      <c r="K52" s="6" t="inlineStr"/>
-      <c r="L52" s="6" t="inlineStr"/>
+      <c r="K54" s="6" t="inlineStr"/>
+      <c r="L54" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14006,18 +14112,18 @@
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>Dining bay (north window)</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E70" s="4" t="n">
-        <v>38.4</v>
+        <v>44.8</v>
       </c>
       <c r="F70" s="4" t="n">
-        <v>22.4</v>
+        <v>9.4</v>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>TV wall: 2 sockets + data + HDMI conduit to the unit</t>
+          <t>TV wall (common-bath wall, dry face): 2 sockets + data + HDMI conduit to the unit</t>
         </is>
       </c>
     </row>
@@ -14039,14 +14145,14 @@
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Dining bay (north window)</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E71" s="4" t="n">
-        <v>38.4</v>
+        <v>43.2</v>
       </c>
       <c r="F71" s="4" t="n">
-        <v>21</v>
+        <v>9.4</v>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
@@ -14083,7 +14189,7 @@
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>above the TV unit, throws east over the seating</t>
+          <t>Bedroom 2's east wall, throws east across the hall and the TV seating</t>
         </is>
       </c>
     </row>
@@ -14898,14 +15004,14 @@
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>Dining bay (north window)</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E98" s="4" t="n">
-        <v>48.2</v>
+        <v>47.9</v>
       </c>
       <c r="F98" s="4" t="n">
-        <v>18.8</v>
+        <v>18</v>
       </c>
       <c r="G98" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Thin precast post-and-panel compound wall
2 in panels in 4 in posts, 5 ft high, set just inside the plot line so
the side strips stay walkable; panels lift out so the north run can move if
the north strip is bought. Added to the specification, quantities (60 m),
site plan notes, brief and the 3D model.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Schedules/KH-P1_Schedules_RevB.xlsx
+++ b/03_Schedules/KH-P1_Schedules_RevB.xlsx
@@ -4911,7 +4911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5056,7 +5056,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Twenty-eighth review: TV lounge reworked: sofa brought forward to about 8 ft from the TV, a 3 ft walk behind it, and a built-in window seat (charupadi-style enclave) under the dining-bay window, so the sofa backs onto a quiet seating nook rather than the entrance and nobody walks in front of the TV.</t>
+          <t>Twenty-ninth review: compound wall made as thin as practical: precast RCC post-and-panel (2 in panels in 4 in posts) set just inside the plot line, so the side strips stay walkable and the north run can be lifted and moved if more land is bought.</t>
         </is>
       </c>
     </row>
@@ -5066,7 +5066,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Twenty-seventh review: TV lounge moves to the open dining space under the ventilator: TV on the north face of the common-bath wall, sofa facing south with its back to the north window, so the main door is in side view, not behind (commanding position) and the TV no longer faces the main door; the dining bay becomes a reading / dining nook with a chair by the window.</t>
+          <t>Twenty-eighth review: TV lounge reworked: sofa brought forward to about 8 ft from the TV, a 3 ft walk behind it, and a built-in window seat (charupadi-style enclave) under the dining-bay window, so the sofa backs onto a quiet seating nook rather than the entrance and nobody walks in front of the TV.</t>
         </is>
       </c>
     </row>
@@ -5076,7 +5076,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Twenty-sixth review: built-in ideas borrowed and adapted (function, not style, in Kerala materials): recessed shower niches, mirror cabinets over basins, genkan-style shoe bench with hooks and a granite threshold band, vilakku madam lamp niche facing the main door, floating bedside shelves (walls too thin for recesses), drawers-first kitchen with a masala pull-out and utensil rail, dish-drying rack over the utility sink, ceiling clothes airer in the wet area.</t>
+          <t>Twenty-seventh review: TV lounge moves to the open dining space under the ventilator: TV on the north face of the common-bath wall, sofa facing south with its back to the north window, so the main door is in side view, not behind (commanding position) and the TV no longer faces the main door; the dining bay becomes a reading / dining nook with a chair by the window.</t>
         </is>
       </c>
     </row>
@@ -5086,7 +5086,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Twenty-fifth review: main door moved 3'-4" south (y 17'-7" to 20'-7"), centred under the front gable and opening straight onto the 5 ft walk between the pooja and the diwan; shoe cupboard to its north on the east wall; window diwan back to 6 ft along the north window, out of the door's line; steps, middle verandah pillars and the swing realigned.</t>
+          <t>Twenty-sixth review: built-in ideas borrowed and adapted (function, not style, in Kerala materials): recessed shower niches, mirror cabinets over basins, genkan-style shoe bench with hooks and a granite threshold band, vilakku madam lamp niche facing the main door, floating bedside shelves (walls too thin for recesses), drawers-first kitchen with a masala pull-out and utensil rail, dish-drying rack over the utility sink, ceiling clothes airer in the wet area.</t>
         </is>
       </c>
     </row>
@@ -5096,7 +5096,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Twenty-fourth review: planned on the 27 ft plot alone (north strip dropped for now): roof eaves cut from 2'-6" to 2'-0" so the north eave stays inside the plot line, septic tank moved under the two-wheeler bay in the front yard with a lined soak pit beside it, all drains rerouted along the south walkway to the front, rainwater to the sump with overflow to the road; north-strip trees and recharge pit removed.</t>
+          <t>Twenty-fifth review: main door moved 3'-4" south (y 17'-7" to 20'-7"), centred under the front gable and opening straight onto the 5 ft walk between the pooja and the diwan; shoe cupboard to its north on the east wall; window diwan back to 6 ft along the north window, out of the door's line; steps, middle verandah pillars and the swing realigned.</t>
         </is>
       </c>
     </row>
@@ -5106,7 +5106,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Twenty-third review: the fridge moves out of the kitchen into the dining alcove beside the kitchen door, against the wet-area wall; the kitchen's north wall is now free.</t>
+          <t>Twenty-fourth review: planned on the 27 ft plot alone (north strip dropped for now): roof eaves cut from 2'-6" to 2'-0" so the north eave stays inside the plot line, septic tank moved under the two-wheeler bay in the front yard with a lined soak pit beside it, all drains rerouted along the south walkway to the front, rainwater to the sump with overflow to the road; north-strip trees and recharge pit removed.</t>
         </is>
       </c>
     </row>
@@ -5116,7 +5116,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Twenty-second review: the kitchen's tall pantry and the dining table and chairs are removed at the owner's request; the dining space under the ventilator stays open (the pendant light and points stay for a table later).</t>
+          <t>Twenty-third review: the fridge moves out of the kitchen into the dining alcove beside the kitchen door, against the wet-area wall; the kitchen's north wall is now free.</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Twenty-first review: the open hall becomes three zones: family TV lounge in the dining bay (5'-6" sofa facing the TV), dining under the ventilator moved 9 in south (about 2 ft behind the chairs on both sides), and guest sitting by the main door with a 4'-6" window diwan (shortened after the walk-through showed a 1'-6" pinch at the shoe cupboard) and an armchair under the living's north window; a clear walk of about 4'-11" from the main door to the dining and kitchen, pooja front kept clear.</t>
+          <t>Twenty-second review: the kitchen's tall pantry and the dining table and chairs are removed at the owner's request; the dining space under the ventilator stays open (the pendant light and points stay for a table later).</t>
         </is>
       </c>
     </row>
@@ -5136,7 +5136,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Twentieth review: Bedroom 2's bed moves to the east wall, head east, leaving an 8 x 14 ft open floor from the door to the bath and window; wardrobe to the west wall (sound buffer to the master), work table north of the bed, AC on the bath's outer wall; dresser dropped (mirror on the wardrobe).</t>
+          <t>Twenty-first review: the open hall becomes three zones: family TV lounge in the dining bay (5'-6" sofa facing the TV), dining under the ventilator moved 9 in south (about 2 ft behind the chairs on both sides), and guest sitting by the main door with a 4'-6" window diwan (shortened after the walk-through showed a 1'-6" pinch at the shoe cupboard) and an armchair under the living's north window; a clear walk of about 4'-11" from the main door to the dining and kitchen, pooja front kept clear.</t>
         </is>
       </c>
     </row>
@@ -5146,7 +5146,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
+          <t>Twentieth review: Bedroom 2's bed moves to the east wall, head east, leaving an 8 x 14 ft open floor from the door to the bath and window; wardrobe to the west wall (sound buffer to the master), work table north of the bed, AC on the bath's outer wall; dresser dropped (mirror on the wardrobe).</t>
         </is>
       </c>
     </row>
@@ -5156,7 +5156,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
+          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
         </is>
       </c>
     </row>
@@ -5166,7 +5166,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
+          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
+          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
         </is>
       </c>
     </row>
@@ -5186,7 +5186,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
+          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
+          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
         </is>
       </c>
     </row>
@@ -5206,7 +5206,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
+          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
         </is>
       </c>
     </row>
@@ -5216,7 +5216,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
+          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
         </is>
       </c>
     </row>
@@ -5226,7 +5226,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
+          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
         </is>
       </c>
     </row>
@@ -5236,7 +5236,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
+          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
         </is>
       </c>
     </row>
@@ -5246,7 +5246,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
+          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
         </is>
       </c>
     </row>
@@ -5256,7 +5256,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
+          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5266,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
+          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
         </is>
       </c>
     </row>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
+          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
         </is>
       </c>
     </row>
@@ -5286,7 +5286,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
+          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
         </is>
       </c>
     </row>
@@ -5296,7 +5296,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
+          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
         </is>
       </c>
     </row>
@@ -5306,7 +5306,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
+          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
         </is>
       </c>
     </row>
@@ -5316,7 +5316,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
+          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
         </is>
       </c>
     </row>
@@ -5326,7 +5326,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
+          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
         </is>
       </c>
     </row>
@@ -5336,7 +5336,7 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
+          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
         </is>
       </c>
     </row>
@@ -5346,7 +5346,7 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
+          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
+          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
         </is>
       </c>
     </row>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
+          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
         </is>
       </c>
     </row>
@@ -5376,7 +5376,7 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
+          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
+          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
         </is>
       </c>
     </row>
@@ -5396,7 +5396,7 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
         </is>
       </c>
     </row>
@@ -5415,6 +5415,16 @@
         <v>49</v>
       </c>
       <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>Roof: Mangalore clay tiles on steel truss over insulated cement-fibre deck; all edge tiles mechanically fixed.</t>
         </is>
@@ -10214,7 +10224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10292,22 +10302,22 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Substructure</t>
+          <t>Site</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Plinth beam + DPC</t>
+          <t>Compound wall</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>RCC plinth beam all round; 40 mm DPC with waterproofing compound at plinth top</t>
+          <t>Precast RCC post-and-panel wall, 5 ft high: 4 in square posts at about 7 ft centres on small pad footings, 2 in slotted panels, set just inside the plot line; panels lift out, so the north run can be moved if the north strip is bought</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Stops rising damp into AAC</t>
+          <t>Thinnest practical wall: keeps the 2 ft north gap and 3 ft south walkway usable; cheap, quick and reusable</t>
         </is>
       </c>
     </row>
@@ -10319,17 +10329,17 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Plinth fill</t>
+          <t>Plinth beam + DPC</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Non-expansive moorum / gravel in 150 mm layers, compacted; no black soil fill</t>
+          <t>RCC plinth beam all round; 40 mm DPC with waterproofing compound at plinth top</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Black soil under the floor will heave the slab</t>
+          <t>Stops rising damp into AAC</t>
         </is>
       </c>
     </row>
@@ -10341,17 +10351,17 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Anti-termite</t>
+          <t>Plinth fill</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Pre-construction chemical treatment (IS 6313) at foundation, plinth fill and around walls</t>
+          <t>Non-expansive moorum / gravel in 150 mm layers, compacted; no black soil fill</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>High termite risk; cannot be redone easily later</t>
+          <t>Black soil under the floor will heave the slab</t>
         </is>
       </c>
     </row>
@@ -10363,61 +10373,61 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Plinth protection</t>
+          <t>Anti-termite</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>3 ft PCC apron with slope away, joint sealed to wall</t>
+          <t>Pre-construction chemical treatment (IS 6313) at foundation, plinth fill and around walls</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Keeps rain off expansive soil next to foundations</t>
+          <t>High termite risk; cannot be redone easily later</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Frame</t>
+          <t>Substructure</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Columns, beams, bands</t>
+          <t>Plinth protection</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>RCC frame; lintel band at door head, ring beam at wall top; seismic zone III detailing (IS 13920 as engineer decides)</t>
+          <t>3 ft PCC apron with slope away, joint sealed to wall</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>AAC infill is not load-bearing for truss + cyclone loads</t>
+          <t>Keeps rain off expansive soil next to foundations</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Walls</t>
+          <t>Frame</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>AAC blocks</t>
+          <t>Columns, beams, bands</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>IS 2185-3, 200 mm outer / 150 mm wet walls / 100 mm inner; thin-bed polymer mortar</t>
+          <t>RCC frame; lintel band at door head, ring beam at wall top; seismic zone III detailing (IS 13920 as engineer decides)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Better insulation than brick; lighter frame</t>
+          <t>AAC infill is not load-bearing for truss + cyclone loads</t>
         </is>
       </c>
     </row>
@@ -10429,17 +10439,17 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>AAC to RCC joints</t>
+          <t>AAC blocks</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Galvanised mesh strip 150 mm wide over every block-concrete joint before plaster</t>
+          <t>IS 2185-3, 200 mm outer / 150 mm wet walls / 100 mm inner; thin-bed polymer mortar</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>The most common AAC crack; cheap to prevent</t>
+          <t>Better insulation than brick; lighter frame</t>
         </is>
       </c>
     </row>
@@ -10451,17 +10461,17 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Chasing</t>
+          <t>AAC to RCC joints</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Cut chases with a groover, never hammer; fill with polymer mortar + mesh</t>
+          <t>Galvanised mesh strip 150 mm wide over every block-concrete joint before plaster</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Hammering cracks AAC blocks</t>
+          <t>The most common AAC crack; cheap to prevent</t>
         </is>
       </c>
     </row>
@@ -10473,39 +10483,39 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>External plaster</t>
+          <t>Chasing</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>20 mm, two coats, waterproof admixture, cured 7 days; elastomeric paint</t>
+          <t>Cut chases with a groover, never hammer; fill with polymer mortar + mesh</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Wind-driven cyclone rain</t>
+          <t>Hammering cracks AAC blocks</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Roof</t>
+          <t>Walls</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>External plaster</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Steel truss (hot-dip galvanised or epoxy primed), 30 deg pitch, bolted to ring beam with holding-down bolts</t>
+          <t>20 mm, two coats, waterproof admixture, cured 7 days; elastomeric paint</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Uplift in cyclone winds</t>
+          <t>Wind-driven cyclone rain</t>
         </is>
       </c>
     </row>
@@ -10517,17 +10527,17 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Deck and insulation</t>
+          <t>Structure</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Cement-fibre board deck + 50 mm PIR/XPS or reflective insulation + membrane, then battens and Mangalore tiles</t>
+          <t>Steel truss (hot-dip galvanised or epoxy primed), 30 deg pitch, bolted to ring beam with holding-down bolts</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Cuts attic heat in 45 C summers</t>
+          <t>Uplift in cyclone winds</t>
         </is>
       </c>
     </row>
@@ -10539,17 +10549,17 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Tile fixing</t>
+          <t>Deck and insulation</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Clip or screw every tile at eaves, verges, ridges and hips, and every 3rd row elsewhere; ridges bedded and pointed</t>
+          <t>Cement-fibre board deck + 50 mm PIR/XPS or reflective insulation + membrane, then battens and Mangalore tiles</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Loose tiles fly in cyclones</t>
+          <t>Cuts attic heat in 45 C summers</t>
         </is>
       </c>
     </row>
@@ -10561,17 +10571,17 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Ventilation</t>
+          <t>Tile fixing</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Ridge / gable vents with bird and insect mesh; soffit vents at eaves</t>
+          <t>Clip or screw every tile at eaves, verges, ridges and hips, and every 3rd row elsewhere; ridges bedded and pointed</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Flushes hot air from the attic</t>
+          <t>Loose tiles fly in cyclones</t>
         </is>
       </c>
     </row>
@@ -10583,17 +10593,17 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Dining ventilator</t>
+          <t>Ventilation</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Steel frame bolted to the truss; hipped tiled cap at 30 deg, 1'-6" overhang; 45 deg timber or aluminium louvres with 4 in lap; SS 304 mesh about 1.2 mm (18 x 16) in a sealed continuous frame; inner shutters with EPDM seals and a winding opener at 5 ft; 9 in upstand with flashing; fibre-cement lined, insulated shaft</t>
+          <t>Ridge / gable vents with bird and insect mesh; soffit vents at eaves</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Lets hot air out, keeps out rain, mosquitoes and attic dust, and closes for AC</t>
+          <t>Flushes hot air from the attic</t>
         </is>
       </c>
     </row>
@@ -10605,39 +10615,39 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Gutters and downpipes</t>
+          <t>Dining ventilator</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>150 mm half-round gutters with leaf guard, 100 mm downpipes at 8 points, to the sump filter, overflow to the road drain</t>
+          <t>Steel frame bolted to the truss; hipped tiled cap at 30 deg, 1'-6" overhang; 45 deg timber or aluminium louvres with 4 in lap; SS 304 mesh about 1.2 mm (18 x 16) in a sealed continuous frame; inner shutters with EPDM seals and a winding opener at 5 ft; 9 in upstand with flashing; fibre-cement lined, insulated shaft</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Short heavy bursts; protects the plinth</t>
+          <t>Lets hot air out, keeps out rain, mosquitoes and attic dust, and closes for AC</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Openings</t>
+          <t>Roof</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Windows</t>
+          <t>Gutters and downpipes</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Hardwood or UPVC frames; mosquito mesh on every opening; MS grill for security</t>
+          <t>150 mm half-round gutters with leaf guard, 100 mm downpipes at 8 points, to the sump filter, overflow to the road drain</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Mosquitoes; ground-floor security</t>
+          <t>Short heavy bursts; protects the plinth</t>
         </is>
       </c>
     </row>
@@ -10649,17 +10659,17 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Sills and sunshades</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>External sills sloped 1:10 with drip groove; 2 ft sunshades with drip groove; 18 in projecting drip under the jali wall</t>
+          <t>Hardwood or UPVC frames; mosquito mesh on every opening; MS grill for security</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Stops staining and water entry</t>
+          <t>Mosquitoes; ground-floor security</t>
         </is>
       </c>
     </row>
@@ -10671,17 +10681,17 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Vents above inner doors</t>
+          <t>Sills and sunshades</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Pooja: open jali; bedrooms and bathrooms: none (the workstation has no door for now). 7'-6" to 9'-0" above the lintel band</t>
+          <t>External sills sloped 1:10 with drip groove; 2 ft sunshades with drip groove; 18 in projecting drip under the jali wall</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Air moves with doors shut where privacy allows; bedrooms rely on their north windows, fans and AC</t>
+          <t>Stops staining and water entry</t>
         </is>
       </c>
     </row>
@@ -10693,39 +10703,39 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Bathroom doors</t>
+          <t>Vents above inner doors</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>WPC / FRP shutters on WPC or granite frame base; no wooden frame touching the wet floor</t>
+          <t>Pooja: open jali; bedrooms and bathrooms: none (the workstation has no door for now). 7'-6" to 9'-0" above the lintel band</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Wood frames rot at the bottom</t>
+          <t>Air moves with doors shut where privacy allows; bedrooms rely on their north windows, fans and AC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Floors</t>
+          <t>Openings</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Bathroom doors</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>4 in skirting flush with the wall plaster (groove in plaster); 3 mm epoxy grout in wet areas</t>
+          <t>WPC / FRP shutters on WPC or granite frame base; no wooden frame touching the wet floor</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>No dust ledge, no black grout lines</t>
+          <t>Wood frames rot at the bottom</t>
         </is>
       </c>
     </row>
@@ -10737,39 +10747,39 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Wet rooms</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Waterproofing (polymer cementitious) floor + 12 in up walls + 7 ft in shower; flood test 48 h before tiling</t>
+          <t>4 in skirting flush with the wall plaster (groove in plaster); 3 mm epoxy grout in wet areas</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Leak into neighbouring rooms is the top complaint</t>
+          <t>No dust ledge, no black grout lines</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Floors</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Supply</t>
+          <t>Wet rooms</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>CPVC hot/cold; supply runs along external walls in clamps or shallow chases; isolation valve per bathroom and kitchen</t>
+          <t>Waterproofing (polymer cementitious) floor + 12 in up walls + 7 ft in shower; flood test 48 h before tiling</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Easy repair without breaking tiles</t>
+          <t>Leak into neighbouring rooms is the top complaint</t>
         </is>
       </c>
     </row>
@@ -10781,17 +10791,17 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>uPVC SWR 110 mm soil, 75 mm waste; inspection chamber at every bend and junction; separate soil and grey-water lines</t>
+          <t>CPVC hot/cold; supply runs along external walls in clamps or shallow chases; isolation valve per bathroom and kitchen</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Easy rodding</t>
+          <t>Easy repair without breaking tiles</t>
         </is>
       </c>
     </row>
@@ -10803,39 +10813,39 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Water treatment</t>
+          <t>Drainage</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>RO for drinking at kitchen; whole-house softener if hardness &gt; 300 mg/l; matt fittings</t>
+          <t>uPVC SWR 110 mm soil, 75 mm waste; inspection chamber at every bend and junction; separate soil and grey-water lines</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Guntur groundwater is often hard with high fluoride</t>
+          <t>Easy rodding</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Wiring</t>
+          <t>Water treatment</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>FR-LSH copper; 1.5 sq mm lights, 2.5 sq mm sockets, 4 sq mm AC / geyser; separate circuits per AC</t>
+          <t>RO for drinking at kitchen; whole-house softener if hardness &gt; 300 mg/l; matt fittings</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>AC loads</t>
+          <t>Guntur groundwater is often hard with high fluoride</t>
         </is>
       </c>
     </row>
@@ -10847,17 +10857,17 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Protection</t>
+          <t>Wiring</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>RCCB 30 mA + MCBs; 2 earth pits; surge protection device; DB in an accessible spot</t>
+          <t>FR-LSH copper; 1.5 sq mm lights, 2.5 sq mm sockets, 4 sq mm AC / geyser; separate circuits per AC</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Shock and lightning safety</t>
+          <t>AC loads</t>
         </is>
       </c>
     </row>
@@ -10869,17 +10879,17 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Backup</t>
+          <t>Protection</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Inverter circuit to lights, fans, office sockets and router; conduit from roof to DB for future solar PV</t>
+          <t>RCCB 30 mA + MCBs; 2 earth pits; surge protection device; DB in an accessible spot</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Power cuts during work-from-home</t>
+          <t>Shock and lightning safety</t>
         </is>
       </c>
     </row>
@@ -10891,15 +10901,37 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
+          <t>Backup</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Inverter circuit to lights, fans, office sockets and router; conduit from roof to DB for future solar PV</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Power cuts during work-from-home</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
           <t>AC provisions</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>16 A socket at 7 ft, 65 mm sleeve through wall, drain pipe to outside, ODU brackets on shaded walls</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>Retrofitting later means breaking walls</t>
         </is>
@@ -10916,7 +10948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11753,20 +11785,20 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Plinth protection apron, 3 ft wide</t>
+          <t>Compound wall, precast RCC post and panel, 5 ft high</t>
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>sq m</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>PCC with slope away</t>
+          <t>Plot perimeter less the gate</t>
         </is>
       </c>
       <c r="F28" s="10" t="n"/>
@@ -11778,25 +11810,25 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Openings</t>
+          <t>Site</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Doors</t>
+          <t>Plinth protection apron, 3 ft wide</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>9</v>
+        <v>51</v>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>no.</t>
+          <t>sq m</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>See Doors tab</t>
+          <t>PCC with slope away</t>
         </is>
       </c>
       <c r="F29" s="10" t="n"/>
@@ -11813,11 +11845,11 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Windows and vents</t>
+          <t>Doors</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
@@ -11826,7 +11858,7 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>See Windows tab</t>
+          <t>See Doors tab</t>
         </is>
       </c>
       <c r="F30" s="10" t="n"/>
@@ -11843,18 +11875,22 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Window area (for mesh and grills)</t>
+          <t>Windows and vents</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>22.8</v>
+        <v>17</v>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>sq m</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr"/>
+          <t>no.</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>See Windows tab</t>
+        </is>
+      </c>
       <c r="F31" s="10" t="n"/>
       <c r="G31" s="11">
         <f>IF(F31="","",C31*F31)</f>
@@ -11862,18 +11898,44 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr"/>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Openings</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Window area (for mesh and grills)</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>sq m</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr"/>
+      <c r="F32" s="10" t="n"/>
+      <c r="G32" s="11">
+        <f>IF(F32="","",C32*F32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr"/>
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>Total of priced items</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr"/>
-      <c r="D32" s="6" t="inlineStr"/>
-      <c r="E32" s="6" t="inlineStr"/>
-      <c r="F32" s="12" t="inlineStr"/>
-      <c r="G32" s="12">
-        <f>SUM(G2:G31)</f>
+      <c r="C33" s="6" t="inlineStr"/>
+      <c r="D33" s="6" t="inlineStr"/>
+      <c r="E33" s="6" t="inlineStr"/>
+      <c r="F33" s="12" t="inlineStr"/>
+      <c r="G33" s="12">
+        <f>SUM(G2:G32)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Proportion clean-up and front facade upgrades
Windows standardised to three sizes with every head at 7 ft; sunshades only
on sunny walls; floors cut to three families plus the verandah; hidden
services, aligned switches, warm layered lighting, handle-less built-ins.
Front: gate and stone forecourt on the door axis with the tulsi at its
centre, charupadi seats flanking the steps, gable barge boards and brass
kalasham, laterite kitchen front with a deep teak window frame, carved main
door with studs, stone surround and nameplate, front lighting, hedges and
palms.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Schedules/KH-P1_Schedules_RevB.xlsx
+++ b/03_Schedules/KH-P1_Schedules_RevB.xlsx
@@ -1491,10 +1491,10 @@
         </is>
       </c>
       <c r="D30" s="4" t="n">
-        <v>71.2</v>
+        <v>74</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>22</v>
+        <v>21.6</v>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
@@ -4911,7 +4911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:B53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5056,7 +5056,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Twenty-ninth review: compound wall made as thin as practical: precast RCC post-and-panel (2 in panels in 4 in posts) set just inside the plot line, so the side strips stay walkable and the north run can be lifted and moved if more land is bought.</t>
+          <t>Thirty-first review (front facade): gate re-centred on the main door with a 6 ft stone forecourt and the tulsi thara on the axis (gate, tulsi, steps, door, hall, lamp niche in one line); charupadi seats with sloping backrests between the verandah pillars, flanking the steps; carved teak barge boards and a brass kalasham finial on the front gable; the kitchen front clad in exposed laterite with a deep projecting teak frame to its window; carved teak main door with brass studs, a stone surround and a nameplate niche; warm uplights at the pillars, a lantern by the door and gate-post lights; low hedges screening the sump and the two-wheeler bay; a pair of potted palms beside the steps.</t>
         </is>
       </c>
     </row>
@@ -5066,7 +5066,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Twenty-eighth review: TV lounge reworked: sofa brought forward to about 8 ft from the TV, a 3 ft walk behind it, and a built-in window seat (charupadi-style enclave) under the dining-bay window, so the sofa backs onto a quiet seating nook rather than the entrance and nobody walks in front of the TV.</t>
+          <t>Thirtieth review (proportion clean-up): windows standardised to three sizes (6 ft rooms, 3 ft small, 2 ft baths) with every head at 7 ft and three sill levels (3 ft rooms, 3'-6" over counters, 5 ft baths); sunshades only on the sunny south, east and west walls (the eaves shade the north); floors cut to three families plus the verandah (red oxide in all public rooms and the pooja, vitrified in bedrooms, anti-skid ceramic in kitchen, baths and wet area, granite on the verandah); services hidden (pipes in chases, outdoor units grouped behind jali on the north wall), switchboards aligned, warm layered lighting, handle-less built-in fronts.</t>
         </is>
       </c>
     </row>
@@ -5076,7 +5076,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Twenty-seventh review: TV lounge moves to the open dining space under the ventilator: TV on the north face of the common-bath wall, sofa facing south with its back to the north window, so the main door is in side view, not behind (commanding position) and the TV no longer faces the main door; the dining bay becomes a reading / dining nook with a chair by the window.</t>
+          <t>Twenty-ninth review: compound wall made as thin as practical: precast RCC post-and-panel (2 in panels in 4 in posts) set just inside the plot line, so the side strips stay walkable and the north run can be lifted and moved if more land is bought.</t>
         </is>
       </c>
     </row>
@@ -5086,7 +5086,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Twenty-sixth review: built-in ideas borrowed and adapted (function, not style, in Kerala materials): recessed shower niches, mirror cabinets over basins, genkan-style shoe bench with hooks and a granite threshold band, vilakku madam lamp niche facing the main door, floating bedside shelves (walls too thin for recesses), drawers-first kitchen with a masala pull-out and utensil rail, dish-drying rack over the utility sink, ceiling clothes airer in the wet area.</t>
+          <t>Twenty-eighth review: TV lounge reworked: sofa brought forward to about 8 ft from the TV, a 3 ft walk behind it, and a built-in window seat (charupadi-style enclave) under the dining-bay window, so the sofa backs onto a quiet seating nook rather than the entrance and nobody walks in front of the TV.</t>
         </is>
       </c>
     </row>
@@ -5096,7 +5096,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Twenty-fifth review: main door moved 3'-4" south (y 17'-7" to 20'-7"), centred under the front gable and opening straight onto the 5 ft walk between the pooja and the diwan; shoe cupboard to its north on the east wall; window diwan back to 6 ft along the north window, out of the door's line; steps, middle verandah pillars and the swing realigned.</t>
+          <t>Twenty-seventh review: TV lounge moves to the open dining space under the ventilator: TV on the north face of the common-bath wall, sofa facing south with its back to the north window, so the main door is in side view, not behind (commanding position) and the TV no longer faces the main door; the dining bay becomes a reading / dining nook with a chair by the window.</t>
         </is>
       </c>
     </row>
@@ -5106,7 +5106,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Twenty-fourth review: planned on the 27 ft plot alone (north strip dropped for now): roof eaves cut from 2'-6" to 2'-0" so the north eave stays inside the plot line, septic tank moved under the two-wheeler bay in the front yard with a lined soak pit beside it, all drains rerouted along the south walkway to the front, rainwater to the sump with overflow to the road; north-strip trees and recharge pit removed.</t>
+          <t>Twenty-sixth review: built-in ideas borrowed and adapted (function, not style, in Kerala materials): recessed shower niches, mirror cabinets over basins, genkan-style shoe bench with hooks and a granite threshold band, vilakku madam lamp niche facing the main door, floating bedside shelves (walls too thin for recesses), drawers-first kitchen with a masala pull-out and utensil rail, dish-drying rack over the utility sink, ceiling clothes airer in the wet area.</t>
         </is>
       </c>
     </row>
@@ -5116,7 +5116,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Twenty-third review: the fridge moves out of the kitchen into the dining alcove beside the kitchen door, against the wet-area wall; the kitchen's north wall is now free.</t>
+          <t>Twenty-fifth review: main door moved 3'-4" south (y 17'-7" to 20'-7"), centred under the front gable and opening straight onto the 5 ft walk between the pooja and the diwan; shoe cupboard to its north on the east wall; window diwan back to 6 ft along the north window, out of the door's line; steps, middle verandah pillars and the swing realigned.</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Twenty-second review: the kitchen's tall pantry and the dining table and chairs are removed at the owner's request; the dining space under the ventilator stays open (the pendant light and points stay for a table later).</t>
+          <t>Twenty-fourth review: planned on the 27 ft plot alone (north strip dropped for now): roof eaves cut from 2'-6" to 2'-0" so the north eave stays inside the plot line, septic tank moved under the two-wheeler bay in the front yard with a lined soak pit beside it, all drains rerouted along the south walkway to the front, rainwater to the sump with overflow to the road; north-strip trees and recharge pit removed.</t>
         </is>
       </c>
     </row>
@@ -5136,7 +5136,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Twenty-first review: the open hall becomes three zones: family TV lounge in the dining bay (5'-6" sofa facing the TV), dining under the ventilator moved 9 in south (about 2 ft behind the chairs on both sides), and guest sitting by the main door with a 4'-6" window diwan (shortened after the walk-through showed a 1'-6" pinch at the shoe cupboard) and an armchair under the living's north window; a clear walk of about 4'-11" from the main door to the dining and kitchen, pooja front kept clear.</t>
+          <t>Twenty-third review: the fridge moves out of the kitchen into the dining alcove beside the kitchen door, against the wet-area wall; the kitchen's north wall is now free.</t>
         </is>
       </c>
     </row>
@@ -5146,7 +5146,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Twentieth review: Bedroom 2's bed moves to the east wall, head east, leaving an 8 x 14 ft open floor from the door to the bath and window; wardrobe to the west wall (sound buffer to the master), work table north of the bed, AC on the bath's outer wall; dresser dropped (mirror on the wardrobe).</t>
+          <t>Twenty-second review: the kitchen's tall pantry and the dining table and chairs are removed at the owner's request; the dining space under the ventilator stays open (the pendant light and points stay for a table later).</t>
         </is>
       </c>
     </row>
@@ -5156,7 +5156,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
+          <t>Twenty-first review: the open hall becomes three zones: family TV lounge in the dining bay (5'-6" sofa facing the TV), dining under the ventilator moved 9 in south (about 2 ft behind the chairs on both sides), and guest sitting by the main door with a 4'-6" window diwan (shortened after the walk-through showed a 1'-6" pinch at the shoe cupboard) and an armchair under the living's north window; a clear walk of about 4'-11" from the main door to the dining and kitchen, pooja front kept clear.</t>
         </is>
       </c>
     </row>
@@ -5166,7 +5166,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
+          <t>Twentieth review: Bedroom 2's bed moves to the east wall, head east, leaving an 8 x 14 ft open floor from the door to the bath and window; wardrobe to the west wall (sound buffer to the master), work table north of the bed, AC on the bath's outer wall; dresser dropped (mirror on the wardrobe).</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
+          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
         </is>
       </c>
     </row>
@@ -5186,7 +5186,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
+          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
+          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
         </is>
       </c>
     </row>
@@ -5206,7 +5206,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
+          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
         </is>
       </c>
     </row>
@@ -5216,7 +5216,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
+          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
         </is>
       </c>
     </row>
@@ -5226,7 +5226,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
+          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
         </is>
       </c>
     </row>
@@ -5236,7 +5236,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
+          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
         </is>
       </c>
     </row>
@@ -5246,7 +5246,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
+          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
         </is>
       </c>
     </row>
@@ -5256,7 +5256,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
+          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5266,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
+          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
         </is>
       </c>
     </row>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
+          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
         </is>
       </c>
     </row>
@@ -5286,7 +5286,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
+          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
         </is>
       </c>
     </row>
@@ -5296,7 +5296,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
+          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
         </is>
       </c>
     </row>
@@ -5306,7 +5306,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
+          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
         </is>
       </c>
     </row>
@@ -5316,7 +5316,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
+          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
         </is>
       </c>
     </row>
@@ -5326,7 +5326,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
+          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
         </is>
       </c>
     </row>
@@ -5336,7 +5336,7 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
+          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
         </is>
       </c>
     </row>
@@ -5346,7 +5346,7 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
+          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
+          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
         </is>
       </c>
     </row>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
+          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
         </is>
       </c>
     </row>
@@ -5376,7 +5376,7 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
+          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
+          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
         </is>
       </c>
     </row>
@@ -5396,7 +5396,7 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
+          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
         </is>
       </c>
     </row>
@@ -5416,7 +5416,7 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
         </is>
       </c>
     </row>
@@ -5425,6 +5425,26 @@
         <v>50</v>
       </c>
       <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
         <is>
           <t>Roof: Mangalore clay tiles on steel truss over insulated cement-fibre deck; all edge tiles mechanically fixed.</t>
         </is>
@@ -6809,7 +6829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6887,7 +6907,7 @@
         </is>
       </c>
       <c r="D2" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E2" s="9" t="n">
         <v>3</v>
@@ -6923,10 +6943,10 @@
         </is>
       </c>
       <c r="D3" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>7</v>
@@ -6945,24 +6965,24 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>W04</t>
+          <t>W17</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Basin and crockery nook</t>
+          <t>Pooja</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>East (to verandah)</t>
         </is>
       </c>
       <c r="D4" s="9" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>3.5</v>
+        <v>5.5</v>
       </c>
       <c r="F4" s="9" t="n">
         <v>7</v>
@@ -6973,7 +6993,7 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Timber jali + glazed shutters (over the serving counter)</t>
+          <t>High vent to the poomukham, jali + mesh (lamp smoke out)</t>
         </is>
       </c>
       <c r="I4" s="8" t="inlineStr"/>
@@ -6981,24 +7001,24 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>W17</t>
+          <t>W19</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Pooja</t>
+          <t>Common bath</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>East (to verandah)</t>
+          <t>South</t>
         </is>
       </c>
       <c r="D5" s="9" t="n">
-        <v>2.8</v>
+        <v>2</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>7</v>
@@ -7009,7 +7029,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>High vent to the poomukham, jali + mesh (lamp smoke out)</t>
+          <t>Frosted casement, top-hung vent</t>
         </is>
       </c>
       <c r="I5" s="8" t="inlineStr"/>
@@ -7017,12 +7037,12 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>W19</t>
+          <t>W05</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Common bath</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -7031,10 +7051,10 @@
         </is>
       </c>
       <c r="D6" s="9" t="n">
-        <v>2.2</v>
+        <v>3</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>5</v>
+        <v>3.5</v>
       </c>
       <c r="F6" s="9" t="n">
         <v>7</v>
@@ -7045,7 +7065,7 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Frosted casement, top-hung vent</t>
+          <t>Timber jali + glazed shutters</t>
         </is>
       </c>
       <c r="I6" s="8" t="inlineStr"/>
@@ -7053,7 +7073,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>W05</t>
+          <t>W07</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -7067,7 +7087,7 @@
         </is>
       </c>
       <c r="D7" s="9" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E7" s="9" t="n">
         <v>3.5</v>
@@ -7089,7 +7109,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>W07</t>
+          <t>W08</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -7099,11 +7119,11 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>East</t>
         </is>
       </c>
       <c r="D8" s="9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E8" s="9" t="n">
         <v>3.5</v>
@@ -7117,7 +7137,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Timber jali + glazed shutters</t>
+          <t>Timber jali + glazed shutters (3 ft, north end; hob wall kept solid)</t>
         </is>
       </c>
       <c r="I8" s="8" t="inlineStr"/>
@@ -7125,24 +7145,24 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>W08</t>
+          <t>W09</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Ensuite</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D9" s="9" t="n">
         <v>2</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>3.5</v>
+        <v>5</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>7</v>
@@ -7153,7 +7173,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Timber jali + glazed shutters (2 ft, north end; hob wall kept solid)</t>
+          <t>Frosted casement</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr"/>
@@ -7161,7 +7181,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>W09</t>
+          <t>W10</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -7171,11 +7191,11 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>West</t>
         </is>
       </c>
       <c r="D10" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E10" s="9" t="n">
         <v>5</v>
@@ -7189,7 +7209,7 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Frosted casement</t>
+          <t>High jali vent</t>
         </is>
       </c>
       <c r="I10" s="8" t="inlineStr"/>
@@ -7197,24 +7217,24 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>W10</t>
+          <t>W11</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Ensuite</t>
+          <t>Master bedroom</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D11" s="9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F11" s="9" t="n">
         <v>7</v>
@@ -7225,7 +7245,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>High jali vent</t>
+          <t>Teak casement, glazed</t>
         </is>
       </c>
       <c r="I11" s="8" t="inlineStr"/>
@@ -7233,12 +7253,12 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>W11</t>
+          <t>W12</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Master bedroom</t>
+          <t>Bedroom 2</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -7261,7 +7281,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Teak casement, glazed</t>
+          <t>Teak casement, glazed (6 ft)</t>
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr"/>
@@ -7269,12 +7289,12 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>W12</t>
+          <t>W13</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Bedroom 2</t>
+          <t>Bath 2</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -7283,10 +7303,10 @@
         </is>
       </c>
       <c r="D13" s="9" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>7</v>
@@ -7297,7 +7317,7 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Teak casement, glazed (6 ft)</t>
+          <t>Frosted casement, top-hung vent</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr"/>
@@ -7305,27 +7325,23 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>W13</t>
+          <t>W20</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Bath 2</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>North</t>
-        </is>
-      </c>
+          <t>Bedroom 2</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr"/>
       <c r="D14" s="9" t="n">
-        <v>2.2</v>
+        <v>4</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>5</v>
+        <v>7.5</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G14" s="9">
         <f>F14-E14</f>
@@ -7333,7 +7349,7 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Frosted casement, top-hung vent</t>
+          <t>High jali vent to the sitting area, above the bed head (cross-ventilation with W12 and W03)</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr"/>
@@ -7341,23 +7357,27 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>W20</t>
+          <t>W18</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Bedroom 2</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr"/>
+          <t>Dining bay</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
       <c r="D15" s="9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G15" s="9">
         <f>F15-E15</f>
@@ -7365,7 +7385,7 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>High jali vent to the sitting area, above the bed head (cross-ventilation with W12 and W03)</t>
+          <t>Teak casement, glazed (north light for the dining)</t>
         </is>
       </c>
       <c r="I15" s="8" t="inlineStr"/>
@@ -7373,12 +7393,12 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>W18</t>
+          <t>W14</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Dining bay</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -7401,7 +7421,7 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Teak casement, glazed (north light for the dining)</t>
+          <t>Teak casement, glazed (6 ft)</t>
         </is>
       </c>
       <c r="I16" s="8" t="inlineStr"/>
@@ -7409,27 +7429,27 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>W16</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Serving counter and hand-wash basin</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>South</t>
         </is>
       </c>
       <c r="D17" s="9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G17" s="9">
         <f>F17-E17</f>
@@ -7437,7 +7457,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Teak casement, tall, glazed</t>
+          <t>Timber jali + glazed shutters (6 ft, over the counter)</t>
         </is>
       </c>
       <c r="I17" s="8" t="inlineStr"/>
@@ -7445,35 +7465,26 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>W16</t>
+          <t>SK1</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Basin and crockery nook</t>
+          <t>Roof</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>South</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E18" s="9" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="F18" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="G18" s="9">
-        <f>F18-E18</f>
-        <v/>
-      </c>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr"/>
+      <c r="E18" s="9" t="inlineStr"/>
+      <c r="F18" s="9" t="inlineStr"/>
+      <c r="G18" s="9" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Timber jali + glazed shutters (over the serving counter)</t>
+          <t>Ventilator over dining, 5 x 5 ft, no glass: hipped tiled cap at 30 deg with 1'-6" overhang; 2 ft band of 45 deg louvres on all four sides; SS insect mesh behind; sealed inner shutters on a winding opener; 9 in upstand; lined shaft to the dining ceiling (see A-503)</t>
         </is>
       </c>
       <c r="I18" s="8" t="inlineStr"/>
@@ -7481,7 +7492,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>SK1</t>
+          <t>GV1-3</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -7500,37 +7511,10 @@
       <c r="G19" s="9" t="inlineStr"/>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Ventilator over dining, 5 x 5 ft, no glass: hipped tiled cap at 30 deg with 1'-6" overhang; 2 ft band of 45 deg louvres on all four sides; SS insect mesh behind; sealed inner shutters on a winding opener; 9 in upstand; lined shaft to the dining ceiling (see A-503)</t>
+          <t>Three glazed/jali vents in front gable (mukhappu), morning light into living</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>GV1-3</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Roof</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Up</t>
-        </is>
-      </c>
-      <c r="D20" s="9" t="inlineStr"/>
-      <c r="E20" s="9" t="inlineStr"/>
-      <c r="F20" s="9" t="inlineStr"/>
-      <c r="G20" s="9" t="inlineStr"/>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>Three glazed/jali vents in front gable (mukhappu), morning light into living</t>
-        </is>
-      </c>
-      <c r="I20" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7543,7 +7527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -9278,7 +9262,7 @@
         </is>
       </c>
       <c r="E40" s="4" t="n">
-        <v>2.2</v>
+        <v>1.7</v>
       </c>
       <c r="F40" s="4" t="n">
         <v>0.15</v>
@@ -9794,7 +9778,7 @@
         </is>
       </c>
       <c r="E52" s="4" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
       <c r="F52" s="4" t="n">
         <v>1.5</v>
@@ -9828,26 +9812,26 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Arugu seat (built-in, south end)</t>
+          <t>Charupadi: built-in teak seat with a sloping backrest between the pillars, south of the steps</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E53" s="4" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="G53" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>Laterite base, teak top</t>
+          <t>Laterite base, teak seat and backrest</t>
         </is>
       </c>
       <c r="I53" s="10" t="n"/>
@@ -9859,28 +9843,71 @@
       <c r="L53" s="8" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="6" t="inlineStr"/>
-      <c r="B54" s="6" t="inlineStr"/>
-      <c r="C54" s="6" t="inlineStr">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>F69</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Poomukham (verandah)</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Charupadi: built-in teak seat with a sloping backrest between the pillars, north of the steps</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Loose furniture</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F54" s="4" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G54" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>Laterite base, teak seat and backrest</t>
+        </is>
+      </c>
+      <c r="I54" s="10" t="n"/>
+      <c r="J54" s="11">
+        <f>G54*I54</f>
+        <v/>
+      </c>
+      <c r="K54" s="8" t="inlineStr"/>
+      <c r="L54" s="8" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr"/>
+      <c r="B55" s="6" t="inlineStr"/>
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D54" s="6" t="inlineStr"/>
-      <c r="E54" s="6" t="inlineStr"/>
-      <c r="F54" s="6" t="inlineStr"/>
-      <c r="G54" s="6">
-        <f>SUM(G2:G53)</f>
+      <c r="D55" s="6" t="inlineStr"/>
+      <c r="E55" s="6" t="inlineStr"/>
+      <c r="F55" s="6" t="inlineStr"/>
+      <c r="G55" s="6">
+        <f>SUM(G2:G54)</f>
         <v/>
       </c>
-      <c r="H54" s="6" t="inlineStr"/>
-      <c r="I54" s="12" t="inlineStr"/>
-      <c r="J54" s="12">
-        <f>SUM(J2:J53)</f>
+      <c r="H55" s="6" t="inlineStr"/>
+      <c r="I55" s="12" t="inlineStr"/>
+      <c r="J55" s="12">
+        <f>SUM(J2:J54)</f>
         <v/>
       </c>
-      <c r="K54" s="6" t="inlineStr"/>
-      <c r="L54" s="6" t="inlineStr"/>
+      <c r="K55" s="6" t="inlineStr"/>
+      <c r="L55" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10948,7 +10975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11009,7 +11036,7 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>22.94</v>
+        <v>23.23</v>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
@@ -11129,7 +11156,7 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>286.5</v>
+        <v>287.9</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
@@ -11159,7 +11186,7 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>146.6</v>
+        <v>148</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
@@ -11219,7 +11246,7 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>10.9</v>
+        <v>24.8</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
@@ -11249,7 +11276,7 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>38.7</v>
+        <v>39.8</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
@@ -11275,11 +11302,11 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Rough Cuddapah / Kota, falls</t>
+          <t>Flamed granite</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>2.4</v>
+        <v>6.1</v>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
@@ -11305,20 +11332,20 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Anti-skid matt vitrified</t>
+          <t>Flush skirting, 4 in</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>11.5</v>
+        <v>111.7</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>sq m</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Clear room areas; add 5-8% wastage</t>
+          <t>Room perimeters (dry rooms), doors not deducted</t>
         </is>
       </c>
       <c r="F12" s="10" t="n"/>
@@ -11330,16 +11357,16 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Floors</t>
+          <t>Wet rooms</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Marble / teak (pooja)</t>
+          <t>Wall tiles to 7 ft, Ensuite</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1.1</v>
+        <v>15.6</v>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
@@ -11348,7 +11375,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Clear room areas; add 5-8% wastage</t>
+          <t>Full height in the shower adds ~2 sq m</t>
         </is>
       </c>
       <c r="F13" s="10" t="n"/>
@@ -11360,16 +11387,16 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Floors</t>
+          <t>Wet rooms</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Flamed granite</t>
+          <t>Waterproofing, Ensuite</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>6.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
@@ -11378,7 +11405,7 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Clear room areas; add 5-8% wastage</t>
+          <t>Floor + 12 in upturn + shower walls to 7 ft</t>
         </is>
       </c>
       <c r="F14" s="10" t="n"/>
@@ -11390,25 +11417,25 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Floors</t>
+          <t>Wet rooms</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Flush skirting, 4 in</t>
+          <t>Wall tiles to 7 ft, Common bath</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>111.7</v>
+        <v>13.2</v>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>sq m</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Room perimeters (dry rooms), doors not deducted</t>
+          <t>Full height in the shower adds ~2 sq m</t>
         </is>
       </c>
       <c r="F15" s="10" t="n"/>
@@ -11425,11 +11452,11 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Wall tiles to 7 ft, Ensuite</t>
+          <t>Waterproofing, Common bath</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>15.6</v>
+        <v>8.5</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
@@ -11438,7 +11465,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Full height in the shower adds ~2 sq m</t>
+          <t>Floor + 12 in upturn + shower walls to 7 ft</t>
         </is>
       </c>
       <c r="F16" s="10" t="n"/>
@@ -11455,11 +11482,11 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Waterproofing, Ensuite</t>
+          <t>Wall tiles to 7 ft, Bath 2 (attached to Bedroom 2)</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>15.1</v>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
@@ -11468,7 +11495,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Floor + 12 in upturn + shower walls to 7 ft</t>
+          <t>Full height in the shower adds ~2 sq m</t>
         </is>
       </c>
       <c r="F17" s="10" t="n"/>
@@ -11485,11 +11512,11 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Wall tiles to 7 ft, Common bath</t>
+          <t>Waterproofing, Bath 2 (attached to Bedroom 2)</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>13.2</v>
+        <v>9.6</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
@@ -11498,7 +11525,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Full height in the shower adds ~2 sq m</t>
+          <t>Floor + 12 in upturn + shower walls to 7 ft</t>
         </is>
       </c>
       <c r="F18" s="10" t="n"/>
@@ -11510,25 +11537,25 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Wet rooms</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Waterproofing, Common bath</t>
+          <t>Granite counter, 2 ft deep</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>8.5</v>
+        <v>5.4</v>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>sq m</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Floor + 12 in upturn + shower walls to 7 ft</t>
+          <t>South and east runs (F34, F35)</t>
         </is>
       </c>
       <c r="F19" s="10" t="n"/>
@@ -11540,16 +11567,16 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Wet rooms</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Wall tiles to 7 ft, Bath 2 (attached to Bedroom 2)</t>
+          <t>Dado between counter and wall cabinets</t>
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>15.1</v>
+        <v>3.3</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
@@ -11558,7 +11585,7 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Full height in the shower adds ~2 sq m</t>
+          <t>2 ft high</t>
         </is>
       </c>
       <c r="F20" s="10" t="n"/>
@@ -11570,16 +11597,16 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Wet rooms</t>
+          <t>Roof</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Waterproofing, Bath 2 (attached to Bedroom 2)</t>
+          <t>Sloped roof area (tiles, deck, insulation, membrane)</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>9.6</v>
+        <v>184.1</v>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
@@ -11588,7 +11615,7 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Floor + 12 in upturn + shower walls to 7 ft</t>
+          <t>Hip outline / cos 30 deg; add ~8% for gable and laps</t>
         </is>
       </c>
       <c r="F21" s="10" t="n"/>
@@ -11600,16 +11627,16 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Roof</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Granite counter, 2 ft deep</t>
+          <t>Gutters</t>
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>5.4</v>
+        <v>40.2</v>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
@@ -11618,7 +11645,7 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>South and east runs (F34, F35)</t>
+          <t>Both long eaves</t>
         </is>
       </c>
       <c r="F22" s="10" t="n"/>
@@ -11630,25 +11657,25 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Roof</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Dado between counter and wall cabinets</t>
+          <t>Downpipes, 100 mm</t>
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>3.3</v>
+        <v>8</v>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>sq m</t>
+          <t>no.</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>2 ft high</t>
+          <t>About 12 ft each</t>
         </is>
       </c>
       <c r="F23" s="10" t="n"/>
@@ -11665,20 +11692,20 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Sloped roof area (tiles, deck, insulation, membrane)</t>
+          <t>Ridge and hip tiles</t>
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>184.1</v>
+        <v>34.6</v>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>sq m</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Hip outline / cos 30 deg; add ~8% for gable and laps</t>
+          <t>Approximate</t>
         </is>
       </c>
       <c r="F24" s="10" t="n"/>
@@ -11690,16 +11717,16 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Roof</t>
+          <t>Site</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Gutters</t>
+          <t>Compound wall, precast RCC post and panel, 5 ft high</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>40.2</v>
+        <v>60</v>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
@@ -11708,7 +11735,7 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Both long eaves</t>
+          <t>Plot perimeter less the gate</t>
         </is>
       </c>
       <c r="F25" s="10" t="n"/>
@@ -11720,25 +11747,25 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Roof</t>
+          <t>Site</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Downpipes, 100 mm</t>
+          <t>Plinth protection apron, 3 ft wide</t>
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>8</v>
+        <v>51</v>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>no.</t>
+          <t>sq m</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>About 12 ft each</t>
+          <t>PCC with slope away</t>
         </is>
       </c>
       <c r="F26" s="10" t="n"/>
@@ -11750,25 +11777,25 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Roof</t>
+          <t>Openings</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Ridge and hip tiles</t>
+          <t>Doors</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>34.6</v>
+        <v>9</v>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>no.</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Approximate</t>
+          <t>See Doors tab</t>
         </is>
       </c>
       <c r="F27" s="10" t="n"/>
@@ -11780,25 +11807,25 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Site</t>
+          <t>Openings</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Compound wall, precast RCC post and panel, 5 ft high</t>
+          <t>Windows and vents</t>
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>no.</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Plot perimeter less the gate</t>
+          <t>See Windows tab</t>
         </is>
       </c>
       <c r="F28" s="10" t="n"/>
@@ -11810,27 +11837,23 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Site</t>
+          <t>Openings</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Plinth protection apron, 3 ft wide</t>
+          <t>Window area (for mesh and grills)</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>51</v>
+        <v>21.4</v>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
           <t>sq m</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>PCC with slope away</t>
-        </is>
-      </c>
+      <c r="E29" s="4" t="inlineStr"/>
       <c r="F29" s="10" t="n"/>
       <c r="G29" s="11">
         <f>IF(F29="","",C29*F29)</f>
@@ -11838,104 +11861,18 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>Openings</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>Doors</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>no.</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>See Doors tab</t>
-        </is>
-      </c>
-      <c r="F30" s="10" t="n"/>
-      <c r="G30" s="11">
-        <f>IF(F30="","",C30*F30)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Openings</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Windows and vents</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>no.</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>See Windows tab</t>
-        </is>
-      </c>
-      <c r="F31" s="10" t="n"/>
-      <c r="G31" s="11">
-        <f>IF(F31="","",C31*F31)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>Openings</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Window area (for mesh and grills)</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="n">
-        <v>22.8</v>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>sq m</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr"/>
-      <c r="F32" s="10" t="n"/>
-      <c r="G32" s="11">
-        <f>IF(F32="","",C32*F32)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr"/>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="A30" s="6" t="inlineStr"/>
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>Total of priced items</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr"/>
-      <c r="D33" s="6" t="inlineStr"/>
-      <c r="E33" s="6" t="inlineStr"/>
-      <c r="F33" s="12" t="inlineStr"/>
-      <c r="G33" s="12">
-        <f>SUM(G2:G32)</f>
+      <c r="C30" s="6" t="inlineStr"/>
+      <c r="D30" s="6" t="inlineStr"/>
+      <c r="E30" s="6" t="inlineStr"/>
+      <c r="F30" s="12" t="inlineStr"/>
+      <c r="G30" s="12">
+        <f>SUM(G2:G29)</f>
         <v/>
       </c>
     </row>
@@ -11951,7 +11888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G114"/>
+  <dimension ref="A1:G117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -13311,64 +13248,60 @@
         </is>
       </c>
       <c r="E43" s="4" t="n">
-        <v>35.15</v>
+        <v>34.5</v>
       </c>
       <c r="F43" s="4" t="n">
         <v>3.4</v>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>serving counter</t>
+          <t>serving counter, on the pier between the windows</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>6 A socket at counter</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area (open)</t>
+          <t>Common bath</t>
         </is>
       </c>
       <c r="E44" s="4" t="n">
-        <v>38.1</v>
+        <v>44.7</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="G44" s="4" t="inlineStr">
-        <is>
-          <t>serving counter</t>
-        </is>
-      </c>
+        <v>6.2</v>
+      </c>
+      <c r="G44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>EF</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Exhaust fan</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>7'-0"</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -13377,27 +13310,31 @@
         </is>
       </c>
       <c r="E45" s="4" t="n">
-        <v>44.7</v>
+        <v>46.9</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="G45" s="4" t="inlineStr"/>
+        <v>3.4</v>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>out through the south wall</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>EF</t>
+          <t>G</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Exhaust fan</t>
+          <t>Geyser (16 A)</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>7'-0"</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -13406,31 +13343,31 @@
         </is>
       </c>
       <c r="E46" s="4" t="n">
-        <v>46.9</v>
+        <v>41.8</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>3.4</v>
+        <v>4.5</v>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>out through the south wall</t>
+          <t>over shower, west wall (clear of the window)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Geyser (16 A)</t>
+          <t>6 A socket at counter</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -13439,97 +13376,97 @@
         </is>
       </c>
       <c r="E47" s="4" t="n">
-        <v>41.8</v>
+        <v>47.6</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>4.5</v>
+        <v>6</v>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>over shower, west wall (clear of the window)</t>
+          <t>by basin</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>6 A socket at counter</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Common bath</t>
+          <t>Sitting and serving area (open)</t>
         </is>
       </c>
       <c r="E48" s="4" t="n">
-        <v>47.6</v>
+        <v>41.1</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t>by basin</t>
+          <t>common bath switches outside the door</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>Ceiling fan point</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area (open)</t>
+          <t>Bedroom 2</t>
         </is>
       </c>
       <c r="E49" s="4" t="n">
-        <v>41.1</v>
+        <v>34.6</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>16.5</v>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>common bath switches outside the door</t>
+          <t>over the bed</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>WL</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Ceiling fan point</t>
+          <t>Wall light / mirror light</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -13538,31 +13475,31 @@
         </is>
       </c>
       <c r="E50" s="4" t="n">
-        <v>34.6</v>
+        <v>37.6</v>
       </c>
       <c r="F50" s="4" t="n">
         <v>16.5</v>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>over the bed</t>
+          <t>reading light over the bed head</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -13571,16 +13508,12 @@
         </is>
       </c>
       <c r="E51" s="4" t="n">
-        <v>37.6</v>
+        <v>24</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>16.5</v>
-      </c>
-      <c r="G51" s="4" t="inlineStr">
-        <is>
-          <t>reading light over the bed head</t>
-        </is>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="G51" s="4" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -13604,7 +13537,7 @@
         </is>
       </c>
       <c r="E52" s="4" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="F52" s="4" t="n">
         <v>14</v>
@@ -13633,27 +13566,27 @@
         </is>
       </c>
       <c r="E53" s="4" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>14</v>
+        <v>20.5</v>
       </c>
       <c r="G53" s="4" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -13662,12 +13595,16 @@
         </is>
       </c>
       <c r="E54" s="4" t="n">
-        <v>33</v>
+        <v>36.8</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="G54" s="4" t="inlineStr"/>
+        <v>11.4</v>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>at the door (latch side, on the corner return), 2-way</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -13691,31 +13628,31 @@
         </is>
       </c>
       <c r="E55" s="4" t="n">
-        <v>36.8</v>
+        <v>37.6</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>11.4</v>
+        <v>13</v>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>at the door (latch side, on the corner return), 2-way</t>
+          <t>bedside, 2-way</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -13727,11 +13664,11 @@
         <v>37.6</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>13</v>
+        <v>13.5</v>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>bedside, 2-way</t>
+          <t>bedside</t>
         </is>
       </c>
     </row>
@@ -13760,7 +13697,7 @@
         <v>37.6</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>13.5</v>
+        <v>19.5</v>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
@@ -13771,17 +13708,17 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -13793,28 +13730,28 @@
         <v>37.6</v>
       </c>
       <c r="F58" s="4" t="n">
-        <v>19.5</v>
+        <v>19.9</v>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>bedside</t>
+          <t>bedside, 2-way</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -13826,23 +13763,23 @@
         <v>37.6</v>
       </c>
       <c r="F59" s="4" t="n">
-        <v>19.9</v>
+        <v>20.8</v>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>bedside, 2-way</t>
+          <t>work table</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Inverter (UPS) socket</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -13859,23 +13796,23 @@
         <v>37.6</v>
       </c>
       <c r="F60" s="4" t="n">
-        <v>20.8</v>
+        <v>21.6</v>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>work table</t>
+          <t>work table, monitor</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Inverter (UPS) socket</t>
+          <t>Data point (Cat6)</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -13892,23 +13829,23 @@
         <v>37.6</v>
       </c>
       <c r="F61" s="4" t="n">
-        <v>21.6</v>
+        <v>22.4</v>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>work table, monitor</t>
+          <t>work table</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Data point (Cat6)</t>
+          <t>Inverter (UPS) socket</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -13925,7 +13862,7 @@
         <v>37.6</v>
       </c>
       <c r="F62" s="4" t="n">
-        <v>22.4</v>
+        <v>23.2</v>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
@@ -13936,17 +13873,17 @@
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Inverter (UPS) socket</t>
+          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>7'-6"</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -13955,125 +13892,121 @@
         </is>
       </c>
       <c r="E63" s="4" t="n">
-        <v>37.6</v>
+        <v>28.4</v>
       </c>
       <c r="F63" s="4" t="n">
-        <v>23.2</v>
+        <v>24</v>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>work table</t>
+          <t>high on the bath's east wall near the north corner, throws east toward the bed foot</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>WL</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
+          <t>Wall light / mirror light</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>7'-6"</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>Bedroom 2</t>
+          <t>Sitting and serving area (open)</t>
         </is>
       </c>
       <c r="E64" s="4" t="n">
-        <v>28.4</v>
+        <v>41.1</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>24</v>
+        <v>4.4</v>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>high on the bath's east wall near the north corner, throws east toward the bed foot</t>
+          <t>over basin, on the common bath wall</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>ODU</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>AC outdoor unit bracket</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>7'-0" outside</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area (open)</t>
+          <t>Bedroom 2</t>
         </is>
       </c>
       <c r="E65" s="4" t="n">
-        <v>41.1</v>
+        <v>29.5</v>
       </c>
       <c r="F65" s="4" t="n">
-        <v>4.4</v>
+        <v>25.6</v>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>over basin, on the common bath wall</t>
+          <t>north wall, shaded</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>ODU</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>AC outdoor unit bracket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>7'-0" outside</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>Bedroom 2</t>
+          <t>Dining bay (north window)</t>
         </is>
       </c>
       <c r="E66" s="4" t="n">
-        <v>29.5</v>
+        <v>41.5</v>
       </c>
       <c r="F66" s="4" t="n">
-        <v>25.6</v>
-      </c>
-      <c r="G66" s="4" t="inlineStr">
-        <is>
-          <t>north wall, shaded</t>
-        </is>
-      </c>
+        <v>21.5</v>
+      </c>
+      <c r="G66" s="4" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Ceiling fan point</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -14087,27 +14020,31 @@
         </is>
       </c>
       <c r="E67" s="4" t="n">
-        <v>41.5</v>
+        <v>45</v>
       </c>
       <c r="F67" s="4" t="n">
         <v>21.5</v>
       </c>
-      <c r="G67" s="4" t="inlineStr"/>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>long downrod, over the seating</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Ceiling fan point</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -14116,60 +14053,60 @@
         </is>
       </c>
       <c r="E68" s="4" t="n">
-        <v>45</v>
+        <v>48.6</v>
       </c>
       <c r="F68" s="4" t="n">
-        <v>21.5</v>
-      </c>
-      <c r="G68" s="4" t="inlineStr">
-        <is>
-          <t>long downrod, over the seating</t>
-        </is>
-      </c>
+        <v>24.6</v>
+      </c>
+      <c r="G68" s="4" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>TV</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>TV + data point</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>Dining bay (north window)</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E69" s="4" t="n">
-        <v>48.6</v>
+        <v>44.8</v>
       </c>
       <c r="F69" s="4" t="n">
-        <v>24.6</v>
-      </c>
-      <c r="G69" s="4" t="inlineStr"/>
+        <v>9.4</v>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>TV wall (common-bath wall, dry face): 2 sockets + data + HDMI conduit to the unit</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>TV</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>TV + data point</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -14178,64 +14115,64 @@
         </is>
       </c>
       <c r="E70" s="4" t="n">
-        <v>44.8</v>
+        <v>43.2</v>
       </c>
       <c r="F70" s="4" t="n">
         <v>9.4</v>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>TV wall (common-bath wall, dry face): 2 sockets + data + HDMI conduit to the unit</t>
+          <t>TV unit</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>7'-6"</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Dining bay (north window)</t>
         </is>
       </c>
       <c r="E71" s="4" t="n">
-        <v>43.2</v>
+        <v>38.4</v>
       </c>
       <c r="F71" s="4" t="n">
-        <v>9.4</v>
+        <v>20</v>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>TV unit</t>
+          <t>Bedroom 2's east wall, throws east across the hall and the TV seating</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>ODU</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>AC indoor unit (16 A socket, sleeve, drain)</t>
+          <t>AC outdoor unit bracket</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>7'-6"</t>
+          <t>7'-0" outside</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
@@ -14244,64 +14181,64 @@
         </is>
       </c>
       <c r="E72" s="4" t="n">
-        <v>38.4</v>
+        <v>40</v>
       </c>
       <c r="F72" s="4" t="n">
-        <v>20</v>
+        <v>25.6</v>
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>Bedroom 2's east wall, throws east across the hall and the TV seating</t>
+          <t>north wall, shaded</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>ODU</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>AC outdoor unit bracket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>7'-0" outside</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Dining bay (north window)</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E73" s="4" t="n">
-        <v>40</v>
+        <v>44.5</v>
       </c>
       <c r="F73" s="4" t="n">
-        <v>25.6</v>
+        <v>15</v>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>north wall, shaded</t>
+          <t>pendant</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>WL</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Wall light / mirror light</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
@@ -14310,31 +14247,31 @@
         </is>
       </c>
       <c r="E74" s="4" t="n">
-        <v>44.5</v>
+        <v>38.4</v>
       </c>
       <c r="F74" s="4" t="n">
-        <v>15</v>
+        <v>17.3</v>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>pendant</t>
+          <t>inside the lamp niche</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -14346,28 +14283,24 @@
         <v>38.4</v>
       </c>
       <c r="F75" s="4" t="n">
-        <v>17.3</v>
-      </c>
-      <c r="G75" s="4" t="inlineStr">
-        <is>
-          <t>inside the lamp niche</t>
-        </is>
-      </c>
+        <v>16.2</v>
+      </c>
+      <c r="G75" s="4" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -14379,57 +14312,57 @@
         <v>38.4</v>
       </c>
       <c r="F76" s="4" t="n">
-        <v>16.2</v>
-      </c>
-      <c r="G76" s="4" t="inlineStr"/>
+        <v>13.7</v>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>dining and bay, at the passage</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Sitting and serving area (open)</t>
         </is>
       </c>
       <c r="E77" s="4" t="n">
-        <v>38.4</v>
+        <v>30.5</v>
       </c>
       <c r="F77" s="4" t="n">
-        <v>13.7</v>
-      </c>
-      <c r="G77" s="4" t="inlineStr">
-        <is>
-          <t>dining and bay, at the passage</t>
-        </is>
-      </c>
+        <v>6.75</v>
+      </c>
+      <c r="G77" s="4" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -14438,27 +14371,27 @@
         </is>
       </c>
       <c r="E78" s="4" t="n">
-        <v>30.5</v>
+        <v>21.4</v>
       </c>
       <c r="F78" s="4" t="n">
-        <v>6.75</v>
+        <v>6</v>
       </c>
       <c r="G78" s="4" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>INV</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>Inverter + battery</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>floor</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -14467,60 +14400,64 @@
         </is>
       </c>
       <c r="E79" s="4" t="n">
-        <v>21.4</v>
+        <v>22</v>
       </c>
       <c r="F79" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="G79" s="4" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>lithium inverter in a ventilated cabinet under the bench</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>INV</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Inverter + battery</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>floor</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>Sitting and serving area (open)</t>
+          <t>Wet area (open to the walkway)</t>
         </is>
       </c>
       <c r="E80" s="4" t="n">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="F80" s="4" t="n">
-        <v>5</v>
+        <v>5.5</v>
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>lithium inverter in a ventilated cabinet under the bench</t>
+          <t>weatherproof</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>16 A power socket</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>varies</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
@@ -14529,31 +14466,31 @@
         </is>
       </c>
       <c r="E81" s="4" t="n">
-        <v>50</v>
+        <v>48.5</v>
       </c>
       <c r="F81" s="4" t="n">
-        <v>5.5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>weatherproof</t>
+          <t>washing machine</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>16 A power socket</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -14562,64 +14499,60 @@
         </is>
       </c>
       <c r="E82" s="4" t="n">
-        <v>48.5</v>
+        <v>52.6</v>
       </c>
       <c r="F82" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>6</v>
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>washing machine</t>
+          <t>utility, weatherproof</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>Wet area (open to the walkway)</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="E83" s="4" t="n">
-        <v>52.6</v>
+        <v>62</v>
       </c>
       <c r="F83" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="G83" s="4" t="inlineStr">
-        <is>
-          <t>utility, weatherproof</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="G83" s="4" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>WL</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Wall light / mirror light</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>6'-6"</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -14628,12 +14561,16 @@
         </is>
       </c>
       <c r="E84" s="4" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F84" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="G84" s="4" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>under-cabinet</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -14657,10 +14594,10 @@
         </is>
       </c>
       <c r="E85" s="4" t="n">
-        <v>61</v>
+        <v>66.5</v>
       </c>
       <c r="F85" s="4" t="n">
-        <v>3.5</v>
+        <v>9.6</v>
       </c>
       <c r="G85" s="4" t="inlineStr">
         <is>
@@ -14671,17 +14608,17 @@
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Wall light / mirror light</t>
+          <t>Kitchen chimney point (16 A)</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>6'-6"</t>
+          <t>7'-0"</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -14690,31 +14627,31 @@
         </is>
       </c>
       <c r="E86" s="4" t="n">
-        <v>66.5</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="F86" s="4" t="n">
-        <v>9.6</v>
+        <v>7.5</v>
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
-          <t>under-cabinet</t>
+          <t>3 ft chimney on solid wall, duct out through the east wall</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Kitchen chimney point (16 A)</t>
+          <t>6 A socket at counter</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>7'-0"</t>
+          <t>3'-6"</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -14723,16 +14660,12 @@
         </is>
       </c>
       <c r="E87" s="4" t="n">
-        <v>66.59999999999999</v>
+        <v>54</v>
       </c>
       <c r="F87" s="4" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="G87" s="4" t="inlineStr">
-        <is>
-          <t>3 ft chimney on solid wall, duct out through the east wall</t>
-        </is>
-      </c>
+        <v>3.5</v>
+      </c>
+      <c r="G87" s="4" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
@@ -14756,12 +14689,16 @@
         </is>
       </c>
       <c r="E88" s="4" t="n">
-        <v>54.5</v>
+        <v>57.8</v>
       </c>
       <c r="F88" s="4" t="n">
         <v>3.5</v>
       </c>
-      <c r="G88" s="4" t="inlineStr"/>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>microwave / OTG</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -14785,14 +14722,14 @@
         </is>
       </c>
       <c r="E89" s="4" t="n">
-        <v>58</v>
+        <v>65.3</v>
       </c>
       <c r="F89" s="4" t="n">
         <v>3.5</v>
       </c>
       <c r="G89" s="4" t="inlineStr">
         <is>
-          <t>microwave / OTG</t>
+          <t>mixer</t>
         </is>
       </c>
     </row>
@@ -14818,16 +14755,12 @@
         </is>
       </c>
       <c r="E90" s="4" t="n">
-        <v>63.5</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="F90" s="4" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="G90" s="4" t="inlineStr">
-        <is>
-          <t>mixer</t>
-        </is>
-      </c>
+        <v>5.6</v>
+      </c>
+      <c r="G90" s="4" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
@@ -14854,7 +14787,7 @@
         <v>66.59999999999999</v>
       </c>
       <c r="F91" s="4" t="n">
-        <v>5.6</v>
+        <v>9.6</v>
       </c>
       <c r="G91" s="4" t="inlineStr"/>
     </row>
@@ -14880,27 +14813,31 @@
         </is>
       </c>
       <c r="E92" s="4" t="n">
-        <v>66.59999999999999</v>
+        <v>58.2</v>
       </c>
       <c r="F92" s="4" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="G92" s="4" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
+          <t>RO purifier, by sink</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>6 A socket at counter</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>3'-6"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
@@ -14909,59 +14846,59 @@
         </is>
       </c>
       <c r="E93" s="4" t="n">
-        <v>59.3</v>
+        <v>53.4</v>
       </c>
       <c r="F93" s="4" t="n">
-        <v>3.5</v>
+        <v>9</v>
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>RO purifier, by sink</t>
+          <t>beside the entry, latch side</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>Ceiling fan point</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="E94" s="4" t="n">
-        <v>53.4</v>
+        <v>55</v>
       </c>
       <c r="F94" s="4" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="G94" s="4" t="inlineStr">
         <is>
-          <t>beside the entry, latch side</t>
+          <t>long downrod</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>Ceiling fan point</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
@@ -14975,14 +14912,14 @@
         </is>
       </c>
       <c r="E95" s="4" t="n">
-        <v>55</v>
+        <v>54.9</v>
       </c>
       <c r="F95" s="4" t="n">
-        <v>19</v>
+        <v>22.8</v>
       </c>
       <c r="G95" s="4" t="inlineStr">
         <is>
-          <t>long downrod</t>
+          <t>over the diwan</t>
         </is>
       </c>
     </row>
@@ -15008,45 +14945,45 @@
         </is>
       </c>
       <c r="E96" s="4" t="n">
-        <v>54.9</v>
+        <v>55</v>
       </c>
       <c r="F96" s="4" t="n">
-        <v>22.8</v>
-      </c>
-      <c r="G96" s="4" t="inlineStr">
-        <is>
-          <t>over the diwan</t>
-        </is>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="G96" s="4" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E97" s="4" t="n">
-        <v>55</v>
+        <v>47.9</v>
       </c>
       <c r="F97" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="G97" s="4" t="inlineStr"/>
+        <v>18</v>
+      </c>
+      <c r="G97" s="4" t="inlineStr">
+        <is>
+          <t>floor socket, sofa end</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
@@ -15066,35 +15003,35 @@
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="E98" s="4" t="n">
-        <v>47.9</v>
+        <v>51</v>
       </c>
       <c r="F98" s="4" t="n">
-        <v>18</v>
+        <v>20.3</v>
       </c>
       <c r="G98" s="4" t="inlineStr">
         <is>
-          <t>floor socket, sofa end</t>
+          <t>floor socket, armchair and diwan (lamp, charger)</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
@@ -15103,64 +15040,64 @@
         </is>
       </c>
       <c r="E99" s="4" t="n">
-        <v>51</v>
+        <v>60.6</v>
       </c>
       <c r="F99" s="4" t="n">
-        <v>20.3</v>
+        <v>21</v>
       </c>
       <c r="G99" s="4" t="inlineStr">
         <is>
-          <t>floor socket, armchair and diwan (lamp, charger)</t>
+          <t>main switch at door</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>Distribution board</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>5'-0" to top</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Dining</t>
         </is>
       </c>
       <c r="E100" s="4" t="n">
-        <v>60.6</v>
+        <v>38.4</v>
       </c>
       <c r="F100" s="4" t="n">
-        <v>21</v>
+        <v>12.6</v>
       </c>
       <c r="G100" s="4" t="inlineStr">
         <is>
-          <t>main switch at door</t>
+          <t>dining face of Bedroom 2's east wall, by the passage; dry wall away from the pooja and wet area</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>Distribution board</t>
+          <t>16 A power socket</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>5'-0" to top</t>
+          <t>varies</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
@@ -15169,31 +15106,31 @@
         </is>
       </c>
       <c r="E101" s="4" t="n">
-        <v>38.4</v>
+        <v>49.55</v>
       </c>
       <c r="F101" s="4" t="n">
-        <v>12.6</v>
+        <v>9.4</v>
       </c>
       <c r="G101" s="4" t="inlineStr">
         <is>
-          <t>dining face of Bedroom 2's east wall, by the passage; dry wall away from the pooja and wet area</t>
+          <t>refrigerator, behind the fridge (dining alcove)</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>16 A power socket</t>
+          <t>Inverter (UPS) socket</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>varies</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
@@ -15202,49 +15139,45 @@
         </is>
       </c>
       <c r="E102" s="4" t="n">
-        <v>49.55</v>
+        <v>38.4</v>
       </c>
       <c r="F102" s="4" t="n">
-        <v>9.4</v>
+        <v>14.6</v>
       </c>
       <c r="G102" s="4" t="inlineStr">
         <is>
-          <t>refrigerator, behind the fridge (dining alcove)</t>
+          <t>router (central)</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>Inverter (UPS) socket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Poomukham (verandah)</t>
         </is>
       </c>
       <c r="E103" s="4" t="n">
-        <v>38.4</v>
+        <v>64</v>
       </c>
       <c r="F103" s="4" t="n">
-        <v>14.6</v>
-      </c>
-      <c r="G103" s="4" t="inlineStr">
-        <is>
-          <t>router (central)</t>
-        </is>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="G103" s="4" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
@@ -15271,24 +15204,24 @@
         <v>64</v>
       </c>
       <c r="F104" s="4" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="G104" s="4" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>BELL</t>
         </is>
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Bell push</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>4'-6"</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
@@ -15297,27 +15230,27 @@
         </is>
       </c>
       <c r="E105" s="4" t="n">
-        <v>64</v>
+        <v>61.4</v>
       </c>
       <c r="F105" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G105" s="4" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>BELL</t>
+          <t>CAM</t>
         </is>
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>Bell push</t>
+          <t>CCTV point</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>4'-6"</t>
+          <t>8'-0"</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
@@ -15326,27 +15259,31 @@
         </is>
       </c>
       <c r="E106" s="4" t="n">
-        <v>61.4</v>
+        <v>66.5</v>
       </c>
       <c r="F106" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="G106" s="4" t="inlineStr"/>
+        <v>24.6</v>
+      </c>
+      <c r="G106" s="4" t="inlineStr">
+        <is>
+          <t>covers gate and door</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>CAM</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>CCTV point</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>8'-0"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
@@ -15355,31 +15292,31 @@
         </is>
       </c>
       <c r="E107" s="4" t="n">
-        <v>66.5</v>
+        <v>61.4</v>
       </c>
       <c r="F107" s="4" t="n">
-        <v>24.6</v>
+        <v>24</v>
       </c>
       <c r="G107" s="4" t="inlineStr">
         <is>
-          <t>covers gate and door</t>
+          <t>outdoor, weatherproof</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
@@ -15391,57 +15328,57 @@
         <v>61.4</v>
       </c>
       <c r="F108" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="G108" s="4" t="inlineStr">
-        <is>
-          <t>outdoor, weatherproof</t>
-        </is>
-      </c>
+        <v>21.5</v>
+      </c>
+      <c r="G108" s="4" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>MTR</t>
         </is>
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>Meter at gate</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>5'-0"</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>Poomukham (verandah)</t>
+          <t>Site</t>
         </is>
       </c>
       <c r="E109" s="4" t="n">
-        <v>61.4</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="F109" s="4" t="n">
-        <v>21.5</v>
-      </c>
-      <c r="G109" s="4" t="inlineStr"/>
+        <v>23.2</v>
+      </c>
+      <c r="G109" s="4" t="inlineStr">
+        <is>
+          <t>meter in compound wall by gate</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>MTR</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>Meter at gate</t>
+          <t>Outdoor / gate light</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>5'-0"</t>
+          <t>7'-0"</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
@@ -15450,14 +15387,14 @@
         </is>
       </c>
       <c r="E110" s="4" t="n">
-        <v>74.59999999999999</v>
+        <v>74.7</v>
       </c>
       <c r="F110" s="4" t="n">
-        <v>23</v>
+        <v>15.3</v>
       </c>
       <c r="G110" s="4" t="inlineStr">
         <is>
-          <t>meter in compound wall by gate</t>
+          <t>gate post light</t>
         </is>
       </c>
     </row>
@@ -15483,111 +15420,210 @@
         </is>
       </c>
       <c r="E111" s="4" t="n">
-        <v>74.59999999999999</v>
+        <v>74.7</v>
       </c>
       <c r="F111" s="4" t="n">
-        <v>14.5</v>
+        <v>22.9</v>
       </c>
       <c r="G111" s="4" t="inlineStr">
         <is>
-          <t>gate light</t>
+          <t>gate post light</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>EP</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>Earth pit</t>
+          <t>Outdoor / gate light</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>ground</t>
+          <t>7'-0"</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>Site</t>
+          <t>Poomukham (verandah)</t>
         </is>
       </c>
       <c r="E112" s="4" t="n">
-        <v>68.2</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="F112" s="4" t="n">
-        <v>1.5</v>
+        <v>16.4</v>
       </c>
       <c r="G112" s="4" t="inlineStr">
         <is>
-          <t>earth pit 1</t>
+          <t>uplight at the pillar base</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>EP</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>Earth pit</t>
+          <t>Outdoor / gate light</t>
         </is>
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>ground</t>
+          <t>7'-0"</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>Site</t>
+          <t>Poomukham (verandah)</t>
         </is>
       </c>
       <c r="E113" s="4" t="n">
-        <v>73.5</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="F113" s="4" t="n">
-        <v>1.5</v>
+        <v>21.8</v>
       </c>
       <c r="G113" s="4" t="inlineStr">
         <is>
-          <t>earth pit 2</t>
+          <t>uplight at the pillar base</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
+          <t>WL</t>
+        </is>
+      </c>
+      <c r="B114" s="4" t="inlineStr">
+        <is>
+          <t>Wall light / mirror light</t>
+        </is>
+      </c>
+      <c r="C114" s="4" t="inlineStr">
+        <is>
+          <t>6'-6"</t>
+        </is>
+      </c>
+      <c r="D114" s="4" t="inlineStr">
+        <is>
+          <t>Poomukham (verandah)</t>
+        </is>
+      </c>
+      <c r="E114" s="4" t="n">
+        <v>61.4</v>
+      </c>
+      <c r="F114" s="4" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="G114" s="4" t="inlineStr">
+        <is>
+          <t>warm lantern beside the main door</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr">
+        <is>
+          <t>EP</t>
+        </is>
+      </c>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
+          <t>Earth pit</t>
+        </is>
+      </c>
+      <c r="C115" s="4" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="E115" s="4" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="F115" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G115" s="4" t="inlineStr">
+        <is>
+          <t>earth pit 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="4" t="inlineStr">
+        <is>
+          <t>EP</t>
+        </is>
+      </c>
+      <c r="B116" s="4" t="inlineStr">
+        <is>
+          <t>Earth pit</t>
+        </is>
+      </c>
+      <c r="C116" s="4" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="E116" s="4" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="F116" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G116" s="4" t="inlineStr">
+        <is>
+          <t>earth pit 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="4" t="inlineStr">
+        <is>
           <t>GL</t>
         </is>
       </c>
-      <c r="B114" s="4" t="inlineStr">
+      <c r="B117" s="4" t="inlineStr">
         <is>
           <t>Outdoor / gate light</t>
         </is>
       </c>
-      <c r="C114" s="4" t="inlineStr">
+      <c r="C117" s="4" t="inlineStr">
         <is>
           <t>7'-0"</t>
         </is>
       </c>
-      <c r="D114" s="4" t="inlineStr">
+      <c r="D117" s="4" t="inlineStr">
         <is>
           <t>Site</t>
         </is>
       </c>
-      <c r="E114" s="4" t="n">
+      <c r="E117" s="4" t="n">
         <v>2.5</v>
       </c>
-      <c r="F114" s="4" t="n">
+      <c r="F117" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="G114" s="4" t="inlineStr">
+      <c r="G117" s="4" t="inlineStr">
         <is>
           <t>rear garden</t>
         </is>

</xml_diff>

<commit_message>
TV back on the west wall of the hall
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Schedules/KH-P1_Schedules_RevB.xlsx
+++ b/03_Schedules/KH-P1_Schedules_RevB.xlsx
@@ -4536,7 +4536,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>TV on the north face of the common-bath wall in the dining space, sofa facing south: confirm screen size (55-65 in at about 8 ft from the sofa) and a concealed HDMI/data conduit; the north window behind the sofa may reflect on the screen (matt screen or sheer blind)</t>
+          <t>TV on the west wall of the hall (Bedroom 2's east wall), sofa facing west: confirm screen size (55 in at about 7'-6") and a concealed HDMI/data conduit</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -4911,7 +4911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5056,7 +5056,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Thirty-first review (front facade): gate re-centred on the main door with a 6 ft stone forecourt and the tulsi thara on the axis (gate, tulsi, steps, door, hall, lamp niche in one line); charupadi seats with sloping backrests between the verandah pillars, flanking the steps; carved teak barge boards and a brass kalasham finial on the front gable; the kitchen front clad in exposed laterite with a deep projecting teak frame to its window; carved teak main door with brass studs, a stone surround and a nameplate niche; warm uplights at the pillars, a lantern by the door and gate-post lights; low hedges screening the sump and the two-wheeler bay; a pair of potted palms beside the steps.</t>
+          <t>Thirty-second review: TV back on the west wall of the hall (Bedroom 2's east wall), sofa facing west about 7'-6" away in the dining bay, coffee table between, the window seat shortened to 4 ft as side seating; the dining space under the ventilator is open again.</t>
         </is>
       </c>
     </row>
@@ -5066,7 +5066,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Thirtieth review (proportion clean-up): windows standardised to three sizes (6 ft rooms, 3 ft small, 2 ft baths) with every head at 7 ft and three sill levels (3 ft rooms, 3'-6" over counters, 5 ft baths); sunshades only on the sunny south, east and west walls (the eaves shade the north); floors cut to three families plus the verandah (red oxide in all public rooms and the pooja, vitrified in bedrooms, anti-skid ceramic in kitchen, baths and wet area, granite on the verandah); services hidden (pipes in chases, outdoor units grouped behind jali on the north wall), switchboards aligned, warm layered lighting, handle-less built-in fronts.</t>
+          <t>Thirty-first review (front facade): gate re-centred on the main door with a 6 ft stone forecourt and the tulsi thara on the axis (gate, tulsi, steps, door, hall, lamp niche in one line); charupadi seats with sloping backrests between the verandah pillars, flanking the steps; carved teak barge boards and a brass kalasham finial on the front gable; the kitchen front clad in exposed laterite with a deep projecting teak frame to its window; carved teak main door with brass studs, a stone surround and a nameplate niche; warm uplights at the pillars, a lantern by the door and gate-post lights; low hedges screening the sump and the two-wheeler bay; a pair of potted palms beside the steps.</t>
         </is>
       </c>
     </row>
@@ -5076,7 +5076,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Twenty-ninth review: compound wall made as thin as practical: precast RCC post-and-panel (2 in panels in 4 in posts) set just inside the plot line, so the side strips stay walkable and the north run can be lifted and moved if more land is bought.</t>
+          <t>Thirtieth review (proportion clean-up): windows standardised to three sizes (6 ft rooms, 3 ft small, 2 ft baths) with every head at 7 ft and three sill levels (3 ft rooms, 3'-6" over counters, 5 ft baths); sunshades only on the sunny south, east and west walls (the eaves shade the north); floors cut to three families plus the verandah (red oxide in all public rooms and the pooja, vitrified in bedrooms, anti-skid ceramic in kitchen, baths and wet area, granite on the verandah); services hidden (pipes in chases, outdoor units grouped behind jali on the north wall), switchboards aligned, warm layered lighting, handle-less built-in fronts.</t>
         </is>
       </c>
     </row>
@@ -5086,7 +5086,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Twenty-eighth review: TV lounge reworked: sofa brought forward to about 8 ft from the TV, a 3 ft walk behind it, and a built-in window seat (charupadi-style enclave) under the dining-bay window, so the sofa backs onto a quiet seating nook rather than the entrance and nobody walks in front of the TV.</t>
+          <t>Twenty-ninth review: compound wall made as thin as practical: precast RCC post-and-panel (2 in panels in 4 in posts) set just inside the plot line, so the side strips stay walkable and the north run can be lifted and moved if more land is bought.</t>
         </is>
       </c>
     </row>
@@ -5096,7 +5096,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Twenty-seventh review: TV lounge moves to the open dining space under the ventilator: TV on the north face of the common-bath wall, sofa facing south with its back to the north window, so the main door is in side view, not behind (commanding position) and the TV no longer faces the main door; the dining bay becomes a reading / dining nook with a chair by the window.</t>
+          <t>Twenty-eighth review: TV lounge reworked: sofa brought forward to about 8 ft from the TV, a 3 ft walk behind it, and a built-in window seat (charupadi-style enclave) under the dining-bay window, so the sofa backs onto a quiet seating nook rather than the entrance and nobody walks in front of the TV.</t>
         </is>
       </c>
     </row>
@@ -5106,7 +5106,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Twenty-sixth review: built-in ideas borrowed and adapted (function, not style, in Kerala materials): recessed shower niches, mirror cabinets over basins, genkan-style shoe bench with hooks and a granite threshold band, vilakku madam lamp niche facing the main door, floating bedside shelves (walls too thin for recesses), drawers-first kitchen with a masala pull-out and utensil rail, dish-drying rack over the utility sink, ceiling clothes airer in the wet area.</t>
+          <t>Twenty-seventh review: TV lounge moves to the open dining space under the ventilator: TV on the north face of the common-bath wall, sofa facing south with its back to the north window, so the main door is in side view, not behind (commanding position) and the TV no longer faces the main door; the dining bay becomes a reading / dining nook with a chair by the window.</t>
         </is>
       </c>
     </row>
@@ -5116,7 +5116,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Twenty-fifth review: main door moved 3'-4" south (y 17'-7" to 20'-7"), centred under the front gable and opening straight onto the 5 ft walk between the pooja and the diwan; shoe cupboard to its north on the east wall; window diwan back to 6 ft along the north window, out of the door's line; steps, middle verandah pillars and the swing realigned.</t>
+          <t>Twenty-sixth review: built-in ideas borrowed and adapted (function, not style, in Kerala materials): recessed shower niches, mirror cabinets over basins, genkan-style shoe bench with hooks and a granite threshold band, vilakku madam lamp niche facing the main door, floating bedside shelves (walls too thin for recesses), drawers-first kitchen with a masala pull-out and utensil rail, dish-drying rack over the utility sink, ceiling clothes airer in the wet area.</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Twenty-fourth review: planned on the 27 ft plot alone (north strip dropped for now): roof eaves cut from 2'-6" to 2'-0" so the north eave stays inside the plot line, septic tank moved under the two-wheeler bay in the front yard with a lined soak pit beside it, all drains rerouted along the south walkway to the front, rainwater to the sump with overflow to the road; north-strip trees and recharge pit removed.</t>
+          <t>Twenty-fifth review: main door moved 3'-4" south (y 17'-7" to 20'-7"), centred under the front gable and opening straight onto the 5 ft walk between the pooja and the diwan; shoe cupboard to its north on the east wall; window diwan back to 6 ft along the north window, out of the door's line; steps, middle verandah pillars and the swing realigned.</t>
         </is>
       </c>
     </row>
@@ -5136,7 +5136,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Twenty-third review: the fridge moves out of the kitchen into the dining alcove beside the kitchen door, against the wet-area wall; the kitchen's north wall is now free.</t>
+          <t>Twenty-fourth review: planned on the 27 ft plot alone (north strip dropped for now): roof eaves cut from 2'-6" to 2'-0" so the north eave stays inside the plot line, septic tank moved under the two-wheeler bay in the front yard with a lined soak pit beside it, all drains rerouted along the south walkway to the front, rainwater to the sump with overflow to the road; north-strip trees and recharge pit removed.</t>
         </is>
       </c>
     </row>
@@ -5146,7 +5146,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Twenty-second review: the kitchen's tall pantry and the dining table and chairs are removed at the owner's request; the dining space under the ventilator stays open (the pendant light and points stay for a table later).</t>
+          <t>Twenty-third review: the fridge moves out of the kitchen into the dining alcove beside the kitchen door, against the wet-area wall; the kitchen's north wall is now free.</t>
         </is>
       </c>
     </row>
@@ -5156,7 +5156,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Twenty-first review: the open hall becomes three zones: family TV lounge in the dining bay (5'-6" sofa facing the TV), dining under the ventilator moved 9 in south (about 2 ft behind the chairs on both sides), and guest sitting by the main door with a 4'-6" window diwan (shortened after the walk-through showed a 1'-6" pinch at the shoe cupboard) and an armchair under the living's north window; a clear walk of about 4'-11" from the main door to the dining and kitchen, pooja front kept clear.</t>
+          <t>Twenty-second review: the kitchen's tall pantry and the dining table and chairs are removed at the owner's request; the dining space under the ventilator stays open (the pendant light and points stay for a table later).</t>
         </is>
       </c>
     </row>
@@ -5166,7 +5166,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Twentieth review: Bedroom 2's bed moves to the east wall, head east, leaving an 8 x 14 ft open floor from the door to the bath and window; wardrobe to the west wall (sound buffer to the master), work table north of the bed, AC on the bath's outer wall; dresser dropped (mirror on the wardrobe).</t>
+          <t>Twenty-first review: the open hall becomes three zones: family TV lounge in the dining bay (5'-6" sofa facing the TV), dining under the ventilator moved 9 in south (about 2 ft behind the chairs on both sides), and guest sitting by the main door with a 4'-6" window diwan (shortened after the walk-through showed a 1'-6" pinch at the shoe cupboard) and an armchair under the living's north window; a clear walk of about 4'-11" from the main door to the dining and kitchen, pooja front kept clear.</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
+          <t>Twentieth review: Bedroom 2's bed moves to the east wall, head east, leaving an 8 x 14 ft open floor from the door to the bath and window; wardrobe to the west wall (sound buffer to the master), work table north of the bed, AC on the bath's outer wall; dresser dropped (mirror on the wardrobe).</t>
         </is>
       </c>
     </row>
@@ -5186,7 +5186,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
+          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
+          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
         </is>
       </c>
     </row>
@@ -5206,7 +5206,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
+          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
         </is>
       </c>
     </row>
@@ -5216,7 +5216,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
+          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
         </is>
       </c>
     </row>
@@ -5226,7 +5226,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
+          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
         </is>
       </c>
     </row>
@@ -5236,7 +5236,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
+          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
         </is>
       </c>
     </row>
@@ -5246,7 +5246,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
+          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
         </is>
       </c>
     </row>
@@ -5256,7 +5256,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
+          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5266,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
+          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
         </is>
       </c>
     </row>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
+          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
         </is>
       </c>
     </row>
@@ -5286,7 +5286,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
+          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
         </is>
       </c>
     </row>
@@ -5296,7 +5296,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
+          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
         </is>
       </c>
     </row>
@@ -5306,7 +5306,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
+          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
         </is>
       </c>
     </row>
@@ -5316,7 +5316,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
+          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
         </is>
       </c>
     </row>
@@ -5326,7 +5326,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
+          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
         </is>
       </c>
     </row>
@@ -5336,7 +5336,7 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
+          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
         </is>
       </c>
     </row>
@@ -5346,7 +5346,7 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
+          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
+          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
         </is>
       </c>
     </row>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
+          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
         </is>
       </c>
     </row>
@@ -5376,7 +5376,7 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
+          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
+          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
         </is>
       </c>
     </row>
@@ -5396,7 +5396,7 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
+          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
+          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
         </is>
       </c>
     </row>
@@ -5416,7 +5416,7 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
+          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
         </is>
       </c>
     </row>
@@ -5426,7 +5426,7 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
         </is>
       </c>
     </row>
@@ -5436,7 +5436,7 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
         </is>
       </c>
     </row>
@@ -5445,6 +5445,16 @@
         <v>52</v>
       </c>
       <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>Roof: Mangalore clay tiles on steel truss over insulated cement-fibre deck; all edge tiles mechanically fixed.</t>
         </is>
@@ -7527,7 +7537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -9377,12 +9387,12 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Dining bay</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Sofa 5'-6" (2-3 seats) facing south to the TV about 8 ft away; behind it a 3 ft walk and the window-seat enclave; main door in side view</t>
+          <t>Sofa 5'-6" (2-3 seats) facing west to the TV about 7'-6" away</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -9391,10 +9401,10 @@
         </is>
       </c>
       <c r="E43" s="4" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="F43" s="4" t="n">
         <v>5.5</v>
-      </c>
-      <c r="F43" s="4" t="n">
-        <v>2.7</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>1</v>
@@ -9420,7 +9430,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Dining bay</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -9434,10 +9444,10 @@
         </is>
       </c>
       <c r="E44" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F44" s="4" t="n">
         <v>3.5</v>
-      </c>
-      <c r="F44" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="G44" s="4" t="n">
         <v>1</v>
@@ -9463,12 +9473,12 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Dining bay</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>TV unit 4'-5" on the north face of the common-bath wall (55-65 in TV wall-mounted above)</t>
+          <t>TV unit 4'-5" on Bedroom 2's east wall, the west wall of the hall (55 in TV wall-mounted above)</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -9477,10 +9487,10 @@
         </is>
       </c>
       <c r="E45" s="4" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F45" s="4" t="n">
         <v>4.4</v>
-      </c>
-      <c r="F45" s="4" t="n">
-        <v>1.25</v>
       </c>
       <c r="G45" s="4" t="n">
         <v>1</v>
@@ -9511,7 +9521,7 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Built-in window seat 6'-5" x 2' under the north window (charupadi-style enclave: cushions, bolsters, drawers below)</t>
+          <t>Built-in window seat 4' x 2' under the north window, side seating for the TV area (cushions, bolsters, drawers below)</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -9520,7 +9530,7 @@
         </is>
       </c>
       <c r="E46" s="4" t="n">
-        <v>6.4</v>
+        <v>4</v>
       </c>
       <c r="F46" s="4" t="n">
         <v>2</v>
@@ -9544,17 +9554,17 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>F66</t>
+          <t>F40</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Dining bay</t>
+          <t>Living</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Reading chair in the north-west corner of the bay</t>
+          <t>Armchair at the west end of the window diwan</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -9587,7 +9597,7 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>F40</t>
+          <t>F58</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -9597,7 +9607,7 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Armchair at the west end of the window diwan</t>
+          <t>Window diwan 6' x 2'-6" under the north window, drawers below (guest seating, day bed); out of the line of the main door</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -9606,17 +9616,17 @@
         </is>
       </c>
       <c r="E48" s="4" t="n">
-        <v>1.8</v>
+        <v>6</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>1.8</v>
+        <v>2.6</v>
       </c>
       <c r="G48" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>Cane / teak</t>
+          <t>Teak frame, cotton mattress and bolsters</t>
         </is>
       </c>
       <c r="I48" s="10" t="n"/>
@@ -9630,7 +9640,7 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>F58</t>
+          <t>F52</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -9640,7 +9650,7 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Window diwan 6' x 2'-6" under the north window, drawers below (guest seating, day bed); out of the line of the main door</t>
+          <t>Shoe bench 3'-3" (Japanese genkan idea): sit to take shoes off, louvred shoe shelves below, hooks and a keys niche above, small cabinet over</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -9649,17 +9659,17 @@
         </is>
       </c>
       <c r="E49" s="4" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>2.6</v>
+        <v>3.2</v>
       </c>
       <c r="G49" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>Teak frame, cotton mattress and bolsters</t>
+          <t>Teak top, ply + laminate, 14 in deep</t>
         </is>
       </c>
       <c r="I49" s="10" t="n"/>
@@ -9673,7 +9683,7 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>F52</t>
+          <t>F59</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -9683,7 +9693,7 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Shoe bench 3'-3" (Japanese genkan idea): sit to take shoes off, louvred shoe shelves below, hooks and a keys niche above, small cabinet over</t>
+          <t>Vilakku madam: carved teak lamp niche with a light inside, on the wall facing the main door</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -9692,17 +9702,17 @@
         </is>
       </c>
       <c r="E50" s="4" t="n">
-        <v>1.2</v>
+        <v>0.34</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>3.2</v>
+        <v>1.8</v>
       </c>
       <c r="G50" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H50" s="4" t="inlineStr">
         <is>
-          <t>Teak top, ply + laminate, 14 in deep</t>
+          <t>Carved teak, brass lamp</t>
         </is>
       </c>
       <c r="I50" s="10" t="n"/>
@@ -9716,17 +9726,17 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>F59</t>
+          <t>F41</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Living</t>
+          <t>Poomukham (verandah)</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Vilakku madam: carved teak lamp niche with a light inside, on the wall facing the main door</t>
+          <t>Oonjal (swing) 3'6", north side of the verandah, clear of the entrance</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -9735,17 +9745,17 @@
         </is>
       </c>
       <c r="E51" s="4" t="n">
-        <v>0.34</v>
+        <v>3.3</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="G51" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>Carved teak, brass lamp</t>
+          <t>Teak, chains to beam</t>
         </is>
       </c>
       <c r="I51" s="10" t="n"/>
@@ -9759,7 +9769,7 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>F41</t>
+          <t>F42</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -9769,7 +9779,7 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Oonjal (swing) 3'6", north side of the verandah, clear of the entrance</t>
+          <t>Charupadi: built-in teak seat with a sloping backrest between the pillars, south of the steps</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -9778,17 +9788,17 @@
         </is>
       </c>
       <c r="E52" s="4" t="n">
-        <v>3.3</v>
+        <v>1.3</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="G52" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H52" s="4" t="inlineStr">
         <is>
-          <t>Teak, chains to beam</t>
+          <t>Laterite base, teak seat and backrest</t>
         </is>
       </c>
       <c r="I52" s="10" t="n"/>
@@ -9802,7 +9812,7 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>F42</t>
+          <t>F69</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
@@ -9812,7 +9822,7 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Charupadi: built-in teak seat with a sloping backrest between the pillars, south of the steps</t>
+          <t>Charupadi: built-in teak seat with a sloping backrest between the pillars, north of the steps</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -9824,7 +9834,7 @@
         <v>1.3</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="G53" s="4" t="n">
         <v>1</v>
@@ -9843,71 +9853,28 @@
       <c r="L53" s="8" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>F69</t>
-        </is>
-      </c>
-      <c r="B54" s="4" t="inlineStr">
-        <is>
-          <t>Poomukham (verandah)</t>
-        </is>
-      </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>Charupadi: built-in teak seat with a sloping backrest between the pillars, north of the steps</t>
-        </is>
-      </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>Loose furniture</t>
-        </is>
-      </c>
-      <c r="E54" s="4" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="F54" s="4" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="G54" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H54" s="4" t="inlineStr">
-        <is>
-          <t>Laterite base, teak seat and backrest</t>
-        </is>
-      </c>
-      <c r="I54" s="10" t="n"/>
-      <c r="J54" s="11">
-        <f>G54*I54</f>
+      <c r="A54" s="6" t="inlineStr"/>
+      <c r="B54" s="6" t="inlineStr"/>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr"/>
+      <c r="E54" s="6" t="inlineStr"/>
+      <c r="F54" s="6" t="inlineStr"/>
+      <c r="G54" s="6">
+        <f>SUM(G2:G53)</f>
         <v/>
       </c>
-      <c r="K54" s="8" t="inlineStr"/>
-      <c r="L54" s="8" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="6" t="inlineStr"/>
-      <c r="B55" s="6" t="inlineStr"/>
-      <c r="C55" s="6" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="D55" s="6" t="inlineStr"/>
-      <c r="E55" s="6" t="inlineStr"/>
-      <c r="F55" s="6" t="inlineStr"/>
-      <c r="G55" s="6">
-        <f>SUM(G2:G54)</f>
+      <c r="H54" s="6" t="inlineStr"/>
+      <c r="I54" s="12" t="inlineStr"/>
+      <c r="J54" s="12">
+        <f>SUM(J2:J53)</f>
         <v/>
       </c>
-      <c r="H55" s="6" t="inlineStr"/>
-      <c r="I55" s="12" t="inlineStr"/>
-      <c r="J55" s="12">
-        <f>SUM(J2:J54)</f>
-        <v/>
-      </c>
-      <c r="K55" s="6" t="inlineStr"/>
-      <c r="L55" s="6" t="inlineStr"/>
+      <c r="K54" s="6" t="inlineStr"/>
+      <c r="L54" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14078,18 +14045,18 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Dining bay (north window)</t>
         </is>
       </c>
       <c r="E69" s="4" t="n">
-        <v>44.8</v>
+        <v>38.4</v>
       </c>
       <c r="F69" s="4" t="n">
-        <v>9.4</v>
+        <v>22.4</v>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>TV wall (common-bath wall, dry face): 2 sockets + data + HDMI conduit to the unit</t>
+          <t>TV wall: 2 sockets + data + HDMI conduit to the unit</t>
         </is>
       </c>
     </row>
@@ -14111,14 +14078,14 @@
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Dining bay (north window)</t>
         </is>
       </c>
       <c r="E70" s="4" t="n">
-        <v>43.2</v>
+        <v>38.4</v>
       </c>
       <c r="F70" s="4" t="n">
-        <v>9.4</v>
+        <v>21</v>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
@@ -14155,7 +14122,7 @@
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>Bedroom 2's east wall, throws east across the hall and the TV seating</t>
+          <t>above the TV unit, throws east over the seating</t>
         </is>
       </c>
     </row>
@@ -14970,14 +14937,14 @@
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>Dining</t>
+          <t>Dining bay (north window)</t>
         </is>
       </c>
       <c r="E97" s="4" t="n">
-        <v>47.9</v>
+        <v>48.4</v>
       </c>
       <c r="F97" s="4" t="n">
-        <v>18</v>
+        <v>18.6</v>
       </c>
       <c r="G97" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Duplex: lounge merged into the upper master, open under-stair, no ridge ventilator
The outdoor lounge becomes the upper master's sitting and study zone,
part-divided by a wardrobe; the space under the upper flight is open to
the lobby where there is 7 ft headroom; the ridge ventilator and its
detail sheet are removed now that the terrace is open-sided.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Schedules/KH-P1_Schedules_RevB.xlsx
+++ b/03_Schedules/KH-P1_Schedules_RevB.xlsx
@@ -1737,7 +1737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E99"/>
+  <dimension ref="A1:E94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Keep 7 ft clear under every part of the stair; the space under the upper flight is a cupboard, not a walkway.</t>
+          <t>Keep 7 ft clear wherever people walk: under the upper flight the first 2 ft is left open as part of the lobby (about 6 ft wide in front of the small bedroom), and only the low part beyond is a cupboard.</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Open stair edges and a lounge rail children can climb.</t>
+          <t>Open stair edges and a terrace rail children can climb.</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -2357,17 +2357,17 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>First-floor outdoor lounge leaking into the bedroom below.</t>
+          <t>West sun on the upper floor.</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Waterproof the slab with upturns, fall 1:80 to a spout away from the wall, flood-test 48 h, then tile.</t>
+          <t>The upper master suite's west wall has only a small high vent; the main roof's 2 ft eave shades the walls; chiks on the terrace's south and east sides.</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>A-109</t>
+          <t>A-202</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr"/>
@@ -2380,17 +2380,17 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>West sun on the upper floor.</t>
+          <t>Covered terrace leaking into the living below.</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>The upper master's west wall is solid; the lounge's open west side gets bamboo chiks; the main roof's 2 ft eave shades the walls.</t>
+          <t>Waterproof the whole terrace slab with upturns at the walls and posts, fall 1:80 to the drain in the south-east corner, flood-test 48 h, then tile.</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>A-202</t>
+          <t>A-109, P-101</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr"/>
@@ -2403,17 +2403,17 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Covered terrace leaking into the living below.</t>
+          <t>Steel roof posts rusting at the base where water sits.</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Waterproof the whole terrace slab with upturns at the walls and posts, fall 1:80 to the drain in the south-east corner, flood-test 48 h, then tile.</t>
+          <t>Hot-dip galvanised posts on RCC stubs 6 in above the terrace tiles, base plates grouted and sealed; repaint every few years.</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>A-109, P-101</t>
+          <t>A-301</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr"/>
@@ -2426,17 +2426,17 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Steel roof posts rusting at the base where water sits.</t>
+          <t>Rain blowing onto the terrace in the monsoon.</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Hot-dip galvanised posts on RCC stubs 6 in above the terrace tiles, base plates grouted and sealed; repaint every few years.</t>
+          <t>The main roof overhangs 2 ft beyond the railings; add bamboo chiks or roll-down blinds on the south and east if needed.</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>A-301</t>
+          <t>A-202</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr"/>
@@ -2444,22 +2444,22 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Stair and first floor</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Rain blowing onto the terrace in the monsoon.</t>
+          <t>Counter at the Western 36 in height: tiring for Indian cooking with tall vessels.</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>The main roof overhangs 2 ft beyond the railings; add bamboo chiks or roll-down blinds on the south and east if needed.</t>
+          <t>Make the counter 34 in, with a 30-31 in section for grinding and rolling chapatis.</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>A-202</t>
+          <t>A-502/6</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr"/>
@@ -2467,22 +2467,22 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Ventilator on the ridge</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Hot air trapped under the tiles over the open terrace.</t>
+          <t>White glossy floor and counter: shows every turmeric stain and is slippery with oil.</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>A raised ventilator on the ridge with louvres on all four sides lets it out; the terrace below is open-sided, so no shutters are needed.</t>
+          <t>Use a mid-tone matt floor and a granite counter (local Chimakurthy / Ongole).</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>A-503, A-110</t>
+          <t>A-108</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr"/>
@@ -2490,22 +2490,22 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Ventilator on the ridge</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Flat-topped roof ventilator: water ponds, leaves and droppings collect, and it leaks first.</t>
+          <t>Chimney duct with long bends: weak suction and grease build-up.</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Give it a small hipped roof at the main roof pitch, tiled and clipped, with a 1'-6" overhang and drip edge.</t>
+          <t>Hob on the east run with the chimney ducted straight out through the east wall.</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>A-503</t>
+          <t>A-502/6, E-103</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr"/>
@@ -2513,22 +2513,22 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Ventilator on the ridge</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Flat or shallow louvres: cyclone rain blows straight through.</t>
+          <t>Too few counter sockets.</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>45 deg blades sloping down and out with a 4 in lap (no straight line through), on a sill sloped out 1:10 with a drip.</t>
+          <t>Fit 5-6 sockets at 42 in plus 16 A for the fridge, microwave / OTG and chimney; RO point by the sink.</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>A-503</t>
+          <t>E-103</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr"/>
@@ -2536,22 +2536,22 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Ventilator on the ridge</t>
+          <t>Kitchen</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Birds nesting in the ventilator.</t>
+          <t>Base cabinets standing on the floor: rot and termites.</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>SS 304 bird mesh behind the louvres in a continuous frame.</t>
+          <t>Put cabinets on 4 in legs or a granite plinth.</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>A-503</t>
+          <t>A-502/6</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr"/>
@@ -2564,17 +2564,17 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Counter at the Western 36 in height: tiring for Indian cooking with tall vessels.</t>
+          <t>Gas cylinder in a closed cabinet under the hob.</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Make the counter 34 in, with a 30-31 in section for grinding and rolling chapatis.</t>
+          <t>Keep the cylinder in the wet area with a fixed copper / steel line and a valve through the wall.</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>A-502/6</t>
+          <t>A-104</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr"/>
@@ -2587,17 +2587,17 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>White glossy floor and counter: shows every turmeric stain and is slippery with oil.</t>
+          <t>Kitchen drain without a grease trap: chokes within a year.</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Use a mid-tone matt floor and a granite counter (local Chimakurthy / Ongole).</t>
+          <t>Put a grease trap outside, before any junction.</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>A-108</t>
+          <t>P-101</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr"/>
@@ -2610,17 +2610,17 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Chimney duct with long bends: weak suction and grease build-up.</t>
+          <t>Fridge beside the hob or in direct sun.</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Hob on the east run with the chimney ducted straight out through the east wall.</t>
+          <t>Fridge on the kitchen's north wall, clear of the entry door and away from the hob.</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>A-502/6, E-103</t>
+          <t>A-104</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr"/>
@@ -2628,22 +2628,22 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Wet area, store and kitchen entry</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Too few counter sockets.</t>
+          <t>A narrow kitchen entry squeezed past a TV wall: two people can't pass and serving is awkward.</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Fit 5-6 sockets at 42 in plus 16 A for the fridge, microwave / OTG and chimney; RO point by the sink.</t>
+          <t>The kitchen is entered through a 3 ft hinged door on its west side, straight off the dining; the wet area opens off the kitchen through a sliding door.</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>E-103</t>
+          <t>A-102</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr"/>
@@ -2651,22 +2651,22 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Wet area, store and kitchen entry</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Base cabinets standing on the floor: rot and termites.</t>
+          <t>Wet area that floods in heavy rain, or a service door that becomes a back door for intruders.</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Put cabinets on 4 in legs or a granite plinth.</t>
+          <t>Floor 3 in below the house sloping to its trap; a lockable steel service door to the walkway with a kerb.</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>A-502/6</t>
+          <t>A-102, A-108</t>
         </is>
       </c>
       <c r="E40" s="8" t="inlineStr"/>
@@ -2674,22 +2674,22 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Wet area, store and kitchen entry</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Gas cylinder in a closed cabinet under the hob.</t>
+          <t>Washing machine with no tap, drain or socket at the right height.</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Keep the cylinder in the wet area with a fixed copper / steel line and a valve through the wall.</t>
+          <t>Provide a tap at 3 ft, a floor drain behind the machine and a splash-proof 16 A socket at 4 ft.</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>A-104</t>
+          <t>P-101, E-103</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr"/>
@@ -2697,22 +2697,22 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Wet area, store and kitchen entry</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Kitchen drain without a grease trap: chokes within a year.</t>
+          <t>No store, so provisions end up on the floor.</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Put a grease trap outside, before any junction.</t>
+          <t>A 4 x 4'-6" store off the dining with full-height racks, a high jali vent and a jali above the door; lofts over the kitchen.</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>P-101</t>
+          <t>A-104</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr"/>
@@ -2720,22 +2720,22 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Wet area, store and kitchen entry</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Fridge beside the hob or in direct sun.</t>
+          <t>Inverter batteries in a bedroom or a closed cupboard.</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Fridge on the kitchen's north wall, clear of the entry door and away from the hob.</t>
+          <t>Lithium inverter in the ventilated under-stair cupboard, away from water and bedrooms.</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>A-104</t>
+          <t>E-103</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr"/>
@@ -2743,22 +2743,22 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>Wet area, store and kitchen entry</t>
+          <t>Pooja</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>A narrow kitchen entry squeezed past a TV wall: two people can't pass and serving is awkward.</t>
+          <t>Lamp smoke blackens the ceiling and the teak panelling.</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>The kitchen is entered through a 3 ft hinged door on its west side, straight off the dining; the wet area opens off the kitchen through a sliding door.</t>
+          <t>Fit a heat-proof granite or brass back panel behind the diya and a small high vent; use a washable ceiling finish.</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>A-102</t>
+          <t>A-108</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr"/>
@@ -2766,22 +2766,22 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>Wet area, store and kitchen entry</t>
+          <t>Pooja</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Wet area that floods in heavy rain, or a service door that becomes a back door for intruders.</t>
+          <t>Pooja sharing a wall with a toilet.</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Floor 3 in below the house sloping to its trap; a lockable steel service door to the walkway with a kerb.</t>
+          <t>Here the pooja sits in the living's south-east corner, back to back with the kitchen (no toilet on any side), opening west into the living with doors that open inward.</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>A-102, A-108</t>
+          <t>A-102</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr"/>
@@ -2789,22 +2789,22 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>Wet area, store and kitchen entry</t>
+          <t>Pooja</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Washing machine with no tap, drain or socket at the right height.</t>
+          <t>Polished marble floor that becomes slippery with oil.</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Provide a tap at 3 ft, a floor drain behind the machine and a splash-proof 16 A socket at 4 ft.</t>
+          <t>Use honed (matt) marble or teak.</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>P-101, E-103</t>
+          <t>A-108</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr"/>
@@ -2812,22 +2812,22 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>Wet area, store and kitchen entry</t>
+          <t>Bedrooms</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>No store, so provisions end up on the floor.</t>
+          <t>AC indoor unit above the bed head: cold air blows on your head all night.</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>A 4 x 4'-6" store off the dining with full-height racks, a high jali vent and a jali above the door; lofts over the kitchen.</t>
+          <t>Mount the AC on a side or opposite wall, throwing across the bed.</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>A-104</t>
+          <t>E-103</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr"/>
@@ -2835,22 +2835,22 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>Wet area, store and kitchen entry</t>
+          <t>Bedrooms</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Inverter batteries in a bedroom or a closed cupboard.</t>
+          <t>Only one switchboard at the door.</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Lithium inverter in the ventilated under-stair cupboard, away from water and bedrooms.</t>
+          <t>Add 2-way switches at the bed for the light and fan, plus bedside sockets.</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>E-103</t>
+          <t>E-101, E-103</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr"/>
@@ -2858,22 +2858,22 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Pooja</t>
+          <t>Bedrooms</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Lamp smoke blackens the ceiling and the teak panelling.</t>
+          <t>Wardrobe shallower than 2 ft: hangers do not fit.</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Fit a heat-proof granite or brass back panel behind the diya and a small high vent; use a washable ceiling finish.</t>
+          <t>Make wardrobes 2 ft deep with lofts above to the false ceiling.</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>A-108</t>
+          <t>A-104, A-105</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr"/>
@@ -2881,22 +2881,22 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Pooja</t>
+          <t>Bedrooms</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Pooja sharing a wall with a toilet.</t>
+          <t>2'-6" bedroom doors: a mattress or cupboard cannot go in later.</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Here the pooja sits in the living's south-east corner, back to back with the kitchen (no toilet on any side), opening west into the living with doors that open inward.</t>
+          <t>Make bedroom doors 3'-0".</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>A-102</t>
+          <t>A-401</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr"/>
@@ -2904,22 +2904,22 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>Pooja</t>
+          <t>Bedrooms</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Polished marble floor that becomes slippery with oil.</t>
+          <t>Curtain rods, TV brackets and fan hooks screwed into plain AAC, which pulls out.</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Use honed (matt) marble or teak.</t>
+          <t>Fix timber grounds or use AAC-rated anchors, marked before plaster.</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>A-108</t>
+          <t>A-001</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr"/>
@@ -2932,17 +2932,17 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>AC indoor unit above the bed head: cold air blows on your head all night.</t>
+          <t>Windows without mesh, so mosquito coils every night.</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Mount the AC on a side or opposite wall, throwing across the bed.</t>
+          <t>Put insect mesh on a separate frame on every opening.</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>E-103</t>
+          <t>A-401</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr"/>
@@ -2950,22 +2950,22 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>Bedrooms</t>
+          <t>Wardrobes and dressing</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Only one switchboard at the door.</t>
+          <t>Clothes stored in a walk-in only one person can use.</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Add 2-way switches at the bed for the light and fan, plus bedside sockets.</t>
+          <t>The upper master has a dressing room between the bedroom and its bath; the ground master and small bedroom have built-in wardrobes with lofts.</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>E-101, E-103</t>
+          <t>A-108</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr"/>
@@ -2973,22 +2973,22 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>Bedrooms</t>
+          <t>Wardrobes and dressing</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Wardrobe shallower than 2 ft: hangers do not fit.</t>
+          <t>Dressing mirror lit from behind.</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Make wardrobes 2 ft deep with lofts above to the false ceiling.</t>
+          <t>Mount the mirror light above or beside the mirror.</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>A-104, A-105</t>
+          <t>E-101, E-102</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr"/>
@@ -2996,22 +2996,22 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>Bedrooms</t>
+          <t>Bathrooms</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>2'-6" bedroom doors: a mattress or cupboard cannot go in later.</t>
+          <t>Raised step at the bathroom door, which people trip on at night.</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Make bedroom doors 3'-0".</t>
+          <t>Drop the bathroom 12 mm with a sloped granite threshold and no step.</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>A-401</t>
+          <t>A-502/5</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr"/>
@@ -3019,22 +3019,22 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>Bedrooms</t>
+          <t>Bathrooms</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Curtain rods, TV brackets and fan hooks screwed into plain AAC, which pulls out.</t>
+          <t>Whole floor sloped to one trap: the entire bathroom is always wet.</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Fix timber grounds or use AAC-rated anchors, marked before plaster.</t>
+          <t>Separate wet and dry zones: a linear drain in the shower, the dry zone nearly flat, and a glass partition.</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>A-001</t>
+          <t>A-502/5</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr"/>
@@ -3042,22 +3042,22 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>Bedrooms</t>
+          <t>Bathrooms</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>Windows without mesh, so mosquito coils every night.</t>
+          <t>No waterproofing or flood test: damp skirting in the next bedroom within a year.</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Put insect mesh on a separate frame on every opening.</t>
+          <t>Waterproof the floor, 12 in up the walls and 7 ft in the shower, then do a 48 h flood test before tiling.</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>A-401</t>
+          <t>A-502/5, A-001</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr"/>
@@ -3065,22 +3065,22 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>Wardrobes and dressing</t>
+          <t>Bathrooms</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Clothes stored in a walk-in only one person can use.</t>
+          <t>Wooden door frame standing in the wet floor.</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>The upper master has a dressing room between the bedroom and its bath; the ground master and small bedroom have built-in wardrobes with lofts.</t>
+          <t>Use a WPC / FRP shutter with the frame on a granite or WPC block.</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>A-108</t>
+          <t>A-401, A-502/9</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr"/>
@@ -3088,22 +3088,22 @@
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>Wardrobes and dressing</t>
+          <t>Bathrooms</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Dressing mirror lit from behind.</t>
+          <t>Exhaust fan blowing into the false ceiling.</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Mount the mirror light above or beside the mirror.</t>
+          <t>Duct the exhaust fan straight out through the outer wall.</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>E-101, E-102</t>
+          <t>E-101</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr"/>
@@ -3116,17 +3116,17 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Raised step at the bathroom door, which people trip on at night.</t>
+          <t>Geyser hidden above the false ceiling, which can't be serviced.</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Drop the bathroom 12 mm with a sloped granite threshold and no step.</t>
+          <t>Wall-mount it at 6'-6" with the switch outside; leave a ceiling access panel at the concealed cistern.</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>A-502/5</t>
+          <t>E-103</t>
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr"/>
@@ -3139,17 +3139,17 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Whole floor sloped to one trap: the entire bathroom is always wet.</t>
+          <t>Black or glossy tiles and chrome fittings with Guntur's hard water: white scale shows everywhere.</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Separate wet and dry zones: a linear drain in the shower, the dry zone nearly flat, and a glass partition.</t>
+          <t>Use light matt tiles and matt / PVD fittings, plus a softener if hardness is high.</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>A-502/5</t>
+          <t>A-108, P-101</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr"/>
@@ -3162,17 +3162,17 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>No waterproofing or flood test: damp skirting in the next bedroom within a year.</t>
+          <t>Bath over a bedroom or the living: a leak shows on the ceiling below.</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Waterproof the floor, 12 in up the walls and 7 ft in the shower, then do a 48 h flood test before tiling.</t>
+          <t>The upper bath sits exactly over the common bath (wet over wet); waterproof its slab, flood-test it and keep its WC stack in the wet wall.</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>A-502/5, A-001</t>
+          <t>A-109, P-101</t>
         </is>
       </c>
       <c r="E62" s="8" t="inlineStr"/>
@@ -3185,17 +3185,17 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Wooden door frame standing in the wet floor.</t>
+          <t>No backing for grab bars later.</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Use a WPC / FRP shutter with the frame on a granite or WPC block.</t>
+          <t>Fix blocking in the walls beside the WC and shower now.</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>A-401, A-502/9</t>
+          <t>A-502/5</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr"/>
@@ -3203,22 +3203,22 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>Bathrooms</t>
+          <t>Study table (small bedroom)</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Exhaust fan blowing into the false ceiling.</t>
+          <t>Window behind the screen (silhouette on video calls) or in front of it (glare).</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Duct the exhaust fan straight out through the outer wall.</t>
+          <t>The study table sits on the south wall with the north window to the side.</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>E-101</t>
+          <t>A-104</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr"/>
@@ -3226,17 +3226,17 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>Bathrooms</t>
+          <t>Study table (small bedroom)</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Geyser hidden above the false ceiling, which can't be serviced.</t>
+          <t>Not enough power or data.</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Wall-mount it at 6'-6" with the switch outside; leave a ceiling access panel at the concealed cistern.</t>
+          <t>Fit a UPS socket, a normal socket and a Cat6 point at the table, with the router on the inverter.</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -3249,22 +3249,22 @@
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>Bathrooms</t>
+          <t>Doors and windows</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Black or glossy tiles and chrome fittings with Guntur's hard water: white scale shows everywhere.</t>
+          <t>Solid walls and closed doors between rooms: no breeze crosses the house at night.</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Use light matt tiles and matt / PVD fittings, plus a softener if hardness is high.</t>
+          <t>Put a vent above inner doors where privacy allows, 7'-6" to 9'-0": open jali for the pooja and the store.</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>A-108, P-101</t>
+          <t>A-401</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr"/>
@@ -3272,22 +3272,22 @@
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>Bathrooms</t>
+          <t>Doors and windows</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Bath over a bedroom or the living: a leak shows on the ceiling below.</t>
+          <t>Open vents above bedroom and bathroom doors: conversation, TV and smells carry.</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>The upper bath sits exactly over the common bath (wet over wet); waterproof its slab, flood-test it and keep its WC stack in the wet wall.</t>
+          <t>No vents at bedrooms (windows, fans and AC are enough) or bathrooms (the door's bottom louvre feeds the exhaust fan).</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>A-109, P-101</t>
+          <t>A-401</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr"/>
@@ -3295,22 +3295,22 @@
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>Bathrooms</t>
+          <t>Doors and windows</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>No backing for grab bars later.</t>
+          <t>A long corridor that wastes area.</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Fix blocking in the walls beside the WC and shower now.</t>
+          <t>Here the lobby opens into the space under the upper flight, so the way to the small bedroom is about 6 ft wide at first, narrowing to a short 2'-6" passage that also serves the linen cupboard.</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>A-502/5</t>
+          <t>A-106</t>
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr"/>
@@ -3318,22 +3318,22 @@
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>Study table (small bedroom)</t>
+          <t>Doors and windows</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Window behind the screen (silhouette on video calls) or in front of it (glare).</t>
+          <t>No drip groove under sills and sunshades: black streaks down the walls.</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>The study table sits on the south wall with the north window to the side.</t>
+          <t>Slope every external sill 1:10 with a drip groove, and give every chajja a drip groove under its edge.</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>A-104</t>
+          <t>A-501/3</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr"/>
@@ -3341,22 +3341,22 @@
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>Study table (small bedroom)</t>
+          <t>Doors and windows</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>Not enough power or data.</t>
+          <t>Unseasoned teak that warps and jams.</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Fit a UPS socket, a normal socket and a Cat6 point at the table, with the router on the inverter.</t>
+          <t>Use kiln-seasoned wood, or sal / pinkado frames and UPVC on the wet side.</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>E-103</t>
+          <t>A-401</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr"/>
@@ -3369,12 +3369,12 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>Solid walls and closed doors between rooms: no breeze crosses the house at night.</t>
+          <t>Mild-steel hinges and screws that rust with humidity and hard water.</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>Put a vent above inner doors where privacy allows, 7'-6" to 9'-0": open jali for the pooja and the store.</t>
+          <t>Use SS 304 hardware, with magnetic stoppers on every door.</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -3392,12 +3392,12 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Open vents above bedroom and bathroom doors: conversation, TV and smells carry.</t>
+          <t>Grill with no openable section: no way out in a fire.</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>No vents at bedrooms (windows, fans and AC are enough) or bathrooms (the door's bottom louvre feeds the exhaust fan).</t>
+          <t>Give each bedroom one escape window with an openable grill.</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
@@ -3410,22 +3410,22 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>Doors and windows</t>
+          <t>Floors, walls and finishes</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>A long corridor that wastes area.</t>
+          <t>Skirting stuck on top of the plaster: a dust ledge that also chips.</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>Here the lobby is 10 x 3'-6" and the passage beside the stair is 2'-6" and only serves the small bedroom and the linen cupboard.</t>
+          <t>Set the skirting flush with the plaster face, with a groove above it.</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>A-106</t>
+          <t>A-501/2</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr"/>
@@ -3433,22 +3433,22 @@
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>Doors and windows</t>
+          <t>Floors, walls and finishes</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>No drip groove under sills and sunshades: black streaks down the walls.</t>
+          <t>Tiles laid tight to the walls: they pop up (tenting) in 45 C summers.</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>Slope every external sill 1:10 with a drip groove, and give every chajja a drip groove under its edge.</t>
+          <t>Leave 5 mm gaps at walls and movement joints every 15-20 ft, hidden by the skirting.</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>A-501/3</t>
+          <t>A-501/2, A-108</t>
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr"/>
@@ -3456,22 +3456,22 @@
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>Doors and windows</t>
+          <t>Floors, walls and finishes</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Unseasoned teak that warps and jams.</t>
+          <t>Cement grout in bathrooms turns black.</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>Use kiln-seasoned wood, or sal / pinkado frames and UPVC on the wet side.</t>
+          <t>Use epoxy grout in wet areas.</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>A-401</t>
+          <t>A-001</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr"/>
@@ -3479,22 +3479,22 @@
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>Doors and windows</t>
+          <t>Floors, walls and finishes</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Mild-steel hinges and screws that rust with humidity and hard water.</t>
+          <t>Exterior paint that chalks and fades in strong sun.</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Use SS 304 hardware, with magnetic stoppers on every door.</t>
+          <t>Use a waterproof plaster additive and elastomeric or UV-stable exterior paint.</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>A-401</t>
+          <t>A-601</t>
         </is>
       </c>
       <c r="E76" s="8" t="inlineStr"/>
@@ -3502,22 +3502,22 @@
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>Doors and windows</t>
+          <t>Roof and rainwater</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Grill with no openable section: no way out in a fire.</t>
+          <t>Clay tiles just resting on battens: a cyclone strips the edges first.</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Give each bedroom one escape window with an openable grill.</t>
+          <t>Clip or screw every eave, verge, hip and ridge tile, plus every third row elsewhere.</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>A-401</t>
+          <t>A-110, A-501/4</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr"/>
@@ -3525,22 +3525,22 @@
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>Floors, walls and finishes</t>
+          <t>Roof and rainwater</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Skirting stuck on top of the plaster: a dust ledge that also chips.</t>
+          <t>Water creeping back under the eave tiles and into the soffit.</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Set the skirting flush with the plaster face, with a groove above it.</t>
+          <t>Use a fascia with drip-edge flashing turned down into the gutter, and raise the first tile row on a tilting fillet.</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>A-501/2</t>
+          <t>A-501/4</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr"/>
@@ -3548,22 +3548,22 @@
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>Floors, walls and finishes</t>
+          <t>Roof and rainwater</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Tiles laid tight to the walls: they pop up (tenting) in 45 C summers.</t>
+          <t>No gutters: roof water splashes the plinth and soaks the foundation.</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Leave 5 mm gaps at walls and movement joints every 15-20 ft, hidden by the skirting.</t>
+          <t>Gutters on both long eaves, downpipes into the sump filter; overflow to the road drain (no recharge pit near the walls on this narrow plot).</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>A-501/2, A-108</t>
+          <t>A-110, P-101</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr"/>
@@ -3571,22 +3571,22 @@
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>Floors, walls and finishes</t>
+          <t>Roof and rainwater</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Cement grout in bathrooms turns black.</t>
+          <t>Where the low front roof meets the two-storey wall: the joint sealed only with mortar.</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Use epoxy grout in wet areas.</t>
+          <t>Use a metal apron flashing chased into the wall with a counter-flashing.</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>A-001</t>
+          <t>A-110</t>
         </is>
       </c>
       <c r="E80" s="8" t="inlineStr"/>
@@ -3594,22 +3594,22 @@
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>Floors, walls and finishes</t>
+          <t>Roof and rainwater</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Exterior paint that chalks and fades in strong sun.</t>
+          <t>No insulation under Mangalore tiles: rooms radiate heat until midnight.</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Use a waterproof plaster additive and elastomeric or UV-stable exterior paint.</t>
+          <t>Add 50 mm insulation on the deck, ventilate the attic at ridge and soffits, and fit insulated false ceilings in bedrooms.</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>A-601</t>
+          <t>A-301, A-501/4</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr"/>
@@ -3622,17 +3622,17 @@
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Clay tiles just resting on battens: a cyclone strips the edges first.</t>
+          <t>Birds, bats and rats nesting in the roof.</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Clip or screw every eave, verge, hip and ridge tile, plus every third row elsewhere.</t>
+          <t>Bird stops at the eaves and mesh at ridge vents and soffits.</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>A-110, A-501/4</t>
+          <t>A-501/4</t>
         </is>
       </c>
       <c r="E82" s="8" t="inlineStr"/>
@@ -3640,22 +3640,22 @@
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>Roof and rainwater</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Water creeping back under the eave tiles and into the soffit.</t>
+          <t>One circuit for everything; cheap wire.</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>Use a fascia with drip-edge flashing turned down into the gutter, and raise the first tile row on a tilting fillet.</t>
+          <t>Separate MCBs for each AC, geyser, kitchen and pump; RCCB 30 mA; FR-LSH copper wire sized per load.</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>A-501/4</t>
+          <t>E-103</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr"/>
@@ -3663,22 +3663,22 @@
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>Roof and rainwater</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>No gutters: roof water splashes the plinth and soaks the foundation.</t>
+          <t>No inverter wiring planned, so it gets rewired later.</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Gutters on both long eaves, downpipes into the sump filter; overflow to the road drain (no recharge pit near the walls on this narrow plot).</t>
+          <t>Put lights, fans, office sockets and the router on a separate inverter circuit from day one.</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>A-110, P-101</t>
+          <t>E-101, E-103</t>
         </is>
       </c>
       <c r="E84" s="8" t="inlineStr"/>
@@ -3686,22 +3686,22 @@
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>Roof and rainwater</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Where the low front roof meets the two-storey wall, and at the ventilator: joints sealed only with mortar.</t>
+          <t>AC drain pipe dripping down the wall and sleeves forgotten.</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Use a metal apron flashing chased into the wall with a counter-flashing, and a 9 in upstand with flashing at the ventilator.</t>
+          <t>Fit a 65 mm sleeve sloping out, a drain to a gully, and ODU brackets on shaded walls.</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>A-110</t>
+          <t>E-103</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr"/>
@@ -3709,22 +3709,22 @@
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>Roof and rainwater</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>No insulation under Mangalore tiles: rooms radiate heat until midnight.</t>
+          <t>No spare conduits for solar PV, CCTV, the sump pump and gate.</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Add 50 mm insulation on the deck, ventilate the attic at ridge and soffits, and fit insulated false ceilings in bedrooms.</t>
+          <t>Run empty 25 mm conduits to the DB now; it costs little at this stage.</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>A-301, A-501/4</t>
+          <t>E-103, A-110</t>
         </is>
       </c>
       <c r="E86" s="8" t="inlineStr"/>
@@ -3732,22 +3732,22 @@
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>Roof and rainwater</t>
+          <t>Plumbing and water</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Birds, bats and rats nesting in the roof.</t>
+          <t>Pipes buried under the floor slab: leaks can't be found without breaking tiles.</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Bird stops at the eaves and mesh at ridge vents and soffits.</t>
+          <t>Run supply lines along the outside walls in clamps or shallow chases, with a valve per room.</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>A-501/4</t>
+          <t>P-101</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr"/>
@@ -3755,22 +3755,22 @@
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Plumbing and water</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>One circuit for everything; cheap wire.</t>
+          <t>Water tank too low over a first-floor shower: no pressure.</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Separate MCBs for each AC, geyser, kitchen and pump; RCCB 30 mA; FR-LSH copper wire sized per load.</t>
+          <t>A 1,000 L loft tank in the roof space over the upper bath, filled from the sump, plus a small pressure pump for the showers.</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>E-103</t>
+          <t>P-101, A-110</t>
         </is>
       </c>
       <c r="E88" s="8" t="inlineStr"/>
@@ -3778,22 +3778,22 @@
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Plumbing and water</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>No inverter wiring planned, so it gets rewired later.</t>
+          <t>All waste going into the septic tank, which overloads it.</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>Put lights, fans, office sockets and the router on a separate inverter circuit from day one.</t>
+          <t>Keep soil and grey water separate: soil to the septic, grey to the soak pit or a road drain, with inspection chambers at every bend.</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>E-101, E-103</t>
+          <t>P-101</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr"/>
@@ -3801,22 +3801,22 @@
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Plumbing and water</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>AC drain pipe dripping down the wall and sleeves forgotten.</t>
+          <t>Drinking borewell water without testing it (fluoride is common around Guntur).</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>Fit a 65 mm sleeve sloping out, a drain to a gully, and ODU brackets on shaded walls.</t>
+          <t>Test the water; RO at the kitchen for drinking, and a softener if hardness exceeds 300 mg/l.</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>E-103</t>
+          <t>P-101</t>
         </is>
       </c>
       <c r="E90" s="8" t="inlineStr"/>
@@ -3824,22 +3824,22 @@
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Plumbing and water</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>No spare conduits for solar PV, CCTV, the sump pump and gate.</t>
+          <t>Sump lid at ground level: surface water and insects get in.</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>Run empty 25 mm conduits to the DB now; it costs little at this stage.</t>
+          <t>Raise the sump cover 6 in above the paving with a locked, sealed lid, and keep it 20 ft+ from the septic.</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>E-103, A-110</t>
+          <t>A-101</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr"/>
@@ -3847,22 +3847,22 @@
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>Plumbing and water</t>
+          <t>Outside: yard, gate and garden</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Pipes buried under the floor slab: leaks can't be found without breaking tiles.</t>
+          <t>Gate swinging out onto the road, or too narrow for two-wheelers.</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>Run supply lines along the outside walls in clamps or shallow chases, with a valve per room.</t>
+          <t>Use a 7 ft gate swinging inward or sliding, with the meter and bell in the pillar.</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>P-101</t>
+          <t>A-101</t>
         </is>
       </c>
       <c r="E92" s="8" t="inlineStr"/>
@@ -3870,22 +3870,22 @@
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>Plumbing and water</t>
+          <t>Outside: yard, gate and garden</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>Water tank too low over a first-floor shower: no pressure.</t>
+          <t>Two-wheeler bay with no slope: puddles.</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>A 1,000 L loft tank in the roof space over the upper bath, filled from the sump, plus a small pressure pump for the showers.</t>
+          <t>Pave it sloping 1:50 toward the road drain.</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>P-101, A-110</t>
+          <t>A-101</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr"/>
@@ -3893,140 +3893,25 @@
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>Plumbing and water</t>
+          <t>Outside: yard, gate and garden</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>All waste going into the septic tank, which overloads it.</t>
+          <t>No outdoor drying space.</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>Keep soil and grey water separate: soil to the septic, grey to the soak pit or a road drain, with inspection chambers at every bend.</t>
+          <t>A fold-away clothesline in the south walkway behind the master, and more room in the spare rear land; the covered terrace also dries clothes in the monsoon.</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>P-101</t>
+          <t>A-104</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="4" t="inlineStr">
-        <is>
-          <t>Plumbing and water</t>
-        </is>
-      </c>
-      <c r="B95" s="4" t="inlineStr">
-        <is>
-          <t>Drinking borewell water without testing it (fluoride is common around Guntur).</t>
-        </is>
-      </c>
-      <c r="C95" s="4" t="inlineStr">
-        <is>
-          <t>Test the water; RO at the kitchen for drinking, and a softener if hardness exceeds 300 mg/l.</t>
-        </is>
-      </c>
-      <c r="D95" s="4" t="inlineStr">
-        <is>
-          <t>P-101</t>
-        </is>
-      </c>
-      <c r="E95" s="8" t="inlineStr"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="4" t="inlineStr">
-        <is>
-          <t>Plumbing and water</t>
-        </is>
-      </c>
-      <c r="B96" s="4" t="inlineStr">
-        <is>
-          <t>Sump lid at ground level: surface water and insects get in.</t>
-        </is>
-      </c>
-      <c r="C96" s="4" t="inlineStr">
-        <is>
-          <t>Raise the sump cover 6 in above the paving with a locked, sealed lid, and keep it 20 ft+ from the septic.</t>
-        </is>
-      </c>
-      <c r="D96" s="4" t="inlineStr">
-        <is>
-          <t>A-101</t>
-        </is>
-      </c>
-      <c r="E96" s="8" t="inlineStr"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="4" t="inlineStr">
-        <is>
-          <t>Outside: yard, gate and garden</t>
-        </is>
-      </c>
-      <c r="B97" s="4" t="inlineStr">
-        <is>
-          <t>Gate swinging out onto the road, or too narrow for two-wheelers.</t>
-        </is>
-      </c>
-      <c r="C97" s="4" t="inlineStr">
-        <is>
-          <t>Use a 7 ft gate swinging inward or sliding, with the meter and bell in the pillar.</t>
-        </is>
-      </c>
-      <c r="D97" s="4" t="inlineStr">
-        <is>
-          <t>A-101</t>
-        </is>
-      </c>
-      <c r="E97" s="8" t="inlineStr"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="4" t="inlineStr">
-        <is>
-          <t>Outside: yard, gate and garden</t>
-        </is>
-      </c>
-      <c r="B98" s="4" t="inlineStr">
-        <is>
-          <t>Two-wheeler bay with no slope: puddles.</t>
-        </is>
-      </c>
-      <c r="C98" s="4" t="inlineStr">
-        <is>
-          <t>Pave it sloping 1:50 toward the road drain.</t>
-        </is>
-      </c>
-      <c r="D98" s="4" t="inlineStr">
-        <is>
-          <t>A-101</t>
-        </is>
-      </c>
-      <c r="E98" s="8" t="inlineStr"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="4" t="inlineStr">
-        <is>
-          <t>Outside: yard, gate and garden</t>
-        </is>
-      </c>
-      <c r="B99" s="4" t="inlineStr">
-        <is>
-          <t>No outdoor drying space.</t>
-        </is>
-      </c>
-      <c r="C99" s="4" t="inlineStr">
-        <is>
-          <t>A fold-away clothesline in the south walkway behind the master, and more room in the spare rear land; the first-floor lounge also dries clothes in the monsoon.</t>
-        </is>
-      </c>
-      <c r="D99" s="4" t="inlineStr">
-        <is>
-          <t>A-104</t>
-        </is>
-      </c>
-      <c r="E99" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4226,7 +4111,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Truss holding-down bolts, membrane and insulation, edge tiles clipped, flashings at the ventilator and valleys</t>
+          <t>Truss holding-down bolts, membrane and insulation, edge tiles clipped, flashing where the front gable meets the two-storey wall</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -4643,7 +4528,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Covered terrace and lounge: deep shade from the main roof keeps the slab over the living cool; the upper master's west wall stays solid; chiks on the open west and south sides</t>
+          <t>Covered terrace: deep shade from the main roof keeps the slab over the living cool; the upper master's west wall has only a small high vent; chiks on the terrace's south and east sides</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -4718,7 +4603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B56"/>
+  <dimension ref="A1:B57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4743,7 +4628,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Duplex option (branch feature/duplex): the house is planned on the front 55 ft of the plot (the back 20 ft stays spare land) as a 44 ft x 22 ft two-level house, 968 sq ft on the ground floor and about 330 sq ft enclosed on the first floor plus a covered outdoor lounge and a 16 x 22 ft covered terrace.</t>
+          <t>Duplex option (branch feature/duplex): the house is planned on the front 55 ft of the plot (the back 20 ft stays spare land) as a 44 ft x 22 ft two-level house, 968 sq ft on the ground floor and about 445 sq ft enclosed on the first floor plus a 16 x 22 ft covered terrace.</t>
         </is>
       </c>
     </row>
@@ -4763,7 +4648,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Ground floor: master bedroom with its bath (south-west), small bedroom, common bath, lobby and a dog-leg stair seen from the living through a timber jali. First floor: upper master with a dressing room and bath, a landing, a passage, a covered outdoor lounge on the north side and the covered terrace.</t>
+          <t>Ground floor: master bedroom with its bath (south-west), small bedroom, common bath, lobby and a dog-leg stair seen from the living through a timber jali. First floor: upper master with a dressing room and bath, a landing, a passage and the covered terrace; the upper master has a sitting and study zone on the north side (the outdoor lounge was merged into it once the terrace was added).</t>
         </is>
       </c>
     </row>
@@ -4783,7 +4668,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>All four bath fittings stack in the south band (two baths over two); the septic tank and soak pit move to the spare rear land behind the baths, freeing the front yard; the water tank goes into the roof space (no tank stand).</t>
+          <t>No ridge ventilator (removed after review): with the terrace open on three sides, hot air under the main roof escapes at its open edges; the attic over the first-floor rooms is vented by meshed ridge and soffit vents.</t>
         </is>
       </c>
     </row>
@@ -4793,7 +4678,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Site is in Guntur, Andhra Pradesh (farm land), not Kerala; Kerala style kept, construction adapted to local climate and soil.</t>
+          <t>All four bath fittings stack in the south band (two baths over two); the septic tank and soak pit move to the spare rear land behind the baths, freeing the front yard; the water tank goes into the roof space (no tank stand).</t>
         </is>
       </c>
     </row>
@@ -4803,7 +4688,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>RCC frame with AAC block walls: 9 in outer, 5 in inner, 7 in where plumbing is concealed.</t>
+          <t>Site is in Guntur, Andhra Pradesh (farm land), not Kerala; Kerala style kept, construction adapted to local climate and soil.</t>
         </is>
       </c>
     </row>
@@ -4813,7 +4698,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Plinth 2 ft above finished ground; poomukham 6 in lower; bathrooms 12 mm lower with no raised threshold.</t>
+          <t>RCC frame with AAC block walls: 9 in outer, 5 in inner, 7 in where plumbing is concealed.</t>
         </is>
       </c>
     </row>
@@ -4823,7 +4708,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>AC provisions (points, sleeves, drain, outdoor-unit brackets) in both bedrooms, the office and living; passive cooling first.</t>
+          <t>Plinth 2 ft above finished ground; poomukham 6 in lower; bathrooms 12 mm lower with no raised threshold.</t>
         </is>
       </c>
     </row>
@@ -4833,7 +4718,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Flat insulated false ceilings in bedrooms, offices, baths and kitchen; sloped ceilings in living, dining and verandah.</t>
+          <t>AC provisions (points, sleeves, drain, outdoor-unit brackets) in both bedrooms, the office and living; passive cooling first.</t>
         </is>
       </c>
     </row>
@@ -4843,7 +4728,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>No glass skylight: the dining gets borrowed daylight from the living, the nook window and the hall; a louvred ventilator lantern above it lets hot air out (no glass, so no greenhouse heat).</t>
+          <t>Flat insulated false ceilings in bedrooms, offices, baths and kitchen; sloped ceilings in living, dining and verandah.</t>
         </is>
       </c>
     </row>
@@ -4853,7 +4738,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Service band on south (heat buffer); bedrooms and living get north light.</t>
+          <t>No glass skylight: the dining gets borrowed daylight from the living, the nook window and the hall; a louvred ventilator lantern above it lets hot air out (no glass, so no greenhouse heat).</t>
         </is>
       </c>
     </row>
@@ -4863,7 +4748,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Kitchen in SE; stove on east wall; open wet area onto the walkway; provisions in bench drawers, kitchen cabinets and lofts (no separate store).</t>
+          <t>Service band on south (heat buffer); bedrooms and living get north light.</t>
         </is>
       </c>
     </row>
@@ -4873,7 +4758,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Bedroom doors widened to 3 ft; bathroom, office and store doors 2 ft 6 in.</t>
+          <t>Kitchen in SE; stove on east wall; open wet area onto the walkway; provisions in bench drawers, kitchen cabinets and lofts (no separate store).</t>
         </is>
       </c>
     </row>
@@ -4883,7 +4768,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Thirty-second review: TV back on the west wall of the hall (Bedroom 2's east wall), sofa facing west about 7'-6" away in the dining bay, coffee table between, the window seat shortened to 4 ft as side seating; the dining space under the ventilator is open again.</t>
+          <t>Bedroom doors widened to 3 ft; bathroom, office and store doors 2 ft 6 in.</t>
         </is>
       </c>
     </row>
@@ -4893,7 +4778,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Thirty-first review (front facade): gate re-centred on the main door with a 6 ft stone forecourt and the tulsi thara on the axis (gate, tulsi, steps, door, hall, lamp niche in one line); charupadi seats with sloping backrests between the verandah pillars, flanking the steps; carved teak barge boards and a brass kalasham finial on the front gable; the kitchen front clad in exposed laterite with a deep projecting teak frame to its window; carved teak main door with brass studs, a stone surround and a nameplate niche; warm uplights at the pillars, a lantern by the door and gate-post lights; low hedges screening the sump and the two-wheeler bay; a pair of potted palms beside the steps.</t>
+          <t>Thirty-second review: TV back on the west wall of the hall (Bedroom 2's east wall), sofa facing west about 7'-6" away in the dining bay, coffee table between, the window seat shortened to 4 ft as side seating; the dining space under the ventilator is open again.</t>
         </is>
       </c>
     </row>
@@ -4903,7 +4788,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Thirtieth review (proportion clean-up): windows standardised to three sizes (6 ft rooms, 3 ft small, 2 ft baths) with every head at 7 ft and three sill levels (3 ft rooms, 3'-6" over counters, 5 ft baths); sunshades only on the sunny south, east and west walls (the eaves shade the north); floors cut to three families plus the verandah (red oxide in all public rooms and the pooja, vitrified in bedrooms, anti-skid ceramic in kitchen, baths and wet area, granite on the verandah); services hidden (pipes in chases, outdoor units grouped behind jali on the north wall), switchboards aligned, warm layered lighting, handle-less built-in fronts.</t>
+          <t>Thirty-first review (front facade): gate re-centred on the main door with a 6 ft stone forecourt and the tulsi thara on the axis (gate, tulsi, steps, door, hall, lamp niche in one line); charupadi seats with sloping backrests between the verandah pillars, flanking the steps; carved teak barge boards and a brass kalasham finial on the front gable; the kitchen front clad in exposed laterite with a deep projecting teak frame to its window; carved teak main door with brass studs, a stone surround and a nameplate niche; warm uplights at the pillars, a lantern by the door and gate-post lights; low hedges screening the sump and the two-wheeler bay; a pair of potted palms beside the steps.</t>
         </is>
       </c>
     </row>
@@ -4913,7 +4798,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Twenty-ninth review: compound wall made as thin as practical: precast RCC post-and-panel (2 in panels in 4 in posts) set just inside the plot line, so the side strips stay walkable and the north run can be lifted and moved if more land is bought.</t>
+          <t>Thirtieth review (proportion clean-up): windows standardised to three sizes (6 ft rooms, 3 ft small, 2 ft baths) with every head at 7 ft and three sill levels (3 ft rooms, 3'-6" over counters, 5 ft baths); sunshades only on the sunny south, east and west walls (the eaves shade the north); floors cut to three families plus the verandah (red oxide in all public rooms and the pooja, vitrified in bedrooms, anti-skid ceramic in kitchen, baths and wet area, granite on the verandah); services hidden (pipes in chases, outdoor units grouped behind jali on the north wall), switchboards aligned, warm layered lighting, handle-less built-in fronts.</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4808,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Twenty-eighth review: TV lounge reworked: sofa brought forward to about 8 ft from the TV, a 3 ft walk behind it, and a built-in window seat (charupadi-style enclave) under the dining-bay window, so the sofa backs onto a quiet seating nook rather than the entrance and nobody walks in front of the TV.</t>
+          <t>Twenty-ninth review: compound wall made as thin as practical: precast RCC post-and-panel (2 in panels in 4 in posts) set just inside the plot line, so the side strips stay walkable and the north run can be lifted and moved if more land is bought.</t>
         </is>
       </c>
     </row>
@@ -4933,7 +4818,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Twenty-seventh review: TV lounge moves to the open dining space under the ventilator: TV on the north face of the common-bath wall, sofa facing south with its back to the north window, so the main door is in side view, not behind (commanding position) and the TV no longer faces the main door; the dining bay becomes a reading / dining nook with a chair by the window.</t>
+          <t>Twenty-eighth review: TV lounge reworked: sofa brought forward to about 8 ft from the TV, a 3 ft walk behind it, and a built-in window seat (charupadi-style enclave) under the dining-bay window, so the sofa backs onto a quiet seating nook rather than the entrance and nobody walks in front of the TV.</t>
         </is>
       </c>
     </row>
@@ -4943,7 +4828,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Twenty-sixth review: built-in ideas borrowed and adapted (function, not style, in Kerala materials): recessed shower niches, mirror cabinets over basins, genkan-style shoe bench with hooks and a granite threshold band, vilakku madam lamp niche facing the main door, floating bedside shelves (walls too thin for recesses), drawers-first kitchen with a masala pull-out and utensil rail, dish-drying rack over the utility sink, ceiling clothes airer in the wet area.</t>
+          <t>Twenty-seventh review: TV lounge moves to the open dining space under the ventilator: TV on the north face of the common-bath wall, sofa facing south with its back to the north window, so the main door is in side view, not behind (commanding position) and the TV no longer faces the main door; the dining bay becomes a reading / dining nook with a chair by the window.</t>
         </is>
       </c>
     </row>
@@ -4953,7 +4838,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Twenty-fifth review: main door moved 3'-4" south (y 17'-7" to 20'-7"), centred under the front gable and opening straight onto the 5 ft walk between the pooja and the diwan; shoe cupboard to its north on the east wall; window diwan back to 6 ft along the north window, out of the door's line; steps, middle verandah pillars and the swing realigned.</t>
+          <t>Twenty-sixth review: built-in ideas borrowed and adapted (function, not style, in Kerala materials): recessed shower niches, mirror cabinets over basins, genkan-style shoe bench with hooks and a granite threshold band, vilakku madam lamp niche facing the main door, floating bedside shelves (walls too thin for recesses), drawers-first kitchen with a masala pull-out and utensil rail, dish-drying rack over the utility sink, ceiling clothes airer in the wet area.</t>
         </is>
       </c>
     </row>
@@ -4963,7 +4848,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Twenty-fourth review: planned on the 27 ft plot alone (north strip dropped for now): roof eaves cut from 2'-6" to 2'-0" so the north eave stays inside the plot line, septic tank moved under the two-wheeler bay in the front yard with a lined soak pit beside it, all drains rerouted along the south walkway to the front, rainwater to the sump with overflow to the road; north-strip trees and recharge pit removed.</t>
+          <t>Twenty-fifth review: main door moved 3'-4" south (y 17'-7" to 20'-7"), centred under the front gable and opening straight onto the 5 ft walk between the pooja and the diwan; shoe cupboard to its north on the east wall; window diwan back to 6 ft along the north window, out of the door's line; steps, middle verandah pillars and the swing realigned.</t>
         </is>
       </c>
     </row>
@@ -4973,7 +4858,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Twenty-third review: the fridge moves out of the kitchen into the dining alcove beside the kitchen door, against the wet-area wall; the kitchen's north wall is now free.</t>
+          <t>Twenty-fourth review: planned on the 27 ft plot alone (north strip dropped for now): roof eaves cut from 2'-6" to 2'-0" so the north eave stays inside the plot line, septic tank moved under the two-wheeler bay in the front yard with a lined soak pit beside it, all drains rerouted along the south walkway to the front, rainwater to the sump with overflow to the road; north-strip trees and recharge pit removed.</t>
         </is>
       </c>
     </row>
@@ -4983,7 +4868,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Twenty-second review: the kitchen's tall pantry and the dining table and chairs are removed at the owner's request; the dining space under the ventilator stays open (the pendant light and points stay for a table later).</t>
+          <t>Twenty-third review: the fridge moves out of the kitchen into the dining alcove beside the kitchen door, against the wet-area wall; the kitchen's north wall is now free.</t>
         </is>
       </c>
     </row>
@@ -4993,7 +4878,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Twenty-first review: the open hall becomes three zones: family TV lounge in the dining bay (5'-6" sofa facing the TV), dining under the ventilator moved 9 in south (about 2 ft behind the chairs on both sides), and guest sitting by the main door with a 4'-6" window diwan (shortened after the walk-through showed a 1'-6" pinch at the shoe cupboard) and an armchair under the living's north window; a clear walk of about 4'-11" from the main door to the dining and kitchen, pooja front kept clear.</t>
+          <t>Twenty-second review: the kitchen's tall pantry and the dining table and chairs are removed at the owner's request; the dining space under the ventilator stays open (the pendant light and points stay for a table later).</t>
         </is>
       </c>
     </row>
@@ -5003,7 +4888,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Twentieth review: Bedroom 2's bed moves to the east wall, head east, leaving an 8 x 14 ft open floor from the door to the bath and window; wardrobe to the west wall (sound buffer to the master), work table north of the bed, AC on the bath's outer wall; dresser dropped (mirror on the wardrobe).</t>
+          <t>Twenty-first review: the open hall becomes three zones: family TV lounge in the dining bay (5'-6" sofa facing the TV), dining under the ventilator moved 9 in south (about 2 ft behind the chairs on both sides), and guest sitting by the main door with a 4'-6" window diwan (shortened after the walk-through showed a 1'-6" pinch at the shoe cupboard) and an armchair under the living's north window; a clear walk of about 4'-11" from the main door to the dining and kitchen, pooja front kept clear.</t>
         </is>
       </c>
     </row>
@@ -5013,7 +4898,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
+          <t>Twentieth review: Bedroom 2's bed moves to the east wall, head east, leaving an 8 x 14 ft open floor from the door to the bath and window; wardrobe to the west wall (sound buffer to the master), work table north of the bed, AC on the bath's outer wall; dresser dropped (mirror on the wardrobe).</t>
         </is>
       </c>
     </row>
@@ -5023,7 +4908,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
+          <t>Nineteenth review: with Bedroom 2 at 17 ft, its bed turns head-south in the middle of the room (2 ft+ on both sides, under the jali); Bath 2 grows to 7' x 7' (6'-7" x 6'-4" clear) with a 3' x 3'-6" wet zone, basin in the dry zone and the door on its east wall; a dresser takes the west wall; work table and wardrobe stay on the east wall.</t>
         </is>
       </c>
     </row>
@@ -5033,7 +4918,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
+          <t>Eighteenth review: house lengthened 2 ft to 62 ft, all of it added to Bedroom 2 (now 17 ft wide; the sitting area below it also gains 2 ft); front yard 10 ft to 8 ft (check the front setback). Bedroom 2 window back to 6 ft.</t>
         </is>
       </c>
     </row>
@@ -5043,7 +4928,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
+          <t>Seventeenth review: sitting area gets a 5 ft tall storage cupboard on the south wall between the bench and the window; the hand-wash basin moves to the east end of the serving counter, just outside the common bath, for washing up after meals.</t>
         </is>
       </c>
     </row>
@@ -5053,7 +4938,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
+          <t>Sixteenth review (independent Indian-architect review): Bath 2 re-planned 7' x 6' so Bedroom 2's bed (head west) has 1'-6" on both sides, work table to the east wall. Kitchen entered only from the dining-side door (hinged, 3 ft); the north sliding door is walled up so the pooja front is quiet, and a tall pantry takes the north wall. East kitchen window cut to 2 ft so the hob and chimney sit on solid wall. Septic tank moved 6 ft+ from the house and the soak pit replaced by a soak trench. Ensuite door opens outward; common bath WC side clearance 17 in, door rehung at the north jamb with a closer, geyser and shower off the window. DB moved to the dining face of Bedroom 2's east wall.</t>
         </is>
       </c>
     </row>
@@ -5063,7 +4948,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
+          <t>Fifteenth review: TV moves to Bedroom 2's east wall facing the dining bay (the bay becomes the TV lounge; sofa faces west, living AC above the TV). Master bed moves 3'-10" south toward the bay, freeing a 9 x 7 ft zone by the north window and ensuite door with a window seat. Bedroom 2's door moves to the east end of its south wall. Bath 2's door moves to its east wall (basin to its south wall) so Bedroom 2's bed sits in the strip between the bath and the sitting area, head west on the master wall, leaving the middle of the room open.</t>
         </is>
       </c>
     </row>
@@ -5073,7 +4958,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
+          <t>Fourteenth review (designer review): Bath 2 moves into Bedroom 2's own north-west corner, made 5'-6" x 7'-6" (about 5'-0" x 6'-11" clear) for a 3' x 3'-6" wet zone and a WC with 15 in each side and the master gets back its full room, bed position and 6 ft window. Bath doors open outward (common bath door moved to the sitting-area side, off the dining). Pooja moves 3'-6" south, back to back with the kitchen, with doors opening inward; the fridge moves into the kitchen; a shoe cupboard takes the freed wall beside the main door. Second kitchen door (sliding) straight to the dining. Bedroom 2's south-east corner is notched 1' x 1'-6" so the way from the dining into the sitting area is about 4'-2" instead of 3'-3"; Bedroom 2 gets a real queen bed, a 6 ft window and a high jali vent to the sitting area. Handrail at the entrance steps, grab bars in the baths.</t>
         </is>
       </c>
     </row>
@@ -5083,7 +4968,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
+          <t>Common bath widened to 6'-6" x 6' (about 6'-0" x 5'-5" clear: 3 x 3 ft shower, WC and basin on the wet wall) by taking 1'-6" from the east end of the sitting area; serving counter now 6 ft.</t>
         </is>
       </c>
     </row>
@@ -5093,7 +4978,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
+          <t>Twelfth review: Bath 2 becomes a common bath in the old pooja bay beside the wet area (5 x 6 ft, door from the sitting area, WC and basin on the shared wet wall, drains straight to the south walkway); Bedroom 2 is a clean room with no attached bath; wet area narrowed to 5 ft. Hall kept on the south so bedrooms keep their north windows.</t>
         </is>
       </c>
     </row>
@@ -5103,7 +4988,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
+          <t>Eleventh review: the corner between the pooja and the kitchen becomes part of the kitchen and holds the fridge; the kitchen entrance moves from the dining side to the north (3 ft sliding glass door from the living); the old fridge spot extends the south counter.</t>
         </is>
       </c>
     </row>
@@ -5113,7 +4998,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
+          <t>Tenth review: main door moved to the north end of the east wall and the pooja 3'-6" north with it, freeing the living's south-east corner beside the kitchen; verandah steps, pillars and swing realigned to the door; TV taken off the east wall (new position open).</t>
         </is>
       </c>
     </row>
@@ -5123,7 +5008,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
+          <t>Ninth review: pooja moved to the east side, in the living's south-east corner beside the main door and back to back with the kitchen (4 x 4 ft, opens west, idols face west, family faces east). Main door moved 2'-4" north and the TV unit trimmed to suit; the old pooja bay joins the sitting area.</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5018,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
+          <t>Eighth review: plot 5 ft longer, so the house grows to 60 ft. The master stays 9'-6" x 14' (bay 7 x 8 ft, full-width wardrobe, light from the workstation window; the bay's own south window dropped). Bedroom 2 grows to 15 ft wide, the sitting area to 20 x 7'-6" (Bedroom 2 gives up 1'-6" of depth, now 15 x 14'-6") and the dining to 11 ft; the plot centre now falls in the dining, west of the ventilator (Vastu to confirm).</t>
         </is>
       </c>
     </row>
@@ -5143,7 +5028,7 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
+          <t>Seventh review: Bedroom 2 enlarged to 12 x 16 ft by taking the hall strip; its door opens from the sitting area (as the master suite does); hand-wash basin back at the west end of the serving counter.</t>
         </is>
       </c>
     </row>
@@ -5153,7 +5038,7 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
+          <t>Sixth review: Office 2 walls and sliding door left out for now (open workstation in the master suite, walls can be added later); Bedroom 2 becomes a study-guest room: work table with monitor beside the bath, sofa-cum-bed instead of a queen bed.</t>
         </is>
       </c>
     </row>
@@ -5163,7 +5048,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
+          <t>Office 1 removed after family review: one office (Office 2) inside the master suite; Bedroom 2 has its own work desk.</t>
         </is>
       </c>
     </row>
@@ -5173,7 +5058,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
+          <t>Common bathroom moved to the north side (old pooja spot), entered from the dining corner next to the hall.</t>
         </is>
       </c>
     </row>
@@ -5183,7 +5068,7 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
+          <t>Second family review: store (8 x 8 ft) moved next to the bedrooms; pooja reduced to a small shrine opening onto the hall (idols face east); wet area moved west (9 x 8 ft); kitchen 14 x 10 ft with a 5 ft sliding entry from the living; dining gains a basin and crockery nook with a south window; TV moved to the living room's east wall.</t>
         </is>
       </c>
     </row>
@@ -5193,7 +5078,7 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
+          <t>Pooja moved beside the wet area and opened to the west (idols face west, the family sits in the nook facing east); shared wall kept dry with no pipes, pooja floor 3 in higher; basin nook shifted west.</t>
         </is>
       </c>
     </row>
@@ -5203,7 +5088,7 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
+          <t>Fifth review: Bedroom 2 made one 12 x 12 ft rectangle with a rectangular private bath (north-west corner, outer wall) and its wardrobe on the east wall; the leftover corner at the hall's west end is an open hand-wash corner; serving counter now 9 ft without a basin.</t>
         </is>
       </c>
     </row>
@@ -5213,7 +5098,7 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
+          <t>Fourth review: Bath 2 made Bedroom 2's private bath (no common toilet); master suite entered through its bay from the sitting area; the old Bath 2 spot opens to the dining with a north window; family store merged back into the master bedroom as a wardrobe bay; inverter under the sitting-area bench.</t>
         </is>
       </c>
     </row>
@@ -5223,7 +5108,7 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
+          <t>Earlier: walk-in wardrobe turned into a family store with a lockable door from the sitting area (inverter inside); built-in sliding wardrobes in the dressing alcove and on the master bedroom's south wall.</t>
         </is>
       </c>
     </row>
@@ -5233,7 +5118,7 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
+          <t>Store wall removed: the strip from the walk-in to the pooja is one open sitting and serving area with a storage bench; hand-wash basin set into the west end of the serving counter, about 8 ft from the pooja, draining straight out to the south walkway.</t>
         </is>
       </c>
     </row>
@@ -5243,7 +5128,7 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
+          <t>Wet area reduced to 6 x 6 ft and left open on its south side to the walkway (service route from the kitchen to the back of the house); kitchen door moved to face the dining (3 ft sliding glass); basin nook widened to 8 ft with a 6 ft serving counter.</t>
         </is>
       </c>
     </row>
@@ -5253,7 +5138,7 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
+          <t>Main door moved to the south part of the living's east wall (still north of the house's centre line); TV on the north part of that wall; steps, swing and arugu seats rearranged on the poomukham.</t>
         </is>
       </c>
     </row>
@@ -5263,7 +5148,7 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
+          <t>Third review: hall widened to about 6 ft clear (store, pooja and basin nook made 6 ft deep) so the family can sit facing the pooja; store left open to the hall for now (a wall and door can be added later); broom closet dropped, tall utility cupboard in the wet area instead.</t>
         </is>
       </c>
     </row>
@@ -5273,7 +5158,7 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+          <t>Earlier: hall widened to 4 ft clear (Bedroom 2 gives up 6 in); vents above the office, walk-in, store, pooja and kitchen doors; none at bedrooms or bathrooms (sound privacy).</t>
         </is>
       </c>
     </row>
@@ -5282,6 +5167,16 @@
         <v>55</v>
       </c>
       <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>Ensuite widened by 1'-6" into the master (about 6'-0" x 7'-4" clear); dressing widened by the same strip; master now 9'-6" x 14'-0".</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
         <is>
           <t>Roof: Mangalore clay tiles on steel truss over insulated cement-fibre deck; all edge tiles mechanically fixed.</t>
         </is>
@@ -6109,7 +6004,7 @@
         <v>11.41</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>11.91</v>
+        <v>12.12</v>
       </c>
       <c r="J15" s="5">
         <f>H15*I15</f>
@@ -6347,7 +6242,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Outdoor lounge (covered) (1st floor)</t>
+          <t>Sitting and study (upper master) (1st floor)</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -6370,10 +6265,10 @@
         <v/>
       </c>
       <c r="H20" s="5" t="n">
-        <v>11.79</v>
+        <v>11.41</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>9.289999999999999</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="J20" s="5">
         <f>H20*I20</f>
@@ -6381,17 +6276,17 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>+11'-9"</t>
+          <t>+12'-0"</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>Sloped (exposed rafters)</t>
+          <t>Flat 9'-6"</t>
         </is>
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>Covered by the main roof, railings on two sides</t>
+          <t>Part of the upper master suite, divided by the wardrobe</t>
         </is>
       </c>
     </row>
@@ -6495,7 +6390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -7014,16 +6909,16 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>D34</t>
+          <t>D36</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Outdoor lounge (from the upper passage)</t>
+          <t>Covered terrace (from the landing, opens outward)</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>7</v>
@@ -7045,76 +6940,6 @@
       </c>
       <c r="H15" s="8" t="inlineStr"/>
       <c r="I15" s="8" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>D35</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Upper master to the outdoor lounge</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D16" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>Hinged, single</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>Teak frame, glazed, 3 ft</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H16" s="8" t="inlineStr"/>
-      <c r="I16" s="8" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>D36</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Covered terrace (from the landing, opens outward)</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="D17" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>Hinged, single</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Teak frame, glazed, 3 ft</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H17" s="8" t="inlineStr"/>
-      <c r="I17" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7772,16 +7597,16 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Upper master bedroom (1st floor)</t>
+          <t>Sitting and study (upper master) (1st floor)</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Inside</t>
+          <t>North</t>
         </is>
       </c>
       <c r="D18" s="9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E18" s="9" t="n">
         <v>3</v>
@@ -7795,7 +7620,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Teak casement, glazed (opens onto the lounge)</t>
+          <t>Teak casement, glazed (6 ft, north light for the desk and reading)</t>
         </is>
       </c>
       <c r="I18" s="8" t="inlineStr"/>
@@ -7803,27 +7628,27 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>W40</t>
+          <t>W41</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Stair (1st floor)</t>
+          <t>Sitting and study (upper master) (1st floor)</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Inside</t>
+          <t>West</t>
         </is>
       </c>
       <c r="D19" s="9" t="n">
-        <v>9.5</v>
+        <v>2</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G19" s="9">
         <f>F19-E19</f>
@@ -7831,7 +7656,7 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Timber jali screen between the stair well and the covered terrace (light and air for the stair)</t>
+          <t>High jali vent (west, cross-ventilation)</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr"/>
@@ -7839,26 +7664,35 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>SK1</t>
+          <t>W40</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Roof</t>
+          <t>Stair (1st floor)</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Up</t>
-        </is>
-      </c>
-      <c r="D20" s="9" t="inlineStr"/>
-      <c r="E20" s="9" t="inlineStr"/>
-      <c r="F20" s="9" t="inlineStr"/>
-      <c r="G20" s="9" t="inlineStr"/>
+          <t>Inside</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="G20" s="9">
+        <f>F20-E20</f>
+        <v/>
+      </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Ventilator on the main ridge over the covered terrace, 4'-6" square, no glass: hipped tiled cap at 30 deg with 1'-6" overhang; 2 ft band of 45 deg louvres on all four sides; SS bird mesh behind; 9 in upstand (see A-503). Lets the hot air under the tiles out</t>
+          <t>Timber jali screen between the stair well and the covered terrace (light and air for the stair)</t>
         </is>
       </c>
       <c r="I20" s="8" t="inlineStr"/>
@@ -7901,7 +7735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8681,7 +8515,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Under-stair cupboard (DB, inverter, brooms), opens to the lobby</t>
+          <t>Under-stair cupboard where the stair drops below 7 ft (DB, inverter, brooms), doors facing the lobby</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -8693,7 +8527,7 @@
         <v>3.4</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="G18" s="4" t="n">
         <v>1</v>
@@ -9918,36 +9752,36 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>F80</t>
+          <t>F90</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Outdoor lounge (covered)</t>
+          <t>Sitting and study (upper master)</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Built-in diwan 6' along the north rail (cushions, bolsters)</t>
+          <t>Built-in wardrobe 6' as a part divider between the sleeping and sitting zones, lofts above</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E47" s="4" t="n">
         <v>6</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="G47" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>Teak, weatherproof cushions</t>
+          <t>Ply + laminate, 2 ft deep</t>
         </is>
       </c>
       <c r="I47" s="10" t="n"/>
@@ -9961,17 +9795,17 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>F81</t>
+          <t>F91</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Outdoor lounge (covered)</t>
+          <t>Sitting and study (upper master)</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Cane armchair</t>
+          <t>Work desk 4' x 2' on the west wall (north window to the side)</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -9980,17 +9814,17 @@
         </is>
       </c>
       <c r="E48" s="4" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>1.8</v>
+        <v>4</v>
       </c>
       <c r="G48" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>Cane</t>
+          <t>Teak / ply, cable tray</t>
         </is>
       </c>
       <c r="I48" s="10" t="n"/>
@@ -10004,17 +9838,17 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>F82</t>
+          <t>F94</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Outdoor lounge (covered)</t>
+          <t>Sitting and study (upper master)</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Low coffee table</t>
+          <t>Window diwan 5' under the north window, drawers below</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -10023,17 +9857,17 @@
         </is>
       </c>
       <c r="E49" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="G49" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>Teak</t>
+          <t>Teak, cotton cushions</t>
         </is>
       </c>
       <c r="I49" s="10" t="n"/>
@@ -10047,36 +9881,36 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>F83</t>
+          <t>F93</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Upper passage</t>
+          <t>Sitting and study (upper master)</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Open bookshelf at the end of the passage (reading nook)</t>
+          <t>Reading chair</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Built-in joinery</t>
+          <t>Loose furniture</t>
         </is>
       </c>
       <c r="E50" s="4" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>4.6</v>
+        <v>1.8</v>
       </c>
       <c r="G50" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H50" s="4" t="inlineStr">
         <is>
-          <t>Teak / ply, open shelves</t>
+          <t>Cane / upholstered</t>
         </is>
       </c>
       <c r="I50" s="10" t="n"/>
@@ -10090,36 +9924,36 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>F84</t>
+          <t>F95</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Covered terrace</t>
+          <t>Sitting and study (upper master)</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Built-in diwan 6' against the stair wall (cushions, bolsters, storage below)</t>
+          <t>Open bookshelf on the passage wall</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E51" s="4" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G51" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>Teak, weatherproof cushions</t>
+          <t>Teak / ply, open shelves</t>
         </is>
       </c>
       <c r="I51" s="10" t="n"/>
@@ -10133,36 +9967,36 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>F85</t>
+          <t>F83</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Covered terrace</t>
+          <t>Upper passage</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Low coffee table</t>
+          <t>Open bookshelf at the end of the passage (reading nook)</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>Loose furniture</t>
+          <t>Built-in joinery</t>
         </is>
       </c>
       <c r="E52" s="4" t="n">
-        <v>2.5</v>
+        <v>1.2</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>3</v>
+        <v>4.6</v>
       </c>
       <c r="G52" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H52" s="4" t="inlineStr">
         <is>
-          <t>Teak</t>
+          <t>Teak / ply, open shelves</t>
         </is>
       </c>
       <c r="I52" s="10" t="n"/>
@@ -10176,7 +10010,7 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>F86</t>
+          <t>F84</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
@@ -10186,7 +10020,7 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Cane armchair</t>
+          <t>Built-in diwan 6' against the stair wall (cushions, bolsters, storage below)</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -10195,17 +10029,17 @@
         </is>
       </c>
       <c r="E53" s="4" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>1.8</v>
+        <v>6</v>
       </c>
       <c r="G53" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>Cane</t>
+          <t>Teak, weatherproof cushions</t>
         </is>
       </c>
       <c r="I53" s="10" t="n"/>
@@ -10219,7 +10053,7 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>F87</t>
+          <t>F85</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -10229,7 +10063,7 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Cane armchair</t>
+          <t>Low coffee table</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -10238,17 +10072,17 @@
         </is>
       </c>
       <c r="E54" s="4" t="n">
-        <v>1.8</v>
+        <v>2.5</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>1.8</v>
+        <v>3</v>
       </c>
       <c r="G54" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t>Cane</t>
+          <t>Teak</t>
         </is>
       </c>
       <c r="I54" s="10" t="n"/>
@@ -10262,7 +10096,7 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>F88</t>
+          <t>F86</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
@@ -10272,7 +10106,7 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Clothes-drying rails hung from the steel frame (dry in the monsoon, out of sight from the road)</t>
+          <t>Cane armchair</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -10281,17 +10115,17 @@
         </is>
       </c>
       <c r="E55" s="4" t="n">
-        <v>8</v>
+        <v>1.8</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="G55" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>Aluminium rails on pulleys</t>
+          <t>Cane</t>
         </is>
       </c>
       <c r="I55" s="10" t="n"/>
@@ -10305,7 +10139,7 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>F89</t>
+          <t>F87</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -10315,7 +10149,7 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Planter boxes along the east railing</t>
+          <t>Cane armchair</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -10324,17 +10158,17 @@
         </is>
       </c>
       <c r="E56" s="4" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>11</v>
+        <v>1.8</v>
       </c>
       <c r="G56" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H56" s="4" t="inlineStr">
         <is>
-          <t>Ferrocement, drained to the terrace drain</t>
+          <t>Cane</t>
         </is>
       </c>
       <c r="I56" s="10" t="n"/>
@@ -10346,28 +10180,114 @@
       <c r="L56" s="8" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="6" t="inlineStr"/>
-      <c r="B57" s="6" t="inlineStr"/>
-      <c r="C57" s="6" t="inlineStr">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>F88</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>Covered terrace</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Clothes-drying rails hung from the steel frame (dry in the monsoon, out of sight from the road)</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>Loose furniture</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F57" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G57" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>Aluminium rails on pulleys</t>
+        </is>
+      </c>
+      <c r="I57" s="10" t="n"/>
+      <c r="J57" s="11">
+        <f>G57*I57</f>
+        <v/>
+      </c>
+      <c r="K57" s="8" t="inlineStr"/>
+      <c r="L57" s="8" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>F89</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Covered terrace</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Planter boxes along the east railing</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Loose furniture</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F58" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="G58" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>Ferrocement, drained to the terrace drain</t>
+        </is>
+      </c>
+      <c r="I58" s="10" t="n"/>
+      <c r="J58" s="11">
+        <f>G58*I58</f>
+        <v/>
+      </c>
+      <c r="K58" s="8" t="inlineStr"/>
+      <c r="L58" s="8" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr"/>
+      <c r="B59" s="6" t="inlineStr"/>
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D57" s="6" t="inlineStr"/>
-      <c r="E57" s="6" t="inlineStr"/>
-      <c r="F57" s="6" t="inlineStr"/>
-      <c r="G57" s="6">
-        <f>SUM(G2:G56)</f>
-        <v/>
-      </c>
-      <c r="H57" s="6" t="inlineStr"/>
-      <c r="I57" s="12" t="inlineStr"/>
-      <c r="J57" s="12">
-        <f>SUM(J2:J56)</f>
-        <v/>
-      </c>
-      <c r="K57" s="6" t="inlineStr"/>
-      <c r="L57" s="6" t="inlineStr"/>
+      <c r="D59" s="6" t="inlineStr"/>
+      <c r="E59" s="6" t="inlineStr"/>
+      <c r="F59" s="6" t="inlineStr"/>
+      <c r="G59" s="6">
+        <f>SUM(G2:G58)</f>
+        <v/>
+      </c>
+      <c r="H59" s="6" t="inlineStr"/>
+      <c r="I59" s="12" t="inlineStr"/>
+      <c r="J59" s="12">
+        <f>SUM(J2:J58)</f>
+        <v/>
+      </c>
+      <c r="K59" s="6" t="inlineStr"/>
+      <c r="L59" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10647,7 +10567,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Outdoor lounge and covered terrace (first floor)</t>
+          <t>Covered terrace (first floor)</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -10657,7 +10577,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Railing 3'-6" on the open sides (teak cap, MS or teak balusters); bamboo chiks on the west and south</t>
+          <t>Railing 3'-6" on the open sides (teak cap, MS or teak balusters); bamboo chiks on the south and east</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -10667,7 +10587,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Slab waterproofing and a 48 h flood test before tiling: both sit over bedrooms and the living</t>
+          <t>Slab waterproofing and a 48 h flood test before tiling: it sits over the living, dining and kitchen</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr"/>
@@ -10767,7 +10687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11202,39 +11122,39 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Ridge ventilator</t>
+          <t>Gutters and downpipes</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Steel frame bolted to the truss on the main ridge; hipped tiled cap at 30 deg, 1'-6" overhang; 45 deg timber or aluminium louvres with 4 in lap; SS 304 mesh about 1.2 mm (18 x 16) in a sealed continuous frame; 9 in upstand with flashing (no shutters needed: it vents the roof over the open terrace)</t>
+          <t>150 mm half-round gutters with leaf guard on the main and front roofs, 100 mm downpipes at 6 points, to the sump filter, overflow to the road drain</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Lets hot air out, keeps out rain, mosquitoes and attic dust, and closes for AC</t>
+          <t>Short heavy bursts; protects the plinth</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Roof</t>
+          <t>Openings</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Gutters and downpipes</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>150 mm half-round gutters with leaf guard on the main and front roofs, 100 mm downpipes at 6 points, to the sump filter, overflow to the road drain</t>
+          <t>Hardwood or UPVC frames; mosquito mesh on every opening; MS grill for security</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Short heavy bursts; protects the plinth</t>
+          <t>Mosquitoes; ground-floor security</t>
         </is>
       </c>
     </row>
@@ -11246,17 +11166,17 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Windows</t>
+          <t>Sills and sunshades</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Hardwood or UPVC frames; mosquito mesh on every opening; MS grill for security</t>
+          <t>External sills sloped 1:10 with drip groove; 2 ft sunshades with drip groove; 18 in projecting drip under the jali wall</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Mosquitoes; ground-floor security</t>
+          <t>Stops staining and water entry</t>
         </is>
       </c>
     </row>
@@ -11268,17 +11188,17 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Sills and sunshades</t>
+          <t>Vents above inner doors</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>External sills sloped 1:10 with drip groove; 2 ft sunshades with drip groove; 18 in projecting drip under the jali wall</t>
+          <t>Pooja: open jali; bedrooms and bathrooms: none (the workstation has no door for now). 7'-6" to 9'-0" above the lintel band</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Stops staining and water entry</t>
+          <t>Air moves with doors shut where privacy allows; bedrooms rely on their north windows, fans and AC</t>
         </is>
       </c>
     </row>
@@ -11290,39 +11210,39 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Vents above inner doors</t>
+          <t>Bathroom doors</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Pooja: open jali; bedrooms and bathrooms: none (the workstation has no door for now). 7'-6" to 9'-0" above the lintel band</t>
+          <t>WPC / FRP shutters on WPC or granite frame base; no wooden frame touching the wet floor</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Air moves with doors shut where privacy allows; bedrooms rely on their north windows, fans and AC</t>
+          <t>Wood frames rot at the bottom</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Openings</t>
+          <t>Floors</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Bathroom doors</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>WPC / FRP shutters on WPC or granite frame base; no wooden frame touching the wet floor</t>
+          <t>4 in skirting flush with the wall plaster (groove in plaster); 3 mm epoxy grout in wet areas</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Wood frames rot at the bottom</t>
+          <t>No dust ledge, no black grout lines</t>
         </is>
       </c>
     </row>
@@ -11334,39 +11254,39 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Wet rooms</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>4 in skirting flush with the wall plaster (groove in plaster); 3 mm epoxy grout in wet areas</t>
+          <t>Waterproofing (polymer cementitious) floor + 12 in up walls + 7 ft in shower; flood test 48 h before tiling</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>No dust ledge, no black grout lines</t>
+          <t>Leak into neighbouring rooms is the top complaint</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Floors</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Wet rooms</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Waterproofing (polymer cementitious) floor + 12 in up walls + 7 ft in shower; flood test 48 h before tiling</t>
+          <t>CPVC hot/cold; supply runs along external walls in clamps or shallow chases; isolation valve per bathroom and kitchen</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Leak into neighbouring rooms is the top complaint</t>
+          <t>Easy repair without breaking tiles</t>
         </is>
       </c>
     </row>
@@ -11378,17 +11298,17 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Supply</t>
+          <t>Drainage</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>CPVC hot/cold; supply runs along external walls in clamps or shallow chases; isolation valve per bathroom and kitchen</t>
+          <t>uPVC SWR 110 mm soil, 75 mm waste; inspection chamber at every bend and junction; separate soil and grey-water lines</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Easy repair without breaking tiles</t>
+          <t>Easy rodding</t>
         </is>
       </c>
     </row>
@@ -11400,39 +11320,39 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Water treatment</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>uPVC SWR 110 mm soil, 75 mm waste; inspection chamber at every bend and junction; separate soil and grey-water lines</t>
+          <t>RO for drinking at kitchen; whole-house softener if hardness &gt; 300 mg/l; matt fittings</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Easy rodding</t>
+          <t>Guntur groundwater is often hard with high fluoride</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Water treatment</t>
+          <t>Wiring</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>RO for drinking at kitchen; whole-house softener if hardness &gt; 300 mg/l; matt fittings</t>
+          <t>FR-LSH copper; 1.5 sq mm lights, 2.5 sq mm sockets, 4 sq mm AC / geyser; separate circuits per AC</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Guntur groundwater is often hard with high fluoride</t>
+          <t>AC loads</t>
         </is>
       </c>
     </row>
@@ -11444,17 +11364,17 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Wiring</t>
+          <t>Protection</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>FR-LSH copper; 1.5 sq mm lights, 2.5 sq mm sockets, 4 sq mm AC / geyser; separate circuits per AC</t>
+          <t>RCCB 30 mA + MCBs; 2 earth pits; surge protection device; DB in an accessible spot</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>AC loads</t>
+          <t>Shock and lightning safety</t>
         </is>
       </c>
     </row>
@@ -11466,17 +11386,17 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Protection</t>
+          <t>Backup</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>RCCB 30 mA + MCBs; 2 earth pits; surge protection device; DB in an accessible spot</t>
+          <t>Inverter circuit to lights, fans, study sockets and router; conduit from roof to DB for future solar PV</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Shock and lightning safety</t>
+          <t>Power cuts during work-from-home</t>
         </is>
       </c>
     </row>
@@ -11488,37 +11408,15 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Backup</t>
+          <t>AC provisions</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Inverter circuit to lights, fans, study sockets and router; conduit from roof to DB for future solar PV</t>
+          <t>16 A socket at 7 ft, 65 mm sleeve through wall, drain pipe to outside, ODU brackets on shaded walls</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>Power cuts during work-from-home</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>Electrical</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>AC provisions</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>16 A socket at 7 ft, 65 mm sleeve through wall, drain pipe to outside, ODU brackets on shaded walls</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>Retrofitting later means breaking walls</t>
         </is>
@@ -11596,7 +11494,7 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>27.68</v>
+        <v>30.65</v>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
@@ -11656,7 +11554,7 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>7.73</v>
+        <v>7.12</v>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
@@ -11686,7 +11584,7 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>112.3</v>
+        <v>114.5</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
@@ -11806,7 +11704,7 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>28</v>
+        <v>21.4</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
@@ -11815,7 +11713,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Lounge open sides and stair well</t>
+          <t>Terrace open sides and stair well</t>
         </is>
       </c>
       <c r="F9" s="10" t="n"/>
@@ -11836,7 +11734,7 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>352.6</v>
+        <v>355.1</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
@@ -11866,7 +11764,7 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>163.6</v>
+        <v>178.5</v>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
@@ -11896,7 +11794,7 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>37.6</v>
+        <v>47.5</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
@@ -12016,7 +11914,7 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>42.1</v>
+        <v>31.9</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
@@ -12046,7 +11944,7 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>140.7</v>
+        <v>130.4</v>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
@@ -12252,11 +12150,11 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Waterproofing, outdoor lounge slab</t>
+          <t>Waterproofing, covered terrace slab</t>
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>14.1</v>
+        <v>38.9</v>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
@@ -12526,7 +12424,7 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
@@ -12556,7 +12454,7 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
@@ -12586,7 +12484,7 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>25.7</v>
+        <v>26.8</v>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
@@ -12628,7 +12526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G118"/>
+  <dimension ref="A1:G121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -13719,18 +13617,18 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Lobby</t>
+          <t>Stair and passage</t>
         </is>
       </c>
       <c r="E34" s="4" t="n">
         <v>39</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>13.7</v>
+        <v>15.9</v>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>in the under-stair cupboard, lobby side (central, dry)</t>
+          <t>in the under-stair cupboard, facing the lobby (central, dry)</t>
         </is>
       </c>
     </row>
@@ -13752,14 +13650,14 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Lobby</t>
+          <t>Stair and passage</t>
         </is>
       </c>
       <c r="E35" s="4" t="n">
         <v>38</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>13.7</v>
+        <v>15.9</v>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
@@ -13792,7 +13690,7 @@
         <v>40.4</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>14.4</v>
+        <v>16.8</v>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
@@ -15617,7 +15515,7 @@
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>east wall, throws west toward the bed foot</t>
+          <t>east wall, throws west toward the bed foot; 1.5 ton for the whole suite</t>
         </is>
       </c>
     </row>
@@ -16052,20 +15950,16 @@
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>Outdoor lounge (covered)</t>
+          <t>Sitting and study (upper master)</t>
         </is>
       </c>
       <c r="E107" s="4" t="n">
-        <v>29</v>
+        <v>29.5</v>
       </c>
       <c r="F107" s="4" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="G107" s="4" t="inlineStr">
-        <is>
-          <t>wet-rated, under the roof</t>
-        </is>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="G107" s="4" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
@@ -16085,20 +15979,16 @@
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>Outdoor lounge (covered)</t>
+          <t>Sitting and study (upper master)</t>
         </is>
       </c>
       <c r="E108" s="4" t="n">
         <v>26</v>
       </c>
       <c r="F108" s="4" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="G108" s="4" t="inlineStr">
-        <is>
-          <t>wet-rated</t>
-        </is>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="G108" s="4" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
@@ -16118,7 +16008,7 @@
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>Outdoor lounge (covered)</t>
+          <t>Sitting and study (upper master)</t>
         </is>
       </c>
       <c r="E109" s="4" t="n">
@@ -16127,186 +16017,182 @@
       <c r="F109" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="G109" s="4" t="inlineStr">
-        <is>
-          <t>wet-rated</t>
-        </is>
-      </c>
+      <c r="G109" s="4" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Switchboard</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>4'-0"</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>Outdoor lounge (covered)</t>
+          <t>Sitting and study (upper master)</t>
         </is>
       </c>
       <c r="E110" s="4" t="n">
-        <v>34.6</v>
+        <v>30</v>
       </c>
       <c r="F110" s="4" t="n">
-        <v>21</v>
+        <v>16.8</v>
       </c>
       <c r="G110" s="4" t="inlineStr">
         <is>
-          <t>weatherproof</t>
+          <t>sitting zone, at the wardrobe end</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>Switchboard</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>4'-0"</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>Upper passage</t>
+          <t>Sitting and study (upper master)</t>
         </is>
       </c>
       <c r="E111" s="4" t="n">
-        <v>35.4</v>
+        <v>23.4</v>
       </c>
       <c r="F111" s="4" t="n">
-        <v>19.4</v>
+        <v>18.4</v>
       </c>
       <c r="G111" s="4" t="inlineStr">
         <is>
-          <t>lounge switches by the door</t>
+          <t>desk</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>Ceiling fan point</t>
+          <t>Inverter (UPS) socket</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>Covered terrace</t>
+          <t>Sitting and study (upper master)</t>
         </is>
       </c>
       <c r="E112" s="4" t="n">
-        <v>51</v>
+        <v>23.4</v>
       </c>
       <c r="F112" s="4" t="n">
-        <v>19</v>
+        <v>19.4</v>
       </c>
       <c r="G112" s="4" t="inlineStr">
         <is>
-          <t>wet-rated, hung from the steel truss</t>
+          <t>desk</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Data point (Cat6)</t>
         </is>
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>Covered terrace</t>
+          <t>Sitting and study (upper master)</t>
         </is>
       </c>
       <c r="E113" s="4" t="n">
-        <v>49</v>
+        <v>23.4</v>
       </c>
       <c r="F113" s="4" t="n">
-        <v>9</v>
+        <v>20.4</v>
       </c>
       <c r="G113" s="4" t="inlineStr">
         <is>
-          <t>wet-rated</t>
+          <t>desk</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>6 A socket</t>
         </is>
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>1'-0"</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>Covered terrace</t>
+          <t>Sitting and study (upper master)</t>
         </is>
       </c>
       <c r="E114" s="4" t="n">
-        <v>56</v>
+        <v>31.6</v>
       </c>
       <c r="F114" s="4" t="n">
-        <v>9</v>
+        <v>24.6</v>
       </c>
       <c r="G114" s="4" t="inlineStr">
         <is>
-          <t>wet-rated</t>
+          <t>reading chair</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>Ceiling light</t>
+          <t>Ceiling fan point</t>
         </is>
       </c>
       <c r="C115" s="4" t="inlineStr">
@@ -16320,31 +16206,31 @@
         </is>
       </c>
       <c r="E115" s="4" t="n">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="F115" s="4" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G115" s="4" t="inlineStr">
         <is>
-          <t>wet-rated</t>
+          <t>wet-rated, hung from the steel truss</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B116" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
@@ -16353,31 +16239,31 @@
         </is>
       </c>
       <c r="E116" s="4" t="n">
-        <v>45.4</v>
+        <v>49</v>
       </c>
       <c r="F116" s="4" t="n">
-        <v>15.2</v>
+        <v>9</v>
       </c>
       <c r="G116" s="4" t="inlineStr">
         <is>
-          <t>weatherproof</t>
+          <t>wet-rated</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>6 A socket</t>
+          <t>Ceiling light</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>1'-0"</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
@@ -16386,45 +16272,144 @@
         </is>
       </c>
       <c r="E117" s="4" t="n">
-        <v>45.4</v>
+        <v>56</v>
       </c>
       <c r="F117" s="4" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G117" s="4" t="inlineStr">
         <is>
-          <t>weatherproof</t>
+          <t>wet-rated</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t>Ceiling light</t>
+        </is>
+      </c>
+      <c r="C118" s="4" t="inlineStr">
+        <is>
+          <t>ceiling</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="inlineStr">
+        <is>
+          <t>Covered terrace</t>
+        </is>
+      </c>
+      <c r="E118" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="F118" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="G118" s="4" t="inlineStr">
+        <is>
+          <t>wet-rated</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t>6 A socket</t>
+        </is>
+      </c>
+      <c r="C119" s="4" t="inlineStr">
+        <is>
+          <t>1'-0"</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="inlineStr">
+        <is>
+          <t>Covered terrace</t>
+        </is>
+      </c>
+      <c r="E119" s="4" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="F119" s="4" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="G119" s="4" t="inlineStr">
+        <is>
+          <t>weatherproof</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="4" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="B120" s="4" t="inlineStr">
+        <is>
+          <t>6 A socket</t>
+        </is>
+      </c>
+      <c r="C120" s="4" t="inlineStr">
+        <is>
+          <t>1'-0"</t>
+        </is>
+      </c>
+      <c r="D120" s="4" t="inlineStr">
+        <is>
+          <t>Covered terrace</t>
+        </is>
+      </c>
+      <c r="E120" s="4" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="F120" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G120" s="4" t="inlineStr">
+        <is>
+          <t>weatherproof</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="4" t="inlineStr">
+        <is>
           <t>S</t>
         </is>
       </c>
-      <c r="B118" s="4" t="inlineStr">
+      <c r="B121" s="4" t="inlineStr">
         <is>
           <t>Switchboard</t>
         </is>
       </c>
-      <c r="C118" s="4" t="inlineStr">
+      <c r="C121" s="4" t="inlineStr">
         <is>
           <t>4'-0"</t>
         </is>
       </c>
-      <c r="D118" s="4" t="inlineStr">
+      <c r="D121" s="4" t="inlineStr">
         <is>
           <t>Landing</t>
         </is>
       </c>
-      <c r="E118" s="4" t="n">
+      <c r="E121" s="4" t="n">
         <v>44.6</v>
       </c>
-      <c r="F118" s="4" t="n">
+      <c r="F121" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="G118" s="4" t="inlineStr">
+      <c r="G121" s="4" t="inlineStr">
         <is>
           <t>terrace switches by the door, landing side</t>
         </is>

</xml_diff>

<commit_message>
Duplex: house lengthened to 50 ft (bigger bedrooms and baths)
2 ft to the bedrooms (14 ft wide on both floors), 3 ft to the bath strip
(all three baths about 6 x 6'-5" clear, dressing 6 ft, passage 5'-6"),
1 ft to the hall. Front yard unchanged; the trial plot grows to 61 ft.
Design spec rewritten for the current design.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Schedules/KH-P1_Schedules_RevB.xlsx
+++ b/03_Schedules/KH-P1_Schedules_RevB.xlsx
@@ -731,7 +731,7 @@
         </is>
       </c>
       <c r="D2" s="4" t="n">
-        <v>39.4</v>
+        <v>36.4</v>
       </c>
       <c r="E2" s="4" t="n">
         <v>4.9</v>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="D3" s="4" t="n">
-        <v>40.2</v>
+        <v>37.2</v>
       </c>
       <c r="E3" s="4" t="n">
         <v>5.7</v>
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>37</v>
+        <v>34.6</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>9.6</v>
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>35.4</v>
+        <v>31.4</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>4.4</v>
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>36.4</v>
+        <v>32.4</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>3.6</v>
@@ -867,7 +867,7 @@
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>37.8</v>
+        <v>35</v>
       </c>
       <c r="E7" s="4" t="n">
         <v>7.4</v>
@@ -895,7 +895,7 @@
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>41.6</v>
+        <v>38.6</v>
       </c>
       <c r="E8" s="4" t="n">
         <v>6.2</v>
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>40.8</v>
+        <v>37.8</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>6.9</v>
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>44.6</v>
+        <v>43.6</v>
       </c>
       <c r="E10" s="4" t="n">
         <v>8</v>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>44.6</v>
+        <v>43.6</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>4.2</v>
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>43.7</v>
+        <v>42.7</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>3.6</v>
@@ -1031,7 +1031,7 @@
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>42.5</v>
+        <v>41.5</v>
       </c>
       <c r="E13" s="4" t="n">
         <v>8.4</v>
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="D15" s="4" t="n">
-        <v>50.25</v>
+        <v>49.25</v>
       </c>
       <c r="E15" s="4" t="n">
         <v>6.4</v>
@@ -1111,7 +1111,7 @@
         </is>
       </c>
       <c r="D16" s="4" t="n">
-        <v>51.5</v>
+        <v>50.5</v>
       </c>
       <c r="E16" s="4" t="n">
         <v>3.6</v>
@@ -1275,7 +1275,7 @@
         </is>
       </c>
       <c r="D22" s="4" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="E22" s="4" t="n">
         <v>10</v>
@@ -1331,7 +1331,7 @@
         </is>
       </c>
       <c r="D24" s="4" t="n">
-        <v>40.5</v>
+        <v>37.5</v>
       </c>
       <c r="E24" s="4" t="n">
         <v>1.8</v>
@@ -1359,7 +1359,7 @@
         </is>
       </c>
       <c r="D25" s="4" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E25" s="4" t="n">
         <v>1.8</v>
@@ -1387,14 +1387,14 @@
         </is>
       </c>
       <c r="D26" s="4" t="n">
-        <v>21.6</v>
+        <v>15.6</v>
       </c>
       <c r="E26" s="4" t="n">
         <v>1.8</v>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>IC-3 soil bend at the 55 ft line</t>
+          <t>IC-3 soil bend at the 61 ft line</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1443,7 @@
         </is>
       </c>
       <c r="D28" s="4" t="n">
-        <v>51.5</v>
+        <v>50.5</v>
       </c>
       <c r="E28" s="4" t="n">
         <v>1</v>
@@ -1471,7 +1471,7 @@
         </is>
       </c>
       <c r="D29" s="4" t="n">
-        <v>43.7</v>
+        <v>42.7</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>1</v>
@@ -1499,7 +1499,7 @@
         </is>
       </c>
       <c r="D30" s="4" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E30" s="4" t="n">
         <v>1</v>
@@ -1527,7 +1527,7 @@
         </is>
       </c>
       <c r="D31" s="4" t="n">
-        <v>43.9</v>
+        <v>42.9</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>4.6</v>
@@ -1555,7 +1555,7 @@
         </is>
       </c>
       <c r="D32" s="4" t="n">
-        <v>44.6</v>
+        <v>43.6</v>
       </c>
       <c r="E32" s="4" t="n">
         <v>5.4</v>
@@ -1579,7 +1579,7 @@
         </is>
       </c>
       <c r="D33" s="4" t="n">
-        <v>44.6</v>
+        <v>43.6</v>
       </c>
       <c r="E33" s="4" t="n">
         <v>6.4</v>
@@ -1603,7 +1603,7 @@
         </is>
       </c>
       <c r="D34" s="4" t="n">
-        <v>44.6</v>
+        <v>43.6</v>
       </c>
       <c r="E34" s="4" t="n">
         <v>8.800000000000001</v>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="D35" s="4" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>9.4</v>
@@ -1659,7 +1659,7 @@
         </is>
       </c>
       <c r="D36" s="4" t="n">
-        <v>42.5</v>
+        <v>41.5</v>
       </c>
       <c r="E36" s="4" t="n">
         <v>6</v>
@@ -1715,7 +1715,7 @@
         </is>
       </c>
       <c r="D38" s="4" t="n">
-        <v>45.4</v>
+        <v>44.4</v>
       </c>
       <c r="E38" s="4" t="n">
         <v>4.2</v>
@@ -4203,7 +4203,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Duplex trial on the front 55 ft of the plot, back 20 ft spare: decide between this and the single-storey 62 ft plan (main branch) before structural design</t>
+          <t>Duplex trial on the front 61 ft of the plot (house 50 ft), back 14 ft spare: decide between this and the single-storey 62 ft plan (main branch) before structural design</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -4428,7 +4428,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Septic tank and soak pit in the spare rear land (percolation test for the soak pit size); if the back 20 ft is ever sold, move them or switch to a bio-digester with treated outflow</t>
+          <t>Septic tank and soak pit in the spare rear land (percolation test for the soak pit size); if the back 14 ft is ever sold, move them or switch to a bio-digester with treated outflow</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -4628,7 +4628,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Duplex option (branch feature/duplex): the house is planned on the front 55 ft of the plot (the back 20 ft stays spare land) as a 44 ft x 22 ft two-level house, 968 sq ft on the ground floor and about 445 sq ft enclosed on the first floor plus a 16 x 22 ft covered terrace.</t>
+          <t>Duplex option (branch feature/duplex): the house is planned on the front 61 ft of the plot (the back 14 ft stays spare land) as a 50 ft x 22 ft two-level house, 1,100 sq ft on the ground floor and about 505 sq ft enclosed on the first floor plus a 17 x 22 ft covered terrace.</t>
         </is>
       </c>
     </row>
@@ -4638,7 +4638,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>No double height (changed after review): a slab covers the whole two-storey block, so the living, dining, kitchen, pooja, store and wet area all have flat ceilings at about 9'-5" and no dead space above the kitchen. Over the front half the first floor is a covered terrace, opening off the landing, with railings on three sides.</t>
+          <t>House lengthened from 44 to 50 ft (after review: rooms felt small): 2 ft to the bedrooms (both now 14 ft wide), 3 ft to the bath strip (master, common and upper baths about 6 x 6'-5" clear, dressing 6 ft wide, passage to the small bedroom 5'-6"), 1 ft to the dining, living and wet area. Front yard unchanged at 8 ft; the trial plot grows from 55 to 61 ft.No double height (changed after review): a slab covers the whole two-storey block, so the living, dining, kitchen, pooja, store and wet area all have flat ceilings at about 9'-5" and no dead space above the kitchen. Over the front half the first floor is a covered terrace, opening off the landing, with railings on three sides.</t>
         </is>
       </c>
     </row>
@@ -5295,7 +5295,7 @@
         </is>
       </c>
       <c r="D2" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E2" s="4" t="n">
         <v>12.5</v>
@@ -5309,7 +5309,7 @@
         <v/>
       </c>
       <c r="H2" s="5" t="n">
-        <v>11.34</v>
+        <v>13.34</v>
       </c>
       <c r="I2" s="5" t="n">
         <v>11.91</v>
@@ -5347,7 +5347,7 @@
         </is>
       </c>
       <c r="D3" s="4" t="n">
-        <v>5.5</v>
+        <v>6.5</v>
       </c>
       <c r="E3" s="4" t="n">
         <v>7</v>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="H3" s="5" t="n">
-        <v>4.92</v>
+        <v>5.92</v>
       </c>
       <c r="I3" s="5" t="n">
         <v>6.33</v>
@@ -5399,7 +5399,7 @@
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>4.5</v>
+        <v>6.5</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>7</v>
@@ -5413,7 +5413,7 @@
         <v/>
       </c>
       <c r="H4" s="5" t="n">
-        <v>3.92</v>
+        <v>5.92</v>
       </c>
       <c r="I4" s="5" t="n">
         <v>6.33</v>
@@ -5451,7 +5451,7 @@
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>9.5</v>
@@ -5465,7 +5465,7 @@
         <v/>
       </c>
       <c r="H5" s="5" t="n">
-        <v>11.41</v>
+        <v>13.41</v>
       </c>
       <c r="I5" s="5" t="n">
         <v>8.91</v>
@@ -5503,7 +5503,7 @@
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>3.5</v>
@@ -5517,7 +5517,7 @@
         <v/>
       </c>
       <c r="H6" s="5" t="n">
-        <v>9.789999999999999</v>
+        <v>12.79</v>
       </c>
       <c r="I6" s="5" t="n">
         <v>3.21</v>
@@ -5555,7 +5555,7 @@
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E7" s="4" t="n">
         <v>11.5</v>
@@ -5569,7 +5569,7 @@
         <v/>
       </c>
       <c r="H7" s="5" t="n">
-        <v>9.58</v>
+        <v>12.58</v>
       </c>
       <c r="I7" s="5" t="n">
         <v>11.12</v>
@@ -5663,7 +5663,7 @@
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>4.5</v>
@@ -5677,7 +5677,7 @@
         <v/>
       </c>
       <c r="H9" s="5" t="n">
-        <v>5.5</v>
+        <v>6.5</v>
       </c>
       <c r="I9" s="5" t="n">
         <v>3.92</v>
@@ -5715,7 +5715,7 @@
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E10" s="4" t="n">
         <v>5</v>
@@ -5729,7 +5729,7 @@
         <v/>
       </c>
       <c r="H10" s="5" t="n">
-        <v>9.5</v>
+        <v>10.5</v>
       </c>
       <c r="I10" s="5" t="n">
         <v>4.79</v>
@@ -5823,7 +5823,7 @@
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>12.5</v>
@@ -5837,7 +5837,7 @@
         <v/>
       </c>
       <c r="H12" s="5" t="n">
-        <v>15.41</v>
+        <v>16.41</v>
       </c>
       <c r="I12" s="5" t="n">
         <v>11.75</v>
@@ -5987,7 +5987,7 @@
         </is>
       </c>
       <c r="D15" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E15" s="4" t="n">
         <v>12.5</v>
@@ -6001,7 +6001,7 @@
         <v/>
       </c>
       <c r="H15" s="5" t="n">
-        <v>11.41</v>
+        <v>13.41</v>
       </c>
       <c r="I15" s="5" t="n">
         <v>12.12</v>
@@ -6039,7 +6039,7 @@
         </is>
       </c>
       <c r="D16" s="4" t="n">
-        <v>5.5</v>
+        <v>6.5</v>
       </c>
       <c r="E16" s="4" t="n">
         <v>7</v>
@@ -6053,7 +6053,7 @@
         <v/>
       </c>
       <c r="H16" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I16" s="5" t="n">
         <v>6.42</v>
@@ -6091,7 +6091,7 @@
         </is>
       </c>
       <c r="D17" s="4" t="n">
-        <v>4.5</v>
+        <v>6.5</v>
       </c>
       <c r="E17" s="4" t="n">
         <v>7</v>
@@ -6105,7 +6105,7 @@
         <v/>
       </c>
       <c r="H17" s="5" t="n">
-        <v>3.83</v>
+        <v>5.83</v>
       </c>
       <c r="I17" s="5" t="n">
         <v>6.42</v>
@@ -6147,7 +6147,7 @@
         </is>
       </c>
       <c r="D18" s="4" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E18" s="4" t="n">
         <v>4</v>
@@ -6161,7 +6161,7 @@
         <v/>
       </c>
       <c r="H18" s="5" t="n">
-        <v>9.41</v>
+        <v>12.41</v>
       </c>
       <c r="I18" s="5" t="n">
         <v>3.79</v>
@@ -6199,7 +6199,7 @@
         </is>
       </c>
       <c r="D19" s="4" t="n">
-        <v>2.5</v>
+        <v>5.5</v>
       </c>
       <c r="E19" s="4" t="n">
         <v>11</v>
@@ -6213,7 +6213,7 @@
         <v/>
       </c>
       <c r="H19" s="5" t="n">
-        <v>2.29</v>
+        <v>5.29</v>
       </c>
       <c r="I19" s="5" t="n">
         <v>10.62</v>
@@ -6251,7 +6251,7 @@
         </is>
       </c>
       <c r="D20" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E20" s="4" t="n">
         <v>9.5</v>
@@ -6265,7 +6265,7 @@
         <v/>
       </c>
       <c r="H20" s="5" t="n">
-        <v>11.41</v>
+        <v>13.41</v>
       </c>
       <c r="I20" s="5" t="n">
         <v>9.119999999999999</v>
@@ -6307,7 +6307,7 @@
         </is>
       </c>
       <c r="D21" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>22</v>
@@ -6321,7 +6321,7 @@
         <v/>
       </c>
       <c r="H21" s="5" t="n">
-        <v>15.62</v>
+        <v>16.62</v>
       </c>
       <c r="I21" s="5" t="n">
         <v>22</v>
@@ -6374,7 +6374,7 @@
       <c r="L22" s="6" t="inlineStr"/>
       <c r="M22" s="6" t="inlineStr">
         <is>
-          <t>Footprint 44' x 22' = 968 sq ft (ground); first floor about 330 sq ft enclosed + lounge</t>
+          <t>Footprint 50' x 22' = 1,100 sq ft (ground); first floor about 505 sq ft enclosed + 375 sq ft covered terrace</t>
         </is>
       </c>
     </row>
@@ -7026,7 +7026,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>Inside</t>
         </is>
       </c>
       <c r="D2" s="9" t="n">
@@ -7170,7 +7170,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>Inside</t>
         </is>
       </c>
       <c r="D6" s="9" t="n">
@@ -7638,7 +7638,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>Inside</t>
         </is>
       </c>
       <c r="D19" s="9" t="n">
@@ -8567,7 +8567,7 @@
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F19" s="4" t="n">
         <v>2</v>
@@ -8782,7 +8782,7 @@
         </is>
       </c>
       <c r="E24" s="4" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="F24" s="4" t="n">
         <v>1.3</v>
@@ -8825,7 +8825,7 @@
         </is>
       </c>
       <c r="E25" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F25" s="4" t="n">
         <v>1.8</v>
@@ -9547,7 +9547,7 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Built-in wardrobes 4'-8", full height, lofts above (north wall)</t>
+          <t>Built-in wardrobes 5'-10", full height, lofts above (north wall)</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -9556,7 +9556,7 @@
         </is>
       </c>
       <c r="E42" s="4" t="n">
-        <v>4.7</v>
+        <v>5.8</v>
       </c>
       <c r="F42" s="4" t="n">
         <v>1.7</v>
@@ -9728,7 +9728,7 @@
         </is>
       </c>
       <c r="E46" s="4" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="F46" s="4" t="n">
         <v>0.15</v>
@@ -10201,7 +10201,7 @@
         </is>
       </c>
       <c r="E57" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F57" s="4" t="n">
         <v>2.5</v>
@@ -11494,7 +11494,7 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>30.65</v>
+        <v>34.22</v>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
@@ -11524,7 +11524,7 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>4.45</v>
+        <v>4.81</v>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
@@ -11554,7 +11554,7 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>7.12</v>
+        <v>7.6</v>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
@@ -11584,7 +11584,7 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>114.5</v>
+        <v>124</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
@@ -11614,7 +11614,7 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>69.59999999999999</v>
+        <v>81.8</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
@@ -11704,7 +11704,7 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>21.4</v>
+        <v>22</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
@@ -11734,7 +11734,7 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>355.1</v>
+        <v>387.7</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
@@ -11764,7 +11764,7 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>178.5</v>
+        <v>198.6</v>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
@@ -11794,7 +11794,7 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>47.5</v>
+        <v>55.9</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
@@ -11824,7 +11824,7 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>18.8</v>
+        <v>22.1</v>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
@@ -11854,7 +11854,7 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>41.8</v>
+        <v>51.3</v>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
@@ -11914,7 +11914,7 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>31.9</v>
+        <v>34</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
@@ -11944,7 +11944,7 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>130.4</v>
+        <v>142.6</v>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
@@ -11974,7 +11974,7 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>13</v>
+        <v>14.3</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
@@ -12004,7 +12004,7 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
@@ -12034,7 +12034,7 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>11.7</v>
+        <v>14.3</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
@@ -12064,7 +12064,7 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>7.6</v>
+        <v>9.1</v>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
@@ -12094,7 +12094,7 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>11.7</v>
+        <v>14.3</v>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
@@ -12124,7 +12124,7 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>7.5</v>
+        <v>9.1</v>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
@@ -12154,7 +12154,7 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>38.9</v>
+        <v>41.2</v>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
@@ -12244,7 +12244,7 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>133.9</v>
+        <v>150.6</v>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
@@ -12274,7 +12274,7 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>29.3</v>
+        <v>32.9</v>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
@@ -12334,7 +12334,7 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>27.3</v>
+        <v>29.1</v>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
@@ -12394,7 +12394,7 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>41</v>
+        <v>44.3</v>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
@@ -12597,7 +12597,7 @@
         </is>
       </c>
       <c r="E2" s="4" t="n">
-        <v>29.5</v>
+        <v>25.5</v>
       </c>
       <c r="F2" s="4" t="n">
         <v>11</v>
@@ -12630,7 +12630,7 @@
         </is>
       </c>
       <c r="E3" s="4" t="n">
-        <v>25.5</v>
+        <v>19.5</v>
       </c>
       <c r="F3" s="4" t="n">
         <v>12</v>
@@ -12659,7 +12659,7 @@
         </is>
       </c>
       <c r="E4" s="4" t="n">
-        <v>32.5</v>
+        <v>28.5</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>7</v>
@@ -12688,7 +12688,7 @@
         </is>
       </c>
       <c r="E5" s="4" t="n">
-        <v>34.6</v>
+        <v>30.6</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>13.9</v>
@@ -12721,7 +12721,7 @@
         </is>
       </c>
       <c r="E6" s="4" t="n">
-        <v>32.6</v>
+        <v>27.4</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>3.4</v>
@@ -12754,7 +12754,7 @@
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>26.5</v>
+        <v>20.5</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>3.4</v>
@@ -12787,7 +12787,7 @@
         </is>
       </c>
       <c r="E8" s="4" t="n">
-        <v>32.6</v>
+        <v>27</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>3.8</v>
@@ -12820,7 +12820,7 @@
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>30.6</v>
+        <v>26.6</v>
       </c>
       <c r="F9" s="4" t="n">
         <v>15.1</v>
@@ -12853,7 +12853,7 @@
         </is>
       </c>
       <c r="E10" s="4" t="n">
-        <v>23.4</v>
+        <v>17.4</v>
       </c>
       <c r="F10" s="4" t="n">
         <v>12.8</v>
@@ -12886,7 +12886,7 @@
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>22.6</v>
+        <v>16.6</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>13.5</v>
@@ -12919,7 +12919,7 @@
         </is>
       </c>
       <c r="E12" s="4" t="n">
-        <v>37.7</v>
+        <v>34.2</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>6.5</v>
@@ -12948,7 +12948,7 @@
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>39.8</v>
+        <v>36.4</v>
       </c>
       <c r="F13" s="4" t="n">
         <v>3.4</v>
@@ -12981,7 +12981,7 @@
         </is>
       </c>
       <c r="E14" s="4" t="n">
-        <v>35.4</v>
+        <v>31.4</v>
       </c>
       <c r="F14" s="4" t="n">
         <v>5.5</v>
@@ -13014,7 +13014,7 @@
         </is>
       </c>
       <c r="E15" s="4" t="n">
-        <v>38.2</v>
+        <v>35.6</v>
       </c>
       <c r="F15" s="4" t="n">
         <v>9.6</v>
@@ -13047,7 +13047,7 @@
         </is>
       </c>
       <c r="E16" s="4" t="n">
-        <v>34.6</v>
+        <v>30.6</v>
       </c>
       <c r="F16" s="4" t="n">
         <v>9.800000000000001</v>
@@ -13080,7 +13080,7 @@
         </is>
       </c>
       <c r="E17" s="4" t="n">
-        <v>42.7</v>
+        <v>41.7</v>
       </c>
       <c r="F17" s="4" t="n">
         <v>7.2</v>
@@ -13109,7 +13109,7 @@
         </is>
       </c>
       <c r="E18" s="4" t="n">
-        <v>44.6</v>
+        <v>43.6</v>
       </c>
       <c r="F18" s="4" t="n">
         <v>3.4</v>
@@ -13142,7 +13142,7 @@
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>44.6</v>
+        <v>43.6</v>
       </c>
       <c r="F19" s="4" t="n">
         <v>4.6</v>
@@ -13175,7 +13175,7 @@
         </is>
       </c>
       <c r="E20" s="4" t="n">
-        <v>44.6</v>
+        <v>43.6</v>
       </c>
       <c r="F20" s="4" t="n">
         <v>7</v>
@@ -13208,7 +13208,7 @@
         </is>
       </c>
       <c r="E21" s="4" t="n">
-        <v>44.3</v>
+        <v>43.3</v>
       </c>
       <c r="F21" s="4" t="n">
         <v>10.4</v>
@@ -13241,7 +13241,7 @@
         </is>
       </c>
       <c r="E22" s="4" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F22" s="4" t="n">
         <v>20</v>
@@ -13270,7 +13270,7 @@
         </is>
       </c>
       <c r="E23" s="4" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F23" s="4" t="n">
         <v>19</v>
@@ -13299,7 +13299,7 @@
         </is>
       </c>
       <c r="E24" s="4" t="n">
-        <v>31.5</v>
+        <v>27.5</v>
       </c>
       <c r="F24" s="4" t="n">
         <v>23.8</v>
@@ -13328,7 +13328,7 @@
         </is>
       </c>
       <c r="E25" s="4" t="n">
-        <v>34.6</v>
+        <v>30.6</v>
       </c>
       <c r="F25" s="4" t="n">
         <v>19</v>
@@ -13361,7 +13361,7 @@
         </is>
       </c>
       <c r="E26" s="4" t="n">
-        <v>34.6</v>
+        <v>30.6</v>
       </c>
       <c r="F26" s="4" t="n">
         <v>20.1</v>
@@ -13394,7 +13394,7 @@
         </is>
       </c>
       <c r="E27" s="4" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F27" s="4" t="n">
         <v>15.9</v>
@@ -13427,7 +13427,7 @@
         </is>
       </c>
       <c r="E28" s="4" t="n">
-        <v>28.5</v>
+        <v>22.5</v>
       </c>
       <c r="F28" s="4" t="n">
         <v>15.9</v>
@@ -13460,7 +13460,7 @@
         </is>
       </c>
       <c r="E29" s="4" t="n">
-        <v>29.4</v>
+        <v>25.4</v>
       </c>
       <c r="F29" s="4" t="n">
         <v>15.9</v>
@@ -13493,7 +13493,7 @@
         </is>
       </c>
       <c r="E30" s="4" t="n">
-        <v>23.4</v>
+        <v>17.4</v>
       </c>
       <c r="F30" s="4" t="n">
         <v>23</v>
@@ -13526,7 +13526,7 @@
         </is>
       </c>
       <c r="E31" s="4" t="n">
-        <v>22.6</v>
+        <v>16.6</v>
       </c>
       <c r="F31" s="4" t="n">
         <v>22.5</v>
@@ -13559,7 +13559,7 @@
         </is>
       </c>
       <c r="E32" s="4" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F32" s="4" t="n">
         <v>11.8</v>
@@ -13588,7 +13588,7 @@
         </is>
       </c>
       <c r="E33" s="4" t="n">
-        <v>44.6</v>
+        <v>43.6</v>
       </c>
       <c r="F33" s="4" t="n">
         <v>13.6</v>
@@ -13621,7 +13621,7 @@
         </is>
       </c>
       <c r="E34" s="4" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F34" s="4" t="n">
         <v>15.9</v>
@@ -13654,7 +13654,7 @@
         </is>
       </c>
       <c r="E35" s="4" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F35" s="4" t="n">
         <v>15.9</v>
@@ -13687,7 +13687,7 @@
         </is>
       </c>
       <c r="E36" s="4" t="n">
-        <v>40.4</v>
+        <v>39.4</v>
       </c>
       <c r="F36" s="4" t="n">
         <v>16.8</v>
@@ -13720,7 +13720,7 @@
         </is>
       </c>
       <c r="E37" s="4" t="n">
-        <v>41.2</v>
+        <v>40.2</v>
       </c>
       <c r="F37" s="4" t="n">
         <v>24.6</v>
@@ -13753,7 +13753,7 @@
         </is>
       </c>
       <c r="E38" s="4" t="n">
-        <v>36.25</v>
+        <v>32.25</v>
       </c>
       <c r="F38" s="4" t="n">
         <v>15.5</v>
@@ -13786,7 +13786,7 @@
         </is>
       </c>
       <c r="E39" s="4" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F39" s="4" t="n">
         <v>5.8</v>
@@ -13815,7 +13815,7 @@
         </is>
       </c>
       <c r="E40" s="4" t="n">
-        <v>48.6</v>
+        <v>47.6</v>
       </c>
       <c r="F40" s="4" t="n">
         <v>7.9</v>
@@ -13877,7 +13877,7 @@
         </is>
       </c>
       <c r="E42" s="4" t="n">
-        <v>49.3</v>
+        <v>48.3</v>
       </c>
       <c r="F42" s="4" t="n">
         <v>7.2</v>
@@ -13943,7 +13943,7 @@
         </is>
       </c>
       <c r="E44" s="4" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F44" s="4" t="n">
         <v>10</v>
@@ -13976,7 +13976,7 @@
         </is>
       </c>
       <c r="E45" s="4" t="n">
-        <v>45.4</v>
+        <v>44.4</v>
       </c>
       <c r="F45" s="4" t="n">
         <v>9.4</v>
@@ -14542,7 +14542,7 @@
         </is>
       </c>
       <c r="E63" s="4" t="n">
-        <v>49.5</v>
+        <v>48.5</v>
       </c>
       <c r="F63" s="4" t="n">
         <v>22</v>
@@ -14608,7 +14608,7 @@
         </is>
       </c>
       <c r="E65" s="4" t="n">
-        <v>45.4</v>
+        <v>44.4</v>
       </c>
       <c r="F65" s="4" t="n">
         <v>18.9</v>
@@ -14641,7 +14641,7 @@
         </is>
       </c>
       <c r="E66" s="4" t="n">
-        <v>45.4</v>
+        <v>44.4</v>
       </c>
       <c r="F66" s="4" t="n">
         <v>22.4</v>
@@ -14674,7 +14674,7 @@
         </is>
       </c>
       <c r="E67" s="4" t="n">
-        <v>45.4</v>
+        <v>44.4</v>
       </c>
       <c r="F67" s="4" t="n">
         <v>21</v>
@@ -15219,7 +15219,7 @@
         </is>
       </c>
       <c r="E84" s="4" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F84" s="4" t="n">
         <v>8</v>
@@ -15252,7 +15252,7 @@
         </is>
       </c>
       <c r="E85" s="4" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="F85" s="4" t="n">
         <v>8.5</v>
@@ -15285,7 +15285,7 @@
         </is>
       </c>
       <c r="E86" s="4" t="n">
-        <v>25.5</v>
+        <v>19.5</v>
       </c>
       <c r="F86" s="4" t="n">
         <v>13.6</v>
@@ -15314,7 +15314,7 @@
         </is>
       </c>
       <c r="E87" s="4" t="n">
-        <v>32.5</v>
+        <v>28.5</v>
       </c>
       <c r="F87" s="4" t="n">
         <v>7</v>
@@ -15343,7 +15343,7 @@
         </is>
       </c>
       <c r="E88" s="4" t="n">
-        <v>34.6</v>
+        <v>30.6</v>
       </c>
       <c r="F88" s="4" t="n">
         <v>13.9</v>
@@ -15376,7 +15376,7 @@
         </is>
       </c>
       <c r="E89" s="4" t="n">
-        <v>23.4</v>
+        <v>17.4</v>
       </c>
       <c r="F89" s="4" t="n">
         <v>12.9</v>
@@ -15409,7 +15409,7 @@
         </is>
       </c>
       <c r="E90" s="4" t="n">
-        <v>23.4</v>
+        <v>17.4</v>
       </c>
       <c r="F90" s="4" t="n">
         <v>4.2</v>
@@ -15442,7 +15442,7 @@
         </is>
       </c>
       <c r="E91" s="4" t="n">
-        <v>23.4</v>
+        <v>17.4</v>
       </c>
       <c r="F91" s="4" t="n">
         <v>12</v>
@@ -15475,7 +15475,7 @@
         </is>
       </c>
       <c r="E92" s="4" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="F92" s="4" t="n">
         <v>3.4</v>
@@ -15508,7 +15508,7 @@
         </is>
       </c>
       <c r="E93" s="4" t="n">
-        <v>34.6</v>
+        <v>30.6</v>
       </c>
       <c r="F93" s="4" t="n">
         <v>8</v>
@@ -15541,7 +15541,7 @@
         </is>
       </c>
       <c r="E94" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F94" s="4" t="n">
         <v>2.4</v>
@@ -15574,7 +15574,7 @@
         </is>
       </c>
       <c r="E95" s="4" t="n">
-        <v>37.7</v>
+        <v>34.2</v>
       </c>
       <c r="F95" s="4" t="n">
         <v>6.5</v>
@@ -15603,7 +15603,7 @@
         </is>
       </c>
       <c r="E96" s="4" t="n">
-        <v>34.6</v>
+        <v>30.6</v>
       </c>
       <c r="F96" s="4" t="n">
         <v>4.6</v>
@@ -15636,7 +15636,7 @@
         </is>
       </c>
       <c r="E97" s="4" t="n">
-        <v>38.8</v>
+        <v>35.6</v>
       </c>
       <c r="F97" s="4" t="n">
         <v>4.2</v>
@@ -15669,7 +15669,7 @@
         </is>
       </c>
       <c r="E98" s="4" t="n">
-        <v>42.7</v>
+        <v>41.7</v>
       </c>
       <c r="F98" s="4" t="n">
         <v>6</v>
@@ -15698,7 +15698,7 @@
         </is>
       </c>
       <c r="E99" s="4" t="n">
-        <v>44.7</v>
+        <v>43.7</v>
       </c>
       <c r="F99" s="4" t="n">
         <v>3.4</v>
@@ -15731,7 +15731,7 @@
         </is>
       </c>
       <c r="E100" s="4" t="n">
-        <v>44.6</v>
+        <v>43.6</v>
       </c>
       <c r="F100" s="4" t="n">
         <v>8.6</v>
@@ -15764,7 +15764,7 @@
         </is>
       </c>
       <c r="E101" s="4" t="n">
-        <v>44.6</v>
+        <v>43.6</v>
       </c>
       <c r="F101" s="4" t="n">
         <v>6.6</v>
@@ -15797,7 +15797,7 @@
         </is>
       </c>
       <c r="E102" s="4" t="n">
-        <v>40.1</v>
+        <v>37.2</v>
       </c>
       <c r="F102" s="4" t="n">
         <v>6.4</v>
@@ -15830,7 +15830,7 @@
         </is>
       </c>
       <c r="E103" s="4" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F103" s="4" t="n">
         <v>12</v>
@@ -15859,7 +15859,7 @@
         </is>
       </c>
       <c r="E104" s="4" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="F104" s="4" t="n">
         <v>10.4</v>
@@ -15892,7 +15892,7 @@
         </is>
       </c>
       <c r="E105" s="4" t="n">
-        <v>36.25</v>
+        <v>32.25</v>
       </c>
       <c r="F105" s="4" t="n">
         <v>19.5</v>
@@ -15921,7 +15921,7 @@
         </is>
       </c>
       <c r="E106" s="4" t="n">
-        <v>36.25</v>
+        <v>32.25</v>
       </c>
       <c r="F106" s="4" t="n">
         <v>24.6</v>
@@ -15954,7 +15954,7 @@
         </is>
       </c>
       <c r="E107" s="4" t="n">
-        <v>29.5</v>
+        <v>25.5</v>
       </c>
       <c r="F107" s="4" t="n">
         <v>20</v>
@@ -15983,7 +15983,7 @@
         </is>
       </c>
       <c r="E108" s="4" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F108" s="4" t="n">
         <v>19</v>
@@ -16012,7 +16012,7 @@
         </is>
       </c>
       <c r="E109" s="4" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F109" s="4" t="n">
         <v>23</v>
@@ -16041,7 +16041,7 @@
         </is>
       </c>
       <c r="E110" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F110" s="4" t="n">
         <v>16.8</v>
@@ -16074,7 +16074,7 @@
         </is>
       </c>
       <c r="E111" s="4" t="n">
-        <v>23.4</v>
+        <v>17.4</v>
       </c>
       <c r="F111" s="4" t="n">
         <v>18.4</v>
@@ -16107,7 +16107,7 @@
         </is>
       </c>
       <c r="E112" s="4" t="n">
-        <v>23.4</v>
+        <v>17.4</v>
       </c>
       <c r="F112" s="4" t="n">
         <v>19.4</v>
@@ -16140,7 +16140,7 @@
         </is>
       </c>
       <c r="E113" s="4" t="n">
-        <v>23.4</v>
+        <v>17.4</v>
       </c>
       <c r="F113" s="4" t="n">
         <v>20.4</v>
@@ -16173,7 +16173,7 @@
         </is>
       </c>
       <c r="E114" s="4" t="n">
-        <v>31.6</v>
+        <v>27.6</v>
       </c>
       <c r="F114" s="4" t="n">
         <v>24.6</v>
@@ -16206,7 +16206,7 @@
         </is>
       </c>
       <c r="E115" s="4" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F115" s="4" t="n">
         <v>19</v>
@@ -16239,7 +16239,7 @@
         </is>
       </c>
       <c r="E116" s="4" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F116" s="4" t="n">
         <v>9</v>
@@ -16338,7 +16338,7 @@
         </is>
       </c>
       <c r="E119" s="4" t="n">
-        <v>45.4</v>
+        <v>44.4</v>
       </c>
       <c r="F119" s="4" t="n">
         <v>15.2</v>
@@ -16371,7 +16371,7 @@
         </is>
       </c>
       <c r="E120" s="4" t="n">
-        <v>45.4</v>
+        <v>44.4</v>
       </c>
       <c r="F120" s="4" t="n">
         <v>5</v>
@@ -16404,7 +16404,7 @@
         </is>
       </c>
       <c r="E121" s="4" t="n">
-        <v>44.6</v>
+        <v>43.6</v>
       </c>
       <c r="F121" s="4" t="n">
         <v>14</v>

</xml_diff>